<commit_message>
fix: make login test cases universal by removing Non Employee from titles
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -46252,7 +46252,7 @@
       <c r="C2" s="47" t="n"/>
       <c r="D2" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Login Non Employee</t>
+          <t>Membuka halaman Login</t>
         </is>
       </c>
       <c r="E2" s="46" t="inlineStr">
@@ -46309,7 +46309,7 @@
       <c r="C3" s="47" t="n"/>
       <c r="D3" s="48" t="inlineStr">
         <is>
-          <t>Melakukan login Non Employee dengan email dan password valid</t>
+          <t>Melakukan login dengan email dan password valid</t>
         </is>
       </c>
       <c r="E3" s="46" t="inlineStr">
@@ -46374,7 +46374,7 @@
       <c r="C4" s="47" t="n"/>
       <c r="D4" s="48" t="inlineStr">
         <is>
-          <t>Melakukan login Non Employee dengan email tidak terdaftar</t>
+          <t>Melakukan login dengan email tidak terdaftar</t>
         </is>
       </c>
       <c r="E4" s="46" t="inlineStr">
@@ -46439,7 +46439,7 @@
       <c r="C5" s="47" t="n"/>
       <c r="D5" s="48" t="inlineStr">
         <is>
-          <t>Melakukan login Non Employee dengan password salah</t>
+          <t>Melakukan login dengan password salah</t>
         </is>
       </c>
       <c r="E5" s="46" t="inlineStr">

</xml_diff>

<commit_message>
fix(web): rename TC 34.14 to 'Membatalkan approval yang sudah di reject'
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -20745,7 +20745,7 @@
       </c>
       <c r="D458" s="4" t="inlineStr">
         <is>
-          <t>Membatalkan pembatalan approval</t>
+          <t>Membatalkan approval yang sudah di reject</t>
         </is>
       </c>
       <c r="E458" s="3" t="inlineStr">
@@ -20760,13 +20760,13 @@
       </c>
       <c r="G458" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Cancel Approval.
-2. Klik No.</t>
+          <t>1. Klik button Cancel Approval pada data yang berstatus Rejected.
+2. Klik Yes pada pop up konfirmasi.</t>
         </is>
       </c>
       <c r="H458" s="4" t="inlineStr">
         <is>
-          <t>Berhasil status approval tidak berubah.</t>
+          <t>Berhasil membatalkan status Rejected dan status approval kembali menjadi Pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(web-report): adopt Opsi B Kondisi naming for Modul 64 & 69, embed all Modul 64 screenshots
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -36083,7 +36083,7 @@
       </c>
       <c r="D809" s="4" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Menambahkan Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E809" s="3" t="inlineStr">
@@ -36098,16 +36098,16 @@
       </c>
       <c r="G809" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Add Condition pada bagian Performance Indicator.
-2. Mengisi semua field mandatory pada condition baru.
-3. Klik button Submit.</t>
+          <t>1. Klik button + Tambah Kondisi pada bagian Indikator Performa.
+2. Mengisi semua field mandatory pada kondisi baru.
+3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H809" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form condition baru pada Performance Indicator.
-2. Berhasil mengisi field mandatory condition.
-3. Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>1. Berhasil menampilkan form kondisi baru pada Indikator Performa.
+2. Berhasil mengisi field mandatory kondisi.
+3. Berhasil menyimpan kondisi baru pada Indikator Performa.</t>
         </is>
       </c>
     </row>
@@ -36129,7 +36129,7 @@
       </c>
       <c r="D810" s="4" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Menghapus Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E810" s="3" t="inlineStr">
@@ -36144,13 +36144,13 @@
       </c>
       <c r="G810" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Remove pada salah satu condition di Performance Indicator.
-2. Klik button Submit.</t>
+          <t>1. Klik button Hapus pada salah satu kondisi di Indikator Performa.
+2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H810" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menghapus condition dari Performance Indicator.
+          <t>1. Berhasil menghapus kondisi dari Indikator Performa.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
@@ -36173,7 +36173,7 @@
       </c>
       <c r="D811" s="4" t="inlineStr">
         <is>
-          <t>Menambahkan Operator pada Condition di Performance Indicator</t>
+          <t>Menambahkan Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E811" s="3" t="inlineStr">
@@ -36188,14 +36188,14 @@
       </c>
       <c r="G811" s="4" t="inlineStr">
         <is>
-          <t>1. Klik link tambah operator pada salah satu condition di Performance Indicator.
+          <t>1. Klik link tambah operator pada salah satu kondisi di Indikator Performa.
 2. Mengisi field operator baru.
 3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H811" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan baris operator baru pada condition.
+          <t>1. Berhasil menampilkan baris operator baru pada kondisi.
 2. Berhasil mengisi data operator.
 3. Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
@@ -36219,7 +36219,7 @@
       </c>
       <c r="D812" s="4" t="inlineStr">
         <is>
-          <t>Menghapus Operator pada Condition di Performance Indicator</t>
+          <t>Menghapus Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E812" s="3" t="inlineStr">
@@ -36234,13 +36234,13 @@
       </c>
       <c r="G812" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button x pada salah satu operator di Performance Indicator.
+          <t>1. Klik button x pada salah satu operator di Indikator Performa.
 2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H812" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menghapus operator dari condition di Performance Indicator.
+          <t>1. Berhasil menghapus operator dari kondisi di Indikator Performa.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
@@ -37861,7 +37861,7 @@
       </c>
       <c r="D849" s="4" t="inlineStr">
         <is>
-          <t>Menampilkan data Pengaturan Funnel Lending berdasarkan section</t>
+          <t>Mengubah data Pengaturan Funnel Lending</t>
         </is>
       </c>
       <c r="E849" s="3" t="inlineStr">
@@ -37871,17 +37871,19 @@
       </c>
       <c r="F849" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G849" s="4" t="inlineStr">
         <is>
-          <t>1. Klik salah satu daftar section pada tabel.</t>
+          <t>1. Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel.
+2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H849" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data pengaturan funnel Lending.</t>
+          <t>1. Berhasil mengisi field Performance Percentage.
+2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -37903,7 +37905,7 @@
       </c>
       <c r="D850" s="4" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending</t>
+          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E850" s="3" t="inlineStr">
@@ -37918,14 +37920,14 @@
       </c>
       <c r="G850" s="4" t="inlineStr">
         <is>
-          <t>1. Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel.
-2. Klik button Submit.</t>
+          <t>1. Mengosongkan field mandatory Performance Percentage.
+2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H850" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi field Performance Percentage.
-2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
+          <t>1. Berhasil mengosongkan field Performance Percentage.
+2. Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
@@ -37947,7 +37949,7 @@
       </c>
       <c r="D851" s="4" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
+          <t>Menambahkan Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E851" s="3" t="inlineStr">
@@ -37962,14 +37964,16 @@
       </c>
       <c r="G851" s="4" t="inlineStr">
         <is>
-          <t>1. Mengosongkan field mandatory Performance Percentage.
-2. Klik button Submit.</t>
+          <t>1. Klik button + Tambah Kondisi pada bagian Indikator Performa.
+2. Mengisi semua field mandatory pada kondisi baru.
+3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H851" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil mengosongkan field Performance Percentage.
-2. Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>1. Berhasil menampilkan form kondisi baru pada Indikator Performa.
+2. Berhasil mengisi field mandatory kondisi.
+3. Berhasil menyimpan kondisi baru pada Indikator Performa.</t>
         </is>
       </c>
     </row>
@@ -37991,7 +37995,7 @@
       </c>
       <c r="D852" s="4" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Menghapus Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E852" s="3" t="inlineStr">
@@ -38006,16 +38010,14 @@
       </c>
       <c r="G852" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Add Condition pada bagian Performance Indicator.
-2. Mengisi semua field mandatory pada condition baru.
-3. Klik button Submit.</t>
+          <t>1. Klik button Hapus pada salah satu kondisi di Indikator Performa.
+2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H852" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form condition baru pada Performance Indicator.
-2. Berhasil mengisi field mandatory condition.
-3. Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>1. Berhasil menghapus kondisi dari Indikator Performa.
+2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -38037,7 +38039,7 @@
       </c>
       <c r="D853" s="4" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
+          <t>Menambahkan Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E853" s="3" t="inlineStr">
@@ -38052,16 +38054,16 @@
       </c>
       <c r="G853" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Add Condition pada bagian Performance Indicator.
-2. Mengosongkan field mandatory pada condition baru.
-3. Klik button Submit.</t>
+          <t>1. Klik link tambah operator pada salah satu kondisi di Indikator Performa.
+2. Mengisi field operator baru.
+3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H853" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form condition baru pada Performance Indicator.
-2. Berhasil mengosongkan field mandatory condition.
-3. Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>1. Berhasil menampilkan baris operator baru pada kondisi.
+2. Berhasil mengisi data operator.
+3. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -38083,7 +38085,7 @@
       </c>
       <c r="D854" s="4" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Menghapus Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E854" s="3" t="inlineStr">
@@ -38098,13 +38100,13 @@
       </c>
       <c r="G854" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Remove pada salah satu condition di Performance Indicator.
-2. Klik button Submit.</t>
+          <t>1. Klik button x pada salah satu operator di Indikator Performa.
+2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
       <c r="H854" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menghapus condition dari Performance Indicator.
+          <t>1. Berhasil menghapus operator dari kondisi di Indikator Performa.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat(web-report): add TC 65.2 for tab Non PKS & PKS and renumber Modul 65
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z909"/>
+  <dimension ref="A1:Z910"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -37073,509 +37073,553 @@
       </c>
       <c r="D831" s="4" t="inlineStr">
         <is>
+          <t>Menampilkan data tab Non PKS dan PKS</t>
+        </is>
+      </c>
+      <c r="E831" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F831" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G831" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik tab Non PKS.
+2. Klik tab PKS.</t>
+        </is>
+      </c>
+      <c r="H831" s="4" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan data pada tab Non PKS.
+2. Berhasil menampilkan data pada tab PKS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="832" ht="28" customHeight="1">
+      <c r="A832" s="43" t="inlineStr">
+        <is>
+          <t>65.3</t>
+        </is>
+      </c>
+      <c r="B832" s="3" t="inlineStr">
+        <is>
+          <t>Report Lending</t>
+        </is>
+      </c>
+      <c r="C832" s="3" t="inlineStr">
+        <is>
+          <t>Personal Funnel</t>
+        </is>
+      </c>
+      <c r="D832" s="4" t="inlineStr">
+        <is>
           <t>Melakukan filter data Personal Funnel</t>
         </is>
       </c>
-      <c r="E831" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F831" s="3" t="inlineStr">
+      <c r="E832" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F832" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G831" s="4" t="inlineStr">
+      <c r="G832" s="4" t="inlineStr">
         <is>
           <t>1. Mengisi semua field filter mandatory.
 2. Klik button Submit.</t>
         </is>
       </c>
-      <c r="H831" s="4" t="inlineStr">
+      <c r="H832" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field filter mandatory.
 2. Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="832" ht="28" customHeight="1">
-      <c r="A832" s="43" t="inlineStr">
-        <is>
-          <t>65.3</t>
-        </is>
-      </c>
-      <c r="B832" s="3" t="inlineStr">
+    <row r="833" ht="14" customHeight="1">
+      <c r="A833" s="43" t="inlineStr">
+        <is>
+          <t>65.4</t>
+        </is>
+      </c>
+      <c r="B833" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C832" s="3" t="inlineStr">
+      <c r="C833" s="3" t="inlineStr">
         <is>
           <t>Personal Funnel</t>
         </is>
       </c>
-      <c r="D832" s="4" t="inlineStr">
+      <c r="D833" s="4" t="inlineStr">
         <is>
           <t>Melakukan filter data Personal Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
-      <c r="E832" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F832" s="3" t="inlineStr">
+      <c r="E833" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F833" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G832" s="4" t="inlineStr">
+      <c r="G833" s="4" t="inlineStr">
         <is>
           <t>1. Mengosongkan field filter mandatory.
 2. Klik button Submit.</t>
         </is>
       </c>
-      <c r="H832" s="4" t="inlineStr">
+      <c r="H833" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan field filter mandatory.
 2. Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
-    <row r="833" ht="14" customHeight="1">
-      <c r="A833" s="43" t="inlineStr">
-        <is>
-          <t>65.4</t>
-        </is>
-      </c>
-      <c r="B833" s="3" t="inlineStr">
+    <row r="834" ht="14" customHeight="1">
+      <c r="A834" s="43" t="inlineStr">
+        <is>
+          <t>65.5</t>
+        </is>
+      </c>
+      <c r="B834" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C833" s="3" t="inlineStr">
+      <c r="C834" s="3" t="inlineStr">
         <is>
           <t>Personal Funnel</t>
         </is>
       </c>
-      <c r="D833" s="4" t="inlineStr">
+      <c r="D834" s="4" t="inlineStr">
         <is>
           <t>Mengekspor data Personal Funnel</t>
         </is>
       </c>
-      <c r="E833" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F833" s="3" t="inlineStr">
+      <c r="E834" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F834" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G833" s="4" t="inlineStr">
+      <c r="G834" s="4" t="inlineStr">
         <is>
           <t>1. Klik button Export.
 2. Klik icon download pada panel Download Export.</t>
         </is>
       </c>
-      <c r="H833" s="4" t="inlineStr">
+      <c r="H834" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan panel Download Export.
 2. Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
-    <row r="834" ht="14" customHeight="1">
-      <c r="A834" s="43" t="inlineStr">
+    <row r="835" ht="14" customHeight="1">
+      <c r="A835" s="43" t="inlineStr">
         <is>
           <t>66.1</t>
         </is>
       </c>
-      <c r="B834" s="3" t="inlineStr">
+      <c r="B835" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C834" s="3" t="inlineStr">
+      <c r="C835" s="3" t="inlineStr">
         <is>
           <t>Rekap Funnel</t>
         </is>
       </c>
-      <c r="D834" s="4" t="inlineStr">
+      <c r="D835" s="4" t="inlineStr">
         <is>
           <t>Membuka halaman Rekap Funnel</t>
         </is>
       </c>
-      <c r="E834" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F834" s="3" t="inlineStr">
+      <c r="E835" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F835" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G834" s="4" t="inlineStr">
+      <c r="G835" s="4" t="inlineStr">
         <is>
           <t>1. Klik menu Report Lending.
 2. Klik sub menu Rekap Funnel.</t>
         </is>
       </c>
-      <c r="H834" s="4" t="inlineStr">
+      <c r="H835" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu Report Lending.
 2. Berhasil menampilkan halaman Rekap Funnel.</t>
         </is>
       </c>
     </row>
-    <row r="835" ht="14" customHeight="1">
-      <c r="A835" s="43" t="inlineStr">
+    <row r="836" ht="42" customHeight="1">
+      <c r="A836" s="43" t="inlineStr">
         <is>
           <t>66.2</t>
         </is>
       </c>
-      <c r="B835" s="3" t="inlineStr">
+      <c r="B836" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C835" s="3" t="inlineStr">
+      <c r="C836" s="3" t="inlineStr">
         <is>
           <t>Rekap Funnel</t>
         </is>
       </c>
-      <c r="D835" s="4" t="inlineStr">
+      <c r="D836" s="4" t="inlineStr">
         <is>
           <t>Menampilkan data Rekap Funnel</t>
         </is>
       </c>
-      <c r="E835" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F835" s="3" t="inlineStr">
+      <c r="E836" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F836" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G835" s="4" t="inlineStr">
+      <c r="G836" s="4" t="inlineStr">
         <is>
           <t>1. Mengisi field filter mandatory (Kantor Wilayah, Unit Bisnis, Produk, Info Bulan, Info Tahun).
 2. Klik button Filter Data.</t>
         </is>
       </c>
-      <c r="H835" s="4" t="inlineStr">
+      <c r="H836" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field filter mandatory.
 2. Berhasil menampilkan daftar data Rekap Funnel di dalam tabel.</t>
         </is>
       </c>
     </row>
-    <row r="836" ht="42" customHeight="1">
-      <c r="A836" s="43" t="inlineStr">
+    <row r="837" ht="28" customHeight="1">
+      <c r="A837" s="43" t="inlineStr">
         <is>
           <t>66.3</t>
         </is>
       </c>
-      <c r="B836" s="3" t="inlineStr">
+      <c r="B837" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C836" s="3" t="inlineStr">
+      <c r="C837" s="3" t="inlineStr">
         <is>
           <t>Rekap Funnel</t>
         </is>
       </c>
-      <c r="D836" s="4" t="inlineStr">
+      <c r="D837" s="4" t="inlineStr">
         <is>
           <t>Melakukan filter data Rekap Funnel</t>
         </is>
       </c>
-      <c r="E836" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F836" s="3" t="inlineStr">
+      <c r="E837" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F837" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G836" s="4" t="inlineStr">
+      <c r="G837" s="4" t="inlineStr">
         <is>
           <t>1. Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role).
 2. Klik button Filter Data.</t>
         </is>
       </c>
-      <c r="H836" s="4" t="inlineStr">
+      <c r="H837" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi kriteria filter.
 2. Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="837" ht="28" customHeight="1">
-      <c r="A837" s="43" t="inlineStr">
+    <row r="838" ht="28" customHeight="1">
+      <c r="A838" s="43" t="inlineStr">
         <is>
           <t>66.4</t>
         </is>
       </c>
-      <c r="B837" s="3" t="inlineStr">
+      <c r="B838" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C837" s="3" t="inlineStr">
+      <c r="C838" s="3" t="inlineStr">
         <is>
           <t>Rekap Funnel</t>
         </is>
       </c>
-      <c r="D837" s="4" t="inlineStr">
+      <c r="D838" s="4" t="inlineStr">
         <is>
           <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
-      <c r="E837" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F837" s="3" t="inlineStr">
+      <c r="E838" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F838" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G837" s="4" t="inlineStr">
+      <c r="G838" s="4" t="inlineStr">
         <is>
           <t>1. Mengosongkan field filter mandatory.
 2. Klik button Filter Data.</t>
         </is>
       </c>
-      <c r="H837" s="4" t="inlineStr">
+      <c r="H838" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan field filter mandatory.
 2. Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
-    <row r="838" ht="28" customHeight="1">
-      <c r="A838" s="43" t="inlineStr">
-        <is>
-          <t>66.5</t>
-        </is>
-      </c>
-      <c r="B838" s="3" t="inlineStr">
-        <is>
-          <t>Report Lending</t>
-        </is>
-      </c>
-      <c r="C838" s="3" t="inlineStr">
-        <is>
-          <t>Rekap Funnel</t>
-        </is>
-      </c>
-      <c r="D838" s="4" t="inlineStr">
-        <is>
-          <t>Mengunduh data Rekap Funnel</t>
-        </is>
-      </c>
-      <c r="E838" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F838" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G838" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik button Download Excel.</t>
-        </is>
-      </c>
-      <c r="H838" s="4" t="inlineStr">
-        <is>
-          <t>1. Berhasil mendownload file Excel data Rekap Funnel.</t>
-        </is>
-      </c>
-    </row>
     <row r="839" ht="70" customHeight="1">
       <c r="A839" s="43" t="inlineStr">
         <is>
+          <t>66.5</t>
+        </is>
+      </c>
+      <c r="B839" s="3" t="inlineStr">
+        <is>
+          <t>Report Lending</t>
+        </is>
+      </c>
+      <c r="C839" s="3" t="inlineStr">
+        <is>
+          <t>Rekap Funnel</t>
+        </is>
+      </c>
+      <c r="D839" s="4" t="inlineStr">
+        <is>
+          <t>Mengunduh data Rekap Funnel</t>
+        </is>
+      </c>
+      <c r="E839" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F839" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G839" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik button Download Excel.</t>
+        </is>
+      </c>
+      <c r="H839" s="4" t="inlineStr">
+        <is>
+          <t>1. Berhasil mendownload file Excel data Rekap Funnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="840" ht="28" customHeight="1">
+      <c r="A840" s="43" t="inlineStr">
+        <is>
           <t>67.1</t>
         </is>
       </c>
-      <c r="B839" s="3" t="inlineStr">
+      <c r="B840" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C839" s="3" t="inlineStr">
+      <c r="C840" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D839" s="4" t="inlineStr">
+      <c r="D840" s="4" t="inlineStr">
         <is>
           <t>Membuka halaman Pengaturan Funnel Lending</t>
         </is>
       </c>
-      <c r="E839" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F839" s="3" t="inlineStr">
+      <c r="E840" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F840" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G839" s="4" t="inlineStr">
+      <c r="G840" s="4" t="inlineStr">
         <is>
           <t>1. Klik menu Report Lending.
 2. Klik sub menu Pengaturan Funnel.</t>
         </is>
       </c>
-      <c r="H839" s="4" t="inlineStr">
+      <c r="H840" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu Report Lending.
 2. Berhasil menampilkan halaman Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
-    <row r="840" ht="28" customHeight="1">
-      <c r="A840" s="43" t="inlineStr">
+    <row r="841" ht="84" customHeight="1">
+      <c r="A841" s="43" t="inlineStr">
         <is>
           <t>67.2</t>
         </is>
       </c>
-      <c r="B840" s="3" t="inlineStr">
+      <c r="B841" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C840" s="3" t="inlineStr">
+      <c r="C841" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D840" s="4" t="inlineStr">
+      <c r="D841" s="4" t="inlineStr">
         <is>
           <t>Mengubah data Pengaturan Funnel Lending</t>
         </is>
       </c>
-      <c r="E840" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F840" s="3" t="inlineStr">
+      <c r="E841" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F841" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G840" s="4" t="inlineStr">
+      <c r="G841" s="4" t="inlineStr">
         <is>
           <t>1. Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel.
 2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H840" s="4" t="inlineStr">
+      <c r="H841" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field Performance Percentage.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
-    <row r="841" ht="84" customHeight="1">
-      <c r="A841" s="43" t="inlineStr">
+    <row r="842" ht="28" customHeight="1">
+      <c r="A842" s="43" t="inlineStr">
         <is>
           <t>67.3</t>
         </is>
       </c>
-      <c r="B841" s="3" t="inlineStr">
+      <c r="B842" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C841" s="3" t="inlineStr">
+      <c r="C842" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D841" s="4" t="inlineStr">
+      <c r="D842" s="4" t="inlineStr">
         <is>
           <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
         </is>
       </c>
-      <c r="E841" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F841" s="3" t="inlineStr">
+      <c r="E842" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F842" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G841" s="4" t="inlineStr">
+      <c r="G842" s="4" t="inlineStr">
         <is>
           <t>1. Mengosongkan field mandatory Performance Percentage.
 2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H841" s="4" t="inlineStr">
+      <c r="H842" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan field Performance Percentage.
 2. Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
-    <row r="842" ht="28" customHeight="1">
-      <c r="A842" s="43" t="inlineStr">
+    <row r="843" ht="28" customHeight="1">
+      <c r="A843" s="43" t="inlineStr">
         <is>
           <t>67.4</t>
         </is>
       </c>
-      <c r="B842" s="3" t="inlineStr">
+      <c r="B843" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C842" s="3" t="inlineStr">
+      <c r="C843" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D842" s="4" t="inlineStr">
+      <c r="D843" s="4" t="inlineStr">
         <is>
           <t>Menambahkan Kondisi pada Indikator Performa</t>
         </is>
       </c>
-      <c r="E842" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F842" s="3" t="inlineStr">
+      <c r="E843" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F843" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G842" s="4" t="inlineStr">
+      <c r="G843" s="4" t="inlineStr">
         <is>
           <t>1. Klik button + Tambah Kondisi pada bagian Indikator Performa.
 2. Mengisi semua field mandatory pada kondisi baru.
 3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H842" s="4" t="inlineStr">
+      <c r="H843" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan form kondisi baru pada Indikator Performa.
 2. Berhasil mengisi field mandatory kondisi.
@@ -37583,89 +37627,89 @@
         </is>
       </c>
     </row>
-    <row r="843" ht="28" customHeight="1">
-      <c r="A843" s="43" t="inlineStr">
+    <row r="844" ht="28" customHeight="1">
+      <c r="A844" s="43" t="inlineStr">
         <is>
           <t>67.5</t>
         </is>
       </c>
-      <c r="B843" s="3" t="inlineStr">
+      <c r="B844" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C843" s="3" t="inlineStr">
+      <c r="C844" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D843" s="4" t="inlineStr">
+      <c r="D844" s="4" t="inlineStr">
         <is>
           <t>Menghapus Kondisi pada Indikator Performa</t>
         </is>
       </c>
-      <c r="E843" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F843" s="3" t="inlineStr">
+      <c r="E844" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F844" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G843" s="4" t="inlineStr">
+      <c r="G844" s="4" t="inlineStr">
         <is>
           <t>1. Klik button Hapus pada salah satu kondisi di Indikator Performa.
 2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H843" s="4" t="inlineStr">
+      <c r="H844" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menghapus kondisi dari Indikator Performa.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
-    <row r="844" ht="28" customHeight="1">
-      <c r="A844" s="43" t="inlineStr">
+    <row r="845" ht="42" customHeight="1">
+      <c r="A845" s="43" t="inlineStr">
         <is>
           <t>67.6</t>
         </is>
       </c>
-      <c r="B844" s="3" t="inlineStr">
+      <c r="B845" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C844" s="3" t="inlineStr">
+      <c r="C845" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D844" s="4" t="inlineStr">
+      <c r="D845" s="4" t="inlineStr">
         <is>
           <t>Menambahkan Operator pada Kondisi</t>
         </is>
       </c>
-      <c r="E844" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F844" s="3" t="inlineStr">
+      <c r="E845" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F845" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G844" s="4" t="inlineStr">
+      <c r="G845" s="4" t="inlineStr">
         <is>
           <t>1. Klik link tambah operator pada salah satu kondisi di Indikator Performa.
 2. Mengisi field operator baru.
 3. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H844" s="4" t="inlineStr">
+      <c r="H845" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan baris operator baru pada kondisi.
 2. Berhasil mengisi data operator.
@@ -37673,170 +37717,170 @@
         </is>
       </c>
     </row>
-    <row r="845" ht="42" customHeight="1">
-      <c r="A845" s="43" t="inlineStr">
+    <row r="846" ht="28" customHeight="1">
+      <c r="A846" s="43" t="inlineStr">
         <is>
           <t>67.7</t>
         </is>
       </c>
-      <c r="B845" s="3" t="inlineStr">
+      <c r="B846" s="3" t="inlineStr">
         <is>
           <t>Report Lending</t>
         </is>
       </c>
-      <c r="C845" s="3" t="inlineStr">
+      <c r="C846" s="3" t="inlineStr">
         <is>
           <t>Pengaturan Funnel</t>
         </is>
       </c>
-      <c r="D845" s="4" t="inlineStr">
+      <c r="D846" s="4" t="inlineStr">
         <is>
           <t>Menghapus Operator pada Kondisi</t>
         </is>
       </c>
-      <c r="E845" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F845" s="3" t="inlineStr">
+      <c r="E846" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F846" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G845" s="4" t="inlineStr">
+      <c r="G846" s="4" t="inlineStr">
         <is>
           <t>1. Klik button x pada salah satu operator di Indikator Performa.
 2. Klik button Simpan Pengaturan.</t>
         </is>
       </c>
-      <c r="H845" s="4" t="inlineStr">
+      <c r="H846" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menghapus operator dari kondisi di Indikator Performa.
 2. Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
-    <row r="846" ht="28" customHeight="1">
-      <c r="A846" s="43" t="inlineStr">
+    <row r="847" ht="14" customHeight="1">
+      <c r="A847" s="43" t="inlineStr">
         <is>
           <t>68.1</t>
         </is>
       </c>
-      <c r="B846" s="3" t="inlineStr">
+      <c r="B847" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C846" s="3" t="inlineStr">
+      <c r="C847" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D846" s="4" t="inlineStr">
+      <c r="D847" s="4" t="inlineStr">
         <is>
           <t>Membuka halaman Approval non Banking</t>
         </is>
       </c>
-      <c r="E846" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F846" s="3" t="inlineStr">
+      <c r="E847" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F847" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G846" s="4" t="inlineStr">
+      <c r="G847" s="4" t="inlineStr">
         <is>
           <t>1. Klik menu Re-Assign &amp; Approval 
 2. Klik submenu Approval non banking</t>
         </is>
       </c>
-      <c r="H846" s="4" t="inlineStr">
+      <c r="H847" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan submenu Re-Assign &amp; Approval 
 2. Menampilkan halaman Approval non banking</t>
         </is>
       </c>
     </row>
-    <row r="847" ht="14" customHeight="1">
-      <c r="A847" s="43" t="inlineStr">
+    <row r="848" ht="14" customHeight="1">
+      <c r="A848" s="43" t="inlineStr">
         <is>
           <t>68.2</t>
         </is>
       </c>
-      <c r="B847" s="3" t="inlineStr">
+      <c r="B848" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C847" s="3" t="inlineStr">
+      <c r="C848" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D847" s="4" t="inlineStr">
+      <c r="D848" s="4" t="inlineStr">
         <is>
           <t>Melihat Detail data Approval non banking</t>
         </is>
       </c>
-      <c r="E847" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F847" s="3" t="inlineStr">
+      <c r="E848" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F848" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G847" s="4" t="inlineStr">
+      <c r="G848" s="4" t="inlineStr">
         <is>
           <t>1. Klik titik tiga 
 2. Klik Detail</t>
         </is>
       </c>
-      <c r="H847" s="4" t="inlineStr">
+      <c r="H848" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan beberapa action (detail, setujui, tolak)
 2. Menampilkan halaman detail data approval non banking</t>
         </is>
       </c>
     </row>
-    <row r="848" ht="14" customHeight="1">
-      <c r="A848" s="43" t="inlineStr">
+    <row r="849" ht="42" customHeight="1">
+      <c r="A849" s="43" t="inlineStr">
         <is>
           <t>68.3</t>
         </is>
       </c>
-      <c r="B848" s="3" t="inlineStr">
+      <c r="B849" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C848" s="3" t="inlineStr">
+      <c r="C849" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D848" s="4" t="inlineStr">
+      <c r="D849" s="4" t="inlineStr">
         <is>
           <t>Menyetujui Prospek</t>
         </is>
       </c>
-      <c r="E848" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F848" s="3" t="inlineStr">
+      <c r="E849" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F849" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G848" s="4" t="inlineStr">
+      <c r="G849" s="4" t="inlineStr">
         <is>
           <t>1. Klik titik tiga 
 2. Klik Setujui 
@@ -37845,7 +37889,7 @@
 5. Klik button Setujui</t>
         </is>
       </c>
-      <c r="H848" s="4" t="inlineStr">
+      <c r="H849" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan beberapa action (detail, setujui, tolak)
 2. Menampilkan modal approve 
@@ -37855,87 +37899,87 @@
         </is>
       </c>
     </row>
-    <row r="849" ht="42" customHeight="1">
-      <c r="A849" s="43" t="inlineStr">
-        <is>
-          <t>68.4</t>
-        </is>
-      </c>
-      <c r="B849" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C849" s="3" t="inlineStr">
-        <is>
-          <t>Approval Non Banking</t>
-        </is>
-      </c>
-      <c r="D849" s="4" t="inlineStr">
-        <is>
-          <t>Batal menyetujui Prospek</t>
-        </is>
-      </c>
-      <c r="E849" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F849" s="3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G849" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik button Batalkan pada modal approve</t>
-        </is>
-      </c>
-      <c r="H849" s="4" t="inlineStr">
-        <is>
-          <t>1. Modal approve tertutup dan tetap di halaman approval non banking</t>
-        </is>
-      </c>
-    </row>
     <row r="850" ht="28" customHeight="1">
       <c r="A850" s="43" t="inlineStr">
         <is>
+          <t>68.4</t>
+        </is>
+      </c>
+      <c r="B850" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C850" s="3" t="inlineStr">
+        <is>
+          <t>Approval Non Banking</t>
+        </is>
+      </c>
+      <c r="D850" s="4" t="inlineStr">
+        <is>
+          <t>Batal menyetujui Prospek</t>
+        </is>
+      </c>
+      <c r="E850" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F850" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G850" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik button Batalkan pada modal approve</t>
+        </is>
+      </c>
+      <c r="H850" s="4" t="inlineStr">
+        <is>
+          <t>1. Modal approve tertutup dan tetap di halaman approval non banking</t>
+        </is>
+      </c>
+    </row>
+    <row r="851" ht="28" customHeight="1">
+      <c r="A851" s="43" t="inlineStr">
+        <is>
           <t>68.5</t>
         </is>
       </c>
-      <c r="B850" s="3" t="inlineStr">
+      <c r="B851" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C850" s="3" t="inlineStr">
+      <c r="C851" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D850" s="4" t="inlineStr">
+      <c r="D851" s="4" t="inlineStr">
         <is>
           <t>Tidak menginput nilai realisasi pada modal approve</t>
         </is>
       </c>
-      <c r="E850" s="3" t="inlineStr">
+      <c r="E851" s="3" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F850" s="3" t="inlineStr">
+      <c r="F851" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G850" s="4" t="inlineStr">
+      <c r="G851" s="4" t="inlineStr">
         <is>
           <t>1. Kosongkan nilai realisasi 
 2. Input remark 
 3. Klik button Setujui</t>
         </is>
       </c>
-      <c r="H850" s="4" t="inlineStr">
+      <c r="H851" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan field realisasi 
 2. Berhasil menginput remark 
@@ -37943,52 +37987,10 @@
         </is>
       </c>
     </row>
-    <row r="851" ht="28" customHeight="1">
-      <c r="A851" s="43" t="inlineStr">
-        <is>
-          <t>68.6</t>
-        </is>
-      </c>
-      <c r="B851" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C851" s="3" t="inlineStr">
-        <is>
-          <t>Approval Non Banking</t>
-        </is>
-      </c>
-      <c r="D851" s="4" t="inlineStr">
-        <is>
-          <t>Tidak menginput remark pada modal approve</t>
-        </is>
-      </c>
-      <c r="E851" s="3" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F851" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G851" s="4" t="inlineStr">
-        <is>
-          <t>1. Kosongkan remark</t>
-        </is>
-      </c>
-      <c r="H851" s="4" t="inlineStr">
-        <is>
-          <t>1. Menampilkan alert 'Remark dibutuhkan!'</t>
-        </is>
-      </c>
-    </row>
     <row r="852" ht="28" customHeight="1">
       <c r="A852" s="43" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>68.6</t>
         </is>
       </c>
       <c r="B852" s="3" t="inlineStr">
@@ -38003,7 +38005,7 @@
       </c>
       <c r="D852" s="4" t="inlineStr">
         <is>
-          <t>Menginput huruf pada field realisasi</t>
+          <t>Tidak menginput remark pada modal approve</t>
         </is>
       </c>
       <c r="E852" s="3" t="inlineStr">
@@ -38013,52 +38015,94 @@
       </c>
       <c r="F852" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G852" s="4" t="inlineStr">
         <is>
-          <t>1. Input huruf pada field realisasi kemudian pindah ke filed lain</t>
+          <t>1. Kosongkan remark</t>
         </is>
       </c>
       <c r="H852" s="4" t="inlineStr">
         <is>
-          <t>1. Sistem menghapus input non-numerik secara otomatis saat field kehilangan fokus. Field Realiasi menjadi kosong</t>
+          <t>1. Menampilkan alert 'Remark dibutuhkan!'</t>
         </is>
       </c>
     </row>
     <row r="853" ht="28" customHeight="1">
       <c r="A853" s="43" t="inlineStr">
         <is>
+          <t>68.7</t>
+        </is>
+      </c>
+      <c r="B853" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C853" s="3" t="inlineStr">
+        <is>
+          <t>Approval Non Banking</t>
+        </is>
+      </c>
+      <c r="D853" s="4" t="inlineStr">
+        <is>
+          <t>Menginput huruf pada field realisasi</t>
+        </is>
+      </c>
+      <c r="E853" s="3" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F853" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G853" s="4" t="inlineStr">
+        <is>
+          <t>1. Input huruf pada field realisasi kemudian pindah ke filed lain</t>
+        </is>
+      </c>
+      <c r="H853" s="4" t="inlineStr">
+        <is>
+          <t>1. Sistem menghapus input non-numerik secara otomatis saat field kehilangan fokus. Field Realiasi menjadi kosong</t>
+        </is>
+      </c>
+    </row>
+    <row r="854" ht="28" customHeight="1">
+      <c r="A854" s="43" t="inlineStr">
+        <is>
           <t>68.8</t>
         </is>
       </c>
-      <c r="B853" s="3" t="inlineStr">
+      <c r="B854" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C853" s="3" t="inlineStr">
+      <c r="C854" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D853" s="4" t="inlineStr">
+      <c r="D854" s="4" t="inlineStr">
         <is>
           <t>Menolak Prospek</t>
         </is>
       </c>
-      <c r="E853" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F853" s="3" t="inlineStr">
+      <c r="E854" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F854" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G853" s="4" t="inlineStr">
+      <c r="G854" s="4" t="inlineStr">
         <is>
           <t>1. Klik titik tiga 
 2. Klik Tolak 
@@ -38066,7 +38110,7 @@
 4. Klik button Tolak</t>
         </is>
       </c>
-      <c r="H853" s="4" t="inlineStr">
+      <c r="H854" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan beberapa action (detail, setujui, tolak)
 2. Menampilkan modal tolak prospek
@@ -38075,210 +38119,210 @@
         </is>
       </c>
     </row>
-    <row r="854" ht="28" customHeight="1">
-      <c r="A854" s="43" t="inlineStr">
-        <is>
-          <t>68.9</t>
-        </is>
-      </c>
-      <c r="B854" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C854" s="3" t="inlineStr">
-        <is>
-          <t>Approval Non Banking</t>
-        </is>
-      </c>
-      <c r="D854" s="4" t="inlineStr">
-        <is>
-          <t>Batal menolak prospek</t>
-        </is>
-      </c>
-      <c r="E854" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F854" s="3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G854" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik button Batalkan pada moal tolak prospek</t>
-        </is>
-      </c>
-      <c r="H854" s="4" t="inlineStr">
-        <is>
-          <t>1. Modal tolak prospek tertutup dan tetap berada di halaman approval non banking</t>
-        </is>
-      </c>
-    </row>
     <row r="855" ht="28" customHeight="1">
       <c r="A855" s="43" t="inlineStr">
         <is>
+          <t>68.9</t>
+        </is>
+      </c>
+      <c r="B855" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C855" s="3" t="inlineStr">
+        <is>
+          <t>Approval Non Banking</t>
+        </is>
+      </c>
+      <c r="D855" s="4" t="inlineStr">
+        <is>
+          <t>Batal menolak prospek</t>
+        </is>
+      </c>
+      <c r="E855" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F855" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G855" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik button Batalkan pada moal tolak prospek</t>
+        </is>
+      </c>
+      <c r="H855" s="4" t="inlineStr">
+        <is>
+          <t>1. Modal tolak prospek tertutup dan tetap berada di halaman approval non banking</t>
+        </is>
+      </c>
+    </row>
+    <row r="856" ht="28" customHeight="1">
+      <c r="A856" s="43" t="inlineStr">
+        <is>
           <t>68.10</t>
         </is>
       </c>
-      <c r="B855" s="3" t="inlineStr">
+      <c r="B856" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C855" s="3" t="inlineStr">
+      <c r="C856" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D855" s="4" t="inlineStr">
+      <c r="D856" s="4" t="inlineStr">
         <is>
           <t>Tidak menginput remark pada modal tolak prospek</t>
         </is>
       </c>
-      <c r="E855" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F855" s="3" t="inlineStr">
+      <c r="E856" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F856" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G855" s="4" t="inlineStr">
+      <c r="G856" s="4" t="inlineStr">
         <is>
           <t>1. Kosongkan remark 
 2. Klik button Tolak</t>
         </is>
       </c>
-      <c r="H855" s="4" t="inlineStr">
+      <c r="H856" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan remark 
 2. Menampilkan alert 'Remark dibutuhkan!'</t>
         </is>
       </c>
     </row>
-    <row r="856" ht="28" customHeight="1">
-      <c r="A856" s="43" t="inlineStr">
+    <row r="857" ht="28" customHeight="1">
+      <c r="A857" s="43" t="inlineStr">
         <is>
           <t>68.11</t>
         </is>
       </c>
-      <c r="B856" s="3" t="inlineStr">
+      <c r="B857" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C856" s="3" t="inlineStr">
+      <c r="C857" s="3" t="inlineStr">
         <is>
           <t>Approval Non Banking</t>
         </is>
       </c>
-      <c r="D856" s="4" t="inlineStr">
+      <c r="D857" s="4" t="inlineStr">
         <is>
           <t>Filter kolom</t>
         </is>
       </c>
-      <c r="E856" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F856" s="3" t="inlineStr">
+      <c r="E857" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F857" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G856" s="4" t="inlineStr">
+      <c r="G857" s="4" t="inlineStr">
         <is>
           <t>1. Klik icon filter kolom 
 2. Checklist/unchecklist kolom</t>
         </is>
       </c>
-      <c r="H856" s="4" t="inlineStr">
+      <c r="H857" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan list kolom tabel 
 2. Menampilkan data tabel sesuai dengan kolom yang di ceklis</t>
         </is>
       </c>
     </row>
-    <row r="857" ht="28" customHeight="1">
-      <c r="A857" s="43" t="inlineStr">
-        <is>
-          <t>68.12</t>
-        </is>
-      </c>
-      <c r="B857" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C857" s="3" t="inlineStr">
-        <is>
-          <t>Approval Non Banking</t>
-        </is>
-      </c>
-      <c r="D857" s="4" t="inlineStr">
-        <is>
-          <t>Reset ke Default pada filter kolom</t>
-        </is>
-      </c>
-      <c r="E857" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F857" s="3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G857" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik Reset ke Default</t>
-        </is>
-      </c>
-      <c r="H857" s="4" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan data tabel dengan kolom default</t>
-        </is>
-      </c>
-    </row>
     <row r="858" ht="28" customHeight="1">
       <c r="A858" s="43" t="inlineStr">
         <is>
+          <t>68.12</t>
+        </is>
+      </c>
+      <c r="B858" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C858" s="3" t="inlineStr">
+        <is>
+          <t>Approval Non Banking</t>
+        </is>
+      </c>
+      <c r="D858" s="4" t="inlineStr">
+        <is>
+          <t>Reset ke Default pada filter kolom</t>
+        </is>
+      </c>
+      <c r="E858" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F858" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G858" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik Reset ke Default</t>
+        </is>
+      </c>
+      <c r="H858" s="4" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan data tabel dengan kolom default</t>
+        </is>
+      </c>
+    </row>
+    <row r="859" ht="28" customHeight="1">
+      <c r="A859" s="43" t="inlineStr">
+        <is>
           <t>69.1</t>
         </is>
       </c>
-      <c r="B858" s="3" t="inlineStr">
+      <c r="B859" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C858" s="3" t="inlineStr">
+      <c r="C859" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D858" s="4" t="inlineStr">
+      <c r="D859" s="4" t="inlineStr">
         <is>
           <t>Filter data</t>
         </is>
       </c>
-      <c r="E858" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F858" s="3" t="inlineStr">
+      <c r="E859" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F859" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G858" s="4" t="inlineStr">
+      <c r="G859" s="4" t="inlineStr">
         <is>
           <t>1. Pilih kantor wilayah
 2. Pilih kantor cabang 
@@ -38288,7 +38332,7 @@
 6. Klik button Filter</t>
         </is>
       </c>
-      <c r="H858" s="4" t="inlineStr">
+      <c r="H859" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan dropdown list data filter kantor wilayah dan dapat di pilih
 2. Menampilkan dropdown list data filter kantor cabang dan dapat di pilih
@@ -38299,126 +38343,126 @@
         </is>
       </c>
     </row>
-    <row r="859" ht="28" customHeight="1">
-      <c r="A859" s="43" t="inlineStr">
+    <row r="860" ht="28" customHeight="1">
+      <c r="A860" s="43" t="inlineStr">
         <is>
           <t>69.2</t>
         </is>
       </c>
-      <c r="B859" s="3" t="inlineStr">
+      <c r="B860" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C859" s="3" t="inlineStr">
+      <c r="C860" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D859" s="4" t="inlineStr">
+      <c r="D860" s="4" t="inlineStr">
         <is>
           <t>Mencari data</t>
         </is>
       </c>
-      <c r="E859" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F859" s="3" t="inlineStr">
+      <c r="E860" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F860" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G859" s="4" t="inlineStr">
+      <c r="G860" s="4" t="inlineStr">
         <is>
           <t>1. Input keyword pada field search 
 2. Klik icon search yang ada di sebelah field</t>
         </is>
       </c>
-      <c r="H859" s="4" t="inlineStr">
+      <c r="H860" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput keyword 
 2. Menampilkan data Re-Assign Prospek sesuai dengan keyword yang di cari</t>
         </is>
       </c>
     </row>
-    <row r="860" ht="28" customHeight="1">
-      <c r="A860" s="43" t="inlineStr">
+    <row r="861" ht="28" customHeight="1">
+      <c r="A861" s="43" t="inlineStr">
         <is>
           <t>69.3</t>
         </is>
       </c>
-      <c r="B860" s="3" t="inlineStr">
+      <c r="B861" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C860" s="3" t="inlineStr">
+      <c r="C861" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D860" s="4" t="inlineStr">
+      <c r="D861" s="4" t="inlineStr">
         <is>
           <t>Membuka halaman Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="E860" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F860" s="3" t="inlineStr">
+      <c r="E861" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F861" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G860" s="4" t="inlineStr">
+      <c r="G861" s="4" t="inlineStr">
         <is>
           <t>1. Klik menu Re-Assign &amp; Approval 
 2. Klik submenu Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="H860" s="4" t="inlineStr">
+      <c r="H861" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan submenu Re-Assign &amp; Approval 
 2. Menampilkan halaman Re-Assign Prospek</t>
         </is>
       </c>
     </row>
-    <row r="861" ht="28" customHeight="1">
-      <c r="A861" s="43" t="inlineStr">
+    <row r="862" ht="28" customHeight="1">
+      <c r="A862" s="43" t="inlineStr">
         <is>
           <t>69.4</t>
         </is>
       </c>
-      <c r="B861" s="3" t="inlineStr">
+      <c r="B862" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C861" s="3" t="inlineStr">
+      <c r="C862" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D861" s="4" t="inlineStr">
+      <c r="D862" s="4" t="inlineStr">
         <is>
           <t>Filter data</t>
         </is>
       </c>
-      <c r="E861" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F861" s="3" t="inlineStr">
+      <c r="E862" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F862" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G861" s="4" t="inlineStr">
+      <c r="G862" s="4" t="inlineStr">
         <is>
           <t>1. Pilih kantor wilayah
 2. Pilih kantor cabang 
@@ -38428,7 +38472,7 @@
 6. Klik button Filter</t>
         </is>
       </c>
-      <c r="H861" s="4" t="inlineStr">
+      <c r="H862" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan dropdown list data filter kantor wilayah dan dapat di pilih
 2. Menampilkan dropdown list data filter kantor cabang dan dapat di pilih
@@ -38439,96 +38483,54 @@
         </is>
       </c>
     </row>
-    <row r="862" ht="28" customHeight="1">
-      <c r="A862" s="43" t="inlineStr">
+    <row r="863" ht="28" customHeight="1">
+      <c r="A863" s="43" t="inlineStr">
         <is>
           <t>69.5</t>
         </is>
       </c>
-      <c r="B862" s="3" t="inlineStr">
+      <c r="B863" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C862" s="3" t="inlineStr">
+      <c r="C863" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D862" s="4" t="inlineStr">
+      <c r="D863" s="4" t="inlineStr">
         <is>
           <t>Mencari data</t>
         </is>
       </c>
-      <c r="E862" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F862" s="3" t="inlineStr">
+      <c r="E863" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F863" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G862" s="4" t="inlineStr">
+      <c r="G863" s="4" t="inlineStr">
         <is>
           <t>1. Input keyword pada field search 
 2. Klik icon search yang ada di sebelah field</t>
         </is>
       </c>
-      <c r="H862" s="4" t="inlineStr">
+      <c r="H863" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput keyword 
 2. Menampilkan data Re-Assign Prospek sesuai dengan keyword yang di cari</t>
         </is>
       </c>
     </row>
-    <row r="863" ht="28" customHeight="1">
-      <c r="A863" s="43" t="inlineStr">
-        <is>
-          <t>69.6</t>
-        </is>
-      </c>
-      <c r="B863" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C863" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign Prospek</t>
-        </is>
-      </c>
-      <c r="D863" s="4" t="inlineStr">
-        <is>
-          <t>Validasi count checklist data</t>
-        </is>
-      </c>
-      <c r="E863" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F863" s="3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G863" s="4" t="inlineStr">
-        <is>
-          <t>1. Cek informasi yang ada pada button Reassign () data</t>
-        </is>
-      </c>
-      <c r="H863" s="4" t="inlineStr">
-        <is>
-          <t>1. Menampilkan count angka yang sesuai dengan data yang di checklist</t>
-        </is>
-      </c>
-    </row>
     <row r="864" ht="28" customHeight="1">
       <c r="A864" s="43" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.6</t>
         </is>
       </c>
       <c r="B864" s="3" t="inlineStr">
@@ -38543,7 +38545,7 @@
       </c>
       <c r="D864" s="4" t="inlineStr">
         <is>
-          <t>Validasi data yang sudah dii pilih</t>
+          <t>Validasi count checklist data</t>
         </is>
       </c>
       <c r="E864" s="3" t="inlineStr">
@@ -38558,133 +38560,175 @@
       </c>
       <c r="G864" s="4" t="inlineStr">
         <is>
-          <t>1. Cek pada halaman pindah kelolaan, data tabel nya berisi prospek yang di pilih</t>
+          <t>1. Cek informasi yang ada pada button Reassign () data</t>
         </is>
       </c>
       <c r="H864" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data tabel prospek yang di pilih saja</t>
+          <t>1. Menampilkan count angka yang sesuai dengan data yang di checklist</t>
         </is>
       </c>
     </row>
     <row r="865" ht="28" customHeight="1">
       <c r="A865" s="43" t="inlineStr">
         <is>
+          <t>69.7</t>
+        </is>
+      </c>
+      <c r="B865" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C865" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign Prospek</t>
+        </is>
+      </c>
+      <c r="D865" s="4" t="inlineStr">
+        <is>
+          <t>Validasi data yang sudah dii pilih</t>
+        </is>
+      </c>
+      <c r="E865" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F865" s="3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G865" s="4" t="inlineStr">
+        <is>
+          <t>1. Cek pada halaman pindah kelolaan, data tabel nya berisi prospek yang di pilih</t>
+        </is>
+      </c>
+      <c r="H865" s="4" t="inlineStr">
+        <is>
+          <t>1. Menampilkan data tabel prospek yang di pilih saja</t>
+        </is>
+      </c>
+    </row>
+    <row r="866" ht="28" customHeight="1">
+      <c r="A866" s="43" t="inlineStr">
+        <is>
           <t>69.8</t>
         </is>
       </c>
-      <c r="B865" s="3" t="inlineStr">
+      <c r="B866" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C865" s="3" t="inlineStr">
+      <c r="C866" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D865" s="4" t="inlineStr">
+      <c r="D866" s="4" t="inlineStr">
         <is>
           <t>Mengosongkan field inputan mandatory pada reassign prospek</t>
         </is>
       </c>
-      <c r="E865" s="3" t="inlineStr">
+      <c r="E866" s="3" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F865" s="3" t="inlineStr">
+      <c r="F866" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G865" s="4" t="inlineStr">
+      <c r="G866" s="4" t="inlineStr">
         <is>
           <t>1. Kosongkan salah satu atau semua field mandatory 
 2. Klik button Submit</t>
         </is>
       </c>
-      <c r="H865" s="4" t="inlineStr">
+      <c r="H866" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil tidak mengisi/mengosongkan field 
 2. Menampilkan alert pada setiap field mandatory bahwa field tersebut dibutuhkan / wajib diisi</t>
         </is>
       </c>
     </row>
-    <row r="866" ht="28" customHeight="1">
-      <c r="A866" s="43" t="inlineStr">
-        <is>
-          <t>69.9</t>
-        </is>
-      </c>
-      <c r="B866" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C866" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign Prospek</t>
-        </is>
-      </c>
-      <c r="D866" s="4" t="inlineStr">
-        <is>
-          <t>Membatalkan Re-Assign Prospek</t>
-        </is>
-      </c>
-      <c r="E866" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F866" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G866" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik button Batalkan pada halaman pindah kelolaan</t>
-        </is>
-      </c>
-      <c r="H866" s="4" t="inlineStr">
-        <is>
-          <t>1. Kembali ke halaman utama Re-assign Prospek</t>
-        </is>
-      </c>
-    </row>
     <row r="867" ht="28" customHeight="1">
       <c r="A867" s="43" t="inlineStr">
         <is>
+          <t>69.9</t>
+        </is>
+      </c>
+      <c r="B867" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C867" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign Prospek</t>
+        </is>
+      </c>
+      <c r="D867" s="4" t="inlineStr">
+        <is>
+          <t>Membatalkan Re-Assign Prospek</t>
+        </is>
+      </c>
+      <c r="E867" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F867" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G867" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik button Batalkan pada halaman pindah kelolaan</t>
+        </is>
+      </c>
+      <c r="H867" s="4" t="inlineStr">
+        <is>
+          <t>1. Kembali ke halaman utama Re-assign Prospek</t>
+        </is>
+      </c>
+    </row>
+    <row r="868" ht="28" customHeight="1">
+      <c r="A868" s="43" t="inlineStr">
+        <is>
           <t>69.10</t>
         </is>
       </c>
-      <c r="B867" s="3" t="inlineStr">
+      <c r="B868" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C867" s="3" t="inlineStr">
+      <c r="C868" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D867" s="4" t="inlineStr">
+      <c r="D868" s="4" t="inlineStr">
         <is>
           <t>Validasi data prospek yang di re-assign</t>
         </is>
       </c>
-      <c r="E867" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F867" s="3" t="inlineStr">
+      <c r="E868" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F868" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G867" s="4" t="inlineStr">
+      <c r="G868" s="4" t="inlineStr">
         <is>
           <t>1. Login menggunakan user yang sebelumnya sudah dipilih ketika re-assign prospek 
 2. Klik menu Lead Qualification 
@@ -38692,7 +38736,7 @@
 4. Cek data yang sebelum nya di re-assign pada tabel dan pada detail prospek</t>
         </is>
       </c>
-      <c r="H867" s="4" t="inlineStr">
+      <c r="H868" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil login 
 2. Menampilkan dropdown submenu Lead Qualification 
@@ -38701,38 +38745,38 @@
         </is>
       </c>
     </row>
-    <row r="868" ht="28" customHeight="1">
-      <c r="A868" s="43" t="inlineStr">
+    <row r="869" ht="28" customHeight="1">
+      <c r="A869" s="43" t="inlineStr">
         <is>
           <t>69.11</t>
         </is>
       </c>
-      <c r="B868" s="3" t="inlineStr">
+      <c r="B869" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C868" s="3" t="inlineStr">
+      <c r="C869" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D868" s="4" t="inlineStr">
+      <c r="D869" s="4" t="inlineStr">
         <is>
           <t>Melakukan Re-assign prospek semua data</t>
         </is>
       </c>
-      <c r="E868" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F868" s="3" t="inlineStr">
+      <c r="E869" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F869" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G868" s="4" t="inlineStr">
+      <c r="G869" s="4" t="inlineStr">
         <is>
           <t>1. Klik button Reassign semua data 
 2. Klik button Yes 
@@ -38743,7 +38787,7 @@
 7. Klik button Submit</t>
         </is>
       </c>
-      <c r="H868" s="4" t="inlineStr">
+      <c r="H869" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan popup konfirmasi 
 2. Menampilkan halaman pindah kelolaan 
@@ -38755,52 +38799,10 @@
         </is>
       </c>
     </row>
-    <row r="869" ht="28" customHeight="1">
-      <c r="A869" s="43" t="inlineStr">
-        <is>
-          <t>69.12</t>
-        </is>
-      </c>
-      <c r="B869" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C869" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign Prospek</t>
-        </is>
-      </c>
-      <c r="D869" s="4" t="inlineStr">
-        <is>
-          <t>Validasi semua data</t>
-        </is>
-      </c>
-      <c r="E869" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F869" s="3" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G869" s="4" t="inlineStr">
-        <is>
-          <t>1. Cek pada halaman pindah kelolaan, data tabel nya berisi semua prospek</t>
-        </is>
-      </c>
-      <c r="H869" s="4" t="inlineStr">
-        <is>
-          <t>1. Menampilkan data tabel yang berisi semua prospek</t>
-        </is>
-      </c>
-    </row>
     <row r="870" ht="28" customHeight="1">
       <c r="A870" s="43" t="inlineStr">
         <is>
-          <t>69.13</t>
+          <t>69.12</t>
         </is>
       </c>
       <c r="B870" s="3" t="inlineStr">
@@ -38815,7 +38817,7 @@
       </c>
       <c r="D870" s="4" t="inlineStr">
         <is>
-          <t>Membatalkan Re-Assign Prospek</t>
+          <t>Validasi semua data</t>
         </is>
       </c>
       <c r="E870" s="3" t="inlineStr">
@@ -38825,52 +38827,94 @@
       </c>
       <c r="F870" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G870" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button Batalkan pada halaman pindah kelolaan</t>
+          <t>1. Cek pada halaman pindah kelolaan, data tabel nya berisi semua prospek</t>
         </is>
       </c>
       <c r="H870" s="4" t="inlineStr">
         <is>
-          <t>1. Kembali ke halaman utama Re-assign Prospek</t>
+          <t>1. Menampilkan data tabel yang berisi semua prospek</t>
         </is>
       </c>
     </row>
     <row r="871" ht="28" customHeight="1">
       <c r="A871" s="43" t="inlineStr">
         <is>
+          <t>69.13</t>
+        </is>
+      </c>
+      <c r="B871" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C871" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign Prospek</t>
+        </is>
+      </c>
+      <c r="D871" s="4" t="inlineStr">
+        <is>
+          <t>Membatalkan Re-Assign Prospek</t>
+        </is>
+      </c>
+      <c r="E871" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F871" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G871" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik button Batalkan pada halaman pindah kelolaan</t>
+        </is>
+      </c>
+      <c r="H871" s="4" t="inlineStr">
+        <is>
+          <t>1. Kembali ke halaman utama Re-assign Prospek</t>
+        </is>
+      </c>
+    </row>
+    <row r="872" ht="70" customHeight="1">
+      <c r="A872" s="43" t="inlineStr">
+        <is>
           <t>69.14</t>
         </is>
       </c>
-      <c r="B871" s="3" t="inlineStr">
+      <c r="B872" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C871" s="3" t="inlineStr">
+      <c r="C872" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="D871" s="4" t="inlineStr">
+      <c r="D872" s="4" t="inlineStr">
         <is>
           <t>Validasi semua data prospek yang di re-assign</t>
         </is>
       </c>
-      <c r="E871" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F871" s="3" t="inlineStr">
+      <c r="E872" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F872" s="3" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G871" s="4" t="inlineStr">
+      <c r="G872" s="4" t="inlineStr">
         <is>
           <t>1. Login menggunakan user yang sebelumnya sudah dipilih ketika re-assign prospek 
 2. Klik menu Lead Qualification 
@@ -38878,7 +38922,7 @@
 4. Cek data yang sebelum nya di re-assign pada tabel dan pada detail prospek</t>
         </is>
       </c>
-      <c r="H871" s="4" t="inlineStr">
+      <c r="H872" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil login 
 2. Menampilkan dropdown submenu Lead Qualification 
@@ -38887,126 +38931,126 @@
         </is>
       </c>
     </row>
-    <row r="872" ht="70" customHeight="1">
-      <c r="A872" s="43" t="inlineStr">
+    <row r="873" ht="42" customHeight="1">
+      <c r="A873" s="43" t="inlineStr">
         <is>
           <t>70.1</t>
         </is>
       </c>
-      <c r="B872" s="3" t="inlineStr">
+      <c r="B873" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C872" s="3" t="inlineStr">
+      <c r="C873" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D872" s="4" t="inlineStr">
+      <c r="D873" s="4" t="inlineStr">
         <is>
           <t>Pagination</t>
         </is>
       </c>
-      <c r="E872" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F872" s="3" t="inlineStr">
+      <c r="E873" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F873" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G872" s="4" t="inlineStr">
+      <c r="G873" s="4" t="inlineStr">
         <is>
           <t>1. Klik pagination (10/halaman).
 2. Pilih berapa data yang ingin ditampilkan.</t>
         </is>
       </c>
-      <c r="H872" s="4" t="inlineStr">
+      <c r="H873" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengklik pagination.
 2. Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="873" ht="42" customHeight="1">
-      <c r="A873" s="43" t="inlineStr">
+    <row r="874" ht="42" customHeight="1">
+      <c r="A874" s="43" t="inlineStr">
         <is>
           <t>70.2</t>
         </is>
       </c>
-      <c r="B873" s="3" t="inlineStr">
+      <c r="B874" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C873" s="3" t="inlineStr">
+      <c r="C874" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D873" s="4" t="inlineStr">
+      <c r="D874" s="4" t="inlineStr">
         <is>
           <t>Pindah Halaman</t>
         </is>
       </c>
-      <c r="E873" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F873" s="3" t="inlineStr">
+      <c r="E874" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F874" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G873" s="4" t="inlineStr">
+      <c r="G874" s="4" t="inlineStr">
         <is>
           <t>1. Input angka halaman di field pindah halaman.
 2. Klik Enter pada keyboard.</t>
         </is>
       </c>
-      <c r="H873" s="4" t="inlineStr">
+      <c r="H874" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput angka halaman.
 2. Berhasil berpindah ke halaman yang dituju.</t>
         </is>
       </c>
     </row>
-    <row r="874" ht="42" customHeight="1">
-      <c r="A874" s="43" t="inlineStr">
+    <row r="875" ht="70" customHeight="1">
+      <c r="A875" s="43" t="inlineStr">
         <is>
           <t>70.3</t>
         </is>
       </c>
-      <c r="B874" s="3" t="inlineStr">
+      <c r="B875" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C874" s="3" t="inlineStr">
+      <c r="C875" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D874" s="4" t="inlineStr">
+      <c r="D875" s="4" t="inlineStr">
         <is>
           <t>Melakukan Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="E874" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F874" s="3" t="inlineStr">
+      <c r="E875" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F875" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G874" s="4" t="inlineStr">
+      <c r="G875" s="4" t="inlineStr">
         <is>
           <t>1. Pilih prospek dengan klik checkbox yang ada di samping setiap data prospek 
 2. Klik button Reassign () data 
@@ -39015,7 +39059,7 @@
 5. Klik button Submit</t>
         </is>
       </c>
-      <c r="H874" s="4" t="inlineStr">
+      <c r="H875" s="4" t="inlineStr">
         <is>
           <t>1. Checkbox menjadi ceklis dan data berhasil di pilih 
 2. Menampilkan popup konfirmasi 
@@ -39025,258 +39069,258 @@
         </is>
       </c>
     </row>
-    <row r="875" ht="70" customHeight="1">
-      <c r="A875" s="43" t="inlineStr">
+    <row r="876" ht="28" customHeight="1">
+      <c r="A876" s="43" t="inlineStr">
         <is>
           <t>70.4</t>
         </is>
       </c>
-      <c r="B875" s="3" t="inlineStr">
+      <c r="B876" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C875" s="3" t="inlineStr">
+      <c r="C876" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D875" s="4" t="inlineStr">
+      <c r="D876" s="4" t="inlineStr">
         <is>
           <t>Pagination</t>
         </is>
       </c>
-      <c r="E875" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F875" s="3" t="inlineStr">
+      <c r="E876" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F876" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G875" s="4" t="inlineStr">
+      <c r="G876" s="4" t="inlineStr">
         <is>
           <t>1. Klik pagination (10/halaman).
 2. Pilih berapa data yang ingin ditampilkan.</t>
         </is>
       </c>
-      <c r="H875" s="4" t="inlineStr">
+      <c r="H876" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengklik pagination.
 2. Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="876" ht="28" customHeight="1">
-      <c r="A876" s="43" t="inlineStr">
+    <row r="877" ht="42" customHeight="1">
+      <c r="A877" s="43" t="inlineStr">
         <is>
           <t>70.5</t>
         </is>
       </c>
-      <c r="B876" s="3" t="inlineStr">
+      <c r="B877" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C876" s="3" t="inlineStr">
+      <c r="C877" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D876" s="4" t="inlineStr">
+      <c r="D877" s="4" t="inlineStr">
         <is>
           <t>Pindah Halaman</t>
         </is>
       </c>
-      <c r="E876" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F876" s="3" t="inlineStr">
+      <c r="E877" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F877" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G876" s="4" t="inlineStr">
+      <c r="G877" s="4" t="inlineStr">
         <is>
           <t>1. Input angka halaman di field pindah halaman.
 2. Klik Enter pada keyboard.</t>
         </is>
       </c>
-      <c r="H876" s="4" t="inlineStr">
+      <c r="H877" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput angka halaman.
 2. Berhasil berpindah ke halaman yang dituju.</t>
         </is>
       </c>
     </row>
-    <row r="877" ht="42" customHeight="1">
-      <c r="A877" s="43" t="inlineStr">
+    <row r="878" ht="28" customHeight="1">
+      <c r="A878" s="43" t="inlineStr">
         <is>
           <t>70.6</t>
         </is>
       </c>
-      <c r="B877" s="3" t="inlineStr">
+      <c r="B878" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C877" s="3" t="inlineStr">
+      <c r="C878" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D877" s="4" t="inlineStr">
+      <c r="D878" s="4" t="inlineStr">
         <is>
           <t>Membuka halaman Re-Assign Management</t>
         </is>
       </c>
-      <c r="E877" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F877" s="3" t="inlineStr">
+      <c r="E878" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F878" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G877" s="4" t="inlineStr">
+      <c r="G878" s="4" t="inlineStr">
         <is>
           <t>1. Klik menu Re-Assign &amp; Approval 
 2. Klik submenu Re-Assign Management</t>
         </is>
       </c>
-      <c r="H877" s="4" t="inlineStr">
+      <c r="H878" s="4" t="inlineStr">
         <is>
           <t>1. Menampilkan dropdown list submenu Re-Assign &amp; Approval 
 2. Menampilkan halaman Re-Assign Management</t>
         </is>
       </c>
     </row>
-    <row r="878" ht="28" customHeight="1">
-      <c r="A878" s="43" t="inlineStr">
+    <row r="879" ht="28" customHeight="1">
+      <c r="A879" s="43" t="inlineStr">
         <is>
           <t>70.7</t>
         </is>
       </c>
-      <c r="B878" s="3" t="inlineStr">
+      <c r="B879" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C878" s="3" t="inlineStr">
+      <c r="C879" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D878" s="4" t="inlineStr">
+      <c r="D879" s="4" t="inlineStr">
         <is>
           <t>Mencari data prospek pada halaman Re-Assign Management</t>
         </is>
       </c>
-      <c r="E878" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F878" s="3" t="inlineStr">
+      <c r="E879" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F879" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G878" s="4" t="inlineStr">
+      <c r="G879" s="4" t="inlineStr">
         <is>
           <t>1. Input nama nasabah pada field search 
 2. Klik icon search atau klik Enter</t>
         </is>
       </c>
-      <c r="H878" s="4" t="inlineStr">
+      <c r="H879" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput nama nasabah
 2. Menampilkan data prospek Re-Assign Management sesuai dengan nama yang di cari</t>
         </is>
       </c>
     </row>
-    <row r="879" ht="28" customHeight="1">
-      <c r="A879" s="43" t="inlineStr">
+    <row r="880" ht="28" customHeight="1">
+      <c r="A880" s="43" t="inlineStr">
         <is>
           <t>70.8</t>
         </is>
       </c>
-      <c r="B879" s="3" t="inlineStr">
+      <c r="B880" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C879" s="3" t="inlineStr">
+      <c r="C880" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D879" s="4" t="inlineStr">
+      <c r="D880" s="4" t="inlineStr">
         <is>
           <t>Mencari data prospek yang tidak ada pada halaman Re-Assign Management</t>
         </is>
       </c>
-      <c r="E879" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F879" s="3" t="inlineStr">
+      <c r="E880" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F880" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G879" s="4" t="inlineStr">
+      <c r="G880" s="4" t="inlineStr">
         <is>
           <t>1. Input nama nasabah yang datanya tidak ada 
 2. Klik icon search atau klik Enter</t>
         </is>
       </c>
-      <c r="H879" s="4" t="inlineStr">
+      <c r="H880" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput nama nasabah
 2. Menampilkan tabel kosong dengan keterangan no data</t>
         </is>
       </c>
     </row>
-    <row r="880" ht="28" customHeight="1">
-      <c r="A880" s="43" t="inlineStr">
+    <row r="881" ht="14" customHeight="1">
+      <c r="A881" s="43" t="inlineStr">
         <is>
           <t>70.9</t>
         </is>
       </c>
-      <c r="B880" s="3" t="inlineStr">
+      <c r="B881" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C880" s="3" t="inlineStr">
+      <c r="C881" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D880" s="4" t="inlineStr">
+      <c r="D881" s="4" t="inlineStr">
         <is>
           <t>Melakukan Re-Assign Prospek</t>
         </is>
       </c>
-      <c r="E880" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F880" s="3" t="inlineStr">
+      <c r="E881" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F881" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G880" s="4" t="inlineStr">
+      <c r="G881" s="4" t="inlineStr">
         <is>
           <t>1. Pilih prospek dengan klik checkbox yang ada di samping setiap data prospek 
 2. Klik button Reassign () data 
@@ -39285,7 +39329,7 @@
 5. Klik button Submit</t>
         </is>
       </c>
-      <c r="H880" s="4" t="inlineStr">
+      <c r="H881" s="4" t="inlineStr">
         <is>
           <t>1. Checkbox menjadi ceklis dan data berhasil di pilih 
 2. Menampilkan popup konfirmasi 
@@ -39295,80 +39339,80 @@
         </is>
       </c>
     </row>
-    <row r="881" ht="14" customHeight="1">
-      <c r="A881" s="43" t="inlineStr">
-        <is>
-          <t>70.10</t>
-        </is>
-      </c>
-      <c r="B881" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign dan Approval</t>
-        </is>
-      </c>
-      <c r="C881" s="3" t="inlineStr">
-        <is>
-          <t>Re-Assign Management</t>
-        </is>
-      </c>
-      <c r="D881" s="4" t="inlineStr">
-        <is>
-          <t>Validasi jumlah data yang di pilih untuk reassign</t>
-        </is>
-      </c>
-      <c r="E881" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F881" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G881" s="4" t="inlineStr">
-        <is>
-          <t>1. cek jumlah data yang muncul pada button Reassign () data</t>
-        </is>
-      </c>
-      <c r="H881" s="4" t="inlineStr">
-        <is>
-          <t>1. Angka yang muncul pada button sesuai dengan jumlah data yang di pilih</t>
-        </is>
-      </c>
-    </row>
     <row r="882" ht="42" customHeight="1">
       <c r="A882" s="43" t="inlineStr">
         <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="B882" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign dan Approval</t>
+        </is>
+      </c>
+      <c r="C882" s="3" t="inlineStr">
+        <is>
+          <t>Re-Assign Management</t>
+        </is>
+      </c>
+      <c r="D882" s="4" t="inlineStr">
+        <is>
+          <t>Validasi jumlah data yang di pilih untuk reassign</t>
+        </is>
+      </c>
+      <c r="E882" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F882" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G882" s="4" t="inlineStr">
+        <is>
+          <t>1. cek jumlah data yang muncul pada button Reassign () data</t>
+        </is>
+      </c>
+      <c r="H882" s="4" t="inlineStr">
+        <is>
+          <t>1. Angka yang muncul pada button sesuai dengan jumlah data yang di pilih</t>
+        </is>
+      </c>
+    </row>
+    <row r="883" ht="42" customHeight="1">
+      <c r="A883" s="43" t="inlineStr">
+        <is>
           <t>70.11</t>
         </is>
       </c>
-      <c r="B882" s="3" t="inlineStr">
+      <c r="B883" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C882" s="3" t="inlineStr">
+      <c r="C883" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D882" s="4" t="inlineStr">
+      <c r="D883" s="4" t="inlineStr">
         <is>
           <t>Validasi data prospek yang di re-assign ke sales</t>
         </is>
       </c>
-      <c r="E882" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F882" s="3" t="inlineStr">
+      <c r="E883" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F883" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G882" s="4" t="inlineStr">
+      <c r="G883" s="4" t="inlineStr">
         <is>
           <t>1. Login dengan akun sales yang sebelumnya sudah di pilih reassign management
 2. Klik menu Lead Qualification
@@ -39376,7 +39420,7 @@
 4. Cek data prospek yang sudah di reassign</t>
         </is>
       </c>
-      <c r="H882" s="4" t="inlineStr">
+      <c r="H883" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil login akun sales
 2. Menampilkan dropdown submenu Lead Qualification
@@ -39385,140 +39429,98 @@
         </is>
       </c>
     </row>
-    <row r="883" ht="42" customHeight="1">
-      <c r="A883" s="43" t="inlineStr">
+    <row r="884" ht="28" customHeight="1">
+      <c r="A884" s="43" t="inlineStr">
         <is>
           <t>70.12</t>
         </is>
       </c>
-      <c r="B883" s="3" t="inlineStr">
+      <c r="B884" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C883" s="3" t="inlineStr">
+      <c r="C884" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D883" s="4" t="inlineStr">
+      <c r="D884" s="4" t="inlineStr">
         <is>
           <t>Pagination</t>
         </is>
       </c>
-      <c r="E883" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F883" s="3" t="inlineStr">
+      <c r="E884" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F884" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G883" s="4" t="inlineStr">
+      <c r="G884" s="4" t="inlineStr">
         <is>
           <t>1. Klik pagination (10/halaman).
 2. Pilih berapa data yang ingin ditampilkan.</t>
         </is>
       </c>
-      <c r="H883" s="4" t="inlineStr">
+      <c r="H884" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil mengklik pagination.
 2. Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="884" ht="28" customHeight="1">
-      <c r="A884" s="43" t="inlineStr">
+    <row r="885" ht="42" customHeight="1">
+      <c r="A885" s="43" t="inlineStr">
         <is>
           <t>70.13</t>
         </is>
       </c>
-      <c r="B884" s="3" t="inlineStr">
+      <c r="B885" s="3" t="inlineStr">
         <is>
           <t>Re-Assign dan Approval</t>
         </is>
       </c>
-      <c r="C884" s="3" t="inlineStr">
+      <c r="C885" s="3" t="inlineStr">
         <is>
           <t>Re-Assign Management</t>
         </is>
       </c>
-      <c r="D884" s="4" t="inlineStr">
+      <c r="D885" s="4" t="inlineStr">
         <is>
           <t>Pindah Halaman</t>
         </is>
       </c>
-      <c r="E884" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F884" s="3" t="inlineStr">
+      <c r="E885" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F885" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G884" s="4" t="inlineStr">
+      <c r="G885" s="4" t="inlineStr">
         <is>
           <t>1. Input angka halaman di field pindah halaman.
 2. Klik Enter pada keyboard.</t>
         </is>
       </c>
-      <c r="H884" s="4" t="inlineStr">
+      <c r="H885" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menginput angka halaman.
 2. Berhasil berpindah ke halaman yang dituju.</t>
         </is>
       </c>
     </row>
-    <row r="885" ht="42" customHeight="1">
-      <c r="A885" s="43" t="inlineStr">
-        <is>
-          <t>71.1</t>
-        </is>
-      </c>
-      <c r="B885" s="3" t="inlineStr">
-        <is>
-          <t>Export data management</t>
-        </is>
-      </c>
-      <c r="C885" s="3" t="inlineStr">
-        <is>
-          <t>Riwayat export saya</t>
-        </is>
-      </c>
-      <c r="D885" s="4" t="inlineStr">
-        <is>
-          <t>Membuka menu riwayat export saya</t>
-        </is>
-      </c>
-      <c r="E885" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F885" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G885" s="4" t="inlineStr">
-        <is>
-          <t>1. Klik menu exported data management, klik submenu riwayat export saya</t>
-        </is>
-      </c>
-      <c r="H885" s="4" t="inlineStr">
-        <is>
-          <t>1. Menampilkan halaman riwayat export saya</t>
-        </is>
-      </c>
-    </row>
     <row r="886" ht="14" customHeight="1">
       <c r="A886" s="43" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.1</t>
         </is>
       </c>
       <c r="B886" s="3" t="inlineStr">
@@ -39533,7 +39535,7 @@
       </c>
       <c r="D886" s="4" t="inlineStr">
         <is>
-          <t>Validasi card disetujui dengan data table</t>
+          <t>Membuka menu riwayat export saya</t>
         </is>
       </c>
       <c r="E886" s="3" t="inlineStr">
@@ -39548,19 +39550,19 @@
       </c>
       <c r="G886" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data status approval dengan memilih status “Approved”</t>
+          <t>1. Klik menu exported data management, klik submenu riwayat export saya</t>
         </is>
       </c>
       <c r="H886" s="4" t="inlineStr">
         <is>
-          <t>1. Jumlah data pada card dan table sesuai</t>
+          <t>1. Menampilkan halaman riwayat export saya</t>
         </is>
       </c>
     </row>
     <row r="887" ht="42" customHeight="1">
       <c r="A887" s="43" t="inlineStr">
         <is>
-          <t>71.3</t>
+          <t>71.2</t>
         </is>
       </c>
       <c r="B887" s="3" t="inlineStr">
@@ -39575,7 +39577,7 @@
       </c>
       <c r="D887" s="4" t="inlineStr">
         <is>
-          <t>Validasi card ditolak dengan data table</t>
+          <t>Validasi card disetujui dengan data table</t>
         </is>
       </c>
       <c r="E887" s="3" t="inlineStr">
@@ -39590,7 +39592,7 @@
       </c>
       <c r="G887" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data status approval dengan memilih status “Rejected”</t>
+          <t>1. Melakukan filter data status approval dengan memilih status “Approved”</t>
         </is>
       </c>
       <c r="H887" s="4" t="inlineStr">
@@ -39602,7 +39604,7 @@
     <row r="888" ht="42" customHeight="1">
       <c r="A888" s="43" t="inlineStr">
         <is>
-          <t>71.4</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="B888" s="3" t="inlineStr">
@@ -39617,7 +39619,7 @@
       </c>
       <c r="D888" s="4" t="inlineStr">
         <is>
-          <t>Validasi card kadaluwarsa dengan data table</t>
+          <t>Validasi card ditolak dengan data table</t>
         </is>
       </c>
       <c r="E888" s="3" t="inlineStr">
@@ -39627,12 +39629,12 @@
       </c>
       <c r="F888" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G888" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data status approval dengan memilih status “Expired”</t>
+          <t>1. Melakukan filter data status approval dengan memilih status “Rejected”</t>
         </is>
       </c>
       <c r="H888" s="4" t="inlineStr">
@@ -39644,7 +39646,7 @@
     <row r="889" ht="28" customHeight="1">
       <c r="A889" s="43" t="inlineStr">
         <is>
-          <t>71.5</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="B889" s="3" t="inlineStr">
@@ -39659,7 +39661,7 @@
       </c>
       <c r="D889" s="4" t="inlineStr">
         <is>
-          <t>Mengunduh data yang sudah di approve</t>
+          <t>Validasi card kadaluwarsa dengan data table</t>
         </is>
       </c>
       <c r="E889" s="3" t="inlineStr">
@@ -39669,24 +39671,24 @@
       </c>
       <c r="F889" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G889" s="4" t="inlineStr">
         <is>
-          <t>1. Klik button download</t>
+          <t>1. Melakukan filter data status approval dengan memilih status “Expired”</t>
         </is>
       </c>
       <c r="H889" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil mengunduh data</t>
+          <t>1. Jumlah data pada card dan table sesuai</t>
         </is>
       </c>
     </row>
     <row r="890" ht="42" customHeight="1">
       <c r="A890" s="43" t="inlineStr">
         <is>
-          <t>71.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="B890" s="3" t="inlineStr">
@@ -39701,7 +39703,7 @@
       </c>
       <c r="D890" s="4" t="inlineStr">
         <is>
-          <t>Membuka dokumen hasil download</t>
+          <t>Mengunduh data yang sudah di approve</t>
         </is>
       </c>
       <c r="E890" s="3" t="inlineStr">
@@ -39716,19 +39718,19 @@
       </c>
       <c r="G890" s="4" t="inlineStr">
         <is>
-          <t>1. Extract file, kemudian masukan password yang terkirim pada email user yang mengajukan, input password maka file berhasil di extract, kemudian buka file</t>
+          <t>1. Klik button download</t>
         </is>
       </c>
       <c r="H890" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka file hasil download</t>
+          <t>1. Berhasil mengunduh data</t>
         </is>
       </c>
     </row>
     <row r="891" ht="14" customHeight="1">
       <c r="A891" s="43" t="inlineStr">
         <is>
-          <t>72.1</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="B891" s="3" t="inlineStr">
@@ -39738,12 +39740,12 @@
       </c>
       <c r="C891" s="3" t="inlineStr">
         <is>
-          <t>Management export</t>
+          <t>Riwayat export saya</t>
         </is>
       </c>
       <c r="D891" s="4" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Membuka dokumen hasil download</t>
         </is>
       </c>
       <c r="E891" s="3" t="inlineStr">
@@ -39753,24 +39755,24 @@
       </c>
       <c r="F891" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G891" s="4" t="inlineStr">
         <is>
-          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
+          <t>1. Extract file, kemudian masukan password yang terkirim pada email user yang mengajukan, input password maka file berhasil di extract, kemudian buka file</t>
         </is>
       </c>
       <c r="H891" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai filter yang dipilih</t>
+          <t>1. Berhasil membuka file hasil download</t>
         </is>
       </c>
     </row>
     <row r="892" ht="42" customHeight="1">
       <c r="A892" s="43" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.1</t>
         </is>
       </c>
       <c r="B892" s="3" t="inlineStr">
@@ -39785,7 +39787,7 @@
       </c>
       <c r="D892" s="4" t="inlineStr">
         <is>
-          <t>Validasi card menunggu approval dengan data table</t>
+          <t>Melakukan filter data</t>
         </is>
       </c>
       <c r="E892" s="3" t="inlineStr">
@@ -39795,24 +39797,24 @@
       </c>
       <c r="F892" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G892" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data dengan memilih status approvalnya “pending” dan status exportnya “Generate”</t>
+          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
         </is>
       </c>
       <c r="H892" s="4" t="inlineStr">
         <is>
-          <t>1. Jumlah data pada card dan table sesuai</t>
+          <t>1. Menampilkan data sesuai filter yang dipilih</t>
         </is>
       </c>
     </row>
     <row r="893" ht="42" customHeight="1">
       <c r="A893" s="43" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="B893" s="3" t="inlineStr">
@@ -39827,7 +39829,7 @@
       </c>
       <c r="D893" s="4" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Validasi card menunggu approval dengan data table</t>
         </is>
       </c>
       <c r="E893" s="3" t="inlineStr">
@@ -39842,19 +39844,19 @@
       </c>
       <c r="G893" s="4" t="inlineStr">
         <is>
-          <t>1. Input data pada kolom pencarian</t>
+          <t>1. Melakukan filter data dengan memilih status approvalnya “pending” dan status exportnya “Generate”</t>
         </is>
       </c>
       <c r="H893" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai kata kunci</t>
+          <t>1. Jumlah data pada card dan table sesuai</t>
         </is>
       </c>
     </row>
     <row r="894" ht="28" customHeight="1">
       <c r="A894" s="43" t="inlineStr">
         <is>
-          <t>72.4</t>
+          <t>72.3</t>
         </is>
       </c>
       <c r="B894" s="3" t="inlineStr">
@@ -39869,12 +39871,12 @@
       </c>
       <c r="D894" s="4" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Mencari data pada kolom pencarian</t>
         </is>
       </c>
       <c r="E894" s="3" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F894" s="3" t="inlineStr">
@@ -39884,19 +39886,19 @@
       </c>
       <c r="G894" s="4" t="inlineStr">
         <is>
-          <t>1. Input data yang belum terdaftar</t>
+          <t>1. Input data pada kolom pencarian</t>
         </is>
       </c>
       <c r="H894" s="4" t="inlineStr">
         <is>
-          <t>1. Data tidak ditemukan</t>
+          <t>1. Menampilkan data sesuai kata kunci</t>
         </is>
       </c>
     </row>
     <row r="895" ht="42" customHeight="1">
       <c r="A895" s="43" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>72.4</t>
         </is>
       </c>
       <c r="B895" s="3" t="inlineStr">
@@ -39911,34 +39913,34 @@
       </c>
       <c r="D895" s="4" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Mencari data kata kunci salah</t>
         </is>
       </c>
       <c r="E895" s="3" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F895" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G895" s="4" t="inlineStr">
         <is>
-          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
+          <t>1. Input data yang belum terdaftar</t>
         </is>
       </c>
       <c r="H895" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai filter yang dipilih</t>
+          <t>1. Data tidak ditemukan</t>
         </is>
       </c>
     </row>
     <row r="896" ht="14" customHeight="1">
       <c r="A896" s="43" t="inlineStr">
         <is>
-          <t>72.6</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="B896" s="3" t="inlineStr">
@@ -39953,7 +39955,7 @@
       </c>
       <c r="D896" s="4" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Melakukan filter data</t>
         </is>
       </c>
       <c r="E896" s="3" t="inlineStr">
@@ -39963,24 +39965,24 @@
       </c>
       <c r="F896" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G896" s="4" t="inlineStr">
         <is>
-          <t>1. Input data pada kolom pencarian</t>
+          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
         </is>
       </c>
       <c r="H896" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai kata kunci</t>
+          <t>1. Menampilkan data sesuai filter yang dipilih</t>
         </is>
       </c>
     </row>
     <row r="897" ht="42" customHeight="1">
       <c r="A897" s="43" t="inlineStr">
         <is>
-          <t>72.7</t>
+          <t>72.6</t>
         </is>
       </c>
       <c r="B897" s="3" t="inlineStr">
@@ -39995,12 +39997,12 @@
       </c>
       <c r="D897" s="4" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Mencari data pada kolom pencarian</t>
         </is>
       </c>
       <c r="E897" s="3" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F897" s="3" t="inlineStr">
@@ -40010,19 +40012,19 @@
       </c>
       <c r="G897" s="4" t="inlineStr">
         <is>
-          <t>1. Input data yang belum terdaftar</t>
+          <t>1. Input data pada kolom pencarian</t>
         </is>
       </c>
       <c r="H897" s="4" t="inlineStr">
         <is>
-          <t>1. Data tidak ditemukan</t>
+          <t>1. Menampilkan data sesuai kata kunci</t>
         </is>
       </c>
     </row>
     <row r="898" ht="42" customHeight="1">
       <c r="A898" s="43" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>72.7</t>
         </is>
       </c>
       <c r="B898" s="3" t="inlineStr">
@@ -40037,12 +40039,12 @@
       </c>
       <c r="D898" s="4" t="inlineStr">
         <is>
-          <t>Membuka menu Management Export</t>
+          <t>Mencari data kata kunci salah</t>
         </is>
       </c>
       <c r="E898" s="3" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F898" s="3" t="inlineStr">
@@ -40052,19 +40054,19 @@
       </c>
       <c r="G898" s="4" t="inlineStr">
         <is>
-          <t>1. Klik menu exported data management, klik submenu management export</t>
+          <t>1. Input data yang belum terdaftar</t>
         </is>
       </c>
       <c r="H898" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan halaman management export</t>
+          <t>1. Data tidak ditemukan</t>
         </is>
       </c>
     </row>
     <row r="899" ht="28" customHeight="1">
       <c r="A899" s="43" t="inlineStr">
         <is>
-          <t>72.9</t>
+          <t>72.8</t>
         </is>
       </c>
       <c r="B899" s="3" t="inlineStr">
@@ -40079,7 +40081,7 @@
       </c>
       <c r="D899" s="4" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Membuka menu Management Export</t>
         </is>
       </c>
       <c r="E899" s="3" t="inlineStr">
@@ -40089,24 +40091,24 @@
       </c>
       <c r="F899" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G899" s="4" t="inlineStr">
         <is>
-          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
+          <t>1. Klik menu exported data management, klik submenu management export</t>
         </is>
       </c>
       <c r="H899" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai filter yang dipilih</t>
+          <t>1. Menampilkan halaman management export</t>
         </is>
       </c>
     </row>
     <row r="900" ht="42" customHeight="1">
       <c r="A900" s="43" t="inlineStr">
         <is>
-          <t>72.10</t>
+          <t>72.9</t>
         </is>
       </c>
       <c r="B900" s="3" t="inlineStr">
@@ -40121,7 +40123,7 @@
       </c>
       <c r="D900" s="4" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Melakukan filter data</t>
         </is>
       </c>
       <c r="E900" s="3" t="inlineStr">
@@ -40131,24 +40133,24 @@
       </c>
       <c r="F900" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G900" s="4" t="inlineStr">
         <is>
-          <t>1. Input data pada kolom pencarian</t>
+          <t>1. Pilih kantor wilayah, kantor cabang, cabang pembantu, job role, info user, status approval, status export, modul dan tanggal, klik button filter data</t>
         </is>
       </c>
       <c r="H900" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan data sesuai kata kunci</t>
+          <t>1. Menampilkan data sesuai filter yang dipilih</t>
         </is>
       </c>
     </row>
     <row r="901" ht="28" customHeight="1">
       <c r="A901" s="43" t="inlineStr">
         <is>
-          <t>72.11</t>
+          <t>72.10</t>
         </is>
       </c>
       <c r="B901" s="3" t="inlineStr">
@@ -40163,12 +40165,12 @@
       </c>
       <c r="D901" s="4" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Mencari data pada kolom pencarian</t>
         </is>
       </c>
       <c r="E901" s="3" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F901" s="3" t="inlineStr">
@@ -40178,19 +40180,19 @@
       </c>
       <c r="G901" s="4" t="inlineStr">
         <is>
-          <t>1. Input data yang belum terdaftar</t>
+          <t>1. Input data pada kolom pencarian</t>
         </is>
       </c>
       <c r="H901" s="4" t="inlineStr">
         <is>
-          <t>1. Data tidak ditemukan</t>
+          <t>1. Menampilkan data sesuai kata kunci</t>
         </is>
       </c>
     </row>
     <row r="902" ht="28" customHeight="1">
       <c r="A902" s="43" t="inlineStr">
         <is>
-          <t>72.12</t>
+          <t>72.11</t>
         </is>
       </c>
       <c r="B902" s="3" t="inlineStr">
@@ -40205,12 +40207,12 @@
       </c>
       <c r="D902" s="4" t="inlineStr">
         <is>
-          <t>Validasi card menunggu approval dengan data table</t>
+          <t>Mencari data kata kunci salah</t>
         </is>
       </c>
       <c r="E902" s="3" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F902" s="3" t="inlineStr">
@@ -40220,19 +40222,19 @@
       </c>
       <c r="G902" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data dengan memilih status approvalnya “pending” dan status exportnya “Generate”</t>
+          <t>1. Input data yang belum terdaftar</t>
         </is>
       </c>
       <c r="H902" s="4" t="inlineStr">
         <is>
-          <t>1. Jumlah data pada card dan table sesuai</t>
+          <t>1. Data tidak ditemukan</t>
         </is>
       </c>
     </row>
     <row r="903" ht="28" customHeight="1">
       <c r="A903" s="43" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>72.12</t>
         </is>
       </c>
       <c r="B903" s="3" t="inlineStr">
@@ -40247,7 +40249,7 @@
       </c>
       <c r="D903" s="4" t="inlineStr">
         <is>
-          <t>Validasi card data file aktif dengan data table</t>
+          <t>Validasi card menunggu approval dengan data table</t>
         </is>
       </c>
       <c r="E903" s="3" t="inlineStr">
@@ -40257,12 +40259,12 @@
       </c>
       <c r="F903" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G903" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data dengan memilih status approvalnya “Approved” dan status exportnya “Generate” dengan tanggal sebelum hari berjalan</t>
+          <t>1. Melakukan filter data dengan memilih status approvalnya “pending” dan status exportnya “Generate”</t>
         </is>
       </c>
       <c r="H903" s="4" t="inlineStr">
@@ -40274,7 +40276,7 @@
     <row r="904" ht="28" customHeight="1">
       <c r="A904" s="43" t="inlineStr">
         <is>
-          <t>72.14</t>
+          <t>72.13</t>
         </is>
       </c>
       <c r="B904" s="3" t="inlineStr">
@@ -40289,7 +40291,7 @@
       </c>
       <c r="D904" s="4" t="inlineStr">
         <is>
-          <t>Validasi card file kadaluwarsa dengan data table</t>
+          <t>Validasi card data file aktif dengan data table</t>
         </is>
       </c>
       <c r="E904" s="3" t="inlineStr">
@@ -40304,7 +40306,7 @@
       </c>
       <c r="G904" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data dengan memilih status approvalnya “approve” dan status exportnya “generate” dengan tanggal sesudah hari berjalan</t>
+          <t>1. Melakukan filter data dengan memilih status approvalnya “Approved” dan status exportnya “Generate” dengan tanggal sebelum hari berjalan</t>
         </is>
       </c>
       <c r="H904" s="4" t="inlineStr">
@@ -40316,7 +40318,7 @@
     <row r="905" ht="28" customHeight="1">
       <c r="A905" s="43" t="inlineStr">
         <is>
-          <t>72.15</t>
+          <t>72.14</t>
         </is>
       </c>
       <c r="B905" s="3" t="inlineStr">
@@ -40331,7 +40333,7 @@
       </c>
       <c r="D905" s="4" t="inlineStr">
         <is>
-          <t>Validasi card reject dengan data table</t>
+          <t>Validasi card file kadaluwarsa dengan data table</t>
         </is>
       </c>
       <c r="E905" s="3" t="inlineStr">
@@ -40341,12 +40343,12 @@
       </c>
       <c r="F905" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G905" s="4" t="inlineStr">
         <is>
-          <t>1. Melakukan filter data dengan memilih status approvalnya “reject” dan status exportnya “generate”</t>
+          <t>1. Melakukan filter data dengan memilih status approvalnya “approve” dan status exportnya “generate” dengan tanggal sesudah hari berjalan</t>
         </is>
       </c>
       <c r="H905" s="4" t="inlineStr">
@@ -40358,7 +40360,7 @@
     <row r="906" ht="42" customHeight="1">
       <c r="A906" s="43" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>72.15</t>
         </is>
       </c>
       <c r="B906" s="3" t="inlineStr">
@@ -40368,12 +40370,12 @@
       </c>
       <c r="C906" s="3" t="inlineStr">
         <is>
-          <t>Persetujuan export</t>
+          <t>Management export</t>
         </is>
       </c>
       <c r="D906" s="4" t="inlineStr">
         <is>
-          <t>Lakukan login menggunakan user monitoring</t>
+          <t>Validasi card reject dengan data table</t>
         </is>
       </c>
       <c r="E906" s="3" t="inlineStr">
@@ -40383,24 +40385,24 @@
       </c>
       <c r="F906" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G906" s="4" t="inlineStr">
         <is>
-          <t>1. Login menggunakan user monitoring</t>
+          <t>1. Melakukan filter data dengan memilih status approvalnya “reject” dan status exportnya “generate”</t>
         </is>
       </c>
       <c r="H906" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil melakukan login</t>
+          <t>1. Jumlah data pada card dan table sesuai</t>
         </is>
       </c>
     </row>
     <row r="907" ht="42" customHeight="1">
       <c r="A907" s="43" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B907" s="3" t="inlineStr">
@@ -40415,7 +40417,7 @@
       </c>
       <c r="D907" s="4" t="inlineStr">
         <is>
-          <t>Membuka menu Persetujuan Export</t>
+          <t>Lakukan login menggunakan user monitoring</t>
         </is>
       </c>
       <c r="E907" s="3" t="inlineStr">
@@ -40425,59 +40427,101 @@
       </c>
       <c r="F907" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G907" s="4" t="inlineStr">
         <is>
-          <t>1. Klik menu exported data management, klik submenu persetujuan export</t>
+          <t>1. Login menggunakan user monitoring</t>
         </is>
       </c>
       <c r="H907" s="4" t="inlineStr">
         <is>
-          <t>1. Menampilkan halaman persetujuan export</t>
+          <t>1. Berhasil melakukan login</t>
         </is>
       </c>
     </row>
     <row r="908" ht="28" customHeight="1">
       <c r="A908" s="43" t="inlineStr">
         <is>
+          <t>73.2</t>
+        </is>
+      </c>
+      <c r="B908" s="3" t="inlineStr">
+        <is>
+          <t>Export data management</t>
+        </is>
+      </c>
+      <c r="C908" s="3" t="inlineStr">
+        <is>
+          <t>Persetujuan export</t>
+        </is>
+      </c>
+      <c r="D908" s="4" t="inlineStr">
+        <is>
+          <t>Membuka menu Persetujuan Export</t>
+        </is>
+      </c>
+      <c r="E908" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F908" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G908" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik menu exported data management, klik submenu persetujuan export</t>
+        </is>
+      </c>
+      <c r="H908" s="4" t="inlineStr">
+        <is>
+          <t>1. Menampilkan halaman persetujuan export</t>
+        </is>
+      </c>
+    </row>
+    <row r="909" ht="14" customHeight="1">
+      <c r="A909" s="43" t="inlineStr">
+        <is>
           <t>73.3</t>
         </is>
       </c>
-      <c r="B908" s="3" t="inlineStr">
+      <c r="B909" s="3" t="inlineStr">
         <is>
           <t>Export data management</t>
         </is>
       </c>
-      <c r="C908" s="3" t="inlineStr">
+      <c r="C909" s="3" t="inlineStr">
         <is>
           <t>Persetujuan export</t>
         </is>
       </c>
-      <c r="D908" s="4" t="inlineStr">
+      <c r="D909" s="4" t="inlineStr">
         <is>
           <t>Melakukan approval data pengajuan export</t>
         </is>
       </c>
-      <c r="E908" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F908" s="3" t="inlineStr">
+      <c r="E909" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F909" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G908" s="4" t="inlineStr">
+      <c r="G909" s="4" t="inlineStr">
         <is>
           <t>1. Klik icon titik tiga pada data pengajuan.
 2. Klik menu Setuju.
 3. Klik button YA pada popup konfirmasi.</t>
         </is>
       </c>
-      <c r="H908" s="4" t="inlineStr">
+      <c r="H909" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan menu opsi.
 2. Berhasil menampilkan popup konfirmasi.
@@ -40485,49 +40529,48 @@
         </is>
       </c>
     </row>
-    <row r="909" ht="14" customHeight="1">
-      <c r="A909" s="43" t="inlineStr">
+    <row r="910" ht="28" customHeight="1">
+      <c r="A910" s="43" t="inlineStr">
         <is>
           <t>73.4</t>
         </is>
       </c>
-      <c r="B909" s="3" t="inlineStr">
+      <c r="B910" s="3" t="inlineStr">
         <is>
           <t>Export data management</t>
         </is>
       </c>
-      <c r="C909" s="3" t="inlineStr">
+      <c r="C910" s="3" t="inlineStr">
         <is>
           <t>Persetujuan export</t>
         </is>
       </c>
-      <c r="D909" s="4" t="inlineStr">
+      <c r="D910" s="4" t="inlineStr">
         <is>
           <t>Melakukan reject data pengajuan export</t>
         </is>
       </c>
-      <c r="E909" s="3" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F909" s="3" t="inlineStr">
+      <c r="E910" s="3" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F910" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G909" s="4" t="inlineStr">
+      <c r="G910" s="4" t="inlineStr">
         <is>
           <t>1. Klik icon (titik tiga) klik tolak, input alasan, klik submit</t>
         </is>
       </c>
-      <c r="H909" s="4" t="inlineStr">
+      <c r="H910" s="4" t="inlineStr">
         <is>
           <t>1. Berhasil melakukan reject data</t>
         </is>
       </c>
     </row>
-    <row r="910" ht="28" customHeight="1"/>
     <row r="911" ht="28" customHeight="1"/>
     <row r="912" ht="28" customHeight="1"/>
     <row r="913" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
docs(modul-65): update TC 65.2 title to Menampilkan data Personal Funnel berdasarkan tab
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -37073,7 +37073,7 @@
       </c>
       <c r="D831" s="4" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Non PKS dan PKS</t>
+          <t>Menampilkan data Personal Funnel berdasarkan tab</t>
         </is>
       </c>
       <c r="E831" s="3" t="inlineStr">
@@ -37094,8 +37094,8 @@
       </c>
       <c r="H831" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data pada tab Non PKS.
-2. Berhasil menampilkan data pada tab PKS.</t>
+          <t>1. Berhasil menampilkan data Personal Funnel pada tab Non PKS.
+2. Berhasil menampilkan data Personal Funnel pada tab PKS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(modul-65): sync, crop, and embed screenshots for TC 65.2 into docx and excels
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -37088,14 +37088,16 @@
       </c>
       <c r="G831" s="4" t="inlineStr">
         <is>
-          <t>1. Klik tab Non PKS.
-2. Klik tab PKS.</t>
+          <t>1. Klik tab Semua.
+2. Klik tab Non PKS.
+3. Klik tab PKS.</t>
         </is>
       </c>
       <c r="H831" s="4" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data Personal Funnel pada tab Non PKS.
-2. Berhasil menampilkan data Personal Funnel pada tab PKS.</t>
+          <t>1. Berhasil menampilkan data Personal Funnel pada tab Semua.
+2. Berhasil menampilkan data Personal Funnel pada tab Non PKS.
+3. Berhasil menampilkan data Personal Funnel pada tab PKS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hasil-uji): sync 47 new senior test cases (73 screenshots) across Hasil Uji, SIT docx, and Test Case xlsx
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z982"/>
+  <dimension ref="A1:Z994"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43630,18 +43630,510 @@
         </is>
       </c>
     </row>
-    <row r="983" ht="28" customHeight="1"/>
-    <row r="984" ht="140" customHeight="1"/>
-    <row r="985" ht="14" customHeight="1"/>
-    <row r="986" ht="14" customHeight="1"/>
-    <row r="987" ht="42" customHeight="1"/>
-    <row r="988" ht="14" customHeight="1"/>
-    <row r="989" ht="70" customHeight="1"/>
-    <row r="990" ht="168" customHeight="1"/>
-    <row r="991" ht="14" customHeight="1"/>
-    <row r="992" ht="14" customHeight="1"/>
-    <row r="993" ht="70" customHeight="1"/>
-    <row r="994" ht="28" customHeight="1"/>
+    <row r="983" ht="28" customHeight="1">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>15.11</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Bisnis dan Produk</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Group Produk</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Melakukan validasi data hasil export</t>
+        </is>
+      </c>
+      <c r="E983" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data pada excel sesuai dengan data pada tabel – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="984" ht="140" customHeight="1">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>23.6</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Menampilkan detail batch</t>
+        </is>
+      </c>
+      <c r="E984" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil menampilkan data detail – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="985" ht="14" customHeight="1">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>23.7</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Download source File</t>
+        </is>
+      </c>
+      <c r="E985" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data source berhasil didownload – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="986" ht="14" customHeight="1">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>23.8</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Menampilkan preview data</t>
+        </is>
+      </c>
+      <c r="E986" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil menampilkan detail data hasil upload dan penjelasan jika terdapat validasi error pada file yang diupload – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="987" ht="42" customHeight="1">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>23.9</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Menghapus batch data</t>
+        </is>
+      </c>
+      <c r="E987" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data berhasil dihapus – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="988" ht="14" customHeight="1">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>23.10</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Download error file</t>
+        </is>
+      </c>
+      <c r="E988" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil mendownload error file – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="989" ht="70" customHeight="1">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>23.11</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>Batalkan batch</t>
+        </is>
+      </c>
+      <c r="E989" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil membatalkan batch – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="990" ht="168" customHeight="1">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>23.12</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Upload Bulk</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Upload Target Bulk</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Upload ulang file gagal</t>
+        </is>
+      </c>
+      <c r="E990" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil mengupload ulang file– [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="991" ht="14" customHeight="1">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>46.16</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Approval Target Growth</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Mencari data kata kunci yang tidak sesuai</t>
+        </is>
+      </c>
+      <c r="E991" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data tidak ditemukan – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="992" ht="14" customHeight="1">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>47.6</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Approval Sales Code</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Melihat detail data</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Berhasil menampilkan detail data – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="993" ht="70" customHeight="1">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>47.8</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Approval Sales Code</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Mencari data kata kunci invalid</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data tidak ditemukan – [Success]</t>
+        </is>
+      </c>
+    </row>
+    <row r="994" ht="28" customHeight="1">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>58.7</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Pipeline - Setting Validate Pipeline</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Mencari data kata kunci tidak valid (Negative test)</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>Hasil yang diharapkan [STATUS]: Data Tidak ditemukan – [Success]</t>
+        </is>
+      </c>
+    </row>
     <row r="995" ht="28" customHeight="1"/>
     <row r="996" ht="42" customHeight="1"/>
     <row r="997" ht="42" customHeight="1"/>

</xml_diff>

<commit_message>
feat(mobile): add 14 new test cases for Modul 15 Agenda - Pengingat (empty screenshots)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -49149,7 +49149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA214"/>
+  <dimension ref="A1:AA222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59670,14 +59670,14 @@
       </c>
       <c r="G185" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Pengingat.</t>
+          <t>1. Buka menu Lainnya pada Aksi Cepat di Beranda.
+2. Klik menu Pengingat pada kelompok Agenda.</t>
         </is>
       </c>
       <c r="H185" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Pengingat.</t>
+2. Berhasil menampilkan halaman Pengingat beserta daftar tugas pada tab default (Task).</t>
         </is>
       </c>
       <c r="I185" s="49" t="n"/>
@@ -59718,7 +59718,7 @@
       </c>
       <c r="D186" s="48" t="inlineStr">
         <is>
-          <t>Melihat daftar pengingat pada tab Aktif</t>
+          <t>Melihat daftar agenda pada tab Acara</t>
         </is>
       </c>
       <c r="E186" s="46" t="inlineStr">
@@ -59733,12 +59733,13 @@
       </c>
       <c r="G186" s="48" t="inlineStr">
         <is>
-          <t>1. Klik tab Aktif.</t>
+          <t>1. Pada halaman Pengingat, klik tab Acara.</t>
         </is>
       </c>
       <c r="H186" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan daftar pengingat yang sedang aktif.</t>
+          <t>1. Berhasil berpindah ke tab Acara.
+2. Berhasil menampilkan daftar acara yang terdaftar pada tab Acara.</t>
         </is>
       </c>
       <c r="I186" s="49" t="n"/>
@@ -59779,7 +59780,7 @@
       </c>
       <c r="D187" s="48" t="inlineStr">
         <is>
-          <t>Melihat daftar pengingat pada tab Selesai</t>
+          <t>Melihat detail task</t>
         </is>
       </c>
       <c r="E187" s="46" t="inlineStr">
@@ -59789,17 +59790,18 @@
       </c>
       <c r="F187" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G187" s="48" t="inlineStr">
         <is>
-          <t>1. Klik tab Selesai.</t>
+          <t>1. Pada tab Task, klik salah satu card task yang terdaftar.</t>
         </is>
       </c>
       <c r="H187" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan daftar pengingat yang sudah selesai.</t>
+          <t>1. Berhasil membuka halaman Detail Task.
+2. Berhasil menampilkan informasi status, visibilitas, prioritas, tenggat, zona waktu, pemilik, deskripsi, dan lampiran.</t>
         </is>
       </c>
       <c r="I187" s="49" t="n"/>
@@ -59840,7 +59842,7 @@
       </c>
       <c r="D188" s="48" t="inlineStr">
         <is>
-          <t>Menambahkan pengingat baru dengan data valid</t>
+          <t>Mengubah data task dengan data valid</t>
         </is>
       </c>
       <c r="E188" s="46" t="inlineStr">
@@ -59855,16 +59857,15 @@
       </c>
       <c r="G188" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button + Baru.
-2. Mengisi seluruh field mandatory pada form Tambah Pengingat dengan data valid.
+          <t>1. Pada halaman Detail Task, klik icon Edit (pensil).
+2. Ubah data task pada form Edit Task.
 3. Klik button Simpan.</t>
         </is>
       </c>
       <c r="H188" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Tambah Pengingat.
-2. Berhasil mengisi seluruh field mandatory pada form Tambah Pengingat.
-3. Berhasil menyimpan pengingat dan menampilkan pengingat baru pada daftar.</t>
+          <t>1. Berhasil membuka form Edit Task.
+2. Berhasil menyimpan perubahan data task dengan data yang valid.</t>
         </is>
       </c>
       <c r="I188" s="49" t="n"/>
@@ -59905,31 +59906,30 @@
       </c>
       <c r="D189" s="48" t="inlineStr">
         <is>
-          <t>Menambahkan pengingat baru tanpa mengisi field mandatory</t>
+          <t>Membagikan task kepada user</t>
         </is>
       </c>
       <c r="E189" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F189" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G189" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button + Baru.
-2. Mengosongkan seluruh field mandatory pada form Tambah Pengingat.
-3. Klik button Simpan.</t>
+          <t>1. Pada halaman Detail Task, klik icon Bagikan (share).
+2. Pilih role atau user yang ditugaskan.
+3. Klik button Bagikan.</t>
         </is>
       </c>
       <c r="H189" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Tambah Pengingat.
-2. Field mandatory berhasil dikosongkan.
-3. Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>1. Berhasil membuka form Bagikan Task.
+2. Berhasil membagikan task kepada user dan menampilkan pesan konfirmasi Task berhasil dibagikan.</t>
         </is>
       </c>
       <c r="I189" s="49" t="n"/>
@@ -59970,7 +59970,7 @@
       </c>
       <c r="D190" s="48" t="inlineStr">
         <is>
-          <t>Menandai pengingat sebagai selesai</t>
+          <t>Menghapus penugasan task kepada user</t>
         </is>
       </c>
       <c r="E190" s="46" t="inlineStr">
@@ -59985,14 +59985,15 @@
       </c>
       <c r="G190" s="48" t="inlineStr">
         <is>
-          <t>1. Centang checkbox pada salah satu card pengingat aktif.
-2. Klik button Ya pada pop-up konfirmasi.</t>
+          <t>1. Pada form Bagikan Task, periksa daftar Ditugaskan ke (User).
+2. Klik icon hapus (tempat sampah) pada user yang ditugaskan.
+3. Konfirmasi penghapusan penugasan task.</t>
         </is>
       </c>
       <c r="H190" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan pop-up konfirmasi selesai.
-2. Berhasil menandai pengingat sebagai selesai dan memindahkan pengingat ke tab Selesai.</t>
+          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan penugasan.
+2. Berhasil menghapus penugasan task kepada user dari daftar pembagian task.</t>
         </is>
       </c>
       <c r="I190" s="49" t="n"/>
@@ -60018,538 +60019,402 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
+          <t>15.7</t>
+        </is>
+      </c>
+      <c r="B191" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C191" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D191" s="48" t="inlineStr">
+        <is>
+          <t>Menambahkan komentar pada task</t>
+        </is>
+      </c>
+      <c r="E191" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F191" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G191" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Task, klik tab Aktivitas &amp; Percakapan.
+2. Tulis komentar pada kolom Tulis komentar.
+3. Klik button Kirim.</t>
+        </is>
+      </c>
+      <c r="H191" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menginput teks komentar.
+2. Berhasil mengirimkan komentar dan menampilkan komentar baru pada daftar riwayat aktivitas task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>15.8</t>
+        </is>
+      </c>
+      <c r="B192" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C192" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D192" s="48" t="inlineStr">
+        <is>
+          <t>Menghapus komentar pada task</t>
+        </is>
+      </c>
+      <c r="E192" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F192" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G192" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Task, klik tab Aktivitas &amp; Percakapan.
+2. Klik icon hapus (tempat sampah) pada komentar yang ingin dihapus.
+3. Konfirmasi penghapusan komentar.</t>
+        </is>
+      </c>
+      <c r="H192" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan komentar.
+2. Berhasil menghapus komentar dari daftar aktivitas dan percakapan task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>15.9</t>
+        </is>
+      </c>
+      <c r="B193" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C193" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D193" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail acara</t>
+        </is>
+      </c>
+      <c r="E193" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F193" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G193" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada tab Acara, klik salah satu card acara yang terdaftar.</t>
+        </is>
+      </c>
+      <c r="H193" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka halaman Detail Acara.
+2. Berhasil menampilkan informasi status, visibilitas, tanggal/waktu mulai &amp; selesai, zona waktu, dan pemilik acara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="B194" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C194" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D194" s="48" t="inlineStr">
+        <is>
+          <t>Mengubah data acara dengan data valid</t>
+        </is>
+      </c>
+      <c r="E194" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F194" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G194" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Acara, klik icon Edit (pensil).
+2. Ubah data acara pada form Edit Acara.
+3. Klik button Simpan.</t>
+        </is>
+      </c>
+      <c r="H194" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka form Edit Acara.
+2. Berhasil menyimpan perubahan data acara dengan data yang valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>15.11</t>
+        </is>
+      </c>
+      <c r="B195" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C195" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D195" s="48" t="inlineStr">
+        <is>
+          <t>Membagikan acara kepada user</t>
+        </is>
+      </c>
+      <c r="E195" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F195" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G195" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Acara, klik icon Bagikan (share).
+2. Tentukan user watcher/assignee pada form Bagikan Acara.
+3. Klik button Bagikan.</t>
+        </is>
+      </c>
+      <c r="H195" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka form Bagikan Acara.
+2. Berhasil membagikan acara kepada user dan memicu notifikasi kepada penerima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>15.12</t>
+        </is>
+      </c>
+      <c r="B196" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C196" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D196" s="48" t="inlineStr">
+        <is>
+          <t>Menghapus penugasan acara kepada user</t>
+        </is>
+      </c>
+      <c r="E196" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F196" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G196" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada form Bagikan Acara, periksa daftar Ditugaskan ke (User).
+2. Klik icon hapus (tempat sampah) pada user yang ditugaskan.
+3. Konfirmasi penghapusan penugasan acara.</t>
+        </is>
+      </c>
+      <c r="H196" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan penugasan.
+2. Berhasil menghapus penugasan acara kepada user dari daftar pembagian acara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>15.13</t>
+        </is>
+      </c>
+      <c r="B197" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C197" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D197" s="48" t="inlineStr">
+        <is>
+          <t>Menambahkan komentar pada acara</t>
+        </is>
+      </c>
+      <c r="E197" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F197" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G197" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Acara, klik tab Aktivitas &amp; Percakapan.
+2. Tulis komentar pada kolom Tulis komentar.
+3. Klik button Kirim.</t>
+        </is>
+      </c>
+      <c r="H197" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menginput teks komentar.
+2. Berhasil mengirimkan komentar dan menampilkan komentar baru pada daftar riwayat aktivitas acara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15.14</t>
+        </is>
+      </c>
+      <c r="B198" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C198" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D198" s="48" t="inlineStr">
+        <is>
+          <t>Menghapus komentar pada acara</t>
+        </is>
+      </c>
+      <c r="E198" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F198" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G198" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Acara, klik tab Aktivitas &amp; Percakapan.
+2. Klik icon hapus (tempat sampah) pada komentar yang ingin dihapus.
+3. Konfirmasi penghapusan komentar.</t>
+        </is>
+      </c>
+      <c r="H198" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan komentar.
+2. Berhasil menghapus komentar dari daftar aktivitas dan percakapan acara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
           <t>16.1</t>
         </is>
       </c>
-      <c r="B191" s="46" t="inlineStr">
+      <c r="B199" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C191" s="46" t="inlineStr">
+      <c r="C199" s="46" t="inlineStr">
         <is>
           <t>Daily Sales Agenda</t>
         </is>
       </c>
-      <c r="D191" s="48" t="inlineStr">
+      <c r="D199" s="48" t="inlineStr">
         <is>
           <t>Membuka halaman Daily Sales Agenda</t>
         </is>
       </c>
-      <c r="E191" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F191" s="46" t="inlineStr">
+      <c r="E199" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F199" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G191" s="48" t="inlineStr">
+      <c r="G199" s="48" t="inlineStr">
         <is>
           <t>1. Buka menu Lainnya.
 2. Klik menu Daily Sales Agenda.</t>
         </is>
       </c>
-      <c r="H191" s="48" t="inlineStr">
+      <c r="H199" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu Lainnya.
 2. Berhasil menampilkan halaman Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I191" s="49" t="n"/>
-      <c r="J191" s="49" t="n"/>
-      <c r="K191" s="49" t="n"/>
-      <c r="L191" s="49" t="n"/>
-      <c r="M191" s="49" t="n"/>
-      <c r="N191" s="49" t="n"/>
-      <c r="O191" s="49" t="n"/>
-      <c r="P191" s="49" t="n"/>
-      <c r="Q191" s="49" t="n"/>
-      <c r="R191" s="49" t="n"/>
-      <c r="S191" s="49" t="n"/>
-      <c r="T191" s="49" t="n"/>
-      <c r="U191" s="49" t="n"/>
-      <c r="V191" s="49" t="n"/>
-      <c r="W191" s="49" t="n"/>
-      <c r="X191" s="49" t="n"/>
-      <c r="Y191" s="49" t="n"/>
-      <c r="Z191" s="49" t="n"/>
-      <c r="AA191" s="49" t="n"/>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>16.2</t>
-        </is>
-      </c>
-      <c r="B192" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C192" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D192" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Masuk</t>
-        </is>
-      </c>
-      <c r="E192" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F192" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G192" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Masuk.</t>
-        </is>
-      </c>
-      <c r="H192" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah yang masuk pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I192" s="49" t="n"/>
-      <c r="J192" s="49" t="n"/>
-      <c r="K192" s="49" t="n"/>
-      <c r="L192" s="49" t="n"/>
-      <c r="M192" s="49" t="n"/>
-      <c r="N192" s="49" t="n"/>
-      <c r="O192" s="49" t="n"/>
-      <c r="P192" s="49" t="n"/>
-      <c r="Q192" s="49" t="n"/>
-      <c r="R192" s="49" t="n"/>
-      <c r="S192" s="49" t="n"/>
-      <c r="T192" s="49" t="n"/>
-      <c r="U192" s="49" t="n"/>
-      <c r="V192" s="49" t="n"/>
-      <c r="W192" s="49" t="n"/>
-      <c r="X192" s="49" t="n"/>
-      <c r="Y192" s="49" t="n"/>
-      <c r="Z192" s="49" t="n"/>
-      <c r="AA192" s="49" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>16.3</t>
-        </is>
-      </c>
-      <c r="B193" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C193" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D193" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Closing</t>
-        </is>
-      </c>
-      <c r="E193" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F193" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G193" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Closing.</t>
-        </is>
-      </c>
-      <c r="H193" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah yang closing pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I193" s="49" t="n"/>
-      <c r="J193" s="49" t="n"/>
-      <c r="K193" s="49" t="n"/>
-      <c r="L193" s="49" t="n"/>
-      <c r="M193" s="49" t="n"/>
-      <c r="N193" s="49" t="n"/>
-      <c r="O193" s="49" t="n"/>
-      <c r="P193" s="49" t="n"/>
-      <c r="Q193" s="49" t="n"/>
-      <c r="R193" s="49" t="n"/>
-      <c r="S193" s="49" t="n"/>
-      <c r="T193" s="49" t="n"/>
-      <c r="U193" s="49" t="n"/>
-      <c r="V193" s="49" t="n"/>
-      <c r="W193" s="49" t="n"/>
-      <c r="X193" s="49" t="n"/>
-      <c r="Y193" s="49" t="n"/>
-      <c r="Z193" s="49" t="n"/>
-      <c r="AA193" s="49" t="n"/>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>16.4</t>
-        </is>
-      </c>
-      <c r="B194" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C194" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D194" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Referral</t>
-        </is>
-      </c>
-      <c r="E194" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F194" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G194" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Referral.</t>
-        </is>
-      </c>
-      <c r="H194" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah referral pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I194" s="49" t="n"/>
-      <c r="J194" s="49" t="n"/>
-      <c r="K194" s="49" t="n"/>
-      <c r="L194" s="49" t="n"/>
-      <c r="M194" s="49" t="n"/>
-      <c r="N194" s="49" t="n"/>
-      <c r="O194" s="49" t="n"/>
-      <c r="P194" s="49" t="n"/>
-      <c r="Q194" s="49" t="n"/>
-      <c r="R194" s="49" t="n"/>
-      <c r="S194" s="49" t="n"/>
-      <c r="T194" s="49" t="n"/>
-      <c r="U194" s="49" t="n"/>
-      <c r="V194" s="49" t="n"/>
-      <c r="W194" s="49" t="n"/>
-      <c r="X194" s="49" t="n"/>
-      <c r="Y194" s="49" t="n"/>
-      <c r="Z194" s="49" t="n"/>
-      <c r="AA194" s="49" t="n"/>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>16.5</t>
-        </is>
-      </c>
-      <c r="B195" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C195" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D195" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Ref. Closing</t>
-        </is>
-      </c>
-      <c r="E195" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F195" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G195" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Ref. Closing.</t>
-        </is>
-      </c>
-      <c r="H195" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah referral yang closing pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I195" s="49" t="n"/>
-      <c r="J195" s="49" t="n"/>
-      <c r="K195" s="49" t="n"/>
-      <c r="L195" s="49" t="n"/>
-      <c r="M195" s="49" t="n"/>
-      <c r="N195" s="49" t="n"/>
-      <c r="O195" s="49" t="n"/>
-      <c r="P195" s="49" t="n"/>
-      <c r="Q195" s="49" t="n"/>
-      <c r="R195" s="49" t="n"/>
-      <c r="S195" s="49" t="n"/>
-      <c r="T195" s="49" t="n"/>
-      <c r="U195" s="49" t="n"/>
-      <c r="V195" s="49" t="n"/>
-      <c r="W195" s="49" t="n"/>
-      <c r="X195" s="49" t="n"/>
-      <c r="Y195" s="49" t="n"/>
-      <c r="Z195" s="49" t="n"/>
-      <c r="AA195" s="49" t="n"/>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>16.6</t>
-        </is>
-      </c>
-      <c r="B196" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C196" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D196" s="48" t="inlineStr">
-        <is>
-          <t>Mencari agenda menggunakan Search Bar</t>
-        </is>
-      </c>
-      <c r="E196" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F196" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G196" s="48" t="inlineStr">
-        <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
-        </is>
-      </c>
-      <c r="H196" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan data agenda yang sesuai dengan kata kunci pencarian.</t>
-        </is>
-      </c>
-      <c r="I196" s="49" t="n"/>
-      <c r="J196" s="49" t="n"/>
-      <c r="K196" s="49" t="n"/>
-      <c r="L196" s="49" t="n"/>
-      <c r="M196" s="49" t="n"/>
-      <c r="N196" s="49" t="n"/>
-      <c r="O196" s="49" t="n"/>
-      <c r="P196" s="49" t="n"/>
-      <c r="Q196" s="49" t="n"/>
-      <c r="R196" s="49" t="n"/>
-      <c r="S196" s="49" t="n"/>
-      <c r="T196" s="49" t="n"/>
-      <c r="U196" s="49" t="n"/>
-      <c r="V196" s="49" t="n"/>
-      <c r="W196" s="49" t="n"/>
-      <c r="X196" s="49" t="n"/>
-      <c r="Y196" s="49" t="n"/>
-      <c r="Z196" s="49" t="n"/>
-      <c r="AA196" s="49" t="n"/>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>16.7</t>
-        </is>
-      </c>
-      <c r="B197" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C197" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D197" s="48" t="inlineStr">
-        <is>
-          <t>Mencari agenda dengan keyword tidak valid</t>
-        </is>
-      </c>
-      <c r="E197" s="46" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F197" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G197" s="48" t="inlineStr">
-        <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
-        </is>
-      </c>
-      <c r="H197" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-      <c r="I197" s="49" t="n"/>
-      <c r="J197" s="49" t="n"/>
-      <c r="K197" s="49" t="n"/>
-      <c r="L197" s="49" t="n"/>
-      <c r="M197" s="49" t="n"/>
-      <c r="N197" s="49" t="n"/>
-      <c r="O197" s="49" t="n"/>
-      <c r="P197" s="49" t="n"/>
-      <c r="Q197" s="49" t="n"/>
-      <c r="R197" s="49" t="n"/>
-      <c r="S197" s="49" t="n"/>
-      <c r="T197" s="49" t="n"/>
-      <c r="U197" s="49" t="n"/>
-      <c r="V197" s="49" t="n"/>
-      <c r="W197" s="49" t="n"/>
-      <c r="X197" s="49" t="n"/>
-      <c r="Y197" s="49" t="n"/>
-      <c r="Z197" s="49" t="n"/>
-      <c r="AA197" s="49" t="n"/>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>16.8</t>
-        </is>
-      </c>
-      <c r="B198" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C198" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D198" s="48" t="inlineStr">
-        <is>
-          <t>Melakukan filter data Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="E198" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F198" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G198" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik button Filter.
-2. Pilih kriteria filter pada form Filter (Product, Bulan, Tahun).
-3. Klik button Submit.</t>
-        </is>
-      </c>
-      <c r="H198" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil membuka form Filter.
-2. Berhasil memilih kriteria filter.
-3. Berhasil menampilkan data Daily Sales Agenda sesuai filter yang dipilih.</t>
-        </is>
-      </c>
-      <c r="I198" s="49" t="n"/>
-      <c r="J198" s="49" t="n"/>
-      <c r="K198" s="49" t="n"/>
-      <c r="L198" s="49" t="n"/>
-      <c r="M198" s="49" t="n"/>
-      <c r="N198" s="49" t="n"/>
-      <c r="O198" s="49" t="n"/>
-      <c r="P198" s="49" t="n"/>
-      <c r="Q198" s="49" t="n"/>
-      <c r="R198" s="49" t="n"/>
-      <c r="S198" s="49" t="n"/>
-      <c r="T198" s="49" t="n"/>
-      <c r="U198" s="49" t="n"/>
-      <c r="V198" s="49" t="n"/>
-      <c r="W198" s="49" t="n"/>
-      <c r="X198" s="49" t="n"/>
-      <c r="Y198" s="49" t="n"/>
-      <c r="Z198" s="49" t="n"/>
-      <c r="AA198" s="49" t="n"/>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>17.1</t>
-        </is>
-      </c>
-      <c r="B199" s="46" t="inlineStr">
-        <is>
-          <t>Fitur</t>
-        </is>
-      </c>
-      <c r="C199" s="46" t="inlineStr">
-        <is>
-          <t>Marketing Toolkit</t>
-        </is>
-      </c>
-      <c r="D199" s="48" t="inlineStr">
-        <is>
-          <t>Membuka halaman Marketing Toolkit</t>
-        </is>
-      </c>
-      <c r="E199" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F199" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G199" s="48" t="inlineStr">
-        <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Marketing Toolkit.</t>
-        </is>
-      </c>
-      <c r="H199" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I199" s="49" t="n"/>
@@ -60575,22 +60440,22 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>17.2</t>
+          <t>16.2</t>
         </is>
       </c>
       <c r="B200" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C200" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D200" s="48" t="inlineStr">
         <is>
-          <t>Mengubah tampilan folder menjadi List View</t>
+          <t>Melihat daftar agenda pada tab Masuk</t>
         </is>
       </c>
       <c r="E200" s="46" t="inlineStr">
@@ -60605,12 +60470,12 @@
       </c>
       <c r="G200" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon tampilan List pada halaman Marketing Toolkit.</t>
+          <t>1. Klik tab Masuk.</t>
         </is>
       </c>
       <c r="H200" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengubah tampilan folder menjadi List View.</t>
+          <t>1. Berhasil menampilkan daftar nasabah yang masuk pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I200" s="49" t="n"/>
@@ -60636,22 +60501,22 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>17.3</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="B201" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C201" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D201" s="48" t="inlineStr">
         <is>
-          <t>Mengubah tampilan folder menjadi Grid View</t>
+          <t>Melihat daftar agenda pada tab Closing</t>
         </is>
       </c>
       <c r="E201" s="46" t="inlineStr">
@@ -60666,12 +60531,12 @@
       </c>
       <c r="G201" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon tampilan Grid pada halaman Marketing Toolkit.</t>
+          <t>1. Klik tab Closing.</t>
         </is>
       </c>
       <c r="H201" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengubah tampilan folder menjadi Grid View.</t>
+          <t>1. Berhasil menampilkan daftar nasabah yang closing pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I201" s="49" t="n"/>
@@ -60697,22 +60562,22 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>16.4</t>
         </is>
       </c>
       <c r="B202" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C202" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D202" s="48" t="inlineStr">
         <is>
-          <t>Membuka folder pada Marketing Toolkit</t>
+          <t>Melihat daftar agenda pada tab Referral</t>
         </is>
       </c>
       <c r="E202" s="46" t="inlineStr">
@@ -60722,17 +60587,17 @@
       </c>
       <c r="F202" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G202" s="48" t="inlineStr">
         <is>
-          <t>1. Klik salah satu folder pada daftar Folder.</t>
+          <t>1. Klik tab Referral.</t>
         </is>
       </c>
       <c r="H202" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka folder Marketing Toolkit.</t>
+          <t>1. Berhasil menampilkan daftar nasabah referral pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I202" s="49" t="n"/>
@@ -60758,22 +60623,22 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>17.5</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="B203" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C203" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D203" s="48" t="inlineStr">
         <is>
-          <t>Mencari konten di dalam folder menggunakan Search Bar</t>
+          <t>Melihat daftar agenda pada tab Ref. Closing</t>
         </is>
       </c>
       <c r="E203" s="46" t="inlineStr">
@@ -60783,17 +60648,17 @@
       </c>
       <c r="F203" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G203" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
+          <t>1. Klik tab Ref. Closing.</t>
         </is>
       </c>
       <c r="H203" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data yang sesuai dengan kata kunci pencarian.</t>
+          <t>1. Berhasil menampilkan daftar nasabah referral yang closing pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I203" s="49" t="n"/>
@@ -60819,42 +60684,42 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>17.6</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="B204" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C204" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D204" s="48" t="inlineStr">
         <is>
-          <t>Mencari konten di dalam folder dengan keyword tidak valid</t>
+          <t>Mencari agenda menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E204" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F204" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G204" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H204" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>1. Berhasil menampilkan data agenda yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I204" s="49" t="n"/>
@@ -60880,42 +60745,42 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>17.7</t>
+          <t>16.7</t>
         </is>
       </c>
       <c r="B205" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C205" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D205" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail konten Marketing Toolkit</t>
+          <t>Mencari agenda dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E205" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F205" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G205" s="48" t="inlineStr">
         <is>
-          <t>1. Klik salah satu sub-folder pada daftar folder.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H205" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail konten Marketing Toolkit.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I205" s="49" t="n"/>
@@ -60941,22 +60806,22 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>16.8</t>
         </is>
       </c>
       <c r="B206" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C206" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D206" s="48" t="inlineStr">
         <is>
-          <t>Mengunduh lampiran pada konten Marketing Toolkit</t>
+          <t>Melakukan filter data Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E206" s="46" t="inlineStr">
@@ -60971,14 +60836,16 @@
       </c>
       <c r="G206" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon titik tiga pada salah satu lampiran.
-2. Pilih Download.</t>
+          <t>1. Klik button Filter.
+2. Pilih kriteria filter pada form Filter (Product, Bulan, Tahun).
+3. Klik button Submit.</t>
         </is>
       </c>
       <c r="H206" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
-2. Berhasil mengunduh lampiran ke perangkat.</t>
+          <t>1. Berhasil membuka form Filter.
+2. Berhasil memilih kriteria filter.
+3. Berhasil menampilkan data Daily Sales Agenda sesuai filter yang dipilih.</t>
         </is>
       </c>
       <c r="I206" s="49" t="n"/>
@@ -61004,7 +60871,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>17.9</t>
+          <t>17.1</t>
         </is>
       </c>
       <c r="B207" s="46" t="inlineStr">
@@ -61019,7 +60886,7 @@
       </c>
       <c r="D207" s="48" t="inlineStr">
         <is>
-          <t>Berbagi lampiran pada konten Marketing Toolkit</t>
+          <t>Membuka halaman Marketing Toolkit</t>
         </is>
       </c>
       <c r="E207" s="46" t="inlineStr">
@@ -61029,19 +60896,19 @@
       </c>
       <c r="F207" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G207" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon titik tiga pada salah satu lampiran.
-2. Pilih Share.</t>
+          <t>1. Buka menu Lainnya.
+2. Klik menu Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H207" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
-2. Berhasil menampilkan pilihan aplikasi berbagi.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I207" s="49" t="n"/>
@@ -61067,22 +60934,22 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>17.2</t>
         </is>
       </c>
       <c r="B208" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C208" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D208" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Sales Code</t>
+          <t>Mengubah tampilan folder menjadi List View</t>
         </is>
       </c>
       <c r="E208" s="46" t="inlineStr">
@@ -61092,19 +60959,17 @@
       </c>
       <c r="F208" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G208" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Dashboard Sales Code.</t>
+          <t>1. Klik icon tampilan List pada halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H208" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Dashboard Sales Code.</t>
+          <t>1. Berhasil mengubah tampilan folder menjadi List View.</t>
         </is>
       </c>
       <c r="I208" s="49" t="n"/>
@@ -61130,22 +60995,22 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>18.2</t>
+          <t>17.3</t>
         </is>
       </c>
       <c r="B209" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C209" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D209" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Voa Realization</t>
+          <t>Mengubah tampilan folder menjadi Grid View</t>
         </is>
       </c>
       <c r="E209" s="46" t="inlineStr">
@@ -61155,17 +61020,17 @@
       </c>
       <c r="F209" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G209" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Voa Realization.</t>
+          <t>1. Klik icon tampilan Grid pada halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H209" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Voa Realization.</t>
+          <t>1. Berhasil mengubah tampilan folder menjadi Grid View.</t>
         </is>
       </c>
       <c r="I209" s="49" t="n"/>
@@ -61191,22 +61056,22 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18.3</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="B210" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C210" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D210" s="48" t="inlineStr">
         <is>
-          <t>Melihat Daftar Pipeline pada Voa Realization</t>
+          <t>Membuka folder pada Marketing Toolkit</t>
         </is>
       </c>
       <c r="E210" s="46" t="inlineStr">
@@ -61221,14 +61086,12 @@
       </c>
       <c r="G210" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Voa Realization.
-2. Klik Lihat Daftar Pipeline.</t>
+          <t>1. Klik salah satu folder pada daftar Folder.</t>
         </is>
       </c>
       <c r="H210" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Voa Realization.
-2. Berhasil menampilkan Daftar Pipeline.</t>
+          <t>1. Berhasil membuka folder Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I210" s="49" t="n"/>
@@ -61254,22 +61117,22 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="B211" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C211" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D211" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail CIF Kelolaan</t>
+          <t>Mencari konten di dalam folder menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E211" s="46" t="inlineStr">
@@ -61279,17 +61142,17 @@
       </c>
       <c r="F211" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G211" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card CIF Kelolaan.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H211" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail CIF Kelolaan.</t>
+          <t>1. Berhasil menampilkan data yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I211" s="49" t="n"/>
@@ -61315,42 +61178,42 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>17.6</t>
         </is>
       </c>
       <c r="B212" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C212" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D212" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Realisasi Konek E-Channel</t>
+          <t>Mencari konten di dalam folder dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E212" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F212" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G212" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Realisasi Konek E-Channel.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H212" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Realisasi Konek E-Channel.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I212" s="49" t="n"/>
@@ -61376,22 +61239,22 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>18.6</t>
+          <t>17.7</t>
         </is>
       </c>
       <c r="B213" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C213" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D213" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Realisasi Akuisisi Merchant</t>
+          <t>Melihat detail konten Marketing Toolkit</t>
         </is>
       </c>
       <c r="E213" s="46" t="inlineStr">
@@ -61406,12 +61269,12 @@
       </c>
       <c r="G213" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Realisasi Akuisisi Merchant.</t>
+          <t>1. Klik salah satu sub-folder pada daftar folder.</t>
         </is>
       </c>
       <c r="H213" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Realisasi Akuisisi Merchant.</t>
+          <t>1. Berhasil menampilkan detail konten Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I213" s="49" t="n"/>
@@ -61437,22 +61300,22 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>18.7</t>
+          <t>17.8</t>
         </is>
       </c>
       <c r="B214" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C214" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D214" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Eligible Upgrade to Prospera/Prioritas</t>
+          <t>Mengunduh lampiran pada konten Marketing Toolkit</t>
         </is>
       </c>
       <c r="E214" s="46" t="inlineStr">
@@ -61467,12 +61330,14 @@
       </c>
       <c r="G214" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Eligible Upgrade to Prospera/Prioritas.</t>
+          <t>1. Klik icon titik tiga pada salah satu lampiran.
+2. Pilih Download.</t>
         </is>
       </c>
       <c r="H214" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Eligible Upgrade to Prospera &amp; Prioritas.</t>
+          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
+2. Berhasil mengunduh lampiran ke perangkat.</t>
         </is>
       </c>
       <c r="I214" s="49" t="n"/>
@@ -61495,6 +61360,500 @@
       <c r="Z214" s="49" t="n"/>
       <c r="AA214" s="49" t="n"/>
     </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>17.9</t>
+        </is>
+      </c>
+      <c r="B215" s="46" t="inlineStr">
+        <is>
+          <t>Fitur</t>
+        </is>
+      </c>
+      <c r="C215" s="46" t="inlineStr">
+        <is>
+          <t>Marketing Toolkit</t>
+        </is>
+      </c>
+      <c r="D215" s="48" t="inlineStr">
+        <is>
+          <t>Berbagi lampiran pada konten Marketing Toolkit</t>
+        </is>
+      </c>
+      <c r="E215" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F215" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G215" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon titik tiga pada salah satu lampiran.
+2. Pilih Share.</t>
+        </is>
+      </c>
+      <c r="H215" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
+2. Berhasil menampilkan pilihan aplikasi berbagi.</t>
+        </is>
+      </c>
+      <c r="I215" s="49" t="n"/>
+      <c r="J215" s="49" t="n"/>
+      <c r="K215" s="49" t="n"/>
+      <c r="L215" s="49" t="n"/>
+      <c r="M215" s="49" t="n"/>
+      <c r="N215" s="49" t="n"/>
+      <c r="O215" s="49" t="n"/>
+      <c r="P215" s="49" t="n"/>
+      <c r="Q215" s="49" t="n"/>
+      <c r="R215" s="49" t="n"/>
+      <c r="S215" s="49" t="n"/>
+      <c r="T215" s="49" t="n"/>
+      <c r="U215" s="49" t="n"/>
+      <c r="V215" s="49" t="n"/>
+      <c r="W215" s="49" t="n"/>
+      <c r="X215" s="49" t="n"/>
+      <c r="Y215" s="49" t="n"/>
+      <c r="Z215" s="49" t="n"/>
+      <c r="AA215" s="49" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="B216" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C216" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D216" s="48" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="E216" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F216" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G216" s="48" t="inlineStr">
+        <is>
+          <t>1. Buka menu Lainnya.
+2. Klik menu Dashboard Sales Code.</t>
+        </is>
+      </c>
+      <c r="H216" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Dashboard Sales Code.</t>
+        </is>
+      </c>
+      <c r="I216" s="49" t="n"/>
+      <c r="J216" s="49" t="n"/>
+      <c r="K216" s="49" t="n"/>
+      <c r="L216" s="49" t="n"/>
+      <c r="M216" s="49" t="n"/>
+      <c r="N216" s="49" t="n"/>
+      <c r="O216" s="49" t="n"/>
+      <c r="P216" s="49" t="n"/>
+      <c r="Q216" s="49" t="n"/>
+      <c r="R216" s="49" t="n"/>
+      <c r="S216" s="49" t="n"/>
+      <c r="T216" s="49" t="n"/>
+      <c r="U216" s="49" t="n"/>
+      <c r="V216" s="49" t="n"/>
+      <c r="W216" s="49" t="n"/>
+      <c r="X216" s="49" t="n"/>
+      <c r="Y216" s="49" t="n"/>
+      <c r="Z216" s="49" t="n"/>
+      <c r="AA216" s="49" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="B217" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C217" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D217" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail Voa Realization</t>
+        </is>
+      </c>
+      <c r="E217" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F217" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G217" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card Voa Realization.</t>
+        </is>
+      </c>
+      <c r="H217" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail Voa Realization.</t>
+        </is>
+      </c>
+      <c r="I217" s="49" t="n"/>
+      <c r="J217" s="49" t="n"/>
+      <c r="K217" s="49" t="n"/>
+      <c r="L217" s="49" t="n"/>
+      <c r="M217" s="49" t="n"/>
+      <c r="N217" s="49" t="n"/>
+      <c r="O217" s="49" t="n"/>
+      <c r="P217" s="49" t="n"/>
+      <c r="Q217" s="49" t="n"/>
+      <c r="R217" s="49" t="n"/>
+      <c r="S217" s="49" t="n"/>
+      <c r="T217" s="49" t="n"/>
+      <c r="U217" s="49" t="n"/>
+      <c r="V217" s="49" t="n"/>
+      <c r="W217" s="49" t="n"/>
+      <c r="X217" s="49" t="n"/>
+      <c r="Y217" s="49" t="n"/>
+      <c r="Z217" s="49" t="n"/>
+      <c r="AA217" s="49" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>18.3</t>
+        </is>
+      </c>
+      <c r="B218" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C218" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D218" s="48" t="inlineStr">
+        <is>
+          <t>Melihat Daftar Pipeline pada Voa Realization</t>
+        </is>
+      </c>
+      <c r="E218" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F218" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G218" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card Voa Realization.
+2. Klik Lihat Daftar Pipeline.</t>
+        </is>
+      </c>
+      <c r="H218" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail Voa Realization.
+2. Berhasil menampilkan Daftar Pipeline.</t>
+        </is>
+      </c>
+      <c r="I218" s="49" t="n"/>
+      <c r="J218" s="49" t="n"/>
+      <c r="K218" s="49" t="n"/>
+      <c r="L218" s="49" t="n"/>
+      <c r="M218" s="49" t="n"/>
+      <c r="N218" s="49" t="n"/>
+      <c r="O218" s="49" t="n"/>
+      <c r="P218" s="49" t="n"/>
+      <c r="Q218" s="49" t="n"/>
+      <c r="R218" s="49" t="n"/>
+      <c r="S218" s="49" t="n"/>
+      <c r="T218" s="49" t="n"/>
+      <c r="U218" s="49" t="n"/>
+      <c r="V218" s="49" t="n"/>
+      <c r="W218" s="49" t="n"/>
+      <c r="X218" s="49" t="n"/>
+      <c r="Y218" s="49" t="n"/>
+      <c r="Z218" s="49" t="n"/>
+      <c r="AA218" s="49" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="B219" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C219" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D219" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail CIF Kelolaan</t>
+        </is>
+      </c>
+      <c r="E219" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F219" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G219" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card CIF Kelolaan.</t>
+        </is>
+      </c>
+      <c r="H219" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail CIF Kelolaan.</t>
+        </is>
+      </c>
+      <c r="I219" s="49" t="n"/>
+      <c r="J219" s="49" t="n"/>
+      <c r="K219" s="49" t="n"/>
+      <c r="L219" s="49" t="n"/>
+      <c r="M219" s="49" t="n"/>
+      <c r="N219" s="49" t="n"/>
+      <c r="O219" s="49" t="n"/>
+      <c r="P219" s="49" t="n"/>
+      <c r="Q219" s="49" t="n"/>
+      <c r="R219" s="49" t="n"/>
+      <c r="S219" s="49" t="n"/>
+      <c r="T219" s="49" t="n"/>
+      <c r="U219" s="49" t="n"/>
+      <c r="V219" s="49" t="n"/>
+      <c r="W219" s="49" t="n"/>
+      <c r="X219" s="49" t="n"/>
+      <c r="Y219" s="49" t="n"/>
+      <c r="Z219" s="49" t="n"/>
+      <c r="AA219" s="49" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="B220" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C220" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D220" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail Realisasi Konek E-Channel</t>
+        </is>
+      </c>
+      <c r="E220" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F220" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G220" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card Realisasi Konek E-Channel.</t>
+        </is>
+      </c>
+      <c r="H220" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail Realisasi Konek E-Channel.</t>
+        </is>
+      </c>
+      <c r="I220" s="49" t="n"/>
+      <c r="J220" s="49" t="n"/>
+      <c r="K220" s="49" t="n"/>
+      <c r="L220" s="49" t="n"/>
+      <c r="M220" s="49" t="n"/>
+      <c r="N220" s="49" t="n"/>
+      <c r="O220" s="49" t="n"/>
+      <c r="P220" s="49" t="n"/>
+      <c r="Q220" s="49" t="n"/>
+      <c r="R220" s="49" t="n"/>
+      <c r="S220" s="49" t="n"/>
+      <c r="T220" s="49" t="n"/>
+      <c r="U220" s="49" t="n"/>
+      <c r="V220" s="49" t="n"/>
+      <c r="W220" s="49" t="n"/>
+      <c r="X220" s="49" t="n"/>
+      <c r="Y220" s="49" t="n"/>
+      <c r="Z220" s="49" t="n"/>
+      <c r="AA220" s="49" t="n"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>18.6</t>
+        </is>
+      </c>
+      <c r="B221" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C221" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D221" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail Realisasi Akuisisi Merchant</t>
+        </is>
+      </c>
+      <c r="E221" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F221" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G221" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card Realisasi Akuisisi Merchant.</t>
+        </is>
+      </c>
+      <c r="H221" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail Realisasi Akuisisi Merchant.</t>
+        </is>
+      </c>
+      <c r="I221" s="49" t="n"/>
+      <c r="J221" s="49" t="n"/>
+      <c r="K221" s="49" t="n"/>
+      <c r="L221" s="49" t="n"/>
+      <c r="M221" s="49" t="n"/>
+      <c r="N221" s="49" t="n"/>
+      <c r="O221" s="49" t="n"/>
+      <c r="P221" s="49" t="n"/>
+      <c r="Q221" s="49" t="n"/>
+      <c r="R221" s="49" t="n"/>
+      <c r="S221" s="49" t="n"/>
+      <c r="T221" s="49" t="n"/>
+      <c r="U221" s="49" t="n"/>
+      <c r="V221" s="49" t="n"/>
+      <c r="W221" s="49" t="n"/>
+      <c r="X221" s="49" t="n"/>
+      <c r="Y221" s="49" t="n"/>
+      <c r="Z221" s="49" t="n"/>
+      <c r="AA221" s="49" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="B222" s="46" t="inlineStr">
+        <is>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C222" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
+      <c r="D222" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail Eligible Upgrade to Prospera/Prioritas</t>
+        </is>
+      </c>
+      <c r="E222" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F222" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G222" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik icon expand pada card Eligible Upgrade to Prospera/Prioritas.</t>
+        </is>
+      </c>
+      <c r="H222" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan detail Eligible Upgrade to Prospera &amp; Prioritas.</t>
+        </is>
+      </c>
+      <c r="I222" s="49" t="n"/>
+      <c r="J222" s="49" t="n"/>
+      <c r="K222" s="49" t="n"/>
+      <c r="L222" s="49" t="n"/>
+      <c r="M222" s="49" t="n"/>
+      <c r="N222" s="49" t="n"/>
+      <c r="O222" s="49" t="n"/>
+      <c r="P222" s="49" t="n"/>
+      <c r="Q222" s="49" t="n"/>
+      <c r="R222" s="49" t="n"/>
+      <c r="S222" s="49" t="n"/>
+      <c r="T222" s="49" t="n"/>
+      <c r="U222" s="49" t="n"/>
+      <c r="V222" s="49" t="n"/>
+      <c r="W222" s="49" t="n"/>
+      <c r="X222" s="49" t="n"/>
+      <c r="Y222" s="49" t="n"/>
+      <c r="Z222" s="49" t="n"/>
+      <c r="AA222" s="49" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
style(sit): eliminate numbered list formatting (1. 2.) across all Web TCs to standard dash separator
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -3783,9 +3783,7 @@
       <c r="F79" s="55" t="inlineStr"/>
       <c r="G79" s="56" t="inlineStr">
         <is>
-          <t>1. Buka menu User Authority.
-2. Klik sub menu User.
-3. Periksa tampilan daftar data User.</t>
+          <t>Buka menu User Authority - Klik sub menu User - Periksa tampilan daftar data User</t>
         </is>
       </c>
       <c r="H79" s="56" t="inlineStr">
@@ -4197,9 +4195,7 @@
       <c r="F89" s="55" t="inlineStr"/>
       <c r="G89" s="56" t="inlineStr">
         <is>
-          <t>1. Buka menu User Authority.
-2. Klik sub menu Group Role.
-3. Periksa tampilan daftar data Group Role.</t>
+          <t>Buka menu User Authority - Klik sub menu Group Role - Periksa tampilan daftar data Group Role</t>
         </is>
       </c>
       <c r="H89" s="56" t="inlineStr">
@@ -4611,9 +4607,7 @@
       <c r="F99" s="55" t="inlineStr"/>
       <c r="G99" s="56" t="inlineStr">
         <is>
-          <t>1. Buka menu User Authority.
-2. Klik sub menu Tipe Karyawan.
-3. Periksa tampilan daftar data Tipe Karyawan.</t>
+          <t>Buka menu User Authority - Klik sub menu Tipe Karyawan - Periksa tampilan daftar data Tipe Karyawan</t>
         </is>
       </c>
       <c r="H99" s="56" t="inlineStr">
@@ -4983,9 +4977,7 @@
       <c r="F108" s="55" t="inlineStr"/>
       <c r="G108" s="56" t="inlineStr">
         <is>
-          <t>1. Buka menu User Authority.
-2. Klik sub menu Hak Akses Role.
-3. Periksa tampilan daftar data Hak Akses Role.</t>
+          <t>Buka menu User Authority - Klik sub menu Hak Akses Role - Periksa tampilan daftar data Hak Akses Role</t>
         </is>
       </c>
       <c r="H108" s="56" t="inlineStr">
@@ -5321,13 +5313,12 @@
       </c>
       <c r="G116" s="56" t="inlineStr">
         <is>
-          <t>1. Klik menu User Authority.
-2. Klik sub menu Keamanan Akun.</t>
+          <t>Klik menu User Authority - Klik sub menu Keamanan Akun</t>
         </is>
       </c>
       <c r="H116" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Menampilkan daftar data Akun.</t>
+          <t>Berhasil Menampilkan daftar data Akun.</t>
         </is>
       </c>
     </row>
@@ -6204,13 +6195,12 @@
       </c>
       <c r="G137" s="56" t="inlineStr">
         <is>
-          <t>1. Pilih filter Status dan/atau Rentang Tanggal Permintaan.
-2. Klik button Filter.</t>
+          <t>Pilih filter Status dan/atau Rentang Tanggal Permintaan - Klik button Filter</t>
         </is>
       </c>
       <c r="H137" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Melakukan filter data permintaan reset MFA.</t>
+          <t>Berhasil Melakukan filter data permintaan reset MFA.</t>
         </is>
       </c>
     </row>
@@ -6247,12 +6237,12 @@
       </c>
       <c r="G138" s="56" t="inlineStr">
         <is>
-          <t>1. Klik button Reset Filter.</t>
+          <t>Klik button Reset Filter</t>
         </is>
       </c>
       <c r="H138" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Mereset filter data permintaan reset MFA.</t>
+          <t>Berhasil Mereset filter data permintaan reset MFA.</t>
         </is>
       </c>
     </row>
@@ -6667,13 +6657,12 @@
       </c>
       <c r="G148" s="56" t="inlineStr">
         <is>
-          <t>1. Pilih filter Status Sesi, Perangkat Terpercaya, dan/atau Rentang Tanggal Aktivitas Terakhir.
-2. Klik button Filter.</t>
+          <t>Pilih filter Status Sesi, Perangkat Terpercaya, dan/atau Rentang Tanggal Aktivitas Terakhir - Klik button Filter</t>
         </is>
       </c>
       <c r="H148" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Melakukan filter data perangkat &amp; sesi.</t>
+          <t>Berhasil Melakukan filter data perangkat &amp; sesi.</t>
         </is>
       </c>
     </row>
@@ -6710,12 +6699,12 @@
       </c>
       <c r="G149" s="56" t="inlineStr">
         <is>
-          <t>1. Klik button Reset Filter.</t>
+          <t>Klik button Reset Filter</t>
         </is>
       </c>
       <c r="H149" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Mereset filter data perangkat &amp; sesi.</t>
+          <t>Berhasil Mereset filter data perangkat &amp; sesi.</t>
         </is>
       </c>
     </row>
@@ -7172,13 +7161,12 @@
       </c>
       <c r="G160" s="56" t="inlineStr">
         <is>
-          <t>1. Klik menu Profile Nasabah &amp; Sales.
-2. Klik sub menu Profile Sales.</t>
+          <t>Klik menu Profile Nasabah &amp; Sales - Klik sub menu Profile Sales</t>
         </is>
       </c>
       <c r="H160" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Menampilkan daftar data Sales.</t>
+          <t>Berhasil Menampilkan daftar data Sales.</t>
         </is>
       </c>
     </row>
@@ -7593,13 +7581,12 @@
       </c>
       <c r="G170" s="56" t="inlineStr">
         <is>
-          <t>1. Klik menu Profile Nasabah &amp; Sales.
-2. Klik sub menu Nasabah Perorangan.</t>
+          <t>Klik menu Profile Nasabah &amp; Sales - Klik sub menu Nasabah Perorangan</t>
         </is>
       </c>
       <c r="H170" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Menampilkan daftar data Nasabah Perorangan.</t>
+          <t>Berhasil Menampilkan daftar data Nasabah Perorangan.</t>
         </is>
       </c>
     </row>
@@ -8140,13 +8127,12 @@
       </c>
       <c r="G183" s="56" t="inlineStr">
         <is>
-          <t>1. Pada tab Daftar Rekening, input keyword pada field Search.
-2. Klik button Search.</t>
+          <t>Pada tab Daftar Rekening, input keyword pada field Search - Klik button Search</t>
         </is>
       </c>
       <c r="H183" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Mencari data pada tab Daftar Rekening dengan keyword valid.</t>
+          <t>Berhasil Mencari data pada tab Daftar Rekening dengan keyword valid.</t>
         </is>
       </c>
     </row>
@@ -8183,13 +8169,12 @@
       </c>
       <c r="G184" s="56" t="inlineStr">
         <is>
-          <t>1. Pada tab Daftar Rekening, input keyword yang tidak terdaftar pada field Search.
-2. Klik button Search.</t>
+          <t>Pada tab Daftar Rekening, input keyword yang tidak terdaftar pada field Search - Klik button Search</t>
         </is>
       </c>
       <c r="H184" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Mencari data pada tab Daftar Rekening dengan keyword tidak valid.</t>
+          <t>Berhasil Mencari data pada tab Daftar Rekening dengan keyword tidak valid.</t>
         </is>
       </c>
     </row>
@@ -8226,12 +8211,12 @@
       </c>
       <c r="G185" s="56" t="inlineStr">
         <is>
-          <t>1. Pada tab Daftar Rekening, klik salah satu Nomor Rekening pada tabel.</t>
+          <t>Pada tab Daftar Rekening, klik salah satu Nomor Rekening pada tabel</t>
         </is>
       </c>
       <c r="H185" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Melihat detail load saldo rekening.</t>
+          <t>Berhasil Melihat detail load saldo rekening.</t>
         </is>
       </c>
     </row>
@@ -17279,12 +17264,12 @@
       </c>
       <c r="G403" s="56" t="inlineStr">
         <is>
-          <t>1. Klik salah satu card Kantor Wilayah.</t>
+          <t>Klik salah satu card Kantor Wilayah</t>
         </is>
       </c>
       <c r="H403" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Melihat detail daftar absensi Kantor Wilayah.</t>
+          <t>Berhasil Melihat detail daftar absensi Kantor Wilayah.</t>
         </is>
       </c>
     </row>
@@ -19127,8 +19112,7 @@
       </c>
       <c r="G447" s="56" t="inlineStr">
         <is>
-          <t>1. Klik button Cancel Approval pada data yang berstatus Rejected.
-2. Klik Yes pada pop up konfirmasi.</t>
+          <t>Klik button Cancel Approval pada data yang berstatus Rejected - Klik Yes pada pop up konfirmasi</t>
         </is>
       </c>
       <c r="H447" s="56" t="inlineStr">
@@ -21312,14 +21296,12 @@
       </c>
       <c r="G499" s="56" t="inlineStr">
         <is>
-          <t>1. Klik checkbox pada salah satu data Personnel yang berstatus Tidak Aktif.
-2. Klik toggle Status pada data Personnel tersebut.</t>
+          <t>Klik checkbox pada salah satu data Personnel yang berstatus Tidak Aktif - Klik toggle Status pada data Personnel tersebut</t>
         </is>
       </c>
       <c r="H499" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang checkbox data Personnel.
-2. Berhasil menambahkan/mengaktifkan personnel ke Attendance Spot secara single.</t>
+          <t>Berhasil mencentang checkbox data Personnel. - Berhasil menambahkan/mengaktifkan personnel ke Attendance Spot secara single.</t>
         </is>
       </c>
     </row>
@@ -21356,14 +21338,12 @@
       </c>
       <c r="G500" s="56" t="inlineStr">
         <is>
-          <t>1. Klik checkbox pada salah satu data Personnel yang berstatus Aktif.
-2. Klik toggle Status pada data Personnel tersebut.</t>
+          <t>Klik checkbox pada salah satu data Personnel yang berstatus Aktif - Klik toggle Status pada data Personnel tersebut</t>
         </is>
       </c>
       <c r="H500" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang checkbox data Personnel.
-2. Berhasil menghapus/menonaktifkan personnel dari Attendance Spot secara single.</t>
+          <t>Berhasil mencentang checkbox data Personnel. - Berhasil menghapus/menonaktifkan personnel dari Attendance Spot secara single.</t>
         </is>
       </c>
     </row>
@@ -21400,14 +21380,12 @@
       </c>
       <c r="G501" s="56" t="inlineStr">
         <is>
-          <t>1. Klik beberapa checkbox data Personnel yang berstatus Tidak Aktif.
-2. Klik button Add Personnel.</t>
+          <t>Klik beberapa checkbox data Personnel yang berstatus Tidak Aktif - Klik button Add Personnel</t>
         </is>
       </c>
       <c r="H501" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang beberapa checkbox data Personnel.
-2. Berhasil menambahkan/mengaktifkan seluruh personnel yang dipilih ke Attendance Spot secara bulk.</t>
+          <t>Berhasil mencentang beberapa checkbox data Personnel. - Berhasil menambahkan/mengaktifkan seluruh personnel yang dipilih ke Attendance Spot secara bulk.</t>
         </is>
       </c>
     </row>
@@ -21444,14 +21422,12 @@
       </c>
       <c r="G502" s="56" t="inlineStr">
         <is>
-          <t>1. Klik beberapa checkbox data Personnel yang berstatus Aktif.
-2. Klik button Remove Personnel.</t>
+          <t>Klik beberapa checkbox data Personnel yang berstatus Aktif - Klik button Remove Personnel</t>
         </is>
       </c>
       <c r="H502" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang beberapa checkbox data Personnel.
-2. Berhasil menghapus/menonaktifkan seluruh personnel yang dipilih dari Attendance Spot secara bulk.</t>
+          <t>Berhasil mencentang beberapa checkbox data Personnel. - Berhasil menghapus/menonaktifkan seluruh personnel yang dipilih dari Attendance Spot secara bulk.</t>
         </is>
       </c>
     </row>
@@ -21992,14 +21968,12 @@
       </c>
       <c r="G515" s="56" t="inlineStr">
         <is>
-          <t>1. Pilih data pada salah satu dropdown filter (Kantor Wilayah, Kantor Cabang, dll).
-2. Klik button Filter.</t>
+          <t>Pilih data pada salah satu dropdown filter (Kantor Wilayah, Kantor Cabang, dll) - Klik button Filter</t>
         </is>
       </c>
       <c r="H515" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil memilih data filter.
-2. Berhasil menampilkan data Personnel sesuai filter yang dipilih.</t>
+          <t>Berhasil memilih data filter. - Berhasil menampilkan data Personnel sesuai filter yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -22036,14 +22010,12 @@
       </c>
       <c r="G516" s="56" t="inlineStr">
         <is>
-          <t>1. Input keyword pada field Search di halaman Personnel.
-2. Klik button Search.</t>
+          <t>Input keyword pada field Search di halaman Personnel - Klik button Search</t>
         </is>
       </c>
       <c r="H516" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil menginput keyword.
-2. Berhasil menampilkan data Personnel sesuai keyword.</t>
+          <t>Berhasil menginput keyword. - Berhasil menampilkan data Personnel sesuai keyword.</t>
         </is>
       </c>
     </row>
@@ -22080,14 +22052,12 @@
       </c>
       <c r="G517" s="56" t="inlineStr">
         <is>
-          <t>1. Input keyword yang tidak terdaftar pada field Search di halaman Personnel.
-2. Klik button Search.</t>
+          <t>Input keyword yang tidak terdaftar pada field Search di halaman Personnel - Klik button Search</t>
         </is>
       </c>
       <c r="H517" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil menginput keyword.
-2. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>Berhasil menginput keyword. - Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
@@ -22208,14 +22178,12 @@
       </c>
       <c r="G520" s="56" t="inlineStr">
         <is>
-          <t>1. Klik checkbox pada salah satu data Personnel yang sudah ter-assign.
-2. Klik icon Unassign (merah).</t>
+          <t>Klik checkbox pada salah satu data Personnel yang sudah ter-assign - Klik icon Unassign (merah)</t>
         </is>
       </c>
       <c r="H520" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang checkbox data Personnel.
-2. Berhasil menghapus (unassign) personnel tersebut dari Work Pattern.</t>
+          <t>Berhasil mencentang checkbox data Personnel. - Berhasil menghapus (unassign) personnel tersebut dari Work Pattern.</t>
         </is>
       </c>
     </row>
@@ -22252,14 +22220,12 @@
       </c>
       <c r="G521" s="56" t="inlineStr">
         <is>
-          <t>1. Klik beberapa checkbox data Personnel yang sudah ter-assign.
-2. Klik icon Unassign (merah).</t>
+          <t>Klik beberapa checkbox data Personnel yang sudah ter-assign - Klik icon Unassign (merah)</t>
         </is>
       </c>
       <c r="H521" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil mencentang beberapa checkbox data Personnel.
-2. Berhasil menghapus (unassign) seluruh personnel yang dipilih secara bulk dari Work Pattern.</t>
+          <t>Berhasil mencentang beberapa checkbox data Personnel. - Berhasil menghapus (unassign) seluruh personnel yang dipilih secara bulk dari Work Pattern.</t>
         </is>
       </c>
     </row>
@@ -22338,13 +22304,12 @@
       </c>
       <c r="G523" s="56" t="inlineStr">
         <is>
-          <t>1. Klik menu Setting Absent.
-2. Klik sub menu Holiday.</t>
+          <t>Klik menu Setting Absent - Klik sub menu Holiday</t>
         </is>
       </c>
       <c r="H523" s="56" t="inlineStr">
         <is>
-          <t>1. Berhasil Menampilkan daftar data Holiday.</t>
+          <t>Berhasil Menampilkan daftar data Holiday.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(mobile): add Modul 20 Notifikasi (TC 20.1-20.8) and sync Modul 19 Kunjungan to Excel
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -42887,7 +42887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA222"/>
+  <dimension ref="A1:AA233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55592,6 +55592,424 @@
       <c r="Z222" s="49" t="n"/>
       <c r="AA222" s="49" t="n"/>
     </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="B223" s="46" t="inlineStr">
+        <is>
+          <t>Kunjungan</t>
+        </is>
+      </c>
+      <c r="C223" s="46" t="n"/>
+      <c r="D223" s="48" t="inlineStr">
+        <is>
+          <t>Membuka halaman Kunjungan</t>
+        </is>
+      </c>
+      <c r="E223" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F223" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G223" s="48" t="inlineStr">
+        <is>
+          <t>Buka menu Lainnya - Klik menu Kunjungan</t>
+        </is>
+      </c>
+      <c r="H223" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Kunjungan beserta informasi Periode, ringkasan Realisasi &amp; Target Visit, serta daftar riwayat kunjungan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="B224" s="46" t="inlineStr">
+        <is>
+          <t>Kunjungan</t>
+        </is>
+      </c>
+      <c r="C224" s="46" t="n"/>
+      <c r="D224" s="48" t="inlineStr">
+        <is>
+          <t>Melakukan filter periode tanggal kunjungan</t>
+        </is>
+      </c>
+      <c r="E224" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F224" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G224" s="48" t="inlineStr">
+        <is>
+          <t>Klik dropdown Periode - Pilih rentang tanggal pada kalender (Pilih rentang) - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H224" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil memfilter dan menampilkan daftar data kunjungan sesuai rentang periode tanggal yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>19.3</t>
+        </is>
+      </c>
+      <c r="B225" s="46" t="inlineStr">
+        <is>
+          <t>Kunjungan</t>
+        </is>
+      </c>
+      <c r="C225" s="46" t="n"/>
+      <c r="D225" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail kunjungan</t>
+        </is>
+      </c>
+      <c r="E225" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F225" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G225" s="48" t="inlineStr">
+        <is>
+          <t>Klik salah satu card kunjungan pada daftar - Sistem menampilkan tab default Mulai Kunjungan - Klik tab Selesai Kunjungan</t>
+        </is>
+      </c>
+      <c r="H225" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Detail Kunjungan yang memuat peta lokasi, waktu, tipe kunjungan, dan nama nasabah pada tab Mulai Kunjungan maupun Selesai Kunjungan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="B226" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C226" s="46" t="n"/>
+      <c r="D226" s="48" t="inlineStr">
+        <is>
+          <t>Membuka halaman Notifikasi</t>
+        </is>
+      </c>
+      <c r="E226" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F226" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G226" s="48" t="inlineStr">
+        <is>
+          <t>Buka aplikasi BTN Smart - Masuk ke Beranda - Klik icon Lonceng (Notifikasi)</t>
+        </is>
+      </c>
+      <c r="H226" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Notifikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="B227" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C227" s="46" t="n"/>
+      <c r="D227" s="48" t="inlineStr">
+        <is>
+          <t>Mencari notifikasi dengan kata kunci valid</t>
+        </is>
+      </c>
+      <c r="E227" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F227" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G227" s="48" t="inlineStr">
+        <is>
+          <t>Masukkan kata kunci valid pada Search Bar</t>
+        </is>
+      </c>
+      <c r="H227" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data notifikasi yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20.3</t>
+        </is>
+      </c>
+      <c r="B228" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C228" s="46" t="n"/>
+      <c r="D228" s="48" t="inlineStr">
+        <is>
+          <t>Mencari notifikasi dengan kata kunci tidak valid</t>
+        </is>
+      </c>
+      <c r="E228" s="46" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F228" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G228" s="48" t="inlineStr">
+        <is>
+          <t>Masukkan kata kunci tidak valid pada Search Bar</t>
+        </is>
+      </c>
+      <c r="H228" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="B229" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C229" s="46" t="n"/>
+      <c r="D229" s="48" t="inlineStr">
+        <is>
+          <t>Melihat data notifikasi Belum Dibaca</t>
+        </is>
+      </c>
+      <c r="E229" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F229" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G229" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Notifikasi, klik tab Belum Dibaca</t>
+        </is>
+      </c>
+      <c r="H229" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data notifikasi belum dibaca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="B230" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C230" s="46" t="n"/>
+      <c r="D230" s="48" t="inlineStr">
+        <is>
+          <t>Melihat data notifikasi Diarsipkan</t>
+        </is>
+      </c>
+      <c r="E230" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F230" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G230" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Notifikasi, klik tab Diarsipkan</t>
+        </is>
+      </c>
+      <c r="H230" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data notifikasi diarsipkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>20.6</t>
+        </is>
+      </c>
+      <c r="B231" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C231" s="46" t="n"/>
+      <c r="D231" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail notifikasi</t>
+        </is>
+      </c>
+      <c r="E231" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F231" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G231" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Notifikasi, klik salah satu notifikasi</t>
+        </is>
+      </c>
+      <c r="H231" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan detail notifikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20.7</t>
+        </is>
+      </c>
+      <c r="B232" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C232" s="46" t="n"/>
+      <c r="D232" s="48" t="inlineStr">
+        <is>
+          <t>Mengarsipkan notifikasi</t>
+        </is>
+      </c>
+      <c r="E232" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F232" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G232" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Detail Notifikasi, klik icon Arsipkan</t>
+        </is>
+      </c>
+      <c r="H232" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil mengarsipkan notifikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="B233" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C233" s="46" t="n"/>
+      <c r="D233" s="48" t="inlineStr">
+        <is>
+          <t>Membatalkan arsip notifikasi</t>
+        </is>
+      </c>
+      <c r="E233" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F233" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G233" s="48" t="inlineStr">
+        <is>
+          <t>Pada detail notifikasi di tab Diarsipkan, klik icon Buka Arsip</t>
+        </is>
+      </c>
+      <c r="H233" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil membatalkan arsip notifikasi.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(web): update Export Center (Modul 73-75) with 25 essential TCs and sync across all docs
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -36727,17 +36727,17 @@
       </c>
       <c r="B867" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C867" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D867" s="56" t="inlineStr">
         <is>
-          <t>Membuka menu riwayat export saya</t>
+          <t>Membuka halaman Riwayat Export</t>
         </is>
       </c>
       <c r="E867" s="56" t="inlineStr">
@@ -36752,12 +36752,12 @@
       </c>
       <c r="G867" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Export Center, klik submenu Riwayat export</t>
+          <t>Klik menu Export Center - Klik submenu Riwayat Export</t>
         </is>
       </c>
       <c r="H867" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Riwayat export</t>
+          <t>Berhasil menampilkan halaman Riwayat Export.</t>
         </is>
       </c>
     </row>
@@ -36769,17 +36769,17 @@
       </c>
       <c r="B868" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C868" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D868" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Mencari data riwayat export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E868" s="56" t="inlineStr">
@@ -36794,12 +36794,12 @@
       </c>
       <c r="G868" s="56" t="inlineStr">
         <is>
-          <t>Klik button filter – pilih modul, export status, dan tentan tanggal request – kemudian klik terapkan filter</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H868" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai filter yang dipilih</t>
+          <t>Berhasil menampilkan data riwayat export yang dicari.</t>
         </is>
       </c>
     </row>
@@ -36811,37 +36811,37 @@
       </c>
       <c r="B869" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C869" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D869" s="56" t="inlineStr">
         <is>
-          <t>Validasi card menunggu approval dengan data table</t>
+          <t>Mencari data riwayat export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E869" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F869" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G869" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data dengan memilih status approval 'pending' dan status export 'Generate'</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H869" s="56" t="inlineStr">
         <is>
-          <t>Berhasil Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
@@ -36853,17 +36853,17 @@
       </c>
       <c r="B870" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C870" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D870" s="56" t="inlineStr">
         <is>
-          <t>Validasi card disetujui dengan data table</t>
+          <t>Melihat data riwayat export berdasarkan status</t>
         </is>
       </c>
       <c r="E870" s="56" t="inlineStr">
@@ -36873,17 +36873,17 @@
       </c>
       <c r="F870" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G870" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data status approval dengan memilih status 'Approved'</t>
+          <t>Pada halaman Riwayat Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H870" s="56" t="inlineStr">
         <is>
-          <t>Berhasil Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil menampilkan daftar data riwayat export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -36895,17 +36895,17 @@
       </c>
       <c r="B871" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C871" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D871" s="56" t="inlineStr">
         <is>
-          <t>Validasi card ditolak dengan data table</t>
+          <t>Melakukan filter data riwayat export</t>
         </is>
       </c>
       <c r="E871" s="56" t="inlineStr">
@@ -36915,17 +36915,17 @@
       </c>
       <c r="F871" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G871" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data status approval dengan memilih status 'Rejected'</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H871" s="56" t="inlineStr">
         <is>
-          <t>Berhasil Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil memfilter dan menampilkan data riwayat export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
@@ -36937,17 +36937,17 @@
       </c>
       <c r="B872" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C872" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D872" s="56" t="inlineStr">
         <is>
-          <t>Validasi card kadaluwarsa dengan data table</t>
+          <t>Mereset filter data riwayat export</t>
         </is>
       </c>
       <c r="E872" s="56" t="inlineStr">
@@ -36962,12 +36962,12 @@
       </c>
       <c r="G872" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data status approval dengan memilih status 'Expired'</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H872" s="56" t="inlineStr">
         <is>
-          <t>Berhasil Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data riwayat export.</t>
         </is>
       </c>
     </row>
@@ -36979,17 +36979,17 @@
       </c>
       <c r="B873" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C873" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D873" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Melihat detail riwayat export</t>
         </is>
       </c>
       <c r="E873" s="56" t="inlineStr">
@@ -37004,12 +37004,12 @@
       </c>
       <c r="G873" s="56" t="inlineStr">
         <is>
-          <t>Input data pada kolom pencarian</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H873" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai kata kunci</t>
+          <t>Berhasil menampilkan drawer Export Detail.</t>
         </is>
       </c>
     </row>
@@ -37021,22 +37021,22 @@
       </c>
       <c r="B874" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C874" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D874" s="56" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E874" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F874" s="55" t="inlineStr">
@@ -37046,34 +37046,34 @@
       </c>
       <c r="G874" s="56" t="inlineStr">
         <is>
-          <t>Input data yang belum terdaftar</t>
+          <t>Klik icon Aksi (...) pada baris data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H874" s="56" t="inlineStr">
         <is>
-          <t>Data tidak ditemukan</t>
+          <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>
     <row r="875" ht="70" customHeight="1">
       <c r="A875" s="55" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B875" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C875" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D875" s="56" t="inlineStr">
         <is>
-          <t>Mengunduh data yang sudah di approve</t>
+          <t>Membuka halaman Persetujuan Export</t>
         </is>
       </c>
       <c r="E875" s="56" t="inlineStr">
@@ -37088,34 +37088,34 @@
       </c>
       <c r="G875" s="56" t="inlineStr">
         <is>
-          <t>Klik button download</t>
+          <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
         </is>
       </c>
       <c r="H875" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh data</t>
+          <t>Berhasil menampilkan halaman Persetujuan Export.</t>
         </is>
       </c>
     </row>
     <row r="876" ht="28" customHeight="1">
       <c r="A876" s="55" t="inlineStr">
         <is>
-          <t>73.10</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B876" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C876" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D876" s="56" t="inlineStr">
         <is>
-          <t>Membuka dokumen hasil download</t>
+          <t>Mencari data persetujuan export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E876" s="56" t="inlineStr">
@@ -37125,44 +37125,44 @@
       </c>
       <c r="F876" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G876" s="56" t="inlineStr">
         <is>
-          <t>Extract file, kemudian masukan password yang terkirim pada email user yang mengajukan, input password maka file berhasil di extract, kemudian buka file</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H876" s="56" t="inlineStr">
         <is>
-          <t>Berhasil membuka file hasil download</t>
+          <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="877" ht="42" customHeight="1">
       <c r="A877" s="55" t="inlineStr">
         <is>
-          <t>73.11</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B877" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C877" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D877" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E877" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F877" s="55" t="inlineStr">
@@ -37172,34 +37172,34 @@
       </c>
       <c r="G877" s="56" t="inlineStr">
         <is>
-          <t>Klik button filter – pilih modul, export status, dan tentan tanggal request – kemudian klik terapkan filter</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H877" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai filter yang dipilih</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="878" ht="28" customHeight="1">
       <c r="A878" s="55" t="inlineStr">
         <is>
-          <t>73.12</t>
+          <t>74.4</t>
         </is>
       </c>
       <c r="B878" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C878" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D878" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Melihat data persetujuan export berdasarkan status</t>
         </is>
       </c>
       <c r="E878" s="56" t="inlineStr">
@@ -37209,81 +37209,81 @@
       </c>
       <c r="F878" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G878" s="56" t="inlineStr">
         <is>
-          <t>Input data pada kolom pencarian</t>
+          <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H878" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai kata kunci</t>
+          <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="879" ht="28" customHeight="1">
       <c r="A879" s="55" t="inlineStr">
         <is>
-          <t>73.13</t>
+          <t>74.5</t>
         </is>
       </c>
       <c r="B879" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C879" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D879" s="56" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Melakukan filter data persetujuan export</t>
         </is>
       </c>
       <c r="E879" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F879" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G879" s="56" t="inlineStr">
         <is>
-          <t>Input data yang belum terdaftar</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H879" s="56" t="inlineStr">
         <is>
-          <t>Data tidak ditemukan</t>
+          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="880" ht="28" customHeight="1">
       <c r="A880" s="55" t="inlineStr">
         <is>
-          <t>73.14</t>
+          <t>74.6</t>
         </is>
       </c>
       <c r="B880" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C880" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D880" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Mereset filter data persetujuan export</t>
         </is>
       </c>
       <c r="E880" s="56" t="inlineStr">
@@ -37298,34 +37298,34 @@
       </c>
       <c r="G880" s="56" t="inlineStr">
         <is>
-          <t>Klik button filter – pilih modul, export status, dan tentan tanggal request – kemudian klik terapkan filter</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H880" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai filter yang dipilih</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
         </is>
       </c>
     </row>
     <row r="881" ht="14" customHeight="1">
       <c r="A881" s="55" t="inlineStr">
         <is>
-          <t>73.15</t>
+          <t>74.7</t>
         </is>
       </c>
       <c r="B881" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C881" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D881" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Melakukan approval data pengajuan export</t>
         </is>
       </c>
       <c r="E881" s="56" t="inlineStr">
@@ -37340,39 +37340,39 @@
       </c>
       <c r="G881" s="56" t="inlineStr">
         <is>
-          <t>Input data pada kolom pencarian</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
         </is>
       </c>
       <c r="H881" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai kata kunci</t>
+          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
         </is>
       </c>
     </row>
     <row r="882" ht="42" customHeight="1">
       <c r="A882" s="55" t="inlineStr">
         <is>
-          <t>73.16</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="B882" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C882" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D882" s="56" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci salah</t>
+          <t>Melakukan reject data pengajuan export</t>
         </is>
       </c>
       <c r="E882" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F882" s="55" t="inlineStr">
@@ -37382,34 +37382,34 @@
       </c>
       <c r="G882" s="56" t="inlineStr">
         <is>
-          <t>Input data yang belum terdaftar</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
         </is>
       </c>
       <c r="H882" s="56" t="inlineStr">
         <is>
-          <t>Data tidak ditemukan</t>
+          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
         </is>
       </c>
     </row>
     <row r="883" ht="42" customHeight="1">
       <c r="A883" s="55" t="inlineStr">
         <is>
-          <t>73.17</t>
+          <t>74.9</t>
         </is>
       </c>
       <c r="B883" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C883" s="56" t="inlineStr">
         <is>
-          <t>Riwayat export saya</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D883" s="56" t="inlineStr">
         <is>
-          <t>Validasi card menunggu approval dengan data table</t>
+          <t>Melihat detail pengajuan export</t>
         </is>
       </c>
       <c r="E883" s="56" t="inlineStr">
@@ -37419,39 +37419,39 @@
       </c>
       <c r="F883" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G883" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data dengan memilih status approval 'pending' dan status export 'Generate'</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H883" s="56" t="inlineStr">
         <is>
-          <t>Berhasil Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil menampilkan detail data pengajuan export.</t>
         </is>
       </c>
     </row>
     <row r="884" ht="28" customHeight="1">
       <c r="A884" s="55" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B884" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C884" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D884" s="56" t="inlineStr">
         <is>
-          <t>Lakukan login menggunakan user monitoring</t>
+          <t>Membuka halaman Aktivitas Export</t>
         </is>
       </c>
       <c r="E884" s="56" t="inlineStr">
@@ -37461,39 +37461,39 @@
       </c>
       <c r="F884" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G884" s="56" t="inlineStr">
         <is>
-          <t>Login menggunakan user monitoring</t>
+          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
         </is>
       </c>
       <c r="H884" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan login</t>
+          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
         </is>
       </c>
     </row>
     <row r="885" ht="42" customHeight="1">
       <c r="A885" s="55" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B885" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C885" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D885" s="56" t="inlineStr">
         <is>
-          <t>Membuka menu Persetujuan Export</t>
+          <t>Mencari data aktivitas export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E885" s="56" t="inlineStr">
@@ -37503,81 +37503,81 @@
       </c>
       <c r="F885" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G885" s="56" t="inlineStr">
         <is>
-          <t>Klik menu exported data management, klik submenu persetujuan export</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H885" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman persetujuan export</t>
+          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="886" ht="14" customHeight="1">
       <c r="A886" s="55" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B886" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C886" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D886" s="56" t="inlineStr">
         <is>
-          <t>Melakukan approval data pengajuan export</t>
+          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E886" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F886" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G886" s="56" t="inlineStr">
         <is>
-          <t>Klik icon titik tiga pada data pengajuan - Klik menu Setuju - Klik button YA pada popup konfirmasi</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H886" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyetujui data pengajuan export.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="887" ht="42" customHeight="1">
       <c r="A887" s="55" t="inlineStr">
         <is>
-          <t>74.4</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B887" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C887" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D887" s="56" t="inlineStr">
         <is>
-          <t>Melakukan reject data pengajuan export</t>
+          <t>Melihat data aktivitas export berdasarkan status</t>
         </is>
       </c>
       <c r="E887" s="56" t="inlineStr">
@@ -37587,39 +37587,39 @@
       </c>
       <c r="F887" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G887" s="56" t="inlineStr">
         <is>
-          <t>Klik icon (titik tiga) klik tolak, input alasan, klik submit</t>
+          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H887" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan reject data</t>
+          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="888" ht="42" customHeight="1">
       <c r="A888" s="55" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B888" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C888" s="56" t="inlineStr">
         <is>
-          <t>Management Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D888" s="56" t="inlineStr">
         <is>
-          <t>Membuka menu Management Export</t>
+          <t>Melakukan filter data aktivitas export</t>
         </is>
       </c>
       <c r="E888" s="56" t="inlineStr">
@@ -37629,39 +37629,39 @@
       </c>
       <c r="F888" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G888" s="56" t="inlineStr">
         <is>
-          <t>Klik menu exported data management, klik submenu management export</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H888" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman management export</t>
+          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="889" ht="28" customHeight="1">
       <c r="A889" s="55" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B889" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C889" s="56" t="inlineStr">
         <is>
-          <t>Management Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D889" s="56" t="inlineStr">
         <is>
-          <t>Validasi card data file aktif dengan data table</t>
+          <t>Mereset filter data aktivitas export</t>
         </is>
       </c>
       <c r="E889" s="56" t="inlineStr">
@@ -37676,34 +37676,34 @@
       </c>
       <c r="G889" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data dengan memilih status approvalnya “Approved” dan status exportnya “Generate” dengan tanggal sebelum hari berjalan</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H889" s="56" t="inlineStr">
         <is>
-          <t>Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="890" ht="42" customHeight="1">
       <c r="A890" s="55" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>75.7</t>
         </is>
       </c>
       <c r="B890" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C890" s="56" t="inlineStr">
         <is>
-          <t>Management Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D890" s="56" t="inlineStr">
         <is>
-          <t>Validasi card file kadaluwarsa dengan data table</t>
+          <t>Melihat detail aktivitas export</t>
         </is>
       </c>
       <c r="E890" s="56" t="inlineStr">
@@ -37713,39 +37713,39 @@
       </c>
       <c r="F890" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G890" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data dengan memilih status approvalnya “approve” dan status exportnya “generate” dengan tanggal sesudah hari berjalan</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H890" s="56" t="inlineStr">
         <is>
-          <t>Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil menampilkan detail data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="891" ht="14" customHeight="1">
       <c r="A891" s="55" t="inlineStr">
         <is>
-          <t>75.4</t>
+          <t>75.8</t>
         </is>
       </c>
       <c r="B891" s="56" t="inlineStr">
         <is>
-          <t>Export data management</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C891" s="56" t="inlineStr">
         <is>
-          <t>Management Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D891" s="56" t="inlineStr">
         <is>
-          <t>Validasi card reject dengan data table</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E891" s="56" t="inlineStr">
@@ -37760,12 +37760,12 @@
       </c>
       <c r="G891" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data dengan memilih status approvalnya “reject” dan status exportnya “generate”</t>
+          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H891" s="56" t="inlineStr">
         <is>
-          <t>Jumlah data pada card dan table sesuai</t>
+          <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(notifikasi): reorder TCs 3.1-3.10 to match logical UI flow and sync docs
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -3336,7 +3336,7 @@
       <c r="C69" s="56" t="n"/>
       <c r="D69" s="56" t="inlineStr">
         <is>
-          <t>Melihat data notifikasi Diarsipkan</t>
+          <t>Menandai semua notifikasi telah dibaca</t>
         </is>
       </c>
       <c r="E69" s="56" t="inlineStr">
@@ -3346,17 +3346,17 @@
       </c>
       <c r="F69" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G69" s="56" t="inlineStr">
         <is>
-          <t>Pada halaman Pengaturan Profile - Notifikasi, klik tab Diarsipkan</t>
+          <t>Pada notifikasi, klik tombol Tandai semua dibaca</t>
         </is>
       </c>
       <c r="H69" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data notifikasi diarsipkan.</t>
+          <t>Berhasil menandai seluruh notifikasi telah dibaca.</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       <c r="C70" s="56" t="n"/>
       <c r="D70" s="56" t="inlineStr">
         <is>
-          <t>Menandai semua notifikasi telah dibaca</t>
+          <t>Membuka halaman Notifikasi pada Pengaturan Profile</t>
         </is>
       </c>
       <c r="E70" s="56" t="inlineStr">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="G70" s="56" t="inlineStr">
         <is>
-          <t>Pada notifikasi, klik tombol Tandai semua dibaca</t>
+          <t>Klik tombol Lihat semua pada notifikasi header (atau masuk via menu Pengaturan Profile)</t>
         </is>
       </c>
       <c r="H70" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menandai seluruh notifikasi telah dibaca.</t>
+          <t>Berhasil menampilkan halaman penuh Notifikasi pada Pengaturan Profile.</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       <c r="C71" s="56" t="n"/>
       <c r="D71" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Notifikasi pada Pengaturan Profile</t>
+          <t>Melihat data notifikasi Diarsipkan</t>
         </is>
       </c>
       <c r="E71" s="56" t="inlineStr">
@@ -3422,17 +3422,17 @@
       </c>
       <c r="F71" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G71" s="56" t="inlineStr">
         <is>
-          <t>Klik tombol Lihat semua pada notifikasi header (atau masuk via menu Pengaturan Profile)</t>
+          <t>Pada halaman Pengaturan Profile - Notifikasi, klik tab Diarsipkan</t>
         </is>
       </c>
       <c r="H71" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman penuh Notifikasi pada Pengaturan Profile.</t>
+          <t>Berhasil menampilkan data notifikasi diarsipkan.</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       <c r="C72" s="56" t="n"/>
       <c r="D72" s="56" t="inlineStr">
         <is>
-          <t>Mengarsipkan notifikasi</t>
+          <t>Melihat detail notifikasi</t>
         </is>
       </c>
       <c r="E72" s="56" t="inlineStr">
@@ -3465,12 +3465,12 @@
       </c>
       <c r="G72" s="56" t="inlineStr">
         <is>
-          <t>Pada halaman Detail Notifikasi, klik tombol Arsipkan</t>
+          <t>Pada daftar notifikasi, klik salah satu notifikasi yang ingin dilihat</t>
         </is>
       </c>
       <c r="H72" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengarsipkan notifikasi.</t>
+          <t>Berhasil menampilkan halaman Detail Notifikasi.</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
       <c r="C73" s="56" t="n"/>
       <c r="D73" s="56" t="inlineStr">
         <is>
-          <t>Membatalkan arsip notifikasi</t>
+          <t>Mengarsipkan notifikasi</t>
         </is>
       </c>
       <c r="E73" s="56" t="inlineStr">
@@ -3503,12 +3503,12 @@
       </c>
       <c r="G73" s="56" t="inlineStr">
         <is>
-          <t>Pada halaman Detail Notifikasi yang diarsipkan, klik tombol Kembalikan dari arsip</t>
+          <t>Pada halaman Detail Notifikasi, klik tombol Arsipkan</t>
         </is>
       </c>
       <c r="H73" s="56" t="inlineStr">
         <is>
-          <t>Berhasil membatalkan arsip notifikasi.</t>
+          <t>Berhasil mengarsipkan notifikasi.</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       <c r="C74" s="56" t="n"/>
       <c r="D74" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail notifikasi</t>
+          <t>Membatalkan arsip notifikasi</t>
         </is>
       </c>
       <c r="E74" s="56" t="inlineStr">
@@ -3541,12 +3541,12 @@
       </c>
       <c r="G74" s="56" t="inlineStr">
         <is>
-          <t>Pada daftar notifikasi, klik salah satu notifikasi yang ingin dilihat</t>
+          <t>Pada halaman Detail Notifikasi yang diarsipkan, klik tombol Kembalikan dari arsip</t>
         </is>
       </c>
       <c r="H74" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Detail Notifikasi.</t>
+          <t>Berhasil membatalkan arsip notifikasi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(notifikasi): rename TC 3.6 to Melihat semua notifikasi and sync docs
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -3374,7 +3374,7 @@
       <c r="C70" s="56" t="n"/>
       <c r="D70" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Notifikasi pada Pengaturan Profile</t>
+          <t>Melihat semua notifikasi</t>
         </is>
       </c>
       <c r="E70" s="56" t="inlineStr">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="G70" s="56" t="inlineStr">
         <is>
-          <t>Klik tombol Lihat semua pada notifikasi header (atau masuk via menu Pengaturan Profile)</t>
+          <t>Pada daftar notifikasi, klik tombol Lihat semua</t>
         </is>
       </c>
       <c r="H70" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman penuh Notifikasi pada Pengaturan Profile.</t>
+          <t>Berhasil menampilkan seluruh daftar notifikasi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(reassign): clean up duplicates, restructure TCs, and embed new screenshots for Re-Assign and Approval modules (72, 73, 74)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z915"/>
+  <dimension ref="A1:Z893"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35988,7 +35988,7 @@
       </c>
       <c r="H852" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Approval non banking</t>
+          <t>Menampilkan halaman Approval non banking.</t>
         </is>
       </c>
     </row>
@@ -36010,7 +36010,7 @@
       </c>
       <c r="D853" s="56" t="inlineStr">
         <is>
-          <t>Filter data</t>
+          <t>Melakukan filter data Approval non Banking</t>
         </is>
       </c>
       <c r="E853" s="56" t="inlineStr">
@@ -36025,12 +36025,12 @@
       </c>
       <c r="G853" s="56" t="inlineStr">
         <is>
-          <t>Pilih sales - Pilih produk - Pilih bulan - Pilih tahun - Klik button Submit</t>
+          <t>Pilih filter Sales, Produk, Bulan, Tahun - Klik button Submit</t>
         </is>
       </c>
       <c r="H853" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data approval non banking sesuai dengan filter data yang di pilih</t>
+          <t>Berhasil memfilter dan menampilkan data Approval non banking sesuai filter yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -36052,7 +36052,7 @@
       </c>
       <c r="D854" s="56" t="inlineStr">
         <is>
-          <t>Mencari data</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E854" s="56" t="inlineStr">
@@ -36062,17 +36062,17 @@
       </c>
       <c r="F854" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G854" s="56" t="inlineStr">
         <is>
-          <t>Input keyword pada field search - Klik icon search yang ada di sebelah field search</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H854" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan keyword yang di cari</t>
+          <t>Berhasil menampilkan data Approval non banking yang dicari.</t>
         </is>
       </c>
     </row>
@@ -36094,27 +36094,27 @@
       </c>
       <c r="D855" s="56" t="inlineStr">
         <is>
-          <t>Melihat Detail data Approval non banking</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E855" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F855" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G855" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga - Klik Detail</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H855" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman detail data approval non banking</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
@@ -36136,7 +36136,7 @@
       </c>
       <c r="D856" s="56" t="inlineStr">
         <is>
-          <t>Menyetujui Prospek</t>
+          <t>Melakukan approval data prospek</t>
         </is>
       </c>
       <c r="E856" s="56" t="inlineStr">
@@ -36146,17 +36146,17 @@
       </c>
       <c r="F856" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G856" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga - Klik Setujui - Input Realisasi - Input Remark - Klik button Setujui</t>
+          <t>Klik titik tiga pada data status PENDING - Klik Setujui - Input Realisasi dan Remark - Klik button Setujui</t>
         </is>
       </c>
       <c r="H856" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyetujui prospek, menampilkan popup 'Sukses menyetujui prospek'</t>
+          <t>Berhasil menyetujui prospek.</t>
         </is>
       </c>
     </row>
@@ -36178,7 +36178,7 @@
       </c>
       <c r="D857" s="56" t="inlineStr">
         <is>
-          <t>Batal menyetujui Prospek</t>
+          <t>Melakukan reject data prospek</t>
         </is>
       </c>
       <c r="E857" s="56" t="inlineStr">
@@ -36188,17 +36188,17 @@
       </c>
       <c r="F857" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G857" s="56" t="inlineStr">
         <is>
-          <t>Klik button Batalkan pada modal approve</t>
+          <t>Klik titik tiga pada data status PENDING - Klik Tolak - Input Remark - Klik button Tolak</t>
         </is>
       </c>
       <c r="H857" s="56" t="inlineStr">
         <is>
-          <t>Modal approve tertutup dan tetap di halaman approval non banking</t>
+          <t>Berhasil menolak prospek.</t>
         </is>
       </c>
     </row>
@@ -36220,12 +36220,12 @@
       </c>
       <c r="D858" s="56" t="inlineStr">
         <is>
-          <t>Tidak menginput nilai realisasi pada modal approve</t>
+          <t>Melihat detail data prospek</t>
         </is>
       </c>
       <c r="E858" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F858" s="55" t="inlineStr">
@@ -36235,19 +36235,19 @@
       </c>
       <c r="G858" s="56" t="inlineStr">
         <is>
-          <t>Kosongkan nilai realisasi - Input remark - Klik button Setujui</t>
+          <t>Klik titik tiga pada data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H858" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan alert 'Realisasi dibutuhkan!'</t>
+          <t>Berhasil menampilkan detail data prospek.</t>
         </is>
       </c>
     </row>
     <row r="859" ht="28" customHeight="1">
       <c r="A859" s="55" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B859" s="56" t="inlineStr">
@@ -36257,17 +36257,17 @@
       </c>
       <c r="C859" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D859" s="56" t="inlineStr">
         <is>
-          <t>Tidak menginput remark pada modal approve</t>
+          <t>Membuka halaman Re-Assign Prospek</t>
         </is>
       </c>
       <c r="E859" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F859" s="55" t="inlineStr">
@@ -36277,19 +36277,19 @@
       </c>
       <c r="G859" s="56" t="inlineStr">
         <is>
-          <t>Kosongkan remark</t>
+          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Prospek</t>
         </is>
       </c>
       <c r="H859" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan alert 'Remark dibutuhkan!'</t>
+          <t>Menampilkan halaman Re-Assign Prospek.</t>
         </is>
       </c>
     </row>
     <row r="860" ht="28" customHeight="1">
       <c r="A860" s="55" t="inlineStr">
         <is>
-          <t>72.9</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="B860" s="56" t="inlineStr">
@@ -36299,17 +36299,17 @@
       </c>
       <c r="C860" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D860" s="56" t="inlineStr">
         <is>
-          <t>Menginput huruf pada field realisasi</t>
+          <t>Melakukan filter data Re-Assign Prospek</t>
         </is>
       </c>
       <c r="E860" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F860" s="55" t="inlineStr">
@@ -36319,19 +36319,19 @@
       </c>
       <c r="G860" s="56" t="inlineStr">
         <is>
-          <t>Input huruf pada field realisasi kemudian pindah ke filed lain</t>
+          <t>Klik button Filter - Pilih Produk dan Sales pada drawer Filter - Klik button Filter</t>
         </is>
       </c>
       <c r="H860" s="56" t="inlineStr">
         <is>
-          <t>Sistem menghapus input non-numerik secara otomatis saat field kehilangan fokus. Field Realiasi menjadi kosong</t>
+          <t>Berhasil memfilter dan menampilkan data prospek sesuai kriteria.</t>
         </is>
       </c>
     </row>
     <row r="861" ht="28" customHeight="1">
       <c r="A861" s="55" t="inlineStr">
         <is>
-          <t>72.10</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="B861" s="56" t="inlineStr">
@@ -36341,12 +36341,12 @@
       </c>
       <c r="C861" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D861" s="56" t="inlineStr">
         <is>
-          <t>Menolak Prospek</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E861" s="56" t="inlineStr">
@@ -36361,19 +36361,19 @@
       </c>
       <c r="G861" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga - Klik Tolak - Input Remark - Klik button Tolak</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H861" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menolak prospek, menampilkan popup 'Sukses menolak prospek'</t>
+          <t>Berhasil menampilkan data prospek yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="862" ht="28" customHeight="1">
       <c r="A862" s="55" t="inlineStr">
         <is>
-          <t>72.11</t>
+          <t>73.4</t>
         </is>
       </c>
       <c r="B862" s="56" t="inlineStr">
@@ -36383,17 +36383,17 @@
       </c>
       <c r="C862" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D862" s="56" t="inlineStr">
         <is>
-          <t>Batal menolak prospek</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E862" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F862" s="55" t="inlineStr">
@@ -36403,19 +36403,19 @@
       </c>
       <c r="G862" s="56" t="inlineStr">
         <is>
-          <t>Klik button Batalkan pada moal tolak prospek</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H862" s="56" t="inlineStr">
         <is>
-          <t>Modal tolak prospek tertutup dan tetap berada di halaman approval non banking</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="863" ht="28" customHeight="1">
       <c r="A863" s="55" t="inlineStr">
         <is>
-          <t>72.12</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="B863" s="56" t="inlineStr">
@@ -36425,12 +36425,12 @@
       </c>
       <c r="C863" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D863" s="56" t="inlineStr">
         <is>
-          <t>Tidak menginput remark pada modal tolak prospek</t>
+          <t>Melakukan re-assign beberapa data prospek</t>
         </is>
       </c>
       <c r="E863" s="56" t="inlineStr">
@@ -36445,19 +36445,19 @@
       </c>
       <c r="G863" s="56" t="inlineStr">
         <is>
-          <t>Kosongkan remark - Klik button Tolak</t>
+          <t>Checklist beberapa data prospek - Klik button Reassign () data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H863" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan alert 'Remark dibutuhkan!'</t>
+          <t>Berhasil melakukan re-assign data prospek yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="864" ht="28" customHeight="1">
       <c r="A864" s="55" t="inlineStr">
         <is>
-          <t>72.13</t>
+          <t>73.6</t>
         </is>
       </c>
       <c r="B864" s="56" t="inlineStr">
@@ -36467,12 +36467,12 @@
       </c>
       <c r="C864" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D864" s="56" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Melakukan re-assign semua data prospek</t>
         </is>
       </c>
       <c r="E864" s="56" t="inlineStr">
@@ -36482,24 +36482,24 @@
       </c>
       <c r="F864" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G864" s="56" t="inlineStr">
         <is>
-          <t>Klik pagination (10/halaman) - Pilih berapa data yang ingin ditampilkan</t>
+          <t>Klik button Reassign Semua data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H864" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
+          <t>Berhasil melakukan re-assign seluruh data prospek.</t>
         </is>
       </c>
     </row>
     <row r="865" ht="28" customHeight="1">
       <c r="A865" s="55" t="inlineStr">
         <is>
-          <t>72.14</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B865" s="56" t="inlineStr">
@@ -36509,12 +36509,12 @@
       </c>
       <c r="C865" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D865" s="56" t="inlineStr">
         <is>
-          <t>Pindah Halaman</t>
+          <t>Membuka halaman Re-Assign Management</t>
         </is>
       </c>
       <c r="E865" s="56" t="inlineStr">
@@ -36524,24 +36524,24 @@
       </c>
       <c r="F865" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G865" s="56" t="inlineStr">
         <is>
-          <t>Input angka halaman di field pindah halaman - Klik Enter pada keyboard</t>
+          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Management</t>
         </is>
       </c>
       <c r="H865" s="56" t="inlineStr">
         <is>
-          <t>Berhasil berpindah ke halaman yang dituju.</t>
+          <t>Menampilkan halaman Re-Assign Management.</t>
         </is>
       </c>
     </row>
     <row r="866" ht="28" customHeight="1">
       <c r="A866" s="55" t="inlineStr">
         <is>
-          <t>72.15</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B866" s="56" t="inlineStr">
@@ -36551,12 +36551,12 @@
       </c>
       <c r="C866" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D866" s="56" t="inlineStr">
         <is>
-          <t>Filter kolom</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E866" s="56" t="inlineStr">
@@ -36571,19 +36571,19 @@
       </c>
       <c r="G866" s="56" t="inlineStr">
         <is>
-          <t>Klik icon filter kolom - Checklist/unchecklist kolom</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H866" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tabel sesuai dengan kolom yang di ceklis</t>
+          <t>Berhasil menampilkan data prospek yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="867" ht="28" customHeight="1">
       <c r="A867" s="55" t="inlineStr">
         <is>
-          <t>72.16</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B867" s="56" t="inlineStr">
@@ -36593,17 +36593,17 @@
       </c>
       <c r="C867" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D867" s="56" t="inlineStr">
         <is>
-          <t>Reset ke Default pada filter kolom</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E867" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F867" s="55" t="inlineStr">
@@ -36613,19 +36613,19 @@
       </c>
       <c r="G867" s="56" t="inlineStr">
         <is>
-          <t>Klik Reset ke Default</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H867" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data tabel dengan kolom default</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="868" ht="28" customHeight="1">
       <c r="A868" s="55" t="inlineStr">
         <is>
-          <t>72.17</t>
+          <t>74.4</t>
         </is>
       </c>
       <c r="B868" s="56" t="inlineStr">
@@ -36635,12 +36635,12 @@
       </c>
       <c r="C868" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D868" s="56" t="inlineStr">
         <is>
-          <t>Filter data</t>
+          <t>Melakukan re-assign management</t>
         </is>
       </c>
       <c r="E868" s="56" t="inlineStr">
@@ -36650,39 +36650,39 @@
       </c>
       <c r="F868" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G868" s="56" t="inlineStr">
         <is>
-          <t>Pilih sales - Pilih produk - Pilih bulan - Pilih tahun - Klik button Submit</t>
+          <t>Checklist data prospek - Klik button Reassign () data - Klik button Yes - Pilih Sales tujuan pada modal - Klik button Submit</t>
         </is>
       </c>
       <c r="H868" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data approval non banking sesuai dengan filter data yang di pilih</t>
+          <t>Berhasil melakukan re-assign data prospek referral management.</t>
         </is>
       </c>
     </row>
     <row r="869" ht="28" customHeight="1">
       <c r="A869" s="55" t="inlineStr">
         <is>
-          <t>72.18</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B869" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C869" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D869" s="56" t="inlineStr">
         <is>
-          <t>Mencari data</t>
+          <t>Membuka halaman Riwayat Export</t>
         </is>
       </c>
       <c r="E869" s="56" t="inlineStr">
@@ -36697,34 +36697,34 @@
       </c>
       <c r="G869" s="56" t="inlineStr">
         <is>
-          <t>Input keyword pada field search - Klik icon search yang ada di sebelah field search</t>
+          <t>Klik menu Export Center - Klik submenu Riwayat Export</t>
         </is>
       </c>
       <c r="H869" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan keyword yang di cari</t>
+          <t>Berhasil menampilkan halaman Riwayat Export.</t>
         </is>
       </c>
     </row>
     <row r="870" ht="28" customHeight="1">
       <c r="A870" s="55" t="inlineStr">
         <is>
-          <t>72.19</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B870" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C870" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D870" s="56" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Mencari data riwayat export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E870" s="56" t="inlineStr">
@@ -36734,81 +36734,81 @@
       </c>
       <c r="F870" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G870" s="56" t="inlineStr">
         <is>
-          <t>Klik pagination (10/halaman) - Pilih berapa data yang ingin ditampilkan</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H870" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
+          <t>Berhasil menampilkan data riwayat export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="871" ht="28" customHeight="1">
       <c r="A871" s="55" t="inlineStr">
         <is>
-          <t>72.20</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B871" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C871" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D871" s="56" t="inlineStr">
         <is>
-          <t>Pindah Halaman</t>
+          <t>Mencari data riwayat export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E871" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F871" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G871" s="56" t="inlineStr">
         <is>
-          <t>Input angka halaman di field pindah halaman - Klik Enter pada keyboard</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H871" s="56" t="inlineStr">
         <is>
-          <t>Berhasil berpindah ke halaman yang dituju.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="872" ht="70" customHeight="1">
       <c r="A872" s="55" t="inlineStr">
         <is>
-          <t>72.21</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B872" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C872" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D872" s="56" t="inlineStr">
         <is>
-          <t>Pagination</t>
+          <t>Melihat data riwayat export berdasarkan status</t>
         </is>
       </c>
       <c r="E872" s="56" t="inlineStr">
@@ -36818,39 +36818,39 @@
       </c>
       <c r="F872" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G872" s="56" t="inlineStr">
         <is>
-          <t>Klik pagination (10/halaman) - Pilih berapa data yang ingin ditampilkan</t>
+          <t>Pada halaman Riwayat Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H872" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai jumlah data per halaman yang dipilih.</t>
+          <t>Berhasil menampilkan daftar data riwayat export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="873" ht="42" customHeight="1">
       <c r="A873" s="55" t="inlineStr">
         <is>
-          <t>72.22</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B873" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C873" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D873" s="56" t="inlineStr">
         <is>
-          <t>Pindah Halaman</t>
+          <t>Melakukan filter data riwayat export</t>
         </is>
       </c>
       <c r="E873" s="56" t="inlineStr">
@@ -36860,39 +36860,39 @@
       </c>
       <c r="F873" s="55" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G873" s="56" t="inlineStr">
         <is>
-          <t>Input angka halaman di field pindah halaman - Klik Enter pada keyboard</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H873" s="56" t="inlineStr">
         <is>
-          <t>Berhasil berpindah ke halaman yang dituju.</t>
+          <t>Berhasil memfilter dan menampilkan data riwayat export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="874" ht="42" customHeight="1">
       <c r="A874" s="55" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B874" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C874" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D874" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Re-Assign Prospek</t>
+          <t>Mereset filter data riwayat export</t>
         </is>
       </c>
       <c r="E874" s="56" t="inlineStr">
@@ -36902,39 +36902,39 @@
       </c>
       <c r="F874" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G874" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Prospek</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H874" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Re-Assign Prospek</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data riwayat export.</t>
         </is>
       </c>
     </row>
     <row r="875" ht="70" customHeight="1">
       <c r="A875" s="55" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>75.7</t>
         </is>
       </c>
       <c r="B875" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C875" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D875" s="56" t="inlineStr">
         <is>
-          <t>Melakukan Re-Assign Prospek</t>
+          <t>Melihat detail riwayat export</t>
         </is>
       </c>
       <c r="E875" s="56" t="inlineStr">
@@ -36949,34 +36949,34 @@
       </c>
       <c r="G875" s="56" t="inlineStr">
         <is>
-          <t>Pilih prospek dengan klik checkbox - Klik button Re-Assign () data - Klik button Yes - Pilih kantor wilayah - Pilih kantor cabang - Pilih kantor cabang pembantu - Pilih sales - Klik button Submit</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H875" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign prospek ke sales yang di pilih dan menampilkan popup 'Berhasil melakukan Re-assign Prospek' kemudian data tersebut sudah tidak ada pada tabel re-assign prospek</t>
+          <t>Berhasil menampilkan drawer Export Detail.</t>
         </is>
       </c>
     </row>
     <row r="876" ht="28" customHeight="1">
       <c r="A876" s="55" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>75.8</t>
         </is>
       </c>
       <c r="B876" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C876" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D876" s="56" t="inlineStr">
         <is>
-          <t>Validasi count checklist data</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E876" s="56" t="inlineStr">
@@ -36986,39 +36986,39 @@
       </c>
       <c r="F876" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G876" s="56" t="inlineStr">
         <is>
-          <t>Cek informasi yang ada pada button Reassign () data</t>
+          <t>Klik icon Aksi (...) pada baris data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H876" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan count angka yang sesuai dengan data yang di checklist</t>
+          <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>
     <row r="877" ht="42" customHeight="1">
       <c r="A877" s="55" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="B877" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C877" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D877" s="56" t="inlineStr">
         <is>
-          <t>Validasi data yang sudah dii pilih</t>
+          <t>Membuka halaman Persetujuan Export</t>
         </is>
       </c>
       <c r="E877" s="56" t="inlineStr">
@@ -37028,123 +37028,123 @@
       </c>
       <c r="F877" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G877" s="56" t="inlineStr">
         <is>
-          <t>Cek pada halaman pindah kelolaan, data tabel nya berisi prospek yang di pilih</t>
+          <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
         </is>
       </c>
       <c r="H877" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tabel prospek yang di pilih saja</t>
+          <t>Berhasil menampilkan halaman Persetujuan Export.</t>
         </is>
       </c>
     </row>
     <row r="878" ht="28" customHeight="1">
       <c r="A878" s="55" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>76.2</t>
         </is>
       </c>
       <c r="B878" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C878" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D878" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field inputan mandatory pada reassign prospek</t>
+          <t>Mencari data persetujuan export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E878" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F878" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G878" s="56" t="inlineStr">
         <is>
-          <t>Kosongkan salah satu atau semua field mandatory - Klik button Submit</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H878" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan alert pada setiap field mandatory bahwa field tersebut dibutuhkan / wajib diisi</t>
+          <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="879" ht="28" customHeight="1">
       <c r="A879" s="55" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>76.3</t>
         </is>
       </c>
       <c r="B879" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C879" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D879" s="56" t="inlineStr">
         <is>
-          <t>Membatalkan Re-Assign Prospek</t>
+          <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E879" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F879" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G879" s="56" t="inlineStr">
         <is>
-          <t>Klik button Batalkan pada halaman pindah kelolaan</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H879" s="56" t="inlineStr">
         <is>
-          <t>Kembali ke halaman utama Re-assign Prospek</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="880" ht="28" customHeight="1">
       <c r="A880" s="55" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>76.4</t>
         </is>
       </c>
       <c r="B880" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C880" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D880" s="56" t="inlineStr">
         <is>
-          <t>Validasi data prospek yang di re-assign</t>
+          <t>Melihat data persetujuan export berdasarkan status</t>
         </is>
       </c>
       <c r="E880" s="56" t="inlineStr">
@@ -37154,39 +37154,39 @@
       </c>
       <c r="F880" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G880" s="56" t="inlineStr">
         <is>
-          <t>Login menggunakan user yang sebelumnya sudah dipilih ketika re-assign prospek - Klik menu Lead Qualification - Klik submenu Aktifitas - Cek data yang sebelum nya di re-assign pada tabel dan pada detail prospek</t>
+          <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H880" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek yang sebelumnya di re-assign dan pada detail prospek menampilkan informasi ex. "Re-prospek dari Lead ID: 11370987"</t>
+          <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="881" ht="14" customHeight="1">
       <c r="A881" s="55" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="B881" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C881" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D881" s="56" t="inlineStr">
         <is>
-          <t>Melakukan Re-assign prospek semua data</t>
+          <t>Melakukan filter data persetujuan export</t>
         </is>
       </c>
       <c r="E881" s="56" t="inlineStr">
@@ -37196,39 +37196,39 @@
       </c>
       <c r="F881" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G881" s="56" t="inlineStr">
         <is>
-          <t>Klik button Reassign semua data - Klik button Yes - Pilih kantor wilayah - Pilih kantor cabang - Pilih kantor cabang pembantu - Pilih sales - Klik button Submit</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H881" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign prospek ke sales yang di pilih dan menampilkan popup 'Berhasil melakukan Re-assign Prospek' kemudian data tabel sudah kosong / tidak ada data re-assign prospek</t>
+          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="882" ht="42" customHeight="1">
       <c r="A882" s="55" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>76.6</t>
         </is>
       </c>
       <c r="B882" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C882" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D882" s="56" t="inlineStr">
         <is>
-          <t>Validasi semua data</t>
+          <t>Mereset filter data persetujuan export</t>
         </is>
       </c>
       <c r="E882" s="56" t="inlineStr">
@@ -37243,34 +37243,34 @@
       </c>
       <c r="G882" s="56" t="inlineStr">
         <is>
-          <t>Cek pada halaman pindah kelolaan, data tabel nya berisi semua prospek</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H882" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tabel yang berisi semua prospek</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
         </is>
       </c>
     </row>
     <row r="883" ht="42" customHeight="1">
       <c r="A883" s="55" t="inlineStr">
         <is>
-          <t>73.10</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="B883" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C883" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D883" s="56" t="inlineStr">
         <is>
-          <t>Membatalkan Re-Assign Prospek</t>
+          <t>Melakukan approval data pengajuan export</t>
         </is>
       </c>
       <c r="E883" s="56" t="inlineStr">
@@ -37285,34 +37285,34 @@
       </c>
       <c r="G883" s="56" t="inlineStr">
         <is>
-          <t>Klik button Batalkan pada halaman pindah kelolaan</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
         </is>
       </c>
       <c r="H883" s="56" t="inlineStr">
         <is>
-          <t>Kembali ke halaman utama Re-assign Prospek</t>
+          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
         </is>
       </c>
     </row>
     <row r="884" ht="28" customHeight="1">
       <c r="A884" s="55" t="inlineStr">
         <is>
-          <t>73.11</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="B884" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C884" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D884" s="56" t="inlineStr">
         <is>
-          <t>Validasi semua data prospek yang di re-assign</t>
+          <t>Melakukan reject data pengajuan export</t>
         </is>
       </c>
       <c r="E884" s="56" t="inlineStr">
@@ -37322,39 +37322,39 @@
       </c>
       <c r="F884" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G884" s="56" t="inlineStr">
         <is>
-          <t>Login menggunakan user yang sebelumnya sudah dipilih ketika re-assign prospek - Klik menu Lead Qualification - Klik submenu Aktifitas - Cek data yang sebelum nya di re-assign pada tabel dan pada detail prospek</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
         </is>
       </c>
       <c r="H884" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek yang sebelumnya di re-assign dan pada detail prospek menampilkan informasi ex. "Re-prospek dari Lead ID: 11370987"</t>
+          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
         </is>
       </c>
     </row>
     <row r="885" ht="42" customHeight="1">
       <c r="A885" s="55" t="inlineStr">
         <is>
-          <t>73.12</t>
+          <t>76.9</t>
         </is>
       </c>
       <c r="B885" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C885" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D885" s="56" t="inlineStr">
         <is>
-          <t>Melakukan Re-Assign Prospek</t>
+          <t>Melihat detail pengajuan export</t>
         </is>
       </c>
       <c r="E885" s="56" t="inlineStr">
@@ -37364,39 +37364,39 @@
       </c>
       <c r="F885" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G885" s="56" t="inlineStr">
         <is>
-          <t>Pilih prospek dengan klik checkbox - Klik button Re-Assign () data - Klik button Yes - Pilih kantor wilayah - Pilih kantor cabang - Pilih kantor cabang pembantu - Pilih sales - Klik button Submit</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H885" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign prospek ke sales yang di pilih dan menampilkan popup 'Berhasil melakukan Re-assign Prospek' kemudian data tersebut sudah tidak ada pada tabel re-assign prospek</t>
+          <t>Berhasil menampilkan detail data pengajuan export.</t>
         </is>
       </c>
     </row>
     <row r="886" ht="14" customHeight="1">
       <c r="A886" s="55" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>77.1</t>
         </is>
       </c>
       <c r="B886" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C886" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D886" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Re-Assign Management</t>
+          <t>Membuka halaman Aktivitas Export</t>
         </is>
       </c>
       <c r="E886" s="56" t="inlineStr">
@@ -37411,34 +37411,34 @@
       </c>
       <c r="G886" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Management</t>
+          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
         </is>
       </c>
       <c r="H886" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Re-Assign Management</t>
+          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
         </is>
       </c>
     </row>
     <row r="887" ht="42" customHeight="1">
       <c r="A887" s="55" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="B887" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C887" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D887" s="56" t="inlineStr">
         <is>
-          <t>Mencari data prospek pada halaman Re-Assign Management</t>
+          <t>Mencari data aktivitas export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E887" s="56" t="inlineStr">
@@ -37448,81 +37448,81 @@
       </c>
       <c r="F887" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G887" s="56" t="inlineStr">
         <is>
-          <t>Input nama nasabah pada field search - Klik icon search atau klik Enter</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H887" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data prospek Re-Assign Management sesuai dengan nama yang di cari</t>
+          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="888" ht="42" customHeight="1">
       <c r="A888" s="55" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="B888" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C888" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D888" s="56" t="inlineStr">
         <is>
-          <t>Mencari data prospek yang tidak ada pada halaman Re-Assign Management</t>
+          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E888" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F888" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G888" s="56" t="inlineStr">
         <is>
-          <t>Input nama nasabah yang datanya tidak ada - Klik icon search atau klik Enter</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H888" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan tabel kosong dengan keterangan no data</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="889" ht="28" customHeight="1">
       <c r="A889" s="55" t="inlineStr">
         <is>
-          <t>74.4</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="B889" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C889" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D889" s="56" t="inlineStr">
         <is>
-          <t>Validasi jumlah data yang di pilih untuk reassign</t>
+          <t>Melihat data aktivitas export berdasarkan status</t>
         </is>
       </c>
       <c r="E889" s="56" t="inlineStr">
@@ -37532,39 +37532,39 @@
       </c>
       <c r="F889" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G889" s="56" t="inlineStr">
         <is>
-          <t>cek jumlah data yang muncul pada button Reassign () data</t>
+          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H889" s="56" t="inlineStr">
         <is>
-          <t>Angka yang muncul pada button sesuai dengan jumlah data yang di pilih</t>
+          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="890" ht="42" customHeight="1">
       <c r="A890" s="55" t="inlineStr">
         <is>
-          <t>74.5</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="B890" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C890" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D890" s="56" t="inlineStr">
         <is>
-          <t>Validasi data prospek yang di re-assign ke sales</t>
+          <t>Melakukan filter data aktivitas export</t>
         </is>
       </c>
       <c r="E890" s="56" t="inlineStr">
@@ -37574,24 +37574,24 @@
       </c>
       <c r="F890" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G890" s="56" t="inlineStr">
         <is>
-          <t>Login dengan akun sales yang sebelumnya sudah di pilih reassign management - Klik menu Lead Qualification - Klik submenu Aktifitas Referal - Cek data prospek yang sudah di reassign</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H890" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek yang sesuai dari reassign management</t>
+          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="891" ht="14" customHeight="1">
       <c r="A891" s="55" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>77.6</t>
         </is>
       </c>
       <c r="B891" s="56" t="inlineStr">
@@ -37601,12 +37601,12 @@
       </c>
       <c r="C891" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D891" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Riwayat Export</t>
+          <t>Mereset filter data aktivitas export</t>
         </is>
       </c>
       <c r="E891" s="56" t="inlineStr">
@@ -37616,24 +37616,24 @@
       </c>
       <c r="F891" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G891" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Export Center - Klik submenu Riwayat Export</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H891" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Riwayat Export.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="892" ht="42" customHeight="1">
       <c r="A892" s="55" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="B892" s="56" t="inlineStr">
@@ -37643,12 +37643,12 @@
       </c>
       <c r="C892" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D892" s="56" t="inlineStr">
         <is>
-          <t>Mencari data riwayat export dengan kata kunci valid</t>
+          <t>Melihat detail aktivitas export</t>
         </is>
       </c>
       <c r="E892" s="56" t="inlineStr">
@@ -37658,24 +37658,24 @@
       </c>
       <c r="F892" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G892" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H892" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data riwayat export yang dicari.</t>
+          <t>Berhasil menampilkan detail data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="893" ht="42" customHeight="1">
       <c r="A893" s="55" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>77.8</t>
         </is>
       </c>
       <c r="B893" s="56" t="inlineStr">
@@ -37685,959 +37685,57 @@
       </c>
       <c r="C893" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D893" s="56" t="inlineStr">
         <is>
-          <t>Mencari data riwayat export dengan kata kunci tidak valid</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E893" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F893" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G893" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
+          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H893" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="894" ht="28" customHeight="1">
-      <c r="A894" s="55" t="inlineStr">
-        <is>
-          <t>75.4</t>
-        </is>
-      </c>
-      <c r="B894" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C894" s="56" t="inlineStr">
-        <is>
-          <t>Riwayat Export</t>
-        </is>
-      </c>
-      <c r="D894" s="56" t="inlineStr">
-        <is>
-          <t>Melihat data riwayat export berdasarkan status</t>
-        </is>
-      </c>
-      <c r="E894" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F894" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G894" s="56" t="inlineStr">
-        <is>
-          <t>Pada halaman Riwayat Export, klik salah satu tab status</t>
-        </is>
-      </c>
-      <c r="H894" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan daftar data riwayat export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="895" ht="42" customHeight="1">
-      <c r="A895" s="55" t="inlineStr">
-        <is>
-          <t>75.5</t>
-        </is>
-      </c>
-      <c r="B895" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C895" s="56" t="inlineStr">
-        <is>
-          <t>Riwayat Export</t>
-        </is>
-      </c>
-      <c r="D895" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data riwayat export</t>
-        </is>
-      </c>
-      <c r="E895" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F895" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G895" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H895" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data riwayat export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="896" ht="14" customHeight="1">
-      <c r="A896" s="55" t="inlineStr">
-        <is>
-          <t>75.6</t>
-        </is>
-      </c>
-      <c r="B896" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C896" s="56" t="inlineStr">
-        <is>
-          <t>Riwayat Export</t>
-        </is>
-      </c>
-      <c r="D896" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data riwayat export</t>
-        </is>
-      </c>
-      <c r="E896" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F896" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G896" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
-        </is>
-      </c>
-      <c r="H896" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data riwayat export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="897" ht="42" customHeight="1">
-      <c r="A897" s="55" t="inlineStr">
-        <is>
-          <t>75.7</t>
-        </is>
-      </c>
-      <c r="B897" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C897" s="56" t="inlineStr">
-        <is>
-          <t>Riwayat Export</t>
-        </is>
-      </c>
-      <c r="D897" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail riwayat export</t>
-        </is>
-      </c>
-      <c r="E897" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F897" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G897" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H897" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan drawer Export Detail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="898" ht="42" customHeight="1">
-      <c r="A898" s="55" t="inlineStr">
-        <is>
-          <t>75.8</t>
-        </is>
-      </c>
-      <c r="B898" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C898" s="56" t="inlineStr">
-        <is>
-          <t>Riwayat Export</t>
-        </is>
-      </c>
-      <c r="D898" s="56" t="inlineStr">
-        <is>
-          <t>Mengunduh file data export yang tersedia</t>
-        </is>
-      </c>
-      <c r="E898" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F898" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G898" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada baris data dengan status Tersedia - Klik opsi Download</t>
-        </is>
-      </c>
-      <c r="H898" s="56" t="inlineStr">
-        <is>
           <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>
-    <row r="899" ht="28" customHeight="1">
-      <c r="A899" s="55" t="inlineStr">
-        <is>
-          <t>76.1</t>
-        </is>
-      </c>
-      <c r="B899" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C899" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D899" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="E899" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F899" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G899" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="H899" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Persetujuan Export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="900" ht="42" customHeight="1">
-      <c r="A900" s="55" t="inlineStr">
-        <is>
-          <t>76.2</t>
-        </is>
-      </c>
-      <c r="B900" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C900" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D900" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data persetujuan export dengan kata kunci valid</t>
-        </is>
-      </c>
-      <c r="E900" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F900" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G900" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H900" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
-        </is>
-      </c>
-    </row>
-    <row r="901" ht="28" customHeight="1">
-      <c r="A901" s="55" t="inlineStr">
-        <is>
-          <t>76.3</t>
-        </is>
-      </c>
-      <c r="B901" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C901" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D901" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
-        </is>
-      </c>
-      <c r="E901" s="56" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F901" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G901" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H901" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="902" ht="28" customHeight="1">
-      <c r="A902" s="55" t="inlineStr">
-        <is>
-          <t>76.4</t>
-        </is>
-      </c>
-      <c r="B902" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C902" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D902" s="56" t="inlineStr">
-        <is>
-          <t>Melihat data persetujuan export berdasarkan status</t>
-        </is>
-      </c>
-      <c r="E902" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F902" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G902" s="56" t="inlineStr">
-        <is>
-          <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
-        </is>
-      </c>
-      <c r="H902" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="903" ht="28" customHeight="1">
-      <c r="A903" s="55" t="inlineStr">
-        <is>
-          <t>76.5</t>
-        </is>
-      </c>
-      <c r="B903" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C903" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D903" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data persetujuan export</t>
-        </is>
-      </c>
-      <c r="E903" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F903" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G903" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H903" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="904" ht="28" customHeight="1">
-      <c r="A904" s="55" t="inlineStr">
-        <is>
-          <t>76.6</t>
-        </is>
-      </c>
-      <c r="B904" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C904" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D904" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data persetujuan export</t>
-        </is>
-      </c>
-      <c r="E904" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F904" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G904" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
-        </is>
-      </c>
-      <c r="H904" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="905" ht="28" customHeight="1">
-      <c r="A905" s="55" t="inlineStr">
-        <is>
-          <t>76.7</t>
-        </is>
-      </c>
-      <c r="B905" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C905" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D905" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan approval data pengajuan export</t>
-        </is>
-      </c>
-      <c r="E905" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F905" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G905" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
-        </is>
-      </c>
-      <c r="H905" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
-        </is>
-      </c>
-    </row>
-    <row r="906" ht="42" customHeight="1">
-      <c r="A906" s="55" t="inlineStr">
-        <is>
-          <t>76.8</t>
-        </is>
-      </c>
-      <c r="B906" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C906" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D906" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan reject data pengajuan export</t>
-        </is>
-      </c>
-      <c r="E906" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F906" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G906" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
-        </is>
-      </c>
-      <c r="H906" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
-        </is>
-      </c>
-    </row>
-    <row r="907" ht="42" customHeight="1">
-      <c r="A907" s="55" t="inlineStr">
-        <is>
-          <t>76.9</t>
-        </is>
-      </c>
-      <c r="B907" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C907" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D907" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail pengajuan export</t>
-        </is>
-      </c>
-      <c r="E907" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F907" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G907" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H907" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data pengajuan export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="908" ht="28" customHeight="1">
-      <c r="A908" s="55" t="inlineStr">
-        <is>
-          <t>77.1</t>
-        </is>
-      </c>
-      <c r="B908" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C908" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D908" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="E908" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F908" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G908" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="H908" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="909" ht="14" customHeight="1">
-      <c r="A909" s="55" t="inlineStr">
-        <is>
-          <t>77.2</t>
-        </is>
-      </c>
-      <c r="B909" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C909" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D909" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data aktivitas export dengan kata kunci valid</t>
-        </is>
-      </c>
-      <c r="E909" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F909" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G909" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H909" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
-        </is>
-      </c>
-    </row>
-    <row r="910" ht="28" customHeight="1">
-      <c r="A910" s="55" t="inlineStr">
-        <is>
-          <t>77.3</t>
-        </is>
-      </c>
-      <c r="B910" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C910" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D910" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
-        </is>
-      </c>
-      <c r="E910" s="56" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F910" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G910" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H910" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="911" ht="28" customHeight="1">
-      <c r="A911" s="55" t="inlineStr">
-        <is>
-          <t>77.4</t>
-        </is>
-      </c>
-      <c r="B911" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C911" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D911" s="56" t="inlineStr">
-        <is>
-          <t>Melihat data aktivitas export berdasarkan status</t>
-        </is>
-      </c>
-      <c r="E911" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F911" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G911" s="56" t="inlineStr">
-        <is>
-          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
-        </is>
-      </c>
-      <c r="H911" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="912" ht="28" customHeight="1">
-      <c r="A912" s="55" t="inlineStr">
-        <is>
-          <t>77.5</t>
-        </is>
-      </c>
-      <c r="B912" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C912" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D912" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E912" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F912" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G912" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H912" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="913" ht="28" customHeight="1">
-      <c r="A913" s="55" t="inlineStr">
-        <is>
-          <t>77.6</t>
-        </is>
-      </c>
-      <c r="B913" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C913" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D913" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E913" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F913" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G913" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
-        </is>
-      </c>
-      <c r="H913" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="914" ht="28" customHeight="1">
-      <c r="A914" s="55" t="inlineStr">
-        <is>
-          <t>77.7</t>
-        </is>
-      </c>
-      <c r="B914" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C914" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D914" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail aktivitas export</t>
-        </is>
-      </c>
-      <c r="E914" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F914" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G914" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H914" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="915" ht="14" customHeight="1">
-      <c r="A915" s="55" t="inlineStr">
-        <is>
-          <t>77.8</t>
-        </is>
-      </c>
-      <c r="B915" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C915" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D915" s="56" t="inlineStr">
-        <is>
-          <t>Mengunduh file data export yang tersedia</t>
-        </is>
-      </c>
-      <c r="E915" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F915" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G915" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
-        </is>
-      </c>
-      <c r="H915" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mengunduh file data export.</t>
-        </is>
-      </c>
-    </row>
+    <row r="894" ht="28" customHeight="1"/>
+    <row r="895" ht="42" customHeight="1"/>
+    <row r="896" ht="14" customHeight="1"/>
+    <row r="897" ht="42" customHeight="1"/>
+    <row r="898" ht="42" customHeight="1"/>
+    <row r="899" ht="28" customHeight="1"/>
+    <row r="900" ht="42" customHeight="1"/>
+    <row r="901" ht="28" customHeight="1"/>
+    <row r="902" ht="28" customHeight="1"/>
+    <row r="903" ht="28" customHeight="1"/>
+    <row r="904" ht="28" customHeight="1"/>
+    <row r="905" ht="28" customHeight="1"/>
+    <row r="906" ht="42" customHeight="1"/>
+    <row r="907" ht="42" customHeight="1"/>
+    <row r="908" ht="28" customHeight="1"/>
+    <row r="909" ht="14" customHeight="1"/>
+    <row r="910" ht="28" customHeight="1"/>
+    <row r="911" ht="28" customHeight="1"/>
+    <row r="912" ht="28" customHeight="1"/>
+    <row r="913" ht="28" customHeight="1"/>
+    <row r="914" ht="28" customHeight="1"/>
+    <row r="915" ht="14" customHeight="1"/>
     <row r="916" ht="28" customHeight="1"/>
     <row r="917" ht="14" customHeight="1"/>
     <row r="918" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
chore: remove Regional Funnel (Funding & Lending) and sync Lead Generation & Qualification TCs
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z851"/>
+  <dimension ref="A1:Z842"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30942,12 +30942,12 @@
       </c>
       <c r="C732" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D732" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Regional Funnel</t>
+          <t>Membuka halaman Pengaturan Funnel Funding</t>
         </is>
       </c>
       <c r="E732" s="56" t="inlineStr">
@@ -30962,12 +30962,12 @@
       </c>
       <c r="G732" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Funding - Klik sub menu Regional Funnel</t>
+          <t>Klik menu Report Funding - Klik sub menu Pengaturan Funnel</t>
         </is>
       </c>
       <c r="H732" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Regional Funnel.</t>
+          <t>Berhasil menampilkan halaman Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -30984,12 +30984,12 @@
       </c>
       <c r="C733" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D733" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Regional Funnel</t>
+          <t>Menampilkan data Pengaturan Funnel Funding berdasarkan section</t>
         </is>
       </c>
       <c r="E733" s="56" t="inlineStr">
@@ -31004,12 +31004,12 @@
       </c>
       <c r="G733" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
+          <t>Klik salah satu daftar section pada tabel</t>
         </is>
       </c>
       <c r="H733" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan data pengaturan funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -31026,12 +31026,12 @@
       </c>
       <c r="C734" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D734" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Regional Funnel tanpa mengisi field mandatory</t>
+          <t>Mengubah data Pengaturan Funnel Funding</t>
         </is>
       </c>
       <c r="E734" s="56" t="inlineStr">
@@ -31041,17 +31041,17 @@
       </c>
       <c r="F734" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G734" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
+          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
         </is>
       </c>
       <c r="H734" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -31068,12 +31068,12 @@
       </c>
       <c r="C735" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D735" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Regional Funnel dengan keyword valid</t>
+          <t>Mengubah data Pengaturan Funnel Funding tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E735" s="56" t="inlineStr">
@@ -31083,17 +31083,17 @@
       </c>
       <c r="F735" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G735" s="56" t="inlineStr">
         <is>
-          <t>Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
         </is>
       </c>
       <c r="H735" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
@@ -31110,12 +31110,12 @@
       </c>
       <c r="C736" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D736" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Regional Funnel dengan keyword tidak valid</t>
+          <t>Menambahkan Condition pada Performance Indicator</t>
         </is>
       </c>
       <c r="E736" s="56" t="inlineStr">
@@ -31130,12 +31130,12 @@
       </c>
       <c r="G736" s="56" t="inlineStr">
         <is>
-          <t>Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H736" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
         </is>
       </c>
     </row>
@@ -31152,12 +31152,12 @@
       </c>
       <c r="C737" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D737" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data prospek berdasarkan kantor cabang</t>
+          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E737" s="56" t="inlineStr">
@@ -31172,19 +31172,19 @@
       </c>
       <c r="G737" s="56" t="inlineStr">
         <is>
-          <t>Klik salah satu daftar kantor cabang pada tabel</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H737" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek pada kantor cabang yang dipilih.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
     <row r="738" ht="28" customHeight="1">
       <c r="A738" s="55" t="inlineStr">
         <is>
-          <t>62.1</t>
+          <t>61.7</t>
         </is>
       </c>
       <c r="B738" s="56" t="inlineStr">
@@ -31199,7 +31199,7 @@
       </c>
       <c r="D738" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Pengaturan Funnel Funding</t>
+          <t>Menghapus Condition pada Performance Indicator</t>
         </is>
       </c>
       <c r="E738" s="56" t="inlineStr">
@@ -31209,24 +31209,24 @@
       </c>
       <c r="F738" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G738" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Funding - Klik sub menu Pengaturan Funnel</t>
+          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
         </is>
       </c>
       <c r="H738" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Pengaturan Funnel Funding.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
     <row r="739" ht="28" customHeight="1">
       <c r="A739" s="55" t="inlineStr">
         <is>
-          <t>62.2</t>
+          <t>62.1</t>
         </is>
       </c>
       <c r="B739" s="56" t="inlineStr">
@@ -31236,12 +31236,12 @@
       </c>
       <c r="C739" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D739" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data Pengaturan Funnel Funding berdasarkan section</t>
+          <t>Membuka halaman Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E739" s="56" t="inlineStr">
@@ -31251,24 +31251,24 @@
       </c>
       <c r="F739" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G739" s="56" t="inlineStr">
         <is>
-          <t>Klik salah satu daftar section pada tabel</t>
+          <t>Klik menu Report Funding - Klik sub menu Daily Sales Agenda</t>
         </is>
       </c>
       <c r="H739" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pengaturan funnel Funding.</t>
+          <t>Berhasil menampilkan halaman Daily Sales Agenda.</t>
         </is>
       </c>
     </row>
     <row r="740" ht="56" customHeight="1">
       <c r="A740" s="55" t="inlineStr">
         <is>
-          <t>62.3</t>
+          <t>62.2</t>
         </is>
       </c>
       <c r="B740" s="56" t="inlineStr">
@@ -31278,12 +31278,12 @@
       </c>
       <c r="C740" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D740" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Funding</t>
+          <t>Melakukan filter data Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E740" s="56" t="inlineStr">
@@ -31293,24 +31293,24 @@
       </c>
       <c r="F740" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G740" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
+          <t>Mengisi semua field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H740" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="741" ht="56" customHeight="1">
       <c r="A741" s="55" t="inlineStr">
         <is>
-          <t>62.4</t>
+          <t>62.3</t>
         </is>
       </c>
       <c r="B741" s="56" t="inlineStr">
@@ -31320,12 +31320,12 @@
       </c>
       <c r="C741" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D741" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Funding tanpa mengisi field mandatory</t>
+          <t>Melakukan filter data Daily Sales Agenda tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E741" s="56" t="inlineStr">
@@ -31335,24 +31335,24 @@
       </c>
       <c r="F741" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G741" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
+          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H741" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
     <row r="742" ht="14" customHeight="1">
       <c r="A742" s="55" t="inlineStr">
         <is>
-          <t>62.5</t>
+          <t>62.4</t>
         </is>
       </c>
       <c r="B742" s="56" t="inlineStr">
@@ -31362,12 +31362,12 @@
       </c>
       <c r="C742" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D742" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Menampilkan data tab Prospek Masuk</t>
         </is>
       </c>
       <c r="E742" s="56" t="inlineStr">
@@ -31382,19 +31382,19 @@
       </c>
       <c r="G742" s="56" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk</t>
         </is>
       </c>
       <c r="H742" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Masuk.</t>
         </is>
       </c>
     </row>
     <row r="743" ht="14" customHeight="1">
       <c r="A743" s="55" t="inlineStr">
         <is>
-          <t>62.6</t>
+          <t>62.5</t>
         </is>
       </c>
       <c r="B743" s="56" t="inlineStr">
@@ -31404,12 +31404,12 @@
       </c>
       <c r="C743" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D743" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
+          <t>Mencari data Prospek Masuk dengan keyword valid</t>
         </is>
       </c>
       <c r="E743" s="56" t="inlineStr">
@@ -31419,24 +31419,24 @@
       </c>
       <c r="F743" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G743" s="56" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H743" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="744" ht="14" customHeight="1">
       <c r="A744" s="55" t="inlineStr">
         <is>
-          <t>62.7</t>
+          <t>62.6</t>
         </is>
       </c>
       <c r="B744" s="56" t="inlineStr">
@@ -31446,17 +31446,17 @@
       </c>
       <c r="C744" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D744" s="56" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Mencari data Prospek Masuk dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E744" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F744" s="55" t="inlineStr">
@@ -31466,19 +31466,19 @@
       </c>
       <c r="G744" s="56" t="inlineStr">
         <is>
-          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H744" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="745" ht="14" customHeight="1">
       <c r="A745" s="55" t="inlineStr">
         <is>
-          <t>63.1</t>
+          <t>62.7</t>
         </is>
       </c>
       <c r="B745" s="56" t="inlineStr">
@@ -31493,7 +31493,7 @@
       </c>
       <c r="D745" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Daily Sales Agenda</t>
+          <t>Melihat detail Prospek Masuk</t>
         </is>
       </c>
       <c r="E745" s="56" t="inlineStr">
@@ -31503,24 +31503,24 @@
       </c>
       <c r="F745" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G745" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Funding - Klik sub menu Daily Sales Agenda</t>
+          <t>Klik tab Prospek Masuk - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H745" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Daily Sales Agenda.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="746" ht="28" customHeight="1">
       <c r="A746" s="55" t="inlineStr">
         <is>
-          <t>63.2</t>
+          <t>62.8</t>
         </is>
       </c>
       <c r="B746" s="56" t="inlineStr">
@@ -31535,7 +31535,7 @@
       </c>
       <c r="D746" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Daily Sales Agenda</t>
+          <t>Mengekspor data tab Prospek Masuk</t>
         </is>
       </c>
       <c r="E746" s="56" t="inlineStr">
@@ -31545,24 +31545,24 @@
       </c>
       <c r="F746" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G746" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Filter Data</t>
+          <t>Klik tab Prospek Masuk - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H746" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="747" ht="42" customHeight="1">
       <c r="A747" s="55" t="inlineStr">
         <is>
-          <t>63.3</t>
+          <t>62.9</t>
         </is>
       </c>
       <c r="B747" s="56" t="inlineStr">
@@ -31577,7 +31577,7 @@
       </c>
       <c r="D747" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Daily Sales Agenda tanpa mengisi field mandatory</t>
+          <t>Menampilkan data tab Prospek Closing</t>
         </is>
       </c>
       <c r="E747" s="56" t="inlineStr">
@@ -31592,19 +31592,19 @@
       </c>
       <c r="G747" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
+          <t>Klik tab Prospek Closing</t>
         </is>
       </c>
       <c r="H747" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Closing.</t>
         </is>
       </c>
     </row>
     <row r="748" ht="28" customHeight="1">
       <c r="A748" s="55" t="inlineStr">
         <is>
-          <t>63.4</t>
+          <t>62.10</t>
         </is>
       </c>
       <c r="B748" s="56" t="inlineStr">
@@ -31619,7 +31619,7 @@
       </c>
       <c r="D748" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Masuk</t>
+          <t>Mencari data Prospek Closing dengan keyword valid</t>
         </is>
       </c>
       <c r="E748" s="56" t="inlineStr">
@@ -31629,24 +31629,24 @@
       </c>
       <c r="F748" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G748" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk</t>
+          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H748" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Masuk.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="749" ht="14" customHeight="1">
       <c r="A749" s="55" t="inlineStr">
         <is>
-          <t>63.5</t>
+          <t>62.11</t>
         </is>
       </c>
       <c r="B749" s="56" t="inlineStr">
@@ -31661,34 +31661,34 @@
       </c>
       <c r="D749" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Masuk dengan keyword valid</t>
+          <t>Mencari data Prospek Closing dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E749" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F749" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G749" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H749" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="750" ht="14" customHeight="1">
       <c r="A750" s="55" t="inlineStr">
         <is>
-          <t>63.6</t>
+          <t>62.12</t>
         </is>
       </c>
       <c r="B750" s="56" t="inlineStr">
@@ -31703,12 +31703,12 @@
       </c>
       <c r="D750" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Masuk dengan keyword tidak valid</t>
+          <t>Melihat detail Prospek Closing</t>
         </is>
       </c>
       <c r="E750" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F750" s="55" t="inlineStr">
@@ -31718,19 +31718,19 @@
       </c>
       <c r="G750" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik tab Prospek Closing - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H750" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="751" ht="14" customHeight="1">
       <c r="A751" s="55" t="inlineStr">
         <is>
-          <t>63.7</t>
+          <t>62.13</t>
         </is>
       </c>
       <c r="B751" s="56" t="inlineStr">
@@ -31745,7 +31745,7 @@
       </c>
       <c r="D751" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Masuk</t>
+          <t>Mengekspor data tab Prospek Closing</t>
         </is>
       </c>
       <c r="E751" s="56" t="inlineStr">
@@ -31755,24 +31755,24 @@
       </c>
       <c r="F751" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G751" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik tab Prospek Closing - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H751" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="752" ht="14" customHeight="1">
       <c r="A752" s="55" t="inlineStr">
         <is>
-          <t>63.8</t>
+          <t>62.14</t>
         </is>
       </c>
       <c r="B752" s="56" t="inlineStr">
@@ -31787,7 +31787,7 @@
       </c>
       <c r="D752" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Masuk</t>
+          <t>Menampilkan data tab Prospek Referal</t>
         </is>
       </c>
       <c r="E752" s="56" t="inlineStr">
@@ -31797,24 +31797,24 @@
       </c>
       <c r="F752" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G752" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik tab Prospek Referal</t>
         </is>
       </c>
       <c r="H752" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Referal.</t>
         </is>
       </c>
     </row>
     <row r="753" ht="14" customHeight="1">
       <c r="A753" s="55" t="inlineStr">
         <is>
-          <t>63.9</t>
+          <t>62.15</t>
         </is>
       </c>
       <c r="B753" s="56" t="inlineStr">
@@ -31829,7 +31829,7 @@
       </c>
       <c r="D753" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Closing</t>
+          <t>Mencari data Prospek Referal dengan keyword valid</t>
         </is>
       </c>
       <c r="E753" s="56" t="inlineStr">
@@ -31839,24 +31839,24 @@
       </c>
       <c r="F753" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G753" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing</t>
+          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H753" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Closing.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="754" ht="14" customHeight="1">
       <c r="A754" s="55" t="inlineStr">
         <is>
-          <t>63.10</t>
+          <t>62.16</t>
         </is>
       </c>
       <c r="B754" s="56" t="inlineStr">
@@ -31871,34 +31871,34 @@
       </c>
       <c r="D754" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Closing dengan keyword valid</t>
+          <t>Mencari data Prospek Referal dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E754" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F754" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G754" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H754" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="755" ht="14" customHeight="1">
       <c r="A755" s="55" t="inlineStr">
         <is>
-          <t>63.11</t>
+          <t>62.17</t>
         </is>
       </c>
       <c r="B755" s="56" t="inlineStr">
@@ -31913,12 +31913,12 @@
       </c>
       <c r="D755" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Closing dengan keyword tidak valid</t>
+          <t>Melihat detail Prospek Referal</t>
         </is>
       </c>
       <c r="E755" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F755" s="55" t="inlineStr">
@@ -31928,19 +31928,19 @@
       </c>
       <c r="G755" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H755" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="756" ht="14" customHeight="1">
       <c r="A756" s="55" t="inlineStr">
         <is>
-          <t>63.12</t>
+          <t>62.18</t>
         </is>
       </c>
       <c r="B756" s="56" t="inlineStr">
@@ -31955,7 +31955,7 @@
       </c>
       <c r="D756" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Closing</t>
+          <t>Mengekspor data tab Prospek Referal</t>
         </is>
       </c>
       <c r="E756" s="56" t="inlineStr">
@@ -31965,24 +31965,24 @@
       </c>
       <c r="F756" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G756" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik tab Prospek Referal - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H756" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="757" ht="14" customHeight="1">
       <c r="A757" s="55" t="inlineStr">
         <is>
-          <t>63.13</t>
+          <t>62.19</t>
         </is>
       </c>
       <c r="B757" s="56" t="inlineStr">
@@ -31997,7 +31997,7 @@
       </c>
       <c r="D757" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Closing</t>
+          <t>Menampilkan data tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E757" s="56" t="inlineStr">
@@ -32007,24 +32007,24 @@
       </c>
       <c r="F757" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G757" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="H757" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Referal Closing.</t>
         </is>
       </c>
     </row>
     <row r="758" ht="14" customHeight="1">
       <c r="A758" s="55" t="inlineStr">
         <is>
-          <t>63.14</t>
+          <t>62.20</t>
         </is>
       </c>
       <c r="B758" s="56" t="inlineStr">
@@ -32039,7 +32039,7 @@
       </c>
       <c r="D758" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Referal</t>
+          <t>Mencari data Prospek Referal Closing dengan keyword valid</t>
         </is>
       </c>
       <c r="E758" s="56" t="inlineStr">
@@ -32049,24 +32049,24 @@
       </c>
       <c r="F758" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G758" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal</t>
+          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H758" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Referal.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="759" ht="14" customHeight="1">
       <c r="A759" s="55" t="inlineStr">
         <is>
-          <t>63.15</t>
+          <t>62.21</t>
         </is>
       </c>
       <c r="B759" s="56" t="inlineStr">
@@ -32081,34 +32081,34 @@
       </c>
       <c r="D759" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal dengan keyword valid</t>
+          <t>Mencari data Prospek Referal Closing dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E759" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F759" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G759" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H759" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="760" ht="14" customHeight="1">
       <c r="A760" s="55" t="inlineStr">
         <is>
-          <t>63.16</t>
+          <t>62.22</t>
         </is>
       </c>
       <c r="B760" s="56" t="inlineStr">
@@ -32123,12 +32123,12 @@
       </c>
       <c r="D760" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal dengan keyword tidak valid</t>
+          <t>Melihat detail Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E760" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F760" s="55" t="inlineStr">
@@ -32138,19 +32138,19 @@
       </c>
       <c r="G760" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal Closing - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H760" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="761" ht="14" customHeight="1">
       <c r="A761" s="55" t="inlineStr">
         <is>
-          <t>63.17</t>
+          <t>62.23</t>
         </is>
       </c>
       <c r="B761" s="56" t="inlineStr">
@@ -32165,7 +32165,7 @@
       </c>
       <c r="D761" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Referal</t>
+          <t>Mengekspor data tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E761" s="56" t="inlineStr">
@@ -32175,39 +32175,39 @@
       </c>
       <c r="F761" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G761" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik tab Prospek Referal Closing - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H761" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="762" ht="14" customHeight="1">
       <c r="A762" s="55" t="inlineStr">
         <is>
-          <t>63.18</t>
+          <t>63.1</t>
         </is>
       </c>
       <c r="B762" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C762" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Personal Funnel</t>
         </is>
       </c>
       <c r="D762" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Referal</t>
+          <t>Membuka halaman Personal Funnel</t>
         </is>
       </c>
       <c r="E762" s="56" t="inlineStr">
@@ -32217,39 +32217,39 @@
       </c>
       <c r="F762" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G762" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik menu Report Lending - Klik sub menu Personal Funnel</t>
         </is>
       </c>
       <c r="H762" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman Personal Funnel.</t>
         </is>
       </c>
     </row>
     <row r="763" ht="14" customHeight="1">
       <c r="A763" s="55" t="inlineStr">
         <is>
-          <t>63.19</t>
+          <t>63.2</t>
         </is>
       </c>
       <c r="B763" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C763" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Personal Funnel</t>
         </is>
       </c>
       <c r="D763" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Referal Closing</t>
+          <t>Melakukan filter data Personal Funnel</t>
         </is>
       </c>
       <c r="E763" s="56" t="inlineStr">
@@ -32264,34 +32264,34 @@
       </c>
       <c r="G763" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing</t>
+          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H763" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Referal Closing.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="764" ht="14" customHeight="1">
       <c r="A764" s="55" t="inlineStr">
         <is>
-          <t>63.20</t>
+          <t>63.3</t>
         </is>
       </c>
       <c r="B764" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C764" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Personal Funnel</t>
         </is>
       </c>
       <c r="D764" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal Closing dengan keyword valid</t>
+          <t>Melakukan filter data Personal Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E764" s="56" t="inlineStr">
@@ -32301,81 +32301,81 @@
       </c>
       <c r="F764" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G764" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H764" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
     <row r="765" ht="14" customHeight="1">
       <c r="A765" s="55" t="inlineStr">
         <is>
-          <t>63.21</t>
+          <t>63.4</t>
         </is>
       </c>
       <c r="B765" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C765" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Personal Funnel</t>
         </is>
       </c>
       <c r="D765" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal Closing dengan keyword tidak valid</t>
+          <t>Mengekspor data Personal Funnel</t>
         </is>
       </c>
       <c r="E765" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F765" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G765" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H765" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="766" ht="14" customHeight="1">
       <c r="A766" s="55" t="inlineStr">
         <is>
-          <t>63.22</t>
+          <t>64.1</t>
         </is>
       </c>
       <c r="B766" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C766" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Rekap Funnel</t>
         </is>
       </c>
       <c r="D766" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Referal Closing</t>
+          <t>Membuka halaman Rekap Funnel</t>
         </is>
       </c>
       <c r="E766" s="56" t="inlineStr">
@@ -32385,39 +32385,39 @@
       </c>
       <c r="F766" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G766" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik menu Report Lending - Klik sub menu Rekap Funnel</t>
         </is>
       </c>
       <c r="H766" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil menampilkan halaman Rekap Funnel.</t>
         </is>
       </c>
     </row>
     <row r="767" ht="28" customHeight="1">
       <c r="A767" s="55" t="inlineStr">
         <is>
-          <t>63.23</t>
+          <t>64.2</t>
         </is>
       </c>
       <c r="B767" s="56" t="inlineStr">
         <is>
-          <t>Report Funding</t>
+          <t>Report Lending</t>
         </is>
       </c>
       <c r="C767" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Rekap Funnel</t>
         </is>
       </c>
       <c r="D767" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Referal Closing</t>
+          <t>Menampilkan data Rekap Funnel</t>
         </is>
       </c>
       <c r="E767" s="56" t="inlineStr">
@@ -32427,24 +32427,24 @@
       </c>
       <c r="F767" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G767" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Mengisi field filter mandatory (Kantor Wilayah, Unit Bisnis, Produk, Info Bulan, Info Tahun) - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H767" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan daftar data Rekap Funnel di dalam tabel.</t>
         </is>
       </c>
     </row>
     <row r="768" ht="14" customHeight="1">
       <c r="A768" s="55" t="inlineStr">
         <is>
-          <t>64.1</t>
+          <t>64.3</t>
         </is>
       </c>
       <c r="B768" s="56" t="inlineStr">
@@ -32454,12 +32454,12 @@
       </c>
       <c r="C768" s="56" t="inlineStr">
         <is>
-          <t>Personal Funnel</t>
+          <t>Rekap Funnel</t>
         </is>
       </c>
       <c r="D768" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Personal Funnel</t>
+          <t>Melakukan filter data Rekap Funnel</t>
         </is>
       </c>
       <c r="E768" s="56" t="inlineStr">
@@ -32474,19 +32474,19 @@
       </c>
       <c r="G768" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Lending - Klik sub menu Personal Funnel</t>
+          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H768" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Personal Funnel.</t>
+          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="769" ht="14" customHeight="1">
       <c r="A769" s="55" t="inlineStr">
         <is>
-          <t>64.2</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="B769" s="56" t="inlineStr">
@@ -32496,12 +32496,12 @@
       </c>
       <c r="C769" s="56" t="inlineStr">
         <is>
-          <t>Personal Funnel</t>
+          <t>Rekap Funnel</t>
         </is>
       </c>
       <c r="D769" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Personal Funnel</t>
+          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E769" s="56" t="inlineStr">
@@ -32516,19 +32516,19 @@
       </c>
       <c r="G769" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
+          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H769" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
     <row r="770" ht="14" customHeight="1">
       <c r="A770" s="55" t="inlineStr">
         <is>
-          <t>64.3</t>
+          <t>64.5</t>
         </is>
       </c>
       <c r="B770" s="56" t="inlineStr">
@@ -32538,12 +32538,12 @@
       </c>
       <c r="C770" s="56" t="inlineStr">
         <is>
-          <t>Personal Funnel</t>
+          <t>Rekap Funnel</t>
         </is>
       </c>
       <c r="D770" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Personal Funnel tanpa mengisi field mandatory</t>
+          <t>Mengunduh data Rekap Funnel</t>
         </is>
       </c>
       <c r="E770" s="56" t="inlineStr">
@@ -32558,19 +32558,19 @@
       </c>
       <c r="G770" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
+          <t>Klik button Download Excel</t>
         </is>
       </c>
       <c r="H770" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil mendownload file Excel data Rekap Funnel.</t>
         </is>
       </c>
     </row>
     <row r="771" ht="14" customHeight="1">
       <c r="A771" s="55" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>65.1</t>
         </is>
       </c>
       <c r="B771" s="56" t="inlineStr">
@@ -32580,12 +32580,12 @@
       </c>
       <c r="C771" s="56" t="inlineStr">
         <is>
-          <t>Personal Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D771" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data Personal Funnel</t>
+          <t>Membuka halaman Pengaturan Funnel Lending</t>
         </is>
       </c>
       <c r="E771" s="56" t="inlineStr">
@@ -32600,19 +32600,19 @@
       </c>
       <c r="G771" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik menu Report Lending - Klik sub menu Pengaturan Funnel</t>
         </is>
       </c>
       <c r="H771" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
     <row r="772" ht="14" customHeight="1">
       <c r="A772" s="55" t="inlineStr">
         <is>
-          <t>65.1</t>
+          <t>65.2</t>
         </is>
       </c>
       <c r="B772" s="56" t="inlineStr">
@@ -32622,12 +32622,12 @@
       </c>
       <c r="C772" s="56" t="inlineStr">
         <is>
-          <t>Rekap Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D772" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Rekap Funnel</t>
+          <t>Menampilkan data Pengaturan Funnel Lending berdasarkan section</t>
         </is>
       </c>
       <c r="E772" s="56" t="inlineStr">
@@ -32637,24 +32637,24 @@
       </c>
       <c r="F772" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G772" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Lending - Klik sub menu Rekap Funnel</t>
+          <t>Klik salah satu daftar section pada tabel</t>
         </is>
       </c>
       <c r="H772" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Rekap Funnel.</t>
+          <t>Berhasil menampilkan data pengaturan funnel Lending.</t>
         </is>
       </c>
     </row>
     <row r="773" ht="14" customHeight="1">
       <c r="A773" s="55" t="inlineStr">
         <is>
-          <t>65.2</t>
+          <t>65.3</t>
         </is>
       </c>
       <c r="B773" s="56" t="inlineStr">
@@ -32664,12 +32664,12 @@
       </c>
       <c r="C773" s="56" t="inlineStr">
         <is>
-          <t>Rekap Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D773" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data Rekap Funnel</t>
+          <t>Mengubah data Pengaturan Funnel Lending</t>
         </is>
       </c>
       <c r="E773" s="56" t="inlineStr">
@@ -32679,24 +32679,24 @@
       </c>
       <c r="F773" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G773" s="56" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory (Kantor Wilayah, Unit Bisnis, Produk, Info Bulan, Info Tahun) - Klik button Filter Data</t>
+          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
         </is>
       </c>
       <c r="H773" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan daftar data Rekap Funnel di dalam tabel.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
     <row r="774" ht="14" customHeight="1">
       <c r="A774" s="55" t="inlineStr">
         <is>
-          <t>65.3</t>
+          <t>65.4</t>
         </is>
       </c>
       <c r="B774" s="56" t="inlineStr">
@@ -32706,12 +32706,12 @@
       </c>
       <c r="C774" s="56" t="inlineStr">
         <is>
-          <t>Rekap Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D774" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel</t>
+          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E774" s="56" t="inlineStr">
@@ -32721,24 +32721,24 @@
       </c>
       <c r="F774" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G774" s="56" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
+          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
         </is>
       </c>
       <c r="H774" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
     <row r="775" ht="14" customHeight="1">
       <c r="A775" s="55" t="inlineStr">
         <is>
-          <t>65.4</t>
+          <t>65.5</t>
         </is>
       </c>
       <c r="B775" s="56" t="inlineStr">
@@ -32748,12 +32748,12 @@
       </c>
       <c r="C775" s="56" t="inlineStr">
         <is>
-          <t>Rekap Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D775" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
+          <t>Menambahkan Condition pada Performance Indicator</t>
         </is>
       </c>
       <c r="E775" s="56" t="inlineStr">
@@ -32768,19 +32768,19 @@
       </c>
       <c r="G775" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H775" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
         </is>
       </c>
     </row>
     <row r="776" ht="14" customHeight="1">
       <c r="A776" s="55" t="inlineStr">
         <is>
-          <t>65.5</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="B776" s="56" t="inlineStr">
@@ -32790,12 +32790,12 @@
       </c>
       <c r="C776" s="56" t="inlineStr">
         <is>
-          <t>Rekap Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D776" s="56" t="inlineStr">
         <is>
-          <t>Mengunduh data Rekap Funnel</t>
+          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E776" s="56" t="inlineStr">
@@ -32810,19 +32810,19 @@
       </c>
       <c r="G776" s="56" t="inlineStr">
         <is>
-          <t>Klik button Download Excel</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H776" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file Excel data Rekap Funnel.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
     <row r="777" ht="14" customHeight="1">
       <c r="A777" s="55" t="inlineStr">
         <is>
-          <t>66.1</t>
+          <t>65.7</t>
         </is>
       </c>
       <c r="B777" s="56" t="inlineStr">
@@ -32832,12 +32832,12 @@
       </c>
       <c r="C777" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Pengaturan Funnel</t>
         </is>
       </c>
       <c r="D777" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Regional Funnel</t>
+          <t>Menghapus Condition pada Performance Indicator</t>
         </is>
       </c>
       <c r="E777" s="56" t="inlineStr">
@@ -32852,19 +32852,19 @@
       </c>
       <c r="G777" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Lending - Klik sub menu Regional Funnel</t>
+          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
         </is>
       </c>
       <c r="H777" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Regional Funnel.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
     <row r="778" ht="14" customHeight="1">
       <c r="A778" s="55" t="inlineStr">
         <is>
-          <t>66.2</t>
+          <t>66.1</t>
         </is>
       </c>
       <c r="B778" s="56" t="inlineStr">
@@ -32874,12 +32874,12 @@
       </c>
       <c r="C778" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D778" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Regional Funnel</t>
+          <t>Membuka halaman Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E778" s="56" t="inlineStr">
@@ -32889,24 +32889,24 @@
       </c>
       <c r="F778" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G778" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
+          <t>Klik menu Report Lending - Klik sub menu Daily Sales Agenda</t>
         </is>
       </c>
       <c r="H778" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman Daily Sales Agenda.</t>
         </is>
       </c>
     </row>
     <row r="779" ht="28" customHeight="1">
       <c r="A779" s="55" t="inlineStr">
         <is>
-          <t>66.3</t>
+          <t>66.2</t>
         </is>
       </c>
       <c r="B779" s="56" t="inlineStr">
@@ -32916,12 +32916,12 @@
       </c>
       <c r="C779" s="56" t="inlineStr">
         <is>
-          <t>Regional Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D779" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Regional Funnel tanpa mengisi field mandatory</t>
+          <t>Melakukan filter data Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E779" s="56" t="inlineStr">
@@ -32936,19 +32936,19 @@
       </c>
       <c r="G779" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
+          <t>Mengisi semua field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H779" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="780" ht="14" customHeight="1">
       <c r="A780" s="55" t="inlineStr">
         <is>
-          <t>67.1</t>
+          <t>66.3</t>
         </is>
       </c>
       <c r="B780" s="56" t="inlineStr">
@@ -32958,12 +32958,12 @@
       </c>
       <c r="C780" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D780" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Pengaturan Funnel Lending</t>
+          <t>Melakukan filter data Daily Sales Agenda tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E780" s="56" t="inlineStr">
@@ -32973,24 +32973,24 @@
       </c>
       <c r="F780" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G780" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Lending - Klik sub menu Pengaturan Funnel</t>
+          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H780" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Pengaturan Funnel Lending.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
     <row r="781" ht="28" customHeight="1">
       <c r="A781" s="55" t="inlineStr">
         <is>
-          <t>67.2</t>
+          <t>66.4</t>
         </is>
       </c>
       <c r="B781" s="56" t="inlineStr">
@@ -33000,12 +33000,12 @@
       </c>
       <c r="C781" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D781" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data Pengaturan Funnel Lending berdasarkan section</t>
+          <t>Menampilkan data tab Prospek Masuk</t>
         </is>
       </c>
       <c r="E781" s="56" t="inlineStr">
@@ -33020,19 +33020,19 @@
       </c>
       <c r="G781" s="56" t="inlineStr">
         <is>
-          <t>Klik salah satu daftar section pada tabel</t>
+          <t>Klik tab Prospek Masuk</t>
         </is>
       </c>
       <c r="H781" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pengaturan funnel Lending.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Masuk.</t>
         </is>
       </c>
     </row>
     <row r="782" ht="14" customHeight="1">
       <c r="A782" s="55" t="inlineStr">
         <is>
-          <t>67.3</t>
+          <t>66.5</t>
         </is>
       </c>
       <c r="B782" s="56" t="inlineStr">
@@ -33042,12 +33042,12 @@
       </c>
       <c r="C782" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D782" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending</t>
+          <t>Mencari data Prospek Masuk dengan keyword valid</t>
         </is>
       </c>
       <c r="E782" s="56" t="inlineStr">
@@ -33062,19 +33062,19 @@
       </c>
       <c r="G782" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H782" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="783" ht="14" customHeight="1">
       <c r="A783" s="55" t="inlineStr">
         <is>
-          <t>67.4</t>
+          <t>66.6</t>
         </is>
       </c>
       <c r="B783" s="56" t="inlineStr">
@@ -33084,39 +33084,39 @@
       </c>
       <c r="C783" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D783" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
+          <t>Mencari data Prospek Masuk dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E783" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F783" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G783" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H783" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="784" ht="14" customHeight="1">
       <c r="A784" s="55" t="inlineStr">
         <is>
-          <t>67.5</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="B784" s="56" t="inlineStr">
@@ -33126,12 +33126,12 @@
       </c>
       <c r="C784" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D784" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Melihat detail Prospek Masuk</t>
         </is>
       </c>
       <c r="E784" s="56" t="inlineStr">
@@ -33146,19 +33146,19 @@
       </c>
       <c r="G784" s="56" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H784" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="785" ht="14" customHeight="1">
       <c r="A785" s="55" t="inlineStr">
         <is>
-          <t>67.6</t>
+          <t>66.8</t>
         </is>
       </c>
       <c r="B785" s="56" t="inlineStr">
@@ -33168,12 +33168,12 @@
       </c>
       <c r="C785" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D785" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
+          <t>Mengekspor data tab Prospek Masuk</t>
         </is>
       </c>
       <c r="E785" s="56" t="inlineStr">
@@ -33183,24 +33183,24 @@
       </c>
       <c r="F785" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G785" s="56" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik tab Prospek Masuk - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H785" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="786" ht="14" customHeight="1">
       <c r="A786" s="55" t="inlineStr">
         <is>
-          <t>67.7</t>
+          <t>66.9</t>
         </is>
       </c>
       <c r="B786" s="56" t="inlineStr">
@@ -33210,12 +33210,12 @@
       </c>
       <c r="C786" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Funnel</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D786" s="56" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Menampilkan data tab Prospek Closing</t>
         </is>
       </c>
       <c r="E786" s="56" t="inlineStr">
@@ -33230,19 +33230,19 @@
       </c>
       <c r="G786" s="56" t="inlineStr">
         <is>
-          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
+          <t>Klik tab Prospek Closing</t>
         </is>
       </c>
       <c r="H786" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Closing.</t>
         </is>
       </c>
     </row>
     <row r="787" ht="14" customHeight="1">
       <c r="A787" s="55" t="inlineStr">
         <is>
-          <t>68.1</t>
+          <t>66.10</t>
         </is>
       </c>
       <c r="B787" s="56" t="inlineStr">
@@ -33257,7 +33257,7 @@
       </c>
       <c r="D787" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Daily Sales Agenda</t>
+          <t>Mencari data Prospek Closing dengan keyword valid</t>
         </is>
       </c>
       <c r="E787" s="56" t="inlineStr">
@@ -33272,19 +33272,19 @@
       </c>
       <c r="G787" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Report Lending - Klik sub menu Daily Sales Agenda</t>
+          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H787" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Daily Sales Agenda.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="788" ht="14" customHeight="1">
       <c r="A788" s="55" t="inlineStr">
         <is>
-          <t>68.2</t>
+          <t>66.11</t>
         </is>
       </c>
       <c r="B788" s="56" t="inlineStr">
@@ -33299,12 +33299,12 @@
       </c>
       <c r="D788" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Daily Sales Agenda</t>
+          <t>Mencari data Prospek Closing dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E788" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F788" s="55" t="inlineStr">
@@ -33314,19 +33314,19 @@
       </c>
       <c r="G788" s="56" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Filter Data</t>
+          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H788" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="789" ht="14" customHeight="1">
       <c r="A789" s="55" t="inlineStr">
         <is>
-          <t>68.3</t>
+          <t>66.12</t>
         </is>
       </c>
       <c r="B789" s="56" t="inlineStr">
@@ -33341,7 +33341,7 @@
       </c>
       <c r="D789" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Daily Sales Agenda tanpa mengisi field mandatory</t>
+          <t>Melihat detail Prospek Closing</t>
         </is>
       </c>
       <c r="E789" s="56" t="inlineStr">
@@ -33356,19 +33356,19 @@
       </c>
       <c r="G789" s="56" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
+          <t>Klik tab Prospek Closing - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H789" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="790" ht="14" customHeight="1">
       <c r="A790" s="55" t="inlineStr">
         <is>
-          <t>68.4</t>
+          <t>66.13</t>
         </is>
       </c>
       <c r="B790" s="56" t="inlineStr">
@@ -33383,7 +33383,7 @@
       </c>
       <c r="D790" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Masuk</t>
+          <t>Mengekspor data tab Prospek Closing</t>
         </is>
       </c>
       <c r="E790" s="56" t="inlineStr">
@@ -33393,24 +33393,24 @@
       </c>
       <c r="F790" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G790" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk</t>
+          <t>Klik tab Prospek Closing - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H790" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Masuk.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="791" ht="14" customHeight="1">
       <c r="A791" s="55" t="inlineStr">
         <is>
-          <t>68.5</t>
+          <t>66.14</t>
         </is>
       </c>
       <c r="B791" s="56" t="inlineStr">
@@ -33425,7 +33425,7 @@
       </c>
       <c r="D791" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Masuk dengan keyword valid</t>
+          <t>Menampilkan data tab Prospek Referal</t>
         </is>
       </c>
       <c r="E791" s="56" t="inlineStr">
@@ -33435,24 +33435,24 @@
       </c>
       <c r="F791" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G791" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal</t>
         </is>
       </c>
       <c r="H791" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Referal.</t>
         </is>
       </c>
     </row>
     <row r="792" ht="14" customHeight="1">
       <c r="A792" s="55" t="inlineStr">
         <is>
-          <t>68.6</t>
+          <t>66.15</t>
         </is>
       </c>
       <c r="B792" s="56" t="inlineStr">
@@ -33467,34 +33467,34 @@
       </c>
       <c r="D792" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Masuk dengan keyword tidak valid</t>
+          <t>Mencari data Prospek Referal dengan keyword valid</t>
         </is>
       </c>
       <c r="E792" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F792" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G792" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H792" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="793" ht="14" customHeight="1">
       <c r="A793" s="55" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>66.16</t>
         </is>
       </c>
       <c r="B793" s="56" t="inlineStr">
@@ -33509,12 +33509,12 @@
       </c>
       <c r="D793" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Masuk</t>
+          <t>Mencari data Prospek Referal dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E793" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F793" s="55" t="inlineStr">
@@ -33524,19 +33524,19 @@
       </c>
       <c r="G793" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H793" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="794" ht="14" customHeight="1">
       <c r="A794" s="55" t="inlineStr">
         <is>
-          <t>68.8</t>
+          <t>66.17</t>
         </is>
       </c>
       <c r="B794" s="56" t="inlineStr">
@@ -33551,7 +33551,7 @@
       </c>
       <c r="D794" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Masuk</t>
+          <t>Melihat detail Prospek Referal</t>
         </is>
       </c>
       <c r="E794" s="56" t="inlineStr">
@@ -33561,24 +33561,24 @@
       </c>
       <c r="F794" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G794" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Masuk - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik tab Prospek Referal - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H794" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="795" ht="14" customHeight="1">
       <c r="A795" s="55" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>66.18</t>
         </is>
       </c>
       <c r="B795" s="56" t="inlineStr">
@@ -33593,7 +33593,7 @@
       </c>
       <c r="D795" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Closing</t>
+          <t>Mengekspor data tab Prospek Referal</t>
         </is>
       </c>
       <c r="E795" s="56" t="inlineStr">
@@ -33603,24 +33603,24 @@
       </c>
       <c r="F795" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G795" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing</t>
+          <t>Klik tab Prospek Referal - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H795" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Closing.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="796" ht="14" customHeight="1">
       <c r="A796" s="55" t="inlineStr">
         <is>
-          <t>68.10</t>
+          <t>66.19</t>
         </is>
       </c>
       <c r="B796" s="56" t="inlineStr">
@@ -33635,7 +33635,7 @@
       </c>
       <c r="D796" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Closing dengan keyword valid</t>
+          <t>Menampilkan data tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E796" s="56" t="inlineStr">
@@ -33645,24 +33645,24 @@
       </c>
       <c r="F796" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G796" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="H796" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data pada tab Prospek Referal Closing.</t>
         </is>
       </c>
     </row>
     <row r="797" ht="14" customHeight="1">
       <c r="A797" s="55" t="inlineStr">
         <is>
-          <t>68.11</t>
+          <t>66.20</t>
         </is>
       </c>
       <c r="B797" s="56" t="inlineStr">
@@ -33677,34 +33677,34 @@
       </c>
       <c r="D797" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Closing dengan keyword tidak valid</t>
+          <t>Mencari data Prospek Referal Closing dengan keyword valid</t>
         </is>
       </c>
       <c r="E797" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F797" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G797" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H797" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="798" ht="14" customHeight="1">
       <c r="A798" s="55" t="inlineStr">
         <is>
-          <t>68.12</t>
+          <t>66.21</t>
         </is>
       </c>
       <c r="B798" s="56" t="inlineStr">
@@ -33719,12 +33719,12 @@
       </c>
       <c r="D798" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Closing</t>
+          <t>Mencari data Prospek Referal Closing dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E798" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F798" s="55" t="inlineStr">
@@ -33734,19 +33734,19 @@
       </c>
       <c r="G798" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
         </is>
       </c>
       <c r="H798" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="799" ht="14" customHeight="1">
       <c r="A799" s="55" t="inlineStr">
         <is>
-          <t>68.13</t>
+          <t>66.22</t>
         </is>
       </c>
       <c r="B799" s="56" t="inlineStr">
@@ -33761,7 +33761,7 @@
       </c>
       <c r="D799" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Closing</t>
+          <t>Melihat detail Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E799" s="56" t="inlineStr">
@@ -33771,24 +33771,24 @@
       </c>
       <c r="F799" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G799" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Closing - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik tab Prospek Referal Closing - Klik salah satu nama prospek pada tabel</t>
         </is>
       </c>
       <c r="H799" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman detail prospek.</t>
         </is>
       </c>
     </row>
     <row r="800" ht="14" customHeight="1">
       <c r="A800" s="55" t="inlineStr">
         <is>
-          <t>68.14</t>
+          <t>66.23</t>
         </is>
       </c>
       <c r="B800" s="56" t="inlineStr">
@@ -33803,7 +33803,7 @@
       </c>
       <c r="D800" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Referal</t>
+          <t>Mengekspor data tab Prospek Referal Closing</t>
         </is>
       </c>
       <c r="E800" s="56" t="inlineStr">
@@ -33813,39 +33813,39 @@
       </c>
       <c r="F800" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G800" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal</t>
+          <t>Klik tab Prospek Referal Closing - Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H800" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Referal.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="801" ht="14" customHeight="1">
       <c r="A801" s="55" t="inlineStr">
         <is>
-          <t>68.15</t>
+          <t>67.1</t>
         </is>
       </c>
       <c r="B801" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C801" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D801" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal dengan keyword valid</t>
+          <t>Membuka halaman Approval non Banking</t>
         </is>
       </c>
       <c r="E801" s="56" t="inlineStr">
@@ -33860,39 +33860,39 @@
       </c>
       <c r="G801" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Approval non banking</t>
         </is>
       </c>
       <c r="H801" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Menampilkan halaman Approval non banking.</t>
         </is>
       </c>
     </row>
     <row r="802" ht="14" customHeight="1">
       <c r="A802" s="55" t="inlineStr">
         <is>
-          <t>68.16</t>
+          <t>67.2</t>
         </is>
       </c>
       <c r="B802" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C802" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D802" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal dengan keyword tidak valid</t>
+          <t>Melakukan filter data Approval non Banking</t>
         </is>
       </c>
       <c r="E802" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F802" s="55" t="inlineStr">
@@ -33902,34 +33902,34 @@
       </c>
       <c r="G802" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Pilih filter Sales, Produk, Bulan, Tahun - Klik button Submit</t>
         </is>
       </c>
       <c r="H802" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil memfilter dan menampilkan data Approval non banking sesuai filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="803" ht="14" customHeight="1">
       <c r="A803" s="55" t="inlineStr">
         <is>
-          <t>68.17</t>
+          <t>67.3</t>
         </is>
       </c>
       <c r="B803" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C803" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D803" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Referal</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E803" s="56" t="inlineStr">
@@ -33944,76 +33944,76 @@
       </c>
       <c r="G803" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Klik salah satu nama prospek pada tabel</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H803" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Berhasil menampilkan data Approval non banking yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="804" ht="14" customHeight="1">
       <c r="A804" s="55" t="inlineStr">
         <is>
-          <t>68.18</t>
+          <t>67.4</t>
         </is>
       </c>
       <c r="B804" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C804" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D804" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Referal</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E804" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F804" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G804" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H804" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="805" ht="14" customHeight="1">
       <c r="A805" s="55" t="inlineStr">
         <is>
-          <t>68.19</t>
+          <t>67.5</t>
         </is>
       </c>
       <c r="B805" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C805" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D805" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan data tab Prospek Referal Closing</t>
+          <t>Melakukan approval data prospek</t>
         </is>
       </c>
       <c r="E805" s="56" t="inlineStr">
@@ -34023,39 +34023,39 @@
       </c>
       <c r="F805" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G805" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing</t>
+          <t>Klik titik tiga pada data status PENDING - Klik Setujui - Input Realisasi dan Remark - Klik button Setujui</t>
         </is>
       </c>
       <c r="H805" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek Referal Closing.</t>
+          <t>Berhasil menyetujui prospek.</t>
         </is>
       </c>
     </row>
     <row r="806" ht="14" customHeight="1">
       <c r="A806" s="55" t="inlineStr">
         <is>
-          <t>68.20</t>
+          <t>67.6</t>
         </is>
       </c>
       <c r="B806" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C806" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D806" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal Closing dengan keyword valid</t>
+          <t>Melakukan reject data prospek</t>
         </is>
       </c>
       <c r="E806" s="56" t="inlineStr">
@@ -34070,76 +34070,76 @@
       </c>
       <c r="G806" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword valid - Klik button Search</t>
+          <t>Klik titik tiga pada data status PENDING - Klik Tolak - Input Remark - Klik button Tolak</t>
         </is>
       </c>
       <c r="H806" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menolak prospek.</t>
         </is>
       </c>
     </row>
     <row r="807" ht="14" customHeight="1">
       <c r="A807" s="55" t="inlineStr">
         <is>
-          <t>68.21</t>
+          <t>67.7</t>
         </is>
       </c>
       <c r="B807" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C807" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Approval non Banking</t>
         </is>
       </c>
       <c r="D807" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Prospek Referal Closing dengan keyword tidak valid</t>
+          <t>Melihat detail data prospek</t>
         </is>
       </c>
       <c r="E807" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F807" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G807" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Mengisi field Cari Data dengan keyword tidak valid - Klik button Search</t>
+          <t>Klik titik tiga pada data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H807" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan detail data prospek.</t>
         </is>
       </c>
     </row>
     <row r="808" ht="14" customHeight="1">
       <c r="A808" s="55" t="inlineStr">
         <is>
-          <t>68.22</t>
+          <t>68.1</t>
         </is>
       </c>
       <c r="B808" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C808" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D808" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail Prospek Referal Closing</t>
+          <t>Membuka halaman Re-Assign Prospek</t>
         </is>
       </c>
       <c r="E808" s="56" t="inlineStr">
@@ -34149,39 +34149,39 @@
       </c>
       <c r="F808" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G808" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Klik salah satu nama prospek pada tabel</t>
+          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Prospek</t>
         </is>
       </c>
       <c r="H808" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail prospek.</t>
+          <t>Menampilkan halaman Re-Assign Prospek.</t>
         </is>
       </c>
     </row>
     <row r="809" ht="14" customHeight="1">
       <c r="A809" s="55" t="inlineStr">
         <is>
-          <t>68.23</t>
+          <t>68.2</t>
         </is>
       </c>
       <c r="B809" s="56" t="inlineStr">
         <is>
-          <t>Report Lending</t>
+          <t>Re-Assign dan Approval</t>
         </is>
       </c>
       <c r="C809" s="56" t="inlineStr">
         <is>
-          <t>Daily Sales Agenda</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D809" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tab Prospek Referal Closing</t>
+          <t>Melakukan filter data Re-Assign Prospek</t>
         </is>
       </c>
       <c r="E809" s="56" t="inlineStr">
@@ -34191,24 +34191,24 @@
       </c>
       <c r="F809" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G809" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Prospek Referal Closing - Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik button Filter - Pilih Produk dan Sales pada drawer Filter - Klik button Filter</t>
         </is>
       </c>
       <c r="H809" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil memfilter dan menampilkan data prospek sesuai kriteria.</t>
         </is>
       </c>
     </row>
     <row r="810" ht="42" customHeight="1">
       <c r="A810" s="55" t="inlineStr">
         <is>
-          <t>69.1</t>
+          <t>68.3</t>
         </is>
       </c>
       <c r="B810" s="56" t="inlineStr">
@@ -34218,12 +34218,12 @@
       </c>
       <c r="C810" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D810" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Approval non Banking</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E810" s="56" t="inlineStr">
@@ -34233,24 +34233,24 @@
       </c>
       <c r="F810" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G810" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Approval non banking</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H810" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Approval non banking.</t>
+          <t>Berhasil menampilkan data prospek yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="811" ht="28" customHeight="1">
       <c r="A811" s="55" t="inlineStr">
         <is>
-          <t>69.2</t>
+          <t>68.4</t>
         </is>
       </c>
       <c r="B811" s="56" t="inlineStr">
@@ -34260,17 +34260,17 @@
       </c>
       <c r="C811" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D811" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Approval non Banking</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E811" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F811" s="55" t="inlineStr">
@@ -34280,19 +34280,19 @@
       </c>
       <c r="G811" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Sales, Produk, Bulan, Tahun - Klik button Submit</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H811" s="56" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan data Approval non banking sesuai filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="812" ht="42" customHeight="1">
       <c r="A812" s="55" t="inlineStr">
         <is>
-          <t>69.3</t>
+          <t>68.5</t>
         </is>
       </c>
       <c r="B812" s="56" t="inlineStr">
@@ -34302,12 +34302,12 @@
       </c>
       <c r="C812" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D812" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci valid</t>
+          <t>Melakukan re-assign beberapa data prospek</t>
         </is>
       </c>
       <c r="E812" s="56" t="inlineStr">
@@ -34317,24 +34317,24 @@
       </c>
       <c r="F812" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G812" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
+          <t>Checklist beberapa data prospek - Klik button Reassign () data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H812" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data Approval non banking yang dicari.</t>
+          <t>Berhasil melakukan re-assign data prospek yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="813" ht="28" customHeight="1">
       <c r="A813" s="55" t="inlineStr">
         <is>
-          <t>69.4</t>
+          <t>68.6</t>
         </is>
       </c>
       <c r="B813" s="56" t="inlineStr">
@@ -34344,39 +34344,39 @@
       </c>
       <c r="C813" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Prospek</t>
         </is>
       </c>
       <c r="D813" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci tidak valid</t>
+          <t>Melakukan re-assign semua data prospek</t>
         </is>
       </c>
       <c r="E813" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F813" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G813" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
+          <t>Klik button Reassign Semua data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H813" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>Berhasil melakukan re-assign seluruh data prospek.</t>
         </is>
       </c>
     </row>
     <row r="814" ht="28" customHeight="1">
       <c r="A814" s="55" t="inlineStr">
         <is>
-          <t>69.5</t>
+          <t>69.1</t>
         </is>
       </c>
       <c r="B814" s="56" t="inlineStr">
@@ -34386,12 +34386,12 @@
       </c>
       <c r="C814" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D814" s="56" t="inlineStr">
         <is>
-          <t>Melakukan approval data prospek</t>
+          <t>Membuka halaman Re-Assign Management</t>
         </is>
       </c>
       <c r="E814" s="56" t="inlineStr">
@@ -34406,19 +34406,19 @@
       </c>
       <c r="G814" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga pada data status PENDING - Klik Setujui - Input Realisasi dan Remark - Klik button Setujui</t>
+          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Management</t>
         </is>
       </c>
       <c r="H814" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyetujui prospek.</t>
+          <t>Menampilkan halaman Re-Assign Management.</t>
         </is>
       </c>
     </row>
     <row r="815" ht="56" customHeight="1">
       <c r="A815" s="55" t="inlineStr">
         <is>
-          <t>69.6</t>
+          <t>69.2</t>
         </is>
       </c>
       <c r="B815" s="56" t="inlineStr">
@@ -34428,12 +34428,12 @@
       </c>
       <c r="C815" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D815" s="56" t="inlineStr">
         <is>
-          <t>Melakukan reject data prospek</t>
+          <t>Mencari data dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E815" s="56" t="inlineStr">
@@ -34443,24 +34443,24 @@
       </c>
       <c r="F815" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G815" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga pada data status PENDING - Klik Tolak - Input Remark - Klik button Tolak</t>
+          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H815" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menolak prospek.</t>
+          <t>Berhasil menampilkan data prospek yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="816" ht="56" customHeight="1">
       <c r="A816" s="55" t="inlineStr">
         <is>
-          <t>69.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="B816" s="56" t="inlineStr">
@@ -34470,39 +34470,39 @@
       </c>
       <c r="C816" s="56" t="inlineStr">
         <is>
-          <t>Approval non Banking</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D816" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail data prospek</t>
+          <t>Mencari data dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E816" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F816" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G816" s="56" t="inlineStr">
         <is>
-          <t>Klik titik tiga pada data - Klik opsi Detail</t>
+          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H816" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan detail data prospek.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="817" ht="28" customHeight="1">
       <c r="A817" s="55" t="inlineStr">
         <is>
-          <t>70.1</t>
+          <t>69.4</t>
         </is>
       </c>
       <c r="B817" s="56" t="inlineStr">
@@ -34512,12 +34512,12 @@
       </c>
       <c r="C817" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Re-Assign Management</t>
         </is>
       </c>
       <c r="D817" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Re-Assign Prospek</t>
+          <t>Melakukan re-assign management</t>
         </is>
       </c>
       <c r="E817" s="56" t="inlineStr">
@@ -34532,34 +34532,34 @@
       </c>
       <c r="G817" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Prospek</t>
+          <t>Checklist data prospek - Klik button Reassign () data - Klik button Yes - Pilih Sales tujuan pada modal - Klik button Submit</t>
         </is>
       </c>
       <c r="H817" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Re-Assign Prospek.</t>
+          <t>Berhasil melakukan re-assign data prospek referral management.</t>
         </is>
       </c>
     </row>
     <row r="818" ht="28" customHeight="1">
       <c r="A818" s="55" t="inlineStr">
         <is>
-          <t>70.2</t>
+          <t>70.1</t>
         </is>
       </c>
       <c r="B818" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C818" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D818" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Re-Assign Prospek</t>
+          <t>Membuka halaman Riwayat Export</t>
         </is>
       </c>
       <c r="E818" s="56" t="inlineStr">
@@ -34569,39 +34569,39 @@
       </c>
       <c r="F818" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G818" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Pilih Produk dan Sales pada drawer Filter - Klik button Filter</t>
+          <t>Klik menu Export Center - Klik submenu Riwayat Export</t>
         </is>
       </c>
       <c r="H818" s="56" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan data prospek sesuai kriteria.</t>
+          <t>Berhasil menampilkan halaman Riwayat Export.</t>
         </is>
       </c>
     </row>
     <row r="819" ht="42" customHeight="1">
       <c r="A819" s="55" t="inlineStr">
         <is>
-          <t>70.3</t>
+          <t>70.2</t>
         </is>
       </c>
       <c r="B819" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C819" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D819" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci valid</t>
+          <t>Mencari data riwayat export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E819" s="56" t="inlineStr">
@@ -34616,34 +34616,34 @@
       </c>
       <c r="G819" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H819" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek yang dicari.</t>
+          <t>Berhasil menampilkan data riwayat export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="820" ht="14" customHeight="1">
       <c r="A820" s="55" t="inlineStr">
         <is>
-          <t>70.4</t>
+          <t>70.3</t>
         </is>
       </c>
       <c r="B820" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C820" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D820" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci tidak valid</t>
+          <t>Mencari data riwayat export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E820" s="56" t="inlineStr">
@@ -34658,7 +34658,7 @@
       </c>
       <c r="G820" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H820" s="56" t="inlineStr">
@@ -34670,22 +34670,22 @@
     <row r="821" ht="56" customHeight="1">
       <c r="A821" s="55" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>70.4</t>
         </is>
       </c>
       <c r="B821" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C821" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D821" s="56" t="inlineStr">
         <is>
-          <t>Melakukan re-assign beberapa data prospek</t>
+          <t>Melihat data riwayat export berdasarkan status</t>
         </is>
       </c>
       <c r="E821" s="56" t="inlineStr">
@@ -34695,39 +34695,39 @@
       </c>
       <c r="F821" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G821" s="56" t="inlineStr">
         <is>
-          <t>Checklist beberapa data prospek - Klik button Reassign () data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
+          <t>Pada halaman Riwayat Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H821" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign data prospek yang dipilih.</t>
+          <t>Berhasil menampilkan daftar data riwayat export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="822" ht="56" customHeight="1">
       <c r="A822" s="55" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.5</t>
         </is>
       </c>
       <c r="B822" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C822" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Prospek</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D822" s="56" t="inlineStr">
         <is>
-          <t>Melakukan re-assign semua data prospek</t>
+          <t>Melakukan filter data riwayat export</t>
         </is>
       </c>
       <c r="E822" s="56" t="inlineStr">
@@ -34737,39 +34737,39 @@
       </c>
       <c r="F822" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G822" s="56" t="inlineStr">
         <is>
-          <t>Klik button Reassign Semua data - Klik button Yes - Pilih Wilayah, Cabang, dan Sales baru - Klik button Submit</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H822" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign seluruh data prospek.</t>
+          <t>Berhasil memfilter dan menampilkan data riwayat export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="823" ht="56" customHeight="1">
       <c r="A823" s="55" t="inlineStr">
         <is>
-          <t>71.1</t>
+          <t>70.6</t>
         </is>
       </c>
       <c r="B823" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C823" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D823" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Re-Assign Management</t>
+          <t>Mereset filter data riwayat export</t>
         </is>
       </c>
       <c r="E823" s="56" t="inlineStr">
@@ -34779,39 +34779,39 @@
       </c>
       <c r="F823" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G823" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Re-Assign &amp; Approval - Klik submenu Re-Assign Management</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H823" s="56" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Re-Assign Management.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data riwayat export.</t>
         </is>
       </c>
     </row>
     <row r="824" ht="14" customHeight="1">
       <c r="A824" s="55" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>70.7</t>
         </is>
       </c>
       <c r="B824" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C824" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D824" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci valid</t>
+          <t>Melihat detail riwayat export</t>
         </is>
       </c>
       <c r="E824" s="56" t="inlineStr">
@@ -34821,81 +34821,81 @@
       </c>
       <c r="F824" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G824" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada kolom Cari Data - Klik icon search</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H824" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data prospek yang dicari.</t>
+          <t>Berhasil menampilkan drawer Export Detail.</t>
         </is>
       </c>
     </row>
     <row r="825" ht="14" customHeight="1">
       <c r="A825" s="55" t="inlineStr">
         <is>
-          <t>71.3</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="B825" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C825" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Riwayat Export</t>
         </is>
       </c>
       <c r="D825" s="56" t="inlineStr">
         <is>
-          <t>Mencari data dengan kata kunci tidak valid</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E825" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F825" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G825" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada kolom Cari Data - Klik icon search</t>
+          <t>Klik icon Aksi (...) pada baris data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H825" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>
     <row r="826" ht="14" customHeight="1">
       <c r="A826" s="55" t="inlineStr">
         <is>
-          <t>71.4</t>
+          <t>71.1</t>
         </is>
       </c>
       <c r="B826" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign dan Approval</t>
+          <t>Export Center</t>
         </is>
       </c>
       <c r="C826" s="56" t="inlineStr">
         <is>
-          <t>Re-Assign Management</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D826" s="56" t="inlineStr">
         <is>
-          <t>Melakukan re-assign management</t>
+          <t>Membuka halaman Persetujuan Export</t>
         </is>
       </c>
       <c r="E826" s="56" t="inlineStr">
@@ -34910,19 +34910,19 @@
       </c>
       <c r="G826" s="56" t="inlineStr">
         <is>
-          <t>Checklist data prospek - Klik button Reassign () data - Klik button Yes - Pilih Sales tujuan pada modal - Klik button Submit</t>
+          <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
         </is>
       </c>
       <c r="H826" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan re-assign data prospek referral management.</t>
+          <t>Berhasil menampilkan halaman Persetujuan Export.</t>
         </is>
       </c>
     </row>
     <row r="827" ht="42" customHeight="1">
       <c r="A827" s="55" t="inlineStr">
         <is>
-          <t>72.1</t>
+          <t>71.2</t>
         </is>
       </c>
       <c r="B827" s="56" t="inlineStr">
@@ -34932,12 +34932,12 @@
       </c>
       <c r="C827" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D827" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Riwayat Export</t>
+          <t>Mencari data persetujuan export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E827" s="56" t="inlineStr">
@@ -34947,24 +34947,24 @@
       </c>
       <c r="F827" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G827" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Export Center - Klik submenu Riwayat Export</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H827" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Riwayat Export.</t>
+          <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="828" ht="14" customHeight="1">
       <c r="A828" s="55" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="B828" s="56" t="inlineStr">
@@ -34974,17 +34974,17 @@
       </c>
       <c r="C828" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D828" s="56" t="inlineStr">
         <is>
-          <t>Mencari data riwayat export dengan kata kunci valid</t>
+          <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E828" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F828" s="55" t="inlineStr">
@@ -34994,19 +34994,19 @@
       </c>
       <c r="G828" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H828" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data riwayat export yang dicari.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="829" ht="56" customHeight="1">
       <c r="A829" s="55" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="B829" s="56" t="inlineStr">
@@ -35016,17 +35016,17 @@
       </c>
       <c r="C829" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D829" s="56" t="inlineStr">
         <is>
-          <t>Mencari data riwayat export dengan kata kunci tidak valid</t>
+          <t>Melihat data persetujuan export berdasarkan status</t>
         </is>
       </c>
       <c r="E829" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F829" s="55" t="inlineStr">
@@ -35036,19 +35036,19 @@
       </c>
       <c r="G829" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
+          <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H829" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="830" ht="28" customHeight="1">
       <c r="A830" s="55" t="inlineStr">
         <is>
-          <t>72.4</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="B830" s="56" t="inlineStr">
@@ -35058,12 +35058,12 @@
       </c>
       <c r="C830" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D830" s="56" t="inlineStr">
         <is>
-          <t>Melihat data riwayat export berdasarkan status</t>
+          <t>Melakukan filter data persetujuan export</t>
         </is>
       </c>
       <c r="E830" s="56" t="inlineStr">
@@ -35078,19 +35078,19 @@
       </c>
       <c r="G830" s="56" t="inlineStr">
         <is>
-          <t>Pada halaman Riwayat Export, klik salah satu tab status</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H830" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan daftar data riwayat export sesuai status yang dipilih.</t>
+          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="831" ht="42" customHeight="1">
       <c r="A831" s="55" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="B831" s="56" t="inlineStr">
@@ -35100,12 +35100,12 @@
       </c>
       <c r="C831" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D831" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data riwayat export</t>
+          <t>Mereset filter data persetujuan export</t>
         </is>
       </c>
       <c r="E831" s="56" t="inlineStr">
@@ -35120,19 +35120,19 @@
       </c>
       <c r="G831" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H831" s="56" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan data riwayat export sesuai kriteria filter.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
         </is>
       </c>
     </row>
     <row r="832" ht="28" customHeight="1">
       <c r="A832" s="55" t="inlineStr">
         <is>
-          <t>72.6</t>
+          <t>71.7</t>
         </is>
       </c>
       <c r="B832" s="56" t="inlineStr">
@@ -35142,12 +35142,12 @@
       </c>
       <c r="C832" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D832" s="56" t="inlineStr">
         <is>
-          <t>Mereset filter data riwayat export</t>
+          <t>Melakukan approval data pengajuan export</t>
         </is>
       </c>
       <c r="E832" s="56" t="inlineStr">
@@ -35157,24 +35157,24 @@
       </c>
       <c r="F832" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G832" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
         </is>
       </c>
       <c r="H832" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data riwayat export.</t>
+          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
         </is>
       </c>
     </row>
     <row r="833" ht="14" customHeight="1">
       <c r="A833" s="55" t="inlineStr">
         <is>
-          <t>72.7</t>
+          <t>71.8</t>
         </is>
       </c>
       <c r="B833" s="56" t="inlineStr">
@@ -35184,12 +35184,12 @@
       </c>
       <c r="C833" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D833" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail riwayat export</t>
+          <t>Melakukan reject data pengajuan export</t>
         </is>
       </c>
       <c r="E833" s="56" t="inlineStr">
@@ -35204,19 +35204,19 @@
       </c>
       <c r="G833" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
         </is>
       </c>
       <c r="H833" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan drawer Export Detail.</t>
+          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
         </is>
       </c>
     </row>
     <row r="834" ht="14" customHeight="1">
       <c r="A834" s="55" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>71.9</t>
         </is>
       </c>
       <c r="B834" s="56" t="inlineStr">
@@ -35226,12 +35226,12 @@
       </c>
       <c r="C834" s="56" t="inlineStr">
         <is>
-          <t>Riwayat Export</t>
+          <t>Persetujuan Export</t>
         </is>
       </c>
       <c r="D834" s="56" t="inlineStr">
         <is>
-          <t>Mengunduh file data export yang tersedia</t>
+          <t>Melihat detail pengajuan export</t>
         </is>
       </c>
       <c r="E834" s="56" t="inlineStr">
@@ -35241,24 +35241,24 @@
       </c>
       <c r="F834" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G834" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data dengan status Tersedia - Klik opsi Download</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H834" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh file data export.</t>
+          <t>Berhasil menampilkan detail data pengajuan export.</t>
         </is>
       </c>
     </row>
     <row r="835" ht="14" customHeight="1">
       <c r="A835" s="55" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>72.1</t>
         </is>
       </c>
       <c r="B835" s="56" t="inlineStr">
@@ -35268,12 +35268,12 @@
       </c>
       <c r="C835" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D835" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Persetujuan Export</t>
+          <t>Membuka halaman Aktivitas Export</t>
         </is>
       </c>
       <c r="E835" s="56" t="inlineStr">
@@ -35288,19 +35288,19 @@
       </c>
       <c r="G835" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
+          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
         </is>
       </c>
       <c r="H835" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Persetujuan Export.</t>
+          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
         </is>
       </c>
     </row>
     <row r="836" ht="42" customHeight="1">
       <c r="A836" s="55" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="B836" s="56" t="inlineStr">
@@ -35310,12 +35310,12 @@
       </c>
       <c r="C836" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D836" s="56" t="inlineStr">
         <is>
-          <t>Mencari data persetujuan export dengan kata kunci valid</t>
+          <t>Mencari data aktivitas export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E836" s="56" t="inlineStr">
@@ -35335,14 +35335,14 @@
       </c>
       <c r="H836" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
+          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="837" ht="28" customHeight="1">
       <c r="A837" s="55" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>72.3</t>
         </is>
       </c>
       <c r="B837" s="56" t="inlineStr">
@@ -35352,12 +35352,12 @@
       </c>
       <c r="C837" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D837" s="56" t="inlineStr">
         <is>
-          <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
+          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E837" s="56" t="inlineStr">
@@ -35384,7 +35384,7 @@
     <row r="838" ht="28" customHeight="1">
       <c r="A838" s="55" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>72.4</t>
         </is>
       </c>
       <c r="B838" s="56" t="inlineStr">
@@ -35394,12 +35394,12 @@
       </c>
       <c r="C838" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D838" s="56" t="inlineStr">
         <is>
-          <t>Melihat data persetujuan export berdasarkan status</t>
+          <t>Melihat data aktivitas export berdasarkan status</t>
         </is>
       </c>
       <c r="E838" s="56" t="inlineStr">
@@ -35414,19 +35414,19 @@
       </c>
       <c r="G838" s="56" t="inlineStr">
         <is>
-          <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
+          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H838" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
+          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="839" ht="70" customHeight="1">
       <c r="A839" s="55" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="B839" s="56" t="inlineStr">
@@ -35436,12 +35436,12 @@
       </c>
       <c r="C839" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D839" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data persetujuan export</t>
+          <t>Melakukan filter data aktivitas export</t>
         </is>
       </c>
       <c r="E839" s="56" t="inlineStr">
@@ -35461,14 +35461,14 @@
       </c>
       <c r="H839" s="56" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
+          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="840" ht="28" customHeight="1">
       <c r="A840" s="55" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>72.6</t>
         </is>
       </c>
       <c r="B840" s="56" t="inlineStr">
@@ -35478,12 +35478,12 @@
       </c>
       <c r="C840" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D840" s="56" t="inlineStr">
         <is>
-          <t>Mereset filter data persetujuan export</t>
+          <t>Mereset filter data aktivitas export</t>
         </is>
       </c>
       <c r="E840" s="56" t="inlineStr">
@@ -35503,14 +35503,14 @@
       </c>
       <c r="H840" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="841" ht="84" customHeight="1">
       <c r="A841" s="55" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>72.7</t>
         </is>
       </c>
       <c r="B841" s="56" t="inlineStr">
@@ -35520,12 +35520,12 @@
       </c>
       <c r="C841" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D841" s="56" t="inlineStr">
         <is>
-          <t>Melakukan approval data pengajuan export</t>
+          <t>Melihat detail aktivitas export</t>
         </is>
       </c>
       <c r="E841" s="56" t="inlineStr">
@@ -35540,19 +35540,19 @@
       </c>
       <c r="G841" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H841" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
+          <t>Berhasil menampilkan detail data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="842" ht="28" customHeight="1">
       <c r="A842" s="55" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>72.8</t>
         </is>
       </c>
       <c r="B842" s="56" t="inlineStr">
@@ -35562,12 +35562,12 @@
       </c>
       <c r="C842" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D842" s="56" t="inlineStr">
         <is>
-          <t>Melakukan reject data pengajuan export</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E842" s="56" t="inlineStr">
@@ -35582,393 +35582,24 @@
       </c>
       <c r="G842" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
+          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
         </is>
       </c>
       <c r="H842" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
-        </is>
-      </c>
-    </row>
-    <row r="843" ht="28" customHeight="1">
-      <c r="A843" s="55" t="inlineStr">
-        <is>
-          <t>73.9</t>
-        </is>
-      </c>
-      <c r="B843" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C843" s="56" t="inlineStr">
-        <is>
-          <t>Persetujuan Export</t>
-        </is>
-      </c>
-      <c r="D843" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail pengajuan export</t>
-        </is>
-      </c>
-      <c r="E843" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F843" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G843" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H843" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data pengajuan export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="844" ht="28" customHeight="1">
-      <c r="A844" s="55" t="inlineStr">
-        <is>
-          <t>74.1</t>
-        </is>
-      </c>
-      <c r="B844" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C844" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D844" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="E844" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F844" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G844" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="H844" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="845" ht="42" customHeight="1">
-      <c r="A845" s="55" t="inlineStr">
-        <is>
-          <t>74.2</t>
-        </is>
-      </c>
-      <c r="B845" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C845" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D845" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data aktivitas export dengan kata kunci valid</t>
-        </is>
-      </c>
-      <c r="E845" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F845" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G845" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H845" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
-        </is>
-      </c>
-    </row>
-    <row r="846" ht="28" customHeight="1">
-      <c r="A846" s="55" t="inlineStr">
-        <is>
-          <t>74.3</t>
-        </is>
-      </c>
-      <c r="B846" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C846" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D846" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
-        </is>
-      </c>
-      <c r="E846" s="56" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F846" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G846" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H846" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="847" ht="14" customHeight="1">
-      <c r="A847" s="55" t="inlineStr">
-        <is>
-          <t>74.4</t>
-        </is>
-      </c>
-      <c r="B847" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C847" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D847" s="56" t="inlineStr">
-        <is>
-          <t>Melihat data aktivitas export berdasarkan status</t>
-        </is>
-      </c>
-      <c r="E847" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F847" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G847" s="56" t="inlineStr">
-        <is>
-          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
-        </is>
-      </c>
-      <c r="H847" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="848" ht="14" customHeight="1">
-      <c r="A848" s="55" t="inlineStr">
-        <is>
-          <t>74.5</t>
-        </is>
-      </c>
-      <c r="B848" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C848" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D848" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E848" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F848" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G848" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H848" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="849" ht="42" customHeight="1">
-      <c r="A849" s="55" t="inlineStr">
-        <is>
-          <t>74.6</t>
-        </is>
-      </c>
-      <c r="B849" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C849" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D849" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E849" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F849" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G849" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
-        </is>
-      </c>
-      <c r="H849" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="850" ht="28" customHeight="1">
-      <c r="A850" s="55" t="inlineStr">
-        <is>
-          <t>74.7</t>
-        </is>
-      </c>
-      <c r="B850" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C850" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D850" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail aktivitas export</t>
-        </is>
-      </c>
-      <c r="E850" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F850" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G850" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H850" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="851" ht="28" customHeight="1">
-      <c r="A851" s="55" t="inlineStr">
-        <is>
-          <t>74.8</t>
-        </is>
-      </c>
-      <c r="B851" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C851" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D851" s="56" t="inlineStr">
-        <is>
-          <t>Mengunduh file data export yang tersedia</t>
-        </is>
-      </c>
-      <c r="E851" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F851" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G851" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
-        </is>
-      </c>
-      <c r="H851" s="56" t="inlineStr">
-        <is>
           <t>Berhasil mengunduh file data export.</t>
         </is>
       </c>
     </row>
+    <row r="843" ht="28" customHeight="1"/>
+    <row r="844" ht="28" customHeight="1"/>
+    <row r="845" ht="42" customHeight="1"/>
+    <row r="846" ht="28" customHeight="1"/>
+    <row r="847" ht="14" customHeight="1"/>
+    <row r="848" ht="14" customHeight="1"/>
+    <row r="849" ht="42" customHeight="1"/>
+    <row r="850" ht="28" customHeight="1"/>
+    <row r="851" ht="28" customHeight="1"/>
     <row r="852" ht="28" customHeight="1"/>
     <row r="853" ht="28" customHeight="1"/>
     <row r="854" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
feat(web): add test cases for Modul 72-78 (Ticket Maintenance & Aktivitas Consumer)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -291,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -424,6 +424,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -703,7 +706,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z834"/>
+  <dimension ref="A1:Z881"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35255,53 +35258,1980 @@
         </is>
       </c>
     </row>
-    <row r="835" ht="14" customHeight="1"/>
-    <row r="836" ht="42" customHeight="1"/>
-    <row r="837" ht="28" customHeight="1"/>
-    <row r="838" ht="28" customHeight="1"/>
-    <row r="839" ht="70" customHeight="1"/>
-    <row r="840" ht="28" customHeight="1"/>
-    <row r="841" ht="84" customHeight="1"/>
-    <row r="842" ht="28" customHeight="1"/>
-    <row r="843" ht="28" customHeight="1"/>
-    <row r="844" ht="28" customHeight="1"/>
-    <row r="845" ht="42" customHeight="1"/>
-    <row r="846" ht="28" customHeight="1"/>
-    <row r="847" ht="14" customHeight="1"/>
-    <row r="848" ht="14" customHeight="1"/>
-    <row r="849" ht="42" customHeight="1"/>
-    <row r="850" ht="28" customHeight="1"/>
-    <row r="851" ht="28" customHeight="1"/>
-    <row r="852" ht="28" customHeight="1"/>
-    <row r="853" ht="28" customHeight="1"/>
-    <row r="854" ht="28" customHeight="1"/>
-    <row r="855" ht="28" customHeight="1"/>
-    <row r="856" ht="28" customHeight="1"/>
-    <row r="857" ht="28" customHeight="1"/>
-    <row r="858" ht="28" customHeight="1"/>
-    <row r="859" ht="28" customHeight="1"/>
-    <row r="860" ht="28" customHeight="1"/>
-    <row r="861" ht="28" customHeight="1"/>
-    <row r="862" ht="28" customHeight="1"/>
-    <row r="863" ht="28" customHeight="1"/>
-    <row r="864" ht="28" customHeight="1"/>
-    <row r="865" ht="28" customHeight="1"/>
-    <row r="866" ht="28" customHeight="1"/>
-    <row r="867" ht="28" customHeight="1"/>
-    <row r="868" ht="28" customHeight="1"/>
-    <row r="869" ht="28" customHeight="1"/>
-    <row r="870" ht="28" customHeight="1"/>
-    <row r="871" ht="28" customHeight="1"/>
-    <row r="872" ht="70" customHeight="1"/>
-    <row r="873" ht="42" customHeight="1"/>
-    <row r="874" ht="42" customHeight="1"/>
-    <row r="875" ht="70" customHeight="1"/>
-    <row r="876" ht="28" customHeight="1"/>
-    <row r="877" ht="42" customHeight="1"/>
-    <row r="878" ht="28" customHeight="1"/>
-    <row r="879" ht="28" customHeight="1"/>
-    <row r="880" ht="28" customHeight="1"/>
-    <row r="881" ht="14" customHeight="1"/>
+    <row r="835" ht="14" customHeight="1">
+      <c r="A835" s="57" t="inlineStr">
+        <is>
+          <t>72.1</t>
+        </is>
+      </c>
+      <c r="B835" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C835" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D835" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E835" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F835" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G835" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H835" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="836" ht="42" customHeight="1">
+      <c r="A836" s="57" t="inlineStr">
+        <is>
+          <t>72.2</t>
+        </is>
+      </c>
+      <c r="B836" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C836" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D836" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E836" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F836" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G836" s="56" t="inlineStr">
+        <is>
+          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
+        </is>
+      </c>
+      <c r="H836" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="837" ht="28" customHeight="1">
+      <c r="A837" s="57" t="inlineStr">
+        <is>
+          <t>72.3</t>
+        </is>
+      </c>
+      <c r="B837" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C837" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D837" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E837" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F837" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G837" s="56" t="inlineStr">
+        <is>
+          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H837" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="838" ht="28" customHeight="1">
+      <c r="A838" s="57" t="inlineStr">
+        <is>
+          <t>72.4</t>
+        </is>
+      </c>
+      <c r="B838" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C838" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D838" s="56" t="inlineStr">
+        <is>
+          <t>Menambahkan pelaporan issue baru</t>
+        </is>
+      </c>
+      <c r="E838" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F838" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G838" s="56" t="inlineStr">
+        <is>
+          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
+        </is>
+      </c>
+      <c r="H838" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan data pelaporan issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="839" ht="70" customHeight="1">
+      <c r="A839" s="57" t="inlineStr">
+        <is>
+          <t>72.5</t>
+        </is>
+      </c>
+      <c r="B839" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C839" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D839" s="56" t="inlineStr">
+        <is>
+          <t>Melihat detail pelaporan issue</t>
+        </is>
+      </c>
+      <c r="E839" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F839" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G839" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+        </is>
+      </c>
+      <c r="H839" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman detail issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="840" ht="28" customHeight="1">
+      <c r="A840" s="57" t="inlineStr">
+        <is>
+          <t>72.6</t>
+        </is>
+      </c>
+      <c r="B840" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C840" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D840" s="56" t="inlineStr">
+        <is>
+          <t>Mengubah data pelaporan issue</t>
+        </is>
+      </c>
+      <c r="E840" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F840" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G840" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H840" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan perubahan data issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="841" ht="84" customHeight="1">
+      <c r="A841" s="57" t="inlineStr">
+        <is>
+          <t>72.7</t>
+        </is>
+      </c>
+      <c r="B841" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C841" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D841" s="56" t="inlineStr">
+        <is>
+          <t>Menambahkan komentar pada detail aktivitas issue</t>
+        </is>
+      </c>
+      <c r="E841" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F841" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G841" s="56" t="inlineStr">
+        <is>
+          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
+        </is>
+      </c>
+      <c r="H841" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menambahkan komentar pada detail issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="842" ht="28" customHeight="1">
+      <c r="A842" s="57" t="inlineStr">
+        <is>
+          <t>72.8</t>
+        </is>
+      </c>
+      <c r="B842" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C842" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D842" s="56" t="inlineStr">
+        <is>
+          <t>Mengunduh lampiran bukti issue</t>
+        </is>
+      </c>
+      <c r="E842" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F842" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G842" s="56" t="inlineStr">
+        <is>
+          <t>Buka halaman detail issue - Klik file lampiran bukti screenshot</t>
+        </is>
+      </c>
+      <c r="H842" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mengunduh file lampiran bukti issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="843" ht="28" customHeight="1">
+      <c r="A843" s="57" t="inlineStr">
+        <is>
+          <t>72.9</t>
+        </is>
+      </c>
+      <c r="B843" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C843" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D843" s="56" t="inlineStr">
+        <is>
+          <t>Menghapus data pelaporan issue</t>
+        </is>
+      </c>
+      <c r="E843" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F843" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G843" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
+        </is>
+      </c>
+      <c r="H843" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menghapus data issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="844" ht="28" customHeight="1">
+      <c r="A844" s="57" t="inlineStr">
+        <is>
+          <t>72.10</t>
+        </is>
+      </c>
+      <c r="B844" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C844" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D844" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan update status issue secara massal</t>
+        </is>
+      </c>
+      <c r="E844" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F844" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G844" s="56" t="inlineStr">
+        <is>
+          <t>Checklist data issue - Klik button Mass Update - Pilih status baru - Klik button Update</t>
+        </is>
+      </c>
+      <c r="H844" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil melakukan update status issue secara massal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="845" ht="42" customHeight="1">
+      <c r="A845" s="57" t="inlineStr">
+        <is>
+          <t>73.1</t>
+        </is>
+      </c>
+      <c r="B845" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C845" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D845" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Master Kategori Issue</t>
+        </is>
+      </c>
+      <c r="E845" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F845" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G845" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H845" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="846" ht="28" customHeight="1">
+      <c r="A846" s="57" t="inlineStr">
+        <is>
+          <t>73.2</t>
+        </is>
+      </c>
+      <c r="B846" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C846" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D846" s="56" t="inlineStr">
+        <is>
+          <t>Menambahkan kategori lain melalui pelaporan issue</t>
+        </is>
+      </c>
+      <c r="E846" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F846" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G846" s="56" t="inlineStr">
+        <is>
+          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
+        </is>
+      </c>
+      <c r="H846" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="847" ht="14" customHeight="1">
+      <c r="A847" s="57" t="inlineStr">
+        <is>
+          <t>73.3</t>
+        </is>
+      </c>
+      <c r="B847" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C847" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D847" s="56" t="inlineStr">
+        <is>
+          <t>Menambahkan data master kategori</t>
+        </is>
+      </c>
+      <c r="E847" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F847" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G847" s="56" t="inlineStr">
+        <is>
+          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
+        </is>
+      </c>
+      <c r="H847" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan data master kategori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="848" ht="14" customHeight="1">
+      <c r="A848" s="57" t="inlineStr">
+        <is>
+          <t>73.4</t>
+        </is>
+      </c>
+      <c r="B848" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C848" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D848" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada List Kategori Lain</t>
+        </is>
+      </c>
+      <c r="E848" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F848" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G848" s="56" t="inlineStr">
+        <is>
+          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H848" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="849" ht="42" customHeight="1">
+      <c r="A849" s="57" t="inlineStr">
+        <is>
+          <t>73.5</t>
+        </is>
+      </c>
+      <c r="B849" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C849" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D849" s="56" t="inlineStr">
+        <is>
+          <t>Melihat detail data kategori pada List Kategori Lain</t>
+        </is>
+      </c>
+      <c r="E849" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F849" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G849" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
+        </is>
+      </c>
+      <c r="H849" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan modal detail kategori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="850" ht="28" customHeight="1">
+      <c r="A850" s="57" t="inlineStr">
+        <is>
+          <t>73.6</t>
+        </is>
+      </c>
+      <c r="B850" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C850" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D850" s="56" t="inlineStr">
+        <is>
+          <t>Mengirim data kategori lain ke master kategori</t>
+        </is>
+      </c>
+      <c r="E850" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F850" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G850" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
+        </is>
+      </c>
+      <c r="H850" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="851" ht="28" customHeight="1">
+      <c r="A851" s="57" t="inlineStr">
+        <is>
+          <t>73.7</t>
+        </is>
+      </c>
+      <c r="B851" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C851" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D851" s="56" t="inlineStr">
+        <is>
+          <t>Mengirim data kategori lain ke master kategori secara massal</t>
+        </is>
+      </c>
+      <c r="E851" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F851" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G851" s="56" t="inlineStr">
+        <is>
+          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
+        </is>
+      </c>
+      <c r="H851" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="852" ht="28" customHeight="1">
+      <c r="A852" s="57" t="inlineStr">
+        <is>
+          <t>73.8</t>
+        </is>
+      </c>
+      <c r="B852" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C852" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D852" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada List Kategori</t>
+        </is>
+      </c>
+      <c r="E852" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F852" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G852" s="56" t="inlineStr">
+        <is>
+          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H852" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="853" ht="28" customHeight="1">
+      <c r="A853" s="57" t="inlineStr">
+        <is>
+          <t>73.9</t>
+        </is>
+      </c>
+      <c r="B853" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C853" s="56" t="inlineStr">
+        <is>
+          <t>Kategori Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D853" s="56" t="inlineStr">
+        <is>
+          <t>Melihat dan mengubah data master kategori</t>
+        </is>
+      </c>
+      <c r="E853" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F853" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G853" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
+        </is>
+      </c>
+      <c r="H853" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
+        </is>
+      </c>
+    </row>
+    <row r="854" ht="28" customHeight="1">
+      <c r="A854" s="57" t="inlineStr">
+        <is>
+          <t>74.1</t>
+        </is>
+      </c>
+      <c r="B854" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C854" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D854" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E854" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F854" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G854" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H854" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="855" ht="28" customHeight="1">
+      <c r="A855" s="57" t="inlineStr">
+        <is>
+          <t>74.2</t>
+        </is>
+      </c>
+      <c r="B855" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C855" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D855" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E855" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F855" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G855" s="56" t="inlineStr">
+        <is>
+          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
+        </is>
+      </c>
+      <c r="H855" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="856" ht="28" customHeight="1">
+      <c r="A856" s="57" t="inlineStr">
+        <is>
+          <t>74.3</t>
+        </is>
+      </c>
+      <c r="B856" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C856" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D856" s="56" t="inlineStr">
+        <is>
+          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
+        </is>
+      </c>
+      <c r="E856" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F856" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G856" s="56" t="inlineStr">
+        <is>
+          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
+        </is>
+      </c>
+      <c r="H856" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman detail issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="857" ht="28" customHeight="1">
+      <c r="A857" s="57" t="inlineStr">
+        <is>
+          <t>75.1</t>
+        </is>
+      </c>
+      <c r="B857" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C857" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D857" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E857" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F857" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G857" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H857" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="858" ht="28" customHeight="1">
+      <c r="A858" s="57" t="inlineStr">
+        <is>
+          <t>75.2</t>
+        </is>
+      </c>
+      <c r="B858" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C858" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D858" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E858" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F858" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G858" s="56" t="inlineStr">
+        <is>
+          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
+        </is>
+      </c>
+      <c r="H858" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="859" ht="28" customHeight="1">
+      <c r="A859" s="57" t="inlineStr">
+        <is>
+          <t>75.3</t>
+        </is>
+      </c>
+      <c r="B859" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C859" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D859" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E859" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F859" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G859" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H859" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="860" ht="28" customHeight="1">
+      <c r="A860" s="57" t="inlineStr">
+        <is>
+          <t>75.4</t>
+        </is>
+      </c>
+      <c r="B860" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C860" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D860" s="56" t="inlineStr">
+        <is>
+          <t>Melihat detail report aktivitas issue</t>
+        </is>
+      </c>
+      <c r="E860" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F860" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G860" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+        </is>
+      </c>
+      <c r="H860" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman detail issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="861" ht="28" customHeight="1">
+      <c r="A861" s="57" t="inlineStr">
+        <is>
+          <t>75.5</t>
+        </is>
+      </c>
+      <c r="B861" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C861" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D861" s="56" t="inlineStr">
+        <is>
+          <t>Menghapus data report aktivitas issue secara massal</t>
+        </is>
+      </c>
+      <c r="E861" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F861" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G861" s="56" t="inlineStr">
+        <is>
+          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
+        </is>
+      </c>
+      <c r="H861" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menghapus data report aktivitas issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="862" ht="28" customHeight="1">
+      <c r="A862" s="57" t="inlineStr">
+        <is>
+          <t>75.6</t>
+        </is>
+      </c>
+      <c r="B862" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C862" s="56" t="inlineStr">
+        <is>
+          <t>Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D862" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data Report Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E862" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F862" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G862" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+        </is>
+      </c>
+      <c r="H862" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="863" ht="28" customHeight="1">
+      <c r="A863" s="57" t="inlineStr">
+        <is>
+          <t>76.1</t>
+        </is>
+      </c>
+      <c r="B863" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C863" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D863" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="E863" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F863" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G863" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="H863" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="864" ht="28" customHeight="1">
+      <c r="A864" s="57" t="inlineStr">
+        <is>
+          <t>76.2</t>
+        </is>
+      </c>
+      <c r="B864" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C864" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D864" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="E864" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F864" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G864" s="56" t="inlineStr">
+        <is>
+          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
+        </is>
+      </c>
+      <c r="H864" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="865" ht="28" customHeight="1">
+      <c r="A865" s="57" t="inlineStr">
+        <is>
+          <t>76.3</t>
+        </is>
+      </c>
+      <c r="B865" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C865" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D865" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E865" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F865" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G865" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H865" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="866" ht="28" customHeight="1">
+      <c r="A866" s="57" t="inlineStr">
+        <is>
+          <t>76.4</t>
+        </is>
+      </c>
+      <c r="B866" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C866" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D866" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E866" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F866" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G866" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H866" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="867" ht="28" customHeight="1">
+      <c r="A867" s="57" t="inlineStr">
+        <is>
+          <t>76.5</t>
+        </is>
+      </c>
+      <c r="B867" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C867" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D867" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="E867" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F867" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G867" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="H867" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="868" ht="28" customHeight="1">
+      <c r="A868" s="57" t="inlineStr">
+        <is>
+          <t>76.6</t>
+        </is>
+      </c>
+      <c r="B868" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C868" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D868" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E868" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F868" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G868" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H868" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="869" ht="28" customHeight="1">
+      <c r="A869" s="57" t="inlineStr">
+        <is>
+          <t>76.7</t>
+        </is>
+      </c>
+      <c r="B869" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C869" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D869" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E869" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F869" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G869" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H869" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="870" ht="28" customHeight="1">
+      <c r="A870" s="57" t="inlineStr">
+        <is>
+          <t>76.8</t>
+        </is>
+      </c>
+      <c r="B870" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C870" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="D870" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="E870" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F870" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G870" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="H870" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="871" ht="28" customHeight="1">
+      <c r="A871" s="57" t="inlineStr">
+        <is>
+          <t>77.1</t>
+        </is>
+      </c>
+      <c r="B871" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C871" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D871" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="E871" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F871" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G871" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="H871" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="872" ht="70" customHeight="1">
+      <c r="A872" s="57" t="inlineStr">
+        <is>
+          <t>77.2</t>
+        </is>
+      </c>
+      <c r="B872" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C872" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D872" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="E872" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F872" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G872" s="56" t="inlineStr">
+        <is>
+          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+        </is>
+      </c>
+      <c r="H872" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="873" ht="42" customHeight="1">
+      <c r="A873" s="57" t="inlineStr">
+        <is>
+          <t>77.3</t>
+        </is>
+      </c>
+      <c r="B873" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C873" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D873" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E873" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F873" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G873" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H873" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="874" ht="42" customHeight="1">
+      <c r="A874" s="57" t="inlineStr">
+        <is>
+          <t>77.4</t>
+        </is>
+      </c>
+      <c r="B874" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C874" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D874" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E874" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F874" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G874" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H874" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="875" ht="70" customHeight="1">
+      <c r="A875" s="57" t="inlineStr">
+        <is>
+          <t>77.5</t>
+        </is>
+      </c>
+      <c r="B875" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C875" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D875" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="E875" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F875" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G875" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="H875" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="876" ht="28" customHeight="1">
+      <c r="A876" s="57" t="inlineStr">
+        <is>
+          <t>77.6</t>
+        </is>
+      </c>
+      <c r="B876" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C876" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D876" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E876" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F876" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G876" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H876" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="877" ht="42" customHeight="1">
+      <c r="A877" s="57" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="B877" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C877" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D877" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E877" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F877" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G877" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H877" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="878" ht="28" customHeight="1">
+      <c r="A878" s="57" t="inlineStr">
+        <is>
+          <t>77.8</t>
+        </is>
+      </c>
+      <c r="B878" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C878" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D878" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="E878" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F878" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G878" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="H878" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="879" ht="28" customHeight="1">
+      <c r="A879" s="57" t="inlineStr">
+        <is>
+          <t>78.1</t>
+        </is>
+      </c>
+      <c r="B879" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C879" s="56" t="inlineStr">
+        <is>
+          <t>Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="D879" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="E879" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F879" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G879" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="H879" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="880" ht="28" customHeight="1">
+      <c r="A880" s="57" t="inlineStr">
+        <is>
+          <t>78.2</t>
+        </is>
+      </c>
+      <c r="B880" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C880" s="56" t="inlineStr">
+        <is>
+          <t>Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="D880" s="56" t="inlineStr">
+        <is>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="E880" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F880" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G880" s="56" t="inlineStr">
+        <is>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H880" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="881" ht="14" customHeight="1">
+      <c r="A881" s="57" t="inlineStr">
+        <is>
+          <t>78.3</t>
+        </is>
+      </c>
+      <c r="B881" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C881" s="56" t="inlineStr">
+        <is>
+          <t>Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="D881" s="56" t="inlineStr">
+        <is>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="E881" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F881" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G881" s="56" t="inlineStr">
+        <is>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H881" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
+        </is>
+      </c>
+    </row>
     <row r="882" ht="42" customHeight="1"/>
     <row r="883" ht="42" customHeight="1"/>
     <row r="884" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
feat(web): update and embed screenshots for Modul 72 (Ticket Maintenance - Aktivitas Issue)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z881"/>
+  <dimension ref="A1:Z879"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35570,7 +35570,7 @@
       </c>
       <c r="D842" s="56" t="inlineStr">
         <is>
-          <t>Mengunduh lampiran bukti issue</t>
+          <t>Menghapus data pelaporan issue</t>
         </is>
       </c>
       <c r="E842" s="57" t="inlineStr">
@@ -35580,24 +35580,24 @@
       </c>
       <c r="F842" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G842" s="56" t="inlineStr">
         <is>
-          <t>Buka halaman detail issue - Klik file lampiran bukti screenshot</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
         </is>
       </c>
       <c r="H842" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh file lampiran bukti issue.</t>
+          <t>Berhasil menghapus data issue.</t>
         </is>
       </c>
     </row>
     <row r="843" ht="28" customHeight="1">
       <c r="A843" s="57" t="inlineStr">
         <is>
-          <t>72.9</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B843" s="56" t="inlineStr">
@@ -35607,12 +35607,12 @@
       </c>
       <c r="C843" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D843" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data pelaporan issue</t>
+          <t>Membuka halaman Master Kategori Issue</t>
         </is>
       </c>
       <c r="E843" s="57" t="inlineStr">
@@ -35622,24 +35622,24 @@
       </c>
       <c r="F843" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G843" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="H843" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data issue.</t>
+          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
         </is>
       </c>
     </row>
     <row r="844" ht="28" customHeight="1">
       <c r="A844" s="57" t="inlineStr">
         <is>
-          <t>72.10</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="B844" s="56" t="inlineStr">
@@ -35649,12 +35649,12 @@
       </c>
       <c r="C844" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D844" s="56" t="inlineStr">
         <is>
-          <t>Melakukan update status issue secara massal</t>
+          <t>Menambahkan kategori lain melalui pelaporan issue</t>
         </is>
       </c>
       <c r="E844" s="57" t="inlineStr">
@@ -35669,19 +35669,19 @@
       </c>
       <c r="G844" s="56" t="inlineStr">
         <is>
-          <t>Checklist data issue - Klik button Mass Update - Pilih status baru - Klik button Update</t>
+          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H844" s="56" t="inlineStr">
         <is>
-          <t>Berhasil melakukan update status issue secara massal.</t>
+          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
         </is>
       </c>
     </row>
     <row r="845" ht="42" customHeight="1">
       <c r="A845" s="57" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="B845" s="56" t="inlineStr">
@@ -35696,7 +35696,7 @@
       </c>
       <c r="D845" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Master Kategori Issue</t>
+          <t>Menambahkan data master kategori</t>
         </is>
       </c>
       <c r="E845" s="57" t="inlineStr">
@@ -35711,19 +35711,19 @@
       </c>
       <c r="G845" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
+          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
         </is>
       </c>
       <c r="H845" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
+          <t>Berhasil menyimpan data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="846" ht="28" customHeight="1">
       <c r="A846" s="57" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>73.4</t>
         </is>
       </c>
       <c r="B846" s="56" t="inlineStr">
@@ -35738,7 +35738,7 @@
       </c>
       <c r="D846" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan kategori lain melalui pelaporan issue</t>
+          <t>Mencari data pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E846" s="57" t="inlineStr">
@@ -35753,19 +35753,19 @@
       </c>
       <c r="G846" s="56" t="inlineStr">
         <is>
-          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
+          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
         </is>
       </c>
       <c r="H846" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="847" ht="14" customHeight="1">
       <c r="A847" s="57" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="B847" s="56" t="inlineStr">
@@ -35780,7 +35780,7 @@
       </c>
       <c r="D847" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan data master kategori</t>
+          <t>Melihat detail data kategori pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E847" s="57" t="inlineStr">
@@ -35790,24 +35790,24 @@
       </c>
       <c r="F847" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G847" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H847" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data master kategori.</t>
+          <t>Berhasil menampilkan modal detail kategori.</t>
         </is>
       </c>
     </row>
     <row r="848" ht="14" customHeight="1">
       <c r="A848" s="57" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>73.6</t>
         </is>
       </c>
       <c r="B848" s="56" t="inlineStr">
@@ -35822,7 +35822,7 @@
       </c>
       <c r="D848" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori Lain</t>
+          <t>Mengirim data kategori lain ke master kategori</t>
         </is>
       </c>
       <c r="E848" s="57" t="inlineStr">
@@ -35832,24 +35832,24 @@
       </c>
       <c r="F848" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G848" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
+          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
         </is>
       </c>
       <c r="H848" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="849" ht="42" customHeight="1">
       <c r="A849" s="57" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>73.7</t>
         </is>
       </c>
       <c r="B849" s="56" t="inlineStr">
@@ -35864,7 +35864,7 @@
       </c>
       <c r="D849" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail data kategori pada List Kategori Lain</t>
+          <t>Mengirim data kategori lain ke master kategori secara massal</t>
         </is>
       </c>
       <c r="E849" s="57" t="inlineStr">
@@ -35879,19 +35879,19 @@
       </c>
       <c r="G849" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
+          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
         </is>
       </c>
       <c r="H849" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan modal detail kategori.</t>
+          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="850" ht="28" customHeight="1">
       <c r="A850" s="57" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>73.8</t>
         </is>
       </c>
       <c r="B850" s="56" t="inlineStr">
@@ -35906,7 +35906,7 @@
       </c>
       <c r="D850" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori</t>
+          <t>Mencari data pada List Kategori</t>
         </is>
       </c>
       <c r="E850" s="57" t="inlineStr">
@@ -35916,24 +35916,24 @@
       </c>
       <c r="F850" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G850" s="56" t="inlineStr">
         <is>
-          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
+          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
         </is>
       </c>
       <c r="H850" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="851" ht="28" customHeight="1">
       <c r="A851" s="57" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>73.9</t>
         </is>
       </c>
       <c r="B851" s="56" t="inlineStr">
@@ -35948,7 +35948,7 @@
       </c>
       <c r="D851" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori secara massal</t>
+          <t>Melihat dan mengubah data master kategori</t>
         </is>
       </c>
       <c r="E851" s="57" t="inlineStr">
@@ -35963,19 +35963,19 @@
       </c>
       <c r="G851" s="56" t="inlineStr">
         <is>
-          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
         </is>
       </c>
       <c r="H851" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
+          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="852" ht="28" customHeight="1">
       <c r="A852" s="57" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B852" s="56" t="inlineStr">
@@ -35985,12 +35985,12 @@
       </c>
       <c r="C852" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D852" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori</t>
+          <t>Membuka halaman Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E852" s="57" t="inlineStr">
@@ -36000,24 +36000,24 @@
       </c>
       <c r="F852" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G852" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="H852" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="853" ht="28" customHeight="1">
       <c r="A853" s="57" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B853" s="56" t="inlineStr">
@@ -36027,12 +36027,12 @@
       </c>
       <c r="C853" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D853" s="56" t="inlineStr">
         <is>
-          <t>Melihat dan mengubah data master kategori</t>
+          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E853" s="57" t="inlineStr">
@@ -36047,19 +36047,19 @@
       </c>
       <c r="G853" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
+          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
         </is>
       </c>
       <c r="H853" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="854" ht="28" customHeight="1">
       <c r="A854" s="57" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B854" s="56" t="inlineStr">
@@ -36074,7 +36074,7 @@
       </c>
       <c r="D854" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Issue</t>
+          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
         </is>
       </c>
       <c r="E854" s="57" t="inlineStr">
@@ -36089,19 +36089,19 @@
       </c>
       <c r="G854" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
+          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H854" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="855" ht="28" customHeight="1">
       <c r="A855" s="57" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B855" s="56" t="inlineStr">
@@ -36111,12 +36111,12 @@
       </c>
       <c r="C855" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D855" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
+          <t>Membuka halaman Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E855" s="57" t="inlineStr">
@@ -36126,24 +36126,24 @@
       </c>
       <c r="F855" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G855" s="56" t="inlineStr">
         <is>
-          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="H855" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="856" ht="28" customHeight="1">
       <c r="A856" s="57" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B856" s="56" t="inlineStr">
@@ -36153,12 +36153,12 @@
       </c>
       <c r="C856" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D856" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
+          <t>Melakukan filter data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E856" s="57" t="inlineStr">
@@ -36168,24 +36168,24 @@
       </c>
       <c r="F856" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G856" s="56" t="inlineStr">
         <is>
-          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
+          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H856" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="857" ht="28" customHeight="1">
       <c r="A857" s="57" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B857" s="56" t="inlineStr">
@@ -36200,7 +36200,7 @@
       </c>
       <c r="D857" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Report Aktivitas Issue</t>
+          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
         </is>
       </c>
       <c r="E857" s="57" t="inlineStr">
@@ -36210,24 +36210,24 @@
       </c>
       <c r="F857" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G857" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
+          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H857" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="858" ht="28" customHeight="1">
       <c r="A858" s="57" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B858" s="56" t="inlineStr">
@@ -36242,7 +36242,7 @@
       </c>
       <c r="D858" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Report Aktivitas Issue</t>
+          <t>Melihat detail report aktivitas issue</t>
         </is>
       </c>
       <c r="E858" s="57" t="inlineStr">
@@ -36252,24 +36252,24 @@
       </c>
       <c r="F858" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G858" s="56" t="inlineStr">
         <is>
-          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H858" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="859" ht="28" customHeight="1">
       <c r="A859" s="57" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B859" s="56" t="inlineStr">
@@ -36284,7 +36284,7 @@
       </c>
       <c r="D859" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
+          <t>Menghapus data report aktivitas issue secara massal</t>
         </is>
       </c>
       <c r="E859" s="57" t="inlineStr">
@@ -36299,19 +36299,19 @@
       </c>
       <c r="G859" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
+          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
         </is>
       </c>
       <c r="H859" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menghapus data report aktivitas issue.</t>
         </is>
       </c>
     </row>
     <row r="860" ht="28" customHeight="1">
       <c r="A860" s="57" t="inlineStr">
         <is>
-          <t>75.4</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B860" s="56" t="inlineStr">
@@ -36326,7 +36326,7 @@
       </c>
       <c r="D860" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail report aktivitas issue</t>
+          <t>Mengekspor data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E860" s="57" t="inlineStr">
@@ -36341,34 +36341,34 @@
       </c>
       <c r="G860" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H860" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="861" ht="28" customHeight="1">
       <c r="A861" s="57" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="B861" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C861" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D861" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data report aktivitas issue secara massal</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E861" s="57" t="inlineStr">
@@ -36378,39 +36378,39 @@
       </c>
       <c r="F861" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G861" s="56" t="inlineStr">
         <is>
-          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="H861" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data report aktivitas issue.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="862" ht="28" customHeight="1">
       <c r="A862" s="57" t="inlineStr">
         <is>
-          <t>75.6</t>
+          <t>76.2</t>
         </is>
       </c>
       <c r="B862" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C862" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D862" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data Report Aktivitas Issue</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E862" s="57" t="inlineStr">
@@ -36420,24 +36420,24 @@
       </c>
       <c r="F862" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G862" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
         </is>
       </c>
       <c r="H862" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="863" ht="28" customHeight="1">
       <c r="A863" s="57" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>76.3</t>
         </is>
       </c>
       <c r="B863" s="56" t="inlineStr">
@@ -36452,7 +36452,7 @@
       </c>
       <c r="D863" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E863" s="57" t="inlineStr">
@@ -36462,24 +36462,24 @@
       </c>
       <c r="F863" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G863" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H863" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="864" ht="28" customHeight="1">
       <c r="A864" s="57" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.4</t>
         </is>
       </c>
       <c r="B864" s="56" t="inlineStr">
@@ -36494,12 +36494,12 @@
       </c>
       <c r="D864" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E864" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F864" s="57" t="inlineStr">
@@ -36509,19 +36509,19 @@
       </c>
       <c r="G864" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H864" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="865" ht="28" customHeight="1">
       <c r="A865" s="57" t="inlineStr">
         <is>
-          <t>76.3</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="B865" s="56" t="inlineStr">
@@ -36536,7 +36536,7 @@
       </c>
       <c r="D865" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E865" s="57" t="inlineStr">
@@ -36546,24 +36546,24 @@
       </c>
       <c r="F865" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G865" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H865" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="866" ht="28" customHeight="1">
       <c r="A866" s="57" t="inlineStr">
         <is>
-          <t>76.4</t>
+          <t>76.6</t>
         </is>
       </c>
       <c r="B866" s="56" t="inlineStr">
@@ -36578,12 +36578,12 @@
       </c>
       <c r="D866" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E866" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F866" s="57" t="inlineStr">
@@ -36593,19 +36593,19 @@
       </c>
       <c r="G866" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H866" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="867" ht="28" customHeight="1">
       <c r="A867" s="57" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="B867" s="56" t="inlineStr">
@@ -36620,34 +36620,34 @@
       </c>
       <c r="D867" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E867" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F867" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G867" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H867" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="868" ht="28" customHeight="1">
       <c r="A868" s="57" t="inlineStr">
         <is>
-          <t>76.6</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="B868" s="56" t="inlineStr">
@@ -36662,7 +36662,7 @@
       </c>
       <c r="D868" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E868" s="57" t="inlineStr">
@@ -36672,24 +36672,24 @@
       </c>
       <c r="F868" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G868" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H868" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="869" ht="28" customHeight="1">
       <c r="A869" s="57" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>77.1</t>
         </is>
       </c>
       <c r="B869" s="56" t="inlineStr">
@@ -36699,39 +36699,39 @@
       </c>
       <c r="C869" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D869" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E869" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F869" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G869" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="H869" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
     <row r="870" ht="28" customHeight="1">
       <c r="A870" s="57" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="B870" s="56" t="inlineStr">
@@ -36741,12 +36741,12 @@
       </c>
       <c r="C870" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D870" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E870" s="57" t="inlineStr">
@@ -36756,24 +36756,24 @@
       </c>
       <c r="F870" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G870" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
         </is>
       </c>
       <c r="H870" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="871" ht="28" customHeight="1">
       <c r="A871" s="57" t="inlineStr">
         <is>
-          <t>77.1</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="B871" s="56" t="inlineStr">
@@ -36788,7 +36788,7 @@
       </c>
       <c r="D871" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E871" s="57" t="inlineStr">
@@ -36798,24 +36798,24 @@
       </c>
       <c r="F871" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G871" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H871" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="872" ht="70" customHeight="1">
       <c r="A872" s="57" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="B872" s="56" t="inlineStr">
@@ -36830,12 +36830,12 @@
       </c>
       <c r="D872" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E872" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F872" s="57" t="inlineStr">
@@ -36845,19 +36845,19 @@
       </c>
       <c r="G872" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H872" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="873" ht="42" customHeight="1">
       <c r="A873" s="57" t="inlineStr">
         <is>
-          <t>77.3</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="B873" s="56" t="inlineStr">
@@ -36872,7 +36872,7 @@
       </c>
       <c r="D873" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E873" s="57" t="inlineStr">
@@ -36882,24 +36882,24 @@
       </c>
       <c r="F873" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G873" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H873" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="874" ht="42" customHeight="1">
       <c r="A874" s="57" t="inlineStr">
         <is>
-          <t>77.4</t>
+          <t>77.6</t>
         </is>
       </c>
       <c r="B874" s="56" t="inlineStr">
@@ -36914,12 +36914,12 @@
       </c>
       <c r="D874" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E874" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F874" s="57" t="inlineStr">
@@ -36929,19 +36929,19 @@
       </c>
       <c r="G874" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H874" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="875" ht="70" customHeight="1">
       <c r="A875" s="57" t="inlineStr">
         <is>
-          <t>77.5</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="B875" s="56" t="inlineStr">
@@ -36956,34 +36956,34 @@
       </c>
       <c r="D875" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E875" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F875" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G875" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H875" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="876" ht="28" customHeight="1">
       <c r="A876" s="57" t="inlineStr">
         <is>
-          <t>77.6</t>
+          <t>77.8</t>
         </is>
       </c>
       <c r="B876" s="56" t="inlineStr">
@@ -36998,7 +36998,7 @@
       </c>
       <c r="D876" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E876" s="57" t="inlineStr">
@@ -37008,24 +37008,24 @@
       </c>
       <c r="F876" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G876" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H876" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="877" ht="42" customHeight="1">
       <c r="A877" s="57" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>78.1</t>
         </is>
       </c>
       <c r="B877" s="56" t="inlineStr">
@@ -37035,39 +37035,39 @@
       </c>
       <c r="C877" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D877" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="E877" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F877" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G877" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="H877" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
         </is>
       </c>
     </row>
     <row r="878" ht="28" customHeight="1">
       <c r="A878" s="57" t="inlineStr">
         <is>
-          <t>77.8</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="B878" s="56" t="inlineStr">
@@ -37077,12 +37077,12 @@
       </c>
       <c r="C878" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D878" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E878" s="57" t="inlineStr">
@@ -37092,24 +37092,24 @@
       </c>
       <c r="F878" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G878" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
         </is>
       </c>
       <c r="H878" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="879" ht="28" customHeight="1">
       <c r="A879" s="57" t="inlineStr">
         <is>
-          <t>78.1</t>
+          <t>78.3</t>
         </is>
       </c>
       <c r="B879" s="56" t="inlineStr">
@@ -37124,7 +37124,7 @@
       </c>
       <c r="D879" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E879" s="57" t="inlineStr">
@@ -37134,104 +37134,22 @@
       </c>
       <c r="F879" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G879" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
         </is>
       </c>
       <c r="H879" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="880" ht="28" customHeight="1">
-      <c r="A880" s="57" t="inlineStr">
-        <is>
-          <t>78.2</t>
-        </is>
-      </c>
-      <c r="B880" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C880" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D880" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
-        </is>
-      </c>
-      <c r="E880" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F880" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G880" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H880" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="881" ht="14" customHeight="1">
-      <c r="A881" s="57" t="inlineStr">
-        <is>
-          <t>78.3</t>
-        </is>
-      </c>
-      <c r="B881" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C881" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D881" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="E881" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F881" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G881" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H881" s="56" t="inlineStr">
-        <is>
           <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
+    <row r="880" ht="28" customHeight="1"/>
+    <row r="881" ht="14" customHeight="1"/>
     <row r="882" ht="42" customHeight="1"/>
     <row r="883" ht="42" customHeight="1"/>
     <row r="884" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
feat(web): add test cases and guidance folders for Modul 79 (Dashboard - Optimalisasi Database)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -197,7 +197,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -287,11 +287,25 @@
         <color rgb="00D3D3D3"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -427,6 +441,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -706,7 +726,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z879"/>
+  <dimension ref="A1:Z884"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -37148,11 +37168,216 @@
         </is>
       </c>
     </row>
-    <row r="880" ht="28" customHeight="1"/>
-    <row r="881" ht="14" customHeight="1"/>
-    <row r="882" ht="42" customHeight="1"/>
-    <row r="883" ht="42" customHeight="1"/>
-    <row r="884" ht="28" customHeight="1"/>
+    <row r="880" ht="28" customHeight="1">
+      <c r="A880" s="58" t="inlineStr">
+        <is>
+          <t>79.1</t>
+        </is>
+      </c>
+      <c r="B880" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C880" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D880" s="59" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E880" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F880" s="58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G880" s="59" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
+        </is>
+      </c>
+      <c r="H880" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="881" ht="14" customHeight="1">
+      <c r="A881" s="58" t="inlineStr">
+        <is>
+          <t>79.2</t>
+        </is>
+      </c>
+      <c r="B881" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C881" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D881" s="59" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E881" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F881" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G881" s="59" t="inlineStr">
+        <is>
+          <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
+        </is>
+      </c>
+      <c r="H881" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="882" ht="42" customHeight="1">
+      <c r="A882" s="58" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="B882" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C882" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D882" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E882" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F882" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G882" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H882" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="883" ht="42" customHeight="1">
+      <c r="A883" s="58" t="inlineStr">
+        <is>
+          <t>79.4</t>
+        </is>
+      </c>
+      <c r="B883" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C883" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D883" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E883" s="58" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F883" s="58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G883" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H883" s="59" t="inlineStr">
+        <is>
+          <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="884" ht="28" customHeight="1">
+      <c r="A884" s="58" t="inlineStr">
+        <is>
+          <t>79.5</t>
+        </is>
+      </c>
+      <c r="B884" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C884" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D884" s="59" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E884" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F884" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G884" s="59" t="inlineStr">
+        <is>
+          <t>Klik button Export</t>
+        </is>
+      </c>
+      <c r="H884" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil mengunduh file data tabel dalam format Excel (.xlsx).</t>
+        </is>
+      </c>
+    </row>
     <row r="885" ht="42" customHeight="1"/>
     <row r="886" ht="14" customHeight="1"/>
     <row r="887" ht="42" customHeight="1"/>

</xml_diff>

<commit_message>
fix(web): trim Modul 70 Export Center - Persetujuan Export to 4 TCs (match senior)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z866"/>
+  <dimension ref="A1:Z861"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33982,7 +33982,7 @@
     <row r="804" ht="14" customHeight="1">
       <c r="A804" s="55" t="inlineStr">
         <is>
-          <t>70.5</t>
+          <t>71.1</t>
         </is>
       </c>
       <c r="B804" s="56" t="inlineStr">
@@ -33992,12 +33992,12 @@
       </c>
       <c r="C804" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D804" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data persetujuan export</t>
+          <t>Membuka halaman Aktivitas Export</t>
         </is>
       </c>
       <c r="E804" s="56" t="inlineStr">
@@ -34007,24 +34007,24 @@
       </c>
       <c r="F804" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G804" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
+          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
         </is>
       </c>
       <c r="H804" s="56" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan data persetujuan export sesuai kriteria filter.</t>
+          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
         </is>
       </c>
     </row>
     <row r="805" ht="14" customHeight="1">
       <c r="A805" s="55" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.2</t>
         </is>
       </c>
       <c r="B805" s="56" t="inlineStr">
@@ -34034,12 +34034,12 @@
       </c>
       <c r="C805" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D805" s="56" t="inlineStr">
         <is>
-          <t>Mereset filter data persetujuan export</t>
+          <t>Mencari data aktivitas export dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E805" s="56" t="inlineStr">
@@ -34054,19 +34054,19 @@
       </c>
       <c r="G805" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
+          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H805" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data persetujuan export.</t>
+          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="806" ht="14" customHeight="1">
       <c r="A806" s="55" t="inlineStr">
         <is>
-          <t>70.7</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="B806" s="56" t="inlineStr">
@@ -34076,39 +34076,39 @@
       </c>
       <c r="C806" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D806" s="56" t="inlineStr">
         <is>
-          <t>Melakukan approval data pengajuan export</t>
+          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E806" s="56" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F806" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G806" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Setujui - Klik button Setujui pada modal konfirmasi</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H806" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyetujui pengajuan export dan status berubah menjadi Disetujui.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="807" ht="14" customHeight="1">
       <c r="A807" s="55" t="inlineStr">
         <is>
-          <t>70.8</t>
+          <t>71.4</t>
         </is>
       </c>
       <c r="B807" s="56" t="inlineStr">
@@ -34118,12 +34118,12 @@
       </c>
       <c r="C807" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D807" s="56" t="inlineStr">
         <is>
-          <t>Melakukan reject data pengajuan export</t>
+          <t>Melihat data aktivitas export berdasarkan status</t>
         </is>
       </c>
       <c r="E807" s="56" t="inlineStr">
@@ -34133,24 +34133,24 @@
       </c>
       <c r="F807" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G807" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada data status Menunggu - Pilih opsi Tolak - Masukkan alasan pada field Alasan Penolakan - Klik button Tolak</t>
+          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
         </is>
       </c>
       <c r="H807" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menolak pengajuan export dan status berubah menjadi Ditolak.</t>
+          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="808" ht="14" customHeight="1">
       <c r="A808" s="55" t="inlineStr">
         <is>
-          <t>70.9</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="B808" s="56" t="inlineStr">
@@ -34160,12 +34160,12 @@
       </c>
       <c r="C808" s="56" t="inlineStr">
         <is>
-          <t>Persetujuan Export</t>
+          <t>Aktivitas Export</t>
         </is>
       </c>
       <c r="D808" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail pengajuan export</t>
+          <t>Melakukan filter data aktivitas export</t>
         </is>
       </c>
       <c r="E808" s="56" t="inlineStr">
@@ -34180,19 +34180,19 @@
       </c>
       <c r="G808" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
         </is>
       </c>
       <c r="H808" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan detail data pengajuan export.</t>
+          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
         </is>
       </c>
     </row>
     <row r="809" ht="14" customHeight="1">
       <c r="A809" s="55" t="inlineStr">
         <is>
-          <t>71.1</t>
+          <t>71.6</t>
         </is>
       </c>
       <c r="B809" s="56" t="inlineStr">
@@ -34207,7 +34207,7 @@
       </c>
       <c r="D809" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Aktivitas Export</t>
+          <t>Mereset filter data aktivitas export</t>
         </is>
       </c>
       <c r="E809" s="56" t="inlineStr">
@@ -34217,24 +34217,24 @@
       </c>
       <c r="F809" s="55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G809" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
+          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
         </is>
       </c>
       <c r="H809" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Aktivitas Export.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="810" ht="42" customHeight="1">
       <c r="A810" s="55" t="inlineStr">
         <is>
-          <t>71.2</t>
+          <t>71.7</t>
         </is>
       </c>
       <c r="B810" s="56" t="inlineStr">
@@ -34249,7 +34249,7 @@
       </c>
       <c r="D810" s="56" t="inlineStr">
         <is>
-          <t>Mencari data aktivitas export dengan kata kunci valid</t>
+          <t>Melihat detail aktivitas export</t>
         </is>
       </c>
       <c r="E810" s="56" t="inlineStr">
@@ -34259,24 +34259,24 @@
       </c>
       <c r="F810" s="55" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G810" s="56" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H810" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
+          <t>Berhasil menampilkan detail data aktivitas export.</t>
         </is>
       </c>
     </row>
     <row r="811" ht="28" customHeight="1">
       <c r="A811" s="55" t="inlineStr">
         <is>
-          <t>71.3</t>
+          <t>71.8</t>
         </is>
       </c>
       <c r="B811" s="56" t="inlineStr">
@@ -34291,244 +34291,244 @@
       </c>
       <c r="D811" s="56" t="inlineStr">
         <is>
-          <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
+          <t>Mengunduh file data export yang tersedia</t>
         </is>
       </c>
       <c r="E811" s="56" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F811" s="55" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G811" s="56" t="inlineStr">
+        <is>
+          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
+        </is>
+      </c>
+      <c r="H811" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mengunduh file data export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="812" ht="42" customHeight="1">
+      <c r="A812" s="57" t="inlineStr">
+        <is>
+          <t>72.1</t>
+        </is>
+      </c>
+      <c r="B812" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C812" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D812" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E812" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F812" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G812" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H812" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="813" ht="28" customHeight="1">
+      <c r="A813" s="57" t="inlineStr">
+        <is>
+          <t>72.2</t>
+        </is>
+      </c>
+      <c r="B813" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C813" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D813" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E813" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F813" s="57" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G811" s="56" t="inlineStr">
-        <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H811" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="812" ht="42" customHeight="1">
-      <c r="A812" s="55" t="inlineStr">
-        <is>
-          <t>71.4</t>
-        </is>
-      </c>
-      <c r="B812" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C812" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D812" s="56" t="inlineStr">
-        <is>
-          <t>Melihat data aktivitas export berdasarkan status</t>
-        </is>
-      </c>
-      <c r="E812" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F812" s="55" t="inlineStr">
+      <c r="G813" s="56" t="inlineStr">
+        <is>
+          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
+        </is>
+      </c>
+      <c r="H813" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="814" ht="28" customHeight="1">
+      <c r="A814" s="57" t="inlineStr">
+        <is>
+          <t>72.3</t>
+        </is>
+      </c>
+      <c r="B814" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C814" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D814" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E814" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F814" s="57" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G812" s="56" t="inlineStr">
-        <is>
-          <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
-        </is>
-      </c>
-      <c r="H812" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="813" ht="28" customHeight="1">
-      <c r="A813" s="55" t="inlineStr">
-        <is>
-          <t>71.5</t>
-        </is>
-      </c>
-      <c r="B813" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C813" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D813" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E813" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F813" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G813" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H813" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="814" ht="28" customHeight="1">
-      <c r="A814" s="55" t="inlineStr">
-        <is>
-          <t>71.6</t>
-        </is>
-      </c>
-      <c r="B814" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C814" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D814" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E814" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F814" s="55" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
       <c r="G814" s="56" t="inlineStr">
         <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
+          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H814" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="815" ht="56" customHeight="1">
-      <c r="A815" s="55" t="inlineStr">
-        <is>
-          <t>71.7</t>
+      <c r="A815" s="57" t="inlineStr">
+        <is>
+          <t>72.4</t>
         </is>
       </c>
       <c r="B815" s="56" t="inlineStr">
         <is>
-          <t>Export Center</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C815" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Export</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D815" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail aktivitas export</t>
-        </is>
-      </c>
-      <c r="E815" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F815" s="55" t="inlineStr">
+          <t>Menambahkan pelaporan issue baru</t>
+        </is>
+      </c>
+      <c r="E815" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F815" s="57" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="G815" s="56" t="inlineStr">
         <is>
+          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
+        </is>
+      </c>
+      <c r="H815" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan data pelaporan issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="816" ht="56" customHeight="1">
+      <c r="A816" s="57" t="inlineStr">
+        <is>
+          <t>72.5</t>
+        </is>
+      </c>
+      <c r="B816" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C816" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D816" s="56" t="inlineStr">
+        <is>
+          <t>Melihat detail pelaporan issue</t>
+        </is>
+      </c>
+      <c r="E816" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F816" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G816" s="56" t="inlineStr">
+        <is>
           <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
-      <c r="H815" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="816" ht="56" customHeight="1">
-      <c r="A816" s="55" t="inlineStr">
-        <is>
-          <t>71.8</t>
-        </is>
-      </c>
-      <c r="B816" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C816" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D816" s="56" t="inlineStr">
-        <is>
-          <t>Mengunduh file data export yang tersedia</t>
-        </is>
-      </c>
-      <c r="E816" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F816" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G816" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
-        </is>
-      </c>
       <c r="H816" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh file data export.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="817" ht="28" customHeight="1">
       <c r="A817" s="57" t="inlineStr">
         <is>
-          <t>72.1</t>
+          <t>72.6</t>
         </is>
       </c>
       <c r="B817" s="56" t="inlineStr">
@@ -34543,7 +34543,7 @@
       </c>
       <c r="D817" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Aktivitas Issue</t>
+          <t>Mengubah data pelaporan issue</t>
         </is>
       </c>
       <c r="E817" s="57" t="inlineStr">
@@ -34553,24 +34553,24 @@
       </c>
       <c r="F817" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G817" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
         </is>
       </c>
       <c r="H817" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
+          <t>Berhasil menyimpan perubahan data issue.</t>
         </is>
       </c>
     </row>
     <row r="818" ht="28" customHeight="1">
       <c r="A818" s="57" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.7</t>
         </is>
       </c>
       <c r="B818" s="56" t="inlineStr">
@@ -34585,7 +34585,7 @@
       </c>
       <c r="D818" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Aktivitas Issue</t>
+          <t>Menambahkan komentar pada detail aktivitas issue</t>
         </is>
       </c>
       <c r="E818" s="57" t="inlineStr">
@@ -34600,19 +34600,19 @@
       </c>
       <c r="G818" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
+          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
         </is>
       </c>
       <c r="H818" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menambahkan komentar pada detail issue.</t>
         </is>
       </c>
     </row>
     <row r="819" ht="42" customHeight="1">
       <c r="A819" s="57" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>72.8</t>
         </is>
       </c>
       <c r="B819" s="56" t="inlineStr">
@@ -34627,7 +34627,7 @@
       </c>
       <c r="D819" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
+          <t>Menghapus data pelaporan issue</t>
         </is>
       </c>
       <c r="E819" s="57" t="inlineStr">
@@ -34642,19 +34642,19 @@
       </c>
       <c r="G819" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
         </is>
       </c>
       <c r="H819" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menghapus data issue.</t>
         </is>
       </c>
     </row>
     <row r="820" ht="14" customHeight="1">
       <c r="A820" s="57" t="inlineStr">
         <is>
-          <t>72.4</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B820" s="56" t="inlineStr">
@@ -34664,12 +34664,12 @@
       </c>
       <c r="C820" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D820" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan pelaporan issue baru</t>
+          <t>Membuka halaman Master Kategori Issue</t>
         </is>
       </c>
       <c r="E820" s="57" t="inlineStr">
@@ -34684,19 +34684,19 @@
       </c>
       <c r="G820" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="H820" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data pelaporan issue.</t>
+          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
         </is>
       </c>
     </row>
     <row r="821" ht="56" customHeight="1">
       <c r="A821" s="57" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="B821" s="56" t="inlineStr">
@@ -34706,12 +34706,12 @@
       </c>
       <c r="C821" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D821" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail pelaporan issue</t>
+          <t>Menambahkan kategori lain melalui pelaporan issue</t>
         </is>
       </c>
       <c r="E821" s="57" t="inlineStr">
@@ -34721,24 +34721,24 @@
       </c>
       <c r="F821" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G821" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H821" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
         </is>
       </c>
     </row>
     <row r="822" ht="56" customHeight="1">
       <c r="A822" s="57" t="inlineStr">
         <is>
-          <t>72.6</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="B822" s="56" t="inlineStr">
@@ -34748,12 +34748,12 @@
       </c>
       <c r="C822" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D822" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data pelaporan issue</t>
+          <t>Menambahkan data master kategori</t>
         </is>
       </c>
       <c r="E822" s="57" t="inlineStr">
@@ -34763,24 +34763,24 @@
       </c>
       <c r="F822" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G822" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
+          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
         </is>
       </c>
       <c r="H822" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data issue.</t>
+          <t>Berhasil menyimpan data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="823" ht="56" customHeight="1">
       <c r="A823" s="57" t="inlineStr">
         <is>
-          <t>72.7</t>
+          <t>73.4</t>
         </is>
       </c>
       <c r="B823" s="56" t="inlineStr">
@@ -34790,12 +34790,12 @@
       </c>
       <c r="C823" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D823" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan komentar pada detail aktivitas issue</t>
+          <t>Mencari data pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E823" s="57" t="inlineStr">
@@ -34810,19 +34810,19 @@
       </c>
       <c r="G823" s="56" t="inlineStr">
         <is>
-          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
+          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
         </is>
       </c>
       <c r="H823" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan komentar pada detail issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="824" ht="14" customHeight="1">
       <c r="A824" s="57" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="B824" s="56" t="inlineStr">
@@ -34832,12 +34832,12 @@
       </c>
       <c r="C824" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D824" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data pelaporan issue</t>
+          <t>Melihat detail data kategori pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E824" s="57" t="inlineStr">
@@ -34852,19 +34852,19 @@
       </c>
       <c r="G824" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H824" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data issue.</t>
+          <t>Berhasil menampilkan modal detail kategori.</t>
         </is>
       </c>
     </row>
     <row r="825" ht="14" customHeight="1">
       <c r="A825" s="57" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>73.6</t>
         </is>
       </c>
       <c r="B825" s="56" t="inlineStr">
@@ -34879,7 +34879,7 @@
       </c>
       <c r="D825" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Master Kategori Issue</t>
+          <t>Mengirim data kategori lain ke master kategori</t>
         </is>
       </c>
       <c r="E825" s="57" t="inlineStr">
@@ -34894,19 +34894,19 @@
       </c>
       <c r="G825" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
+          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
         </is>
       </c>
       <c r="H825" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
+          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="826" ht="14" customHeight="1">
       <c r="A826" s="57" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>73.7</t>
         </is>
       </c>
       <c r="B826" s="56" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="D826" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan kategori lain melalui pelaporan issue</t>
+          <t>Mengirim data kategori lain ke master kategori secara massal</t>
         </is>
       </c>
       <c r="E826" s="57" t="inlineStr">
@@ -34936,19 +34936,19 @@
       </c>
       <c r="G826" s="56" t="inlineStr">
         <is>
-          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
+          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
         </is>
       </c>
       <c r="H826" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
+          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="827" ht="42" customHeight="1">
       <c r="A827" s="57" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.8</t>
         </is>
       </c>
       <c r="B827" s="56" t="inlineStr">
@@ -34963,7 +34963,7 @@
       </c>
       <c r="D827" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan data master kategori</t>
+          <t>Mencari data pada List Kategori</t>
         </is>
       </c>
       <c r="E827" s="57" t="inlineStr">
@@ -34973,24 +34973,24 @@
       </c>
       <c r="F827" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G827" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
+          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
         </is>
       </c>
       <c r="H827" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data master kategori.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="828" ht="14" customHeight="1">
       <c r="A828" s="57" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>73.9</t>
         </is>
       </c>
       <c r="B828" s="56" t="inlineStr">
@@ -35005,7 +35005,7 @@
       </c>
       <c r="D828" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori Lain</t>
+          <t>Melihat dan mengubah data master kategori</t>
         </is>
       </c>
       <c r="E828" s="57" t="inlineStr">
@@ -35020,19 +35020,19 @@
       </c>
       <c r="G828" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
         </is>
       </c>
       <c r="H828" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="829" ht="56" customHeight="1">
       <c r="A829" s="57" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B829" s="56" t="inlineStr">
@@ -35042,12 +35042,12 @@
       </c>
       <c r="C829" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D829" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail data kategori pada List Kategori Lain</t>
+          <t>Membuka halaman Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E829" s="57" t="inlineStr">
@@ -35057,24 +35057,24 @@
       </c>
       <c r="F829" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G829" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="H829" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan modal detail kategori.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="830" ht="28" customHeight="1">
       <c r="A830" s="57" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B830" s="56" t="inlineStr">
@@ -35084,12 +35084,12 @@
       </c>
       <c r="C830" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D830" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori</t>
+          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E830" s="57" t="inlineStr">
@@ -35099,24 +35099,24 @@
       </c>
       <c r="F830" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G830" s="56" t="inlineStr">
         <is>
-          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
+          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
         </is>
       </c>
       <c r="H830" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="831" ht="42" customHeight="1">
       <c r="A831" s="57" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B831" s="56" t="inlineStr">
@@ -35126,12 +35126,12 @@
       </c>
       <c r="C831" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D831" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori secara massal</t>
+          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
         </is>
       </c>
       <c r="E831" s="57" t="inlineStr">
@@ -35141,24 +35141,24 @@
       </c>
       <c r="F831" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G831" s="56" t="inlineStr">
         <is>
-          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
+          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H831" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="832" ht="28" customHeight="1">
       <c r="A832" s="57" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B832" s="56" t="inlineStr">
@@ -35168,12 +35168,12 @@
       </c>
       <c r="C832" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D832" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori</t>
+          <t>Membuka halaman Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E832" s="57" t="inlineStr">
@@ -35183,24 +35183,24 @@
       </c>
       <c r="F832" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G832" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="H832" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="833" ht="14" customHeight="1">
       <c r="A833" s="57" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B833" s="56" t="inlineStr">
@@ -35210,12 +35210,12 @@
       </c>
       <c r="C833" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D833" s="56" t="inlineStr">
         <is>
-          <t>Melihat dan mengubah data master kategori</t>
+          <t>Melakukan filter data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E833" s="57" t="inlineStr">
@@ -35230,19 +35230,19 @@
       </c>
       <c r="G833" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
+          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H833" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="834" ht="14" customHeight="1">
       <c r="A834" s="57" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B834" s="56" t="inlineStr">
@@ -35252,12 +35252,12 @@
       </c>
       <c r="C834" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D834" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Issue</t>
+          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
         </is>
       </c>
       <c r="E834" s="57" t="inlineStr">
@@ -35267,24 +35267,24 @@
       </c>
       <c r="F834" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G834" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
+          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H834" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="835" ht="14" customHeight="1">
       <c r="A835" s="57" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B835" s="56" t="inlineStr">
@@ -35294,12 +35294,12 @@
       </c>
       <c r="C835" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D835" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
+          <t>Melihat detail report aktivitas issue</t>
         </is>
       </c>
       <c r="E835" s="57" t="inlineStr">
@@ -35309,24 +35309,24 @@
       </c>
       <c r="F835" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G835" s="56" t="inlineStr">
         <is>
-          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H835" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="836" ht="42" customHeight="1">
       <c r="A836" s="57" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B836" s="56" t="inlineStr">
@@ -35336,12 +35336,12 @@
       </c>
       <c r="C836" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D836" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
+          <t>Menghapus data report aktivitas issue secara massal</t>
         </is>
       </c>
       <c r="E836" s="57" t="inlineStr">
@@ -35351,24 +35351,24 @@
       </c>
       <c r="F836" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G836" s="56" t="inlineStr">
         <is>
-          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
+          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
         </is>
       </c>
       <c r="H836" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menghapus data report aktivitas issue.</t>
         </is>
       </c>
     </row>
     <row r="837" ht="28" customHeight="1">
       <c r="A837" s="57" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B837" s="56" t="inlineStr">
@@ -35383,7 +35383,7 @@
       </c>
       <c r="D837" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Report Aktivitas Issue</t>
+          <t>Mengekspor data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E837" s="57" t="inlineStr">
@@ -35398,34 +35398,34 @@
       </c>
       <c r="G837" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H837" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="838" ht="28" customHeight="1">
       <c r="A838" s="57" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="B838" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C838" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D838" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Report Aktivitas Issue</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E838" s="57" t="inlineStr">
@@ -35435,39 +35435,39 @@
       </c>
       <c r="F838" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G838" s="56" t="inlineStr">
         <is>
-          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="H838" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="839" ht="70" customHeight="1">
       <c r="A839" s="57" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>76.2</t>
         </is>
       </c>
       <c r="B839" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C839" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D839" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E839" s="57" t="inlineStr">
@@ -35482,34 +35482,34 @@
       </c>
       <c r="G839" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
+          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
         </is>
       </c>
       <c r="H839" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="840" ht="28" customHeight="1">
       <c r="A840" s="57" t="inlineStr">
         <is>
-          <t>75.4</t>
+          <t>76.3</t>
         </is>
       </c>
       <c r="B840" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C840" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D840" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail report aktivitas issue</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E840" s="57" t="inlineStr">
@@ -35519,44 +35519,44 @@
       </c>
       <c r="F840" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G840" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H840" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="841" ht="84" customHeight="1">
       <c r="A841" s="57" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>76.4</t>
         </is>
       </c>
       <c r="B841" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C841" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D841" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data report aktivitas issue secara massal</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E841" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F841" s="57" t="inlineStr">
@@ -35566,34 +35566,34 @@
       </c>
       <c r="G841" s="56" t="inlineStr">
         <is>
-          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H841" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data report aktivitas issue.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="842" ht="28" customHeight="1">
       <c r="A842" s="57" t="inlineStr">
         <is>
-          <t>75.6</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="B842" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C842" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D842" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data Report Aktivitas Issue</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E842" s="57" t="inlineStr">
@@ -35608,7 +35608,7 @@
       </c>
       <c r="G842" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H842" s="56" t="inlineStr">
@@ -35620,7 +35620,7 @@
     <row r="843" ht="28" customHeight="1">
       <c r="A843" s="57" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>76.6</t>
         </is>
       </c>
       <c r="B843" s="56" t="inlineStr">
@@ -35635,7 +35635,7 @@
       </c>
       <c r="D843" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E843" s="57" t="inlineStr">
@@ -35645,24 +35645,24 @@
       </c>
       <c r="F843" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G843" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H843" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="844" ht="28" customHeight="1">
       <c r="A844" s="57" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="B844" s="56" t="inlineStr">
@@ -35677,12 +35677,12 @@
       </c>
       <c r="D844" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E844" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F844" s="57" t="inlineStr">
@@ -35692,19 +35692,19 @@
       </c>
       <c r="G844" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H844" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="845" ht="42" customHeight="1">
       <c r="A845" s="57" t="inlineStr">
         <is>
-          <t>76.3</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="B845" s="56" t="inlineStr">
@@ -35719,7 +35719,7 @@
       </c>
       <c r="D845" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E845" s="57" t="inlineStr">
@@ -35729,24 +35729,24 @@
       </c>
       <c r="F845" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G845" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H845" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="846" ht="28" customHeight="1">
       <c r="A846" s="57" t="inlineStr">
         <is>
-          <t>76.4</t>
+          <t>77.1</t>
         </is>
       </c>
       <c r="B846" s="56" t="inlineStr">
@@ -35756,39 +35756,39 @@
       </c>
       <c r="C846" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D846" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E846" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F846" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G846" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="H846" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
     <row r="847" ht="14" customHeight="1">
       <c r="A847" s="57" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="B847" s="56" t="inlineStr">
@@ -35798,12 +35798,12 @@
       </c>
       <c r="C847" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D847" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E847" s="57" t="inlineStr">
@@ -35813,24 +35813,24 @@
       </c>
       <c r="F847" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G847" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
         </is>
       </c>
       <c r="H847" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="848" ht="14" customHeight="1">
       <c r="A848" s="57" t="inlineStr">
         <is>
-          <t>76.6</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="B848" s="56" t="inlineStr">
@@ -35840,12 +35840,12 @@
       </c>
       <c r="C848" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D848" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E848" s="57" t="inlineStr">
@@ -35860,7 +35860,7 @@
       </c>
       <c r="G848" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H848" s="56" t="inlineStr">
@@ -35872,7 +35872,7 @@
     <row r="849" ht="42" customHeight="1">
       <c r="A849" s="57" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="B849" s="56" t="inlineStr">
@@ -35882,12 +35882,12 @@
       </c>
       <c r="C849" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D849" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E849" s="57" t="inlineStr">
@@ -35902,7 +35902,7 @@
       </c>
       <c r="G849" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H849" s="56" t="inlineStr">
@@ -35914,7 +35914,7 @@
     <row r="850" ht="28" customHeight="1">
       <c r="A850" s="57" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="B850" s="56" t="inlineStr">
@@ -35924,12 +35924,12 @@
       </c>
       <c r="C850" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D850" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E850" s="57" t="inlineStr">
@@ -35944,7 +35944,7 @@
       </c>
       <c r="G850" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H850" s="56" t="inlineStr">
@@ -35956,7 +35956,7 @@
     <row r="851" ht="28" customHeight="1">
       <c r="A851" s="57" t="inlineStr">
         <is>
-          <t>77.1</t>
+          <t>77.6</t>
         </is>
       </c>
       <c r="B851" s="56" t="inlineStr">
@@ -35971,7 +35971,7 @@
       </c>
       <c r="D851" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E851" s="57" t="inlineStr">
@@ -35981,24 +35981,24 @@
       </c>
       <c r="F851" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G851" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H851" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="852" ht="28" customHeight="1">
       <c r="A852" s="57" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="B852" s="56" t="inlineStr">
@@ -36013,12 +36013,12 @@
       </c>
       <c r="D852" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E852" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F852" s="57" t="inlineStr">
@@ -36028,19 +36028,19 @@
       </c>
       <c r="G852" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H852" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="853" ht="28" customHeight="1">
       <c r="A853" s="57" t="inlineStr">
         <is>
-          <t>77.3</t>
+          <t>77.8</t>
         </is>
       </c>
       <c r="B853" s="56" t="inlineStr">
@@ -36055,7 +36055,7 @@
       </c>
       <c r="D853" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E853" s="57" t="inlineStr">
@@ -36065,24 +36065,24 @@
       </c>
       <c r="F853" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G853" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H853" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="854" ht="28" customHeight="1">
       <c r="A854" s="57" t="inlineStr">
         <is>
-          <t>77.4</t>
+          <t>78.1</t>
         </is>
       </c>
       <c r="B854" s="56" t="inlineStr">
@@ -36092,39 +36092,39 @@
       </c>
       <c r="C854" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D854" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="E854" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F854" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G854" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="H854" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
         </is>
       </c>
     </row>
     <row r="855" ht="28" customHeight="1">
       <c r="A855" s="57" t="inlineStr">
         <is>
-          <t>77.5</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="B855" s="56" t="inlineStr">
@@ -36134,12 +36134,12 @@
       </c>
       <c r="C855" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D855" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E855" s="57" t="inlineStr">
@@ -36149,24 +36149,24 @@
       </c>
       <c r="F855" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G855" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
         </is>
       </c>
       <c r="H855" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="856" ht="28" customHeight="1">
       <c r="A856" s="57" t="inlineStr">
         <is>
-          <t>77.6</t>
+          <t>78.3</t>
         </is>
       </c>
       <c r="B856" s="56" t="inlineStr">
@@ -36176,12 +36176,12 @@
       </c>
       <c r="C856" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D856" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E856" s="57" t="inlineStr">
@@ -36196,435 +36196,230 @@
       </c>
       <c r="G856" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
         </is>
       </c>
       <c r="H856" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
     <row r="857" ht="28" customHeight="1">
-      <c r="A857" s="57" t="inlineStr">
-        <is>
-          <t>77.7</t>
-        </is>
-      </c>
-      <c r="B857" s="56" t="inlineStr">
+      <c r="A857" s="58" t="inlineStr">
+        <is>
+          <t>79.1</t>
+        </is>
+      </c>
+      <c r="B857" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C857" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="D857" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
-        </is>
-      </c>
-      <c r="E857" s="57" t="inlineStr">
+      <c r="C857" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D857" s="59" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E857" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F857" s="58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G857" s="59" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
+        </is>
+      </c>
+      <c r="H857" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="858" ht="28" customHeight="1">
+      <c r="A858" s="58" t="inlineStr">
+        <is>
+          <t>79.2</t>
+        </is>
+      </c>
+      <c r="B858" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C858" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D858" s="59" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E858" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F858" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G858" s="59" t="inlineStr">
+        <is>
+          <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
+        </is>
+      </c>
+      <c r="H858" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="859" ht="28" customHeight="1">
+      <c r="A859" s="58" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="B859" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C859" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D859" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E859" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F859" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G859" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H859" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="860" ht="28" customHeight="1">
+      <c r="A860" s="58" t="inlineStr">
+        <is>
+          <t>79.4</t>
+        </is>
+      </c>
+      <c r="B860" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C860" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D860" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E860" s="58" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F857" s="57" t="inlineStr">
+      <c r="F860" s="58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G860" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H860" s="59" t="inlineStr">
+        <is>
+          <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="861" ht="28" customHeight="1">
+      <c r="A861" s="58" t="inlineStr">
+        <is>
+          <t>79.5</t>
+        </is>
+      </c>
+      <c r="B861" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C861" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D861" s="59" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E861" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F861" s="58" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G857" s="56" t="inlineStr">
-        <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
-        </is>
-      </c>
-      <c r="H857" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="858" ht="28" customHeight="1">
-      <c r="A858" s="57" t="inlineStr">
-        <is>
-          <t>77.8</t>
-        </is>
-      </c>
-      <c r="B858" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C858" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="D858" s="56" t="inlineStr">
-        <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
-        </is>
-      </c>
-      <c r="E858" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F858" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G858" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
-        </is>
-      </c>
-      <c r="H858" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mendownload file export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="859" ht="28" customHeight="1">
-      <c r="A859" s="57" t="inlineStr">
-        <is>
-          <t>78.1</t>
-        </is>
-      </c>
-      <c r="B859" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C859" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D859" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="E859" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F859" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G859" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="H859" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="860" ht="28" customHeight="1">
-      <c r="A860" s="57" t="inlineStr">
-        <is>
-          <t>78.2</t>
-        </is>
-      </c>
-      <c r="B860" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C860" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D860" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
-        </is>
-      </c>
-      <c r="E860" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F860" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G860" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H860" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="861" ht="28" customHeight="1">
-      <c r="A861" s="57" t="inlineStr">
-        <is>
-          <t>78.3</t>
-        </is>
-      </c>
-      <c r="B861" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C861" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D861" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="E861" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F861" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G861" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H861" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="862" ht="28" customHeight="1">
-      <c r="A862" s="58" t="inlineStr">
-        <is>
-          <t>79.1</t>
-        </is>
-      </c>
-      <c r="B862" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C862" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D862" s="59" t="inlineStr">
-        <is>
-          <t>Membuka halaman Dashboard Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="E862" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F862" s="58" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G862" s="59" t="inlineStr">
-        <is>
-          <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
-        </is>
-      </c>
-      <c r="H862" s="59" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
-        </is>
-      </c>
-    </row>
-    <row r="863" ht="28" customHeight="1">
-      <c r="A863" s="58" t="inlineStr">
-        <is>
-          <t>79.2</t>
-        </is>
-      </c>
-      <c r="B863" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C863" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D863" s="59" t="inlineStr">
-        <is>
-          <t>Melakukan filter data Dashboard Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="E863" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F863" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G863" s="59" t="inlineStr">
-        <is>
-          <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
-        </is>
-      </c>
-      <c r="H863" s="59" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="864" ht="28" customHeight="1">
-      <c r="A864" s="58" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="B864" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C864" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D864" s="59" t="inlineStr">
-        <is>
-          <t>Mencari data pada tabel dengan keyword valid</t>
-        </is>
-      </c>
-      <c r="E864" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F864" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G864" s="59" t="inlineStr">
-        <is>
-          <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H864" s="59" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
-        </is>
-      </c>
-    </row>
-    <row r="865" ht="28" customHeight="1">
-      <c r="A865" s="58" t="inlineStr">
-        <is>
-          <t>79.4</t>
-        </is>
-      </c>
-      <c r="B865" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C865" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D865" s="59" t="inlineStr">
-        <is>
-          <t>Mencari data pada tabel dengan keyword tidak valid</t>
-        </is>
-      </c>
-      <c r="E865" s="58" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F865" s="58" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G865" s="59" t="inlineStr">
-        <is>
-          <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H865" s="59" t="inlineStr">
-        <is>
-          <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="866" ht="28" customHeight="1">
-      <c r="A866" s="58" t="inlineStr">
-        <is>
-          <t>79.5</t>
-        </is>
-      </c>
-      <c r="B866" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C866" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D866" s="59" t="inlineStr">
-        <is>
-          <t>Mengekspor data tabel Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="E866" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F866" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G866" s="59" t="inlineStr">
+      <c r="G861" s="59" t="inlineStr">
         <is>
           <t>Klik button Export</t>
         </is>
       </c>
-      <c r="H866" s="59" t="inlineStr">
+      <c r="H861" s="59" t="inlineStr">
         <is>
           <t>Berhasil mengunduh file data tabel dalam format Excel (.xlsx).</t>
         </is>
       </c>
     </row>
+    <row r="862" ht="28" customHeight="1"/>
+    <row r="863" ht="28" customHeight="1"/>
+    <row r="864" ht="28" customHeight="1"/>
+    <row r="865" ht="28" customHeight="1"/>
+    <row r="866" ht="28" customHeight="1"/>
     <row r="867" ht="28" customHeight="1"/>
     <row r="868" ht="28" customHeight="1"/>
     <row r="869" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
fix(web): trim Modul 71 Export Center - Aktivitas Export to 4 TCs (match senior)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z861"/>
+  <dimension ref="A1:Z857"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34148,177 +34148,177 @@
       </c>
     </row>
     <row r="808" ht="14" customHeight="1">
-      <c r="A808" s="55" t="inlineStr">
-        <is>
-          <t>71.5</t>
+      <c r="A808" s="57" t="inlineStr">
+        <is>
+          <t>72.1</t>
         </is>
       </c>
       <c r="B808" s="56" t="inlineStr">
         <is>
-          <t>Export Center</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C808" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Export</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D808" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E808" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F808" s="55" t="inlineStr">
+          <t>Membuka halaman Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E808" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F808" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G808" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="H808" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="809" ht="14" customHeight="1">
+      <c r="A809" s="57" t="inlineStr">
+        <is>
+          <t>72.2</t>
+        </is>
+      </c>
+      <c r="B809" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C809" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D809" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="E809" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F809" s="57" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G808" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Pilih kriteria filter pada drawer - Klik button Terapkan Filter</t>
-        </is>
-      </c>
-      <c r="H808" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil memfilter dan menampilkan data aktivitas export sesuai kriteria filter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="809" ht="14" customHeight="1">
-      <c r="A809" s="55" t="inlineStr">
-        <is>
-          <t>71.6</t>
-        </is>
-      </c>
-      <c r="B809" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C809" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D809" s="56" t="inlineStr">
-        <is>
-          <t>Mereset filter data aktivitas export</t>
-        </is>
-      </c>
-      <c r="E809" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F809" s="55" t="inlineStr">
+      <c r="G809" s="56" t="inlineStr">
+        <is>
+          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
+        </is>
+      </c>
+      <c r="H809" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="810" ht="42" customHeight="1">
+      <c r="A810" s="57" t="inlineStr">
+        <is>
+          <t>72.3</t>
+        </is>
+      </c>
+      <c r="B810" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C810" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D810" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E810" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F810" s="57" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G809" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Filter - Klik button Reset pada drawer Filter</t>
-        </is>
-      </c>
-      <c r="H809" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mereset filter dan menampilkan seluruh data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="810" ht="42" customHeight="1">
-      <c r="A810" s="55" t="inlineStr">
-        <is>
-          <t>71.7</t>
-        </is>
-      </c>
-      <c r="B810" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C810" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D810" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail aktivitas export</t>
-        </is>
-      </c>
-      <c r="E810" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F810" s="55" t="inlineStr">
+      <c r="G810" s="56" t="inlineStr">
+        <is>
+          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H810" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="811" ht="28" customHeight="1">
+      <c r="A811" s="57" t="inlineStr">
+        <is>
+          <t>72.4</t>
+        </is>
+      </c>
+      <c r="B811" s="56" t="inlineStr">
+        <is>
+          <t>Ticket Maintenance</t>
+        </is>
+      </c>
+      <c r="C811" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Issue</t>
+        </is>
+      </c>
+      <c r="D811" s="56" t="inlineStr">
+        <is>
+          <t>Menambahkan pelaporan issue baru</t>
+        </is>
+      </c>
+      <c r="E811" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F811" s="57" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G810" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H810" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan detail data aktivitas export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="811" ht="28" customHeight="1">
-      <c r="A811" s="55" t="inlineStr">
-        <is>
-          <t>71.8</t>
-        </is>
-      </c>
-      <c r="B811" s="56" t="inlineStr">
-        <is>
-          <t>Export Center</t>
-        </is>
-      </c>
-      <c r="C811" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Export</t>
-        </is>
-      </c>
-      <c r="D811" s="56" t="inlineStr">
-        <is>
-          <t>Mengunduh file data export yang tersedia</t>
-        </is>
-      </c>
-      <c r="E811" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F811" s="55" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
       <c r="G811" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada data dengan status Tersedia - Klik opsi Download</t>
+          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H811" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh file data export.</t>
+          <t>Berhasil menyimpan data pelaporan issue.</t>
         </is>
       </c>
     </row>
     <row r="812" ht="42" customHeight="1">
       <c r="A812" s="57" t="inlineStr">
         <is>
-          <t>72.1</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="B812" s="56" t="inlineStr">
@@ -34333,7 +34333,7 @@
       </c>
       <c r="D812" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Aktivitas Issue</t>
+          <t>Melihat detail pelaporan issue</t>
         </is>
       </c>
       <c r="E812" s="57" t="inlineStr">
@@ -34348,19 +34348,19 @@
       </c>
       <c r="G812" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H812" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="813" ht="28" customHeight="1">
       <c r="A813" s="57" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.6</t>
         </is>
       </c>
       <c r="B813" s="56" t="inlineStr">
@@ -34375,7 +34375,7 @@
       </c>
       <c r="D813" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Aktivitas Issue</t>
+          <t>Mengubah data pelaporan issue</t>
         </is>
       </c>
       <c r="E813" s="57" t="inlineStr">
@@ -34390,19 +34390,19 @@
       </c>
       <c r="G813" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
         </is>
       </c>
       <c r="H813" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menyimpan perubahan data issue.</t>
         </is>
       </c>
     </row>
     <row r="814" ht="28" customHeight="1">
       <c r="A814" s="57" t="inlineStr">
         <is>
-          <t>72.3</t>
+          <t>72.7</t>
         </is>
       </c>
       <c r="B814" s="56" t="inlineStr">
@@ -34417,7 +34417,7 @@
       </c>
       <c r="D814" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
+          <t>Menambahkan komentar pada detail aktivitas issue</t>
         </is>
       </c>
       <c r="E814" s="57" t="inlineStr">
@@ -34432,19 +34432,19 @@
       </c>
       <c r="G814" s="56" t="inlineStr">
         <is>
-          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
+          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
         </is>
       </c>
       <c r="H814" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menambahkan komentar pada detail issue.</t>
         </is>
       </c>
     </row>
     <row r="815" ht="56" customHeight="1">
       <c r="A815" s="57" t="inlineStr">
         <is>
-          <t>72.4</t>
+          <t>72.8</t>
         </is>
       </c>
       <c r="B815" s="56" t="inlineStr">
@@ -34459,7 +34459,7 @@
       </c>
       <c r="D815" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan pelaporan issue baru</t>
+          <t>Menghapus data pelaporan issue</t>
         </is>
       </c>
       <c r="E815" s="57" t="inlineStr">
@@ -34469,24 +34469,24 @@
       </c>
       <c r="F815" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G815" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
         </is>
       </c>
       <c r="H815" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data pelaporan issue.</t>
+          <t>Berhasil menghapus data issue.</t>
         </is>
       </c>
     </row>
     <row r="816" ht="56" customHeight="1">
       <c r="A816" s="57" t="inlineStr">
         <is>
-          <t>72.5</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B816" s="56" t="inlineStr">
@@ -34496,12 +34496,12 @@
       </c>
       <c r="C816" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D816" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail pelaporan issue</t>
+          <t>Membuka halaman Master Kategori Issue</t>
         </is>
       </c>
       <c r="E816" s="57" t="inlineStr">
@@ -34516,19 +34516,19 @@
       </c>
       <c r="G816" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="H816" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
         </is>
       </c>
     </row>
     <row r="817" ht="28" customHeight="1">
       <c r="A817" s="57" t="inlineStr">
         <is>
-          <t>72.6</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="B817" s="56" t="inlineStr">
@@ -34538,12 +34538,12 @@
       </c>
       <c r="C817" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D817" s="56" t="inlineStr">
         <is>
-          <t>Mengubah data pelaporan issue</t>
+          <t>Menambahkan kategori lain melalui pelaporan issue</t>
         </is>
       </c>
       <c r="E817" s="57" t="inlineStr">
@@ -34558,19 +34558,19 @@
       </c>
       <c r="G817" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
+          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H817" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data issue.</t>
+          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
         </is>
       </c>
     </row>
     <row r="818" ht="28" customHeight="1">
       <c r="A818" s="57" t="inlineStr">
         <is>
-          <t>72.7</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="B818" s="56" t="inlineStr">
@@ -34580,12 +34580,12 @@
       </c>
       <c r="C818" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D818" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan komentar pada detail aktivitas issue</t>
+          <t>Menambahkan data master kategori</t>
         </is>
       </c>
       <c r="E818" s="57" t="inlineStr">
@@ -34595,24 +34595,24 @@
       </c>
       <c r="F818" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G818" s="56" t="inlineStr">
         <is>
-          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
+          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
         </is>
       </c>
       <c r="H818" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan komentar pada detail issue.</t>
+          <t>Berhasil menyimpan data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="819" ht="42" customHeight="1">
       <c r="A819" s="57" t="inlineStr">
         <is>
-          <t>72.8</t>
+          <t>73.4</t>
         </is>
       </c>
       <c r="B819" s="56" t="inlineStr">
@@ -34622,12 +34622,12 @@
       </c>
       <c r="C819" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D819" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data pelaporan issue</t>
+          <t>Mencari data pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E819" s="57" t="inlineStr">
@@ -34642,19 +34642,19 @@
       </c>
       <c r="G819" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
+          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
         </is>
       </c>
       <c r="H819" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="820" ht="14" customHeight="1">
       <c r="A820" s="57" t="inlineStr">
         <is>
-          <t>73.1</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="B820" s="56" t="inlineStr">
@@ -34669,7 +34669,7 @@
       </c>
       <c r="D820" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Master Kategori Issue</t>
+          <t>Melihat detail data kategori pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E820" s="57" t="inlineStr">
@@ -34679,24 +34679,24 @@
       </c>
       <c r="F820" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G820" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H820" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
+          <t>Berhasil menampilkan modal detail kategori.</t>
         </is>
       </c>
     </row>
     <row r="821" ht="56" customHeight="1">
       <c r="A821" s="57" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>73.6</t>
         </is>
       </c>
       <c r="B821" s="56" t="inlineStr">
@@ -34711,7 +34711,7 @@
       </c>
       <c r="D821" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan kategori lain melalui pelaporan issue</t>
+          <t>Mengirim data kategori lain ke master kategori</t>
         </is>
       </c>
       <c r="E821" s="57" t="inlineStr">
@@ -34721,24 +34721,24 @@
       </c>
       <c r="F821" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G821" s="56" t="inlineStr">
         <is>
-          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
+          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
         </is>
       </c>
       <c r="H821" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
+          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="822" ht="56" customHeight="1">
       <c r="A822" s="57" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>73.7</t>
         </is>
       </c>
       <c r="B822" s="56" t="inlineStr">
@@ -34753,7 +34753,7 @@
       </c>
       <c r="D822" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan data master kategori</t>
+          <t>Mengirim data kategori lain ke master kategori secara massal</t>
         </is>
       </c>
       <c r="E822" s="57" t="inlineStr">
@@ -34763,24 +34763,24 @@
       </c>
       <c r="F822" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G822" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
+          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
         </is>
       </c>
       <c r="H822" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data master kategori.</t>
+          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="823" ht="56" customHeight="1">
       <c r="A823" s="57" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>73.8</t>
         </is>
       </c>
       <c r="B823" s="56" t="inlineStr">
@@ -34795,7 +34795,7 @@
       </c>
       <c r="D823" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori Lain</t>
+          <t>Mencari data pada List Kategori</t>
         </is>
       </c>
       <c r="E823" s="57" t="inlineStr">
@@ -34810,7 +34810,7 @@
       </c>
       <c r="G823" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
+          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
         </is>
       </c>
       <c r="H823" s="56" t="inlineStr">
@@ -34822,7 +34822,7 @@
     <row r="824" ht="14" customHeight="1">
       <c r="A824" s="57" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>73.9</t>
         </is>
       </c>
       <c r="B824" s="56" t="inlineStr">
@@ -34837,7 +34837,7 @@
       </c>
       <c r="D824" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail data kategori pada List Kategori Lain</t>
+          <t>Melihat dan mengubah data master kategori</t>
         </is>
       </c>
       <c r="E824" s="57" t="inlineStr">
@@ -34852,19 +34852,19 @@
       </c>
       <c r="G824" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
         </is>
       </c>
       <c r="H824" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan modal detail kategori.</t>
+          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="825" ht="14" customHeight="1">
       <c r="A825" s="57" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B825" s="56" t="inlineStr">
@@ -34874,12 +34874,12 @@
       </c>
       <c r="C825" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D825" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori</t>
+          <t>Membuka halaman Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E825" s="57" t="inlineStr">
@@ -34894,19 +34894,19 @@
       </c>
       <c r="G825" s="56" t="inlineStr">
         <is>
-          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="H825" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="826" ht="14" customHeight="1">
       <c r="A826" s="57" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B826" s="56" t="inlineStr">
@@ -34916,12 +34916,12 @@
       </c>
       <c r="C826" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D826" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori secara massal</t>
+          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E826" s="57" t="inlineStr">
@@ -34936,19 +34936,19 @@
       </c>
       <c r="G826" s="56" t="inlineStr">
         <is>
-          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
+          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
         </is>
       </c>
       <c r="H826" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="827" ht="42" customHeight="1">
       <c r="A827" s="57" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B827" s="56" t="inlineStr">
@@ -34958,12 +34958,12 @@
       </c>
       <c r="C827" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D827" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori</t>
+          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
         </is>
       </c>
       <c r="E827" s="57" t="inlineStr">
@@ -34973,24 +34973,24 @@
       </c>
       <c r="F827" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G827" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
+          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H827" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="828" ht="14" customHeight="1">
       <c r="A828" s="57" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B828" s="56" t="inlineStr">
@@ -35000,12 +35000,12 @@
       </c>
       <c r="C828" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D828" s="56" t="inlineStr">
         <is>
-          <t>Melihat dan mengubah data master kategori</t>
+          <t>Membuka halaman Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E828" s="57" t="inlineStr">
@@ -35015,24 +35015,24 @@
       </c>
       <c r="F828" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G828" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="H828" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
+          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="829" ht="56" customHeight="1">
       <c r="A829" s="57" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B829" s="56" t="inlineStr">
@@ -35042,12 +35042,12 @@
       </c>
       <c r="C829" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D829" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Issue</t>
+          <t>Melakukan filter data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E829" s="57" t="inlineStr">
@@ -35057,24 +35057,24 @@
       </c>
       <c r="F829" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G829" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
+          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H829" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="830" ht="28" customHeight="1">
       <c r="A830" s="57" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B830" s="56" t="inlineStr">
@@ -35084,12 +35084,12 @@
       </c>
       <c r="C830" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D830" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
+          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
         </is>
       </c>
       <c r="E830" s="57" t="inlineStr">
@@ -35104,19 +35104,19 @@
       </c>
       <c r="G830" s="56" t="inlineStr">
         <is>
-          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
+          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H830" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="831" ht="42" customHeight="1">
       <c r="A831" s="57" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B831" s="56" t="inlineStr">
@@ -35126,12 +35126,12 @@
       </c>
       <c r="C831" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D831" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
+          <t>Melihat detail report aktivitas issue</t>
         </is>
       </c>
       <c r="E831" s="57" t="inlineStr">
@@ -35146,7 +35146,7 @@
       </c>
       <c r="G831" s="56" t="inlineStr">
         <is>
-          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H831" s="56" t="inlineStr">
@@ -35158,7 +35158,7 @@
     <row r="832" ht="28" customHeight="1">
       <c r="A832" s="57" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B832" s="56" t="inlineStr">
@@ -35173,7 +35173,7 @@
       </c>
       <c r="D832" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Report Aktivitas Issue</t>
+          <t>Menghapus data report aktivitas issue secara massal</t>
         </is>
       </c>
       <c r="E832" s="57" t="inlineStr">
@@ -35183,24 +35183,24 @@
       </c>
       <c r="F832" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G832" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
+          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
         </is>
       </c>
       <c r="H832" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
+          <t>Berhasil menghapus data report aktivitas issue.</t>
         </is>
       </c>
     </row>
     <row r="833" ht="14" customHeight="1">
       <c r="A833" s="57" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B833" s="56" t="inlineStr">
@@ -35215,7 +35215,7 @@
       </c>
       <c r="D833" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Report Aktivitas Issue</t>
+          <t>Mengekspor data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E833" s="57" t="inlineStr">
@@ -35225,39 +35225,39 @@
       </c>
       <c r="F833" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G833" s="56" t="inlineStr">
         <is>
-          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H833" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="834" ht="14" customHeight="1">
       <c r="A834" s="57" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="B834" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C834" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D834" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E834" s="57" t="inlineStr">
@@ -35267,39 +35267,39 @@
       </c>
       <c r="F834" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G834" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="H834" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="835" ht="14" customHeight="1">
       <c r="A835" s="57" t="inlineStr">
         <is>
-          <t>75.4</t>
+          <t>76.2</t>
         </is>
       </c>
       <c r="B835" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C835" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D835" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail report aktivitas issue</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E835" s="57" t="inlineStr">
@@ -35309,39 +35309,39 @@
       </c>
       <c r="F835" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G835" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
         </is>
       </c>
       <c r="H835" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="836" ht="42" customHeight="1">
       <c r="A836" s="57" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>76.3</t>
         </is>
       </c>
       <c r="B836" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C836" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D836" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data report aktivitas issue secara massal</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E836" s="57" t="inlineStr">
@@ -35356,61 +35356,61 @@
       </c>
       <c r="G836" s="56" t="inlineStr">
         <is>
-          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H836" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data report aktivitas issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="837" ht="28" customHeight="1">
       <c r="A837" s="57" t="inlineStr">
         <is>
-          <t>75.6</t>
+          <t>76.4</t>
         </is>
       </c>
       <c r="B837" s="56" t="inlineStr">
         <is>
-          <t>Ticket Maintenance</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="C837" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D837" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data Report Aktivitas Issue</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E837" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F837" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G837" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H837" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="838" ht="28" customHeight="1">
       <c r="A838" s="57" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="B838" s="56" t="inlineStr">
@@ -35425,7 +35425,7 @@
       </c>
       <c r="D838" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E838" s="57" t="inlineStr">
@@ -35440,19 +35440,19 @@
       </c>
       <c r="G838" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H838" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="839" ht="70" customHeight="1">
       <c r="A839" s="57" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>76.6</t>
         </is>
       </c>
       <c r="B839" s="56" t="inlineStr">
@@ -35467,7 +35467,7 @@
       </c>
       <c r="D839" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E839" s="57" t="inlineStr">
@@ -35482,19 +35482,19 @@
       </c>
       <c r="G839" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H839" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="840" ht="28" customHeight="1">
       <c r="A840" s="57" t="inlineStr">
         <is>
-          <t>76.3</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="B840" s="56" t="inlineStr">
@@ -35509,12 +35509,12 @@
       </c>
       <c r="D840" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E840" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F840" s="57" t="inlineStr">
@@ -35524,19 +35524,19 @@
       </c>
       <c r="G840" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H840" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="841" ht="84" customHeight="1">
       <c r="A841" s="57" t="inlineStr">
         <is>
-          <t>76.4</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="B841" s="56" t="inlineStr">
@@ -35551,34 +35551,34 @@
       </c>
       <c r="D841" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E841" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F841" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G841" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H841" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="842" ht="28" customHeight="1">
       <c r="A842" s="57" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>77.1</t>
         </is>
       </c>
       <c r="B842" s="56" t="inlineStr">
@@ -35588,12 +35588,12 @@
       </c>
       <c r="C842" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D842" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E842" s="57" t="inlineStr">
@@ -35608,19 +35608,19 @@
       </c>
       <c r="G842" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="H842" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
     <row r="843" ht="28" customHeight="1">
       <c r="A843" s="57" t="inlineStr">
         <is>
-          <t>76.6</t>
+          <t>77.2</t>
         </is>
       </c>
       <c r="B843" s="56" t="inlineStr">
@@ -35630,12 +35630,12 @@
       </c>
       <c r="C843" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D843" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E843" s="57" t="inlineStr">
@@ -35650,19 +35650,19 @@
       </c>
       <c r="G843" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
         </is>
       </c>
       <c r="H843" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="844" ht="28" customHeight="1">
       <c r="A844" s="57" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="B844" s="56" t="inlineStr">
@@ -35672,17 +35672,17 @@
       </c>
       <c r="C844" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D844" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E844" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F844" s="57" t="inlineStr">
@@ -35692,19 +35692,19 @@
       </c>
       <c r="G844" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H844" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="845" ht="42" customHeight="1">
       <c r="A845" s="57" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="B845" s="56" t="inlineStr">
@@ -35714,39 +35714,39 @@
       </c>
       <c r="C845" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D845" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E845" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F845" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G845" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H845" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="846" ht="28" customHeight="1">
       <c r="A846" s="57" t="inlineStr">
         <is>
-          <t>77.1</t>
+          <t>77.5</t>
         </is>
       </c>
       <c r="B846" s="56" t="inlineStr">
@@ -35761,7 +35761,7 @@
       </c>
       <c r="D846" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E846" s="57" t="inlineStr">
@@ -35776,19 +35776,19 @@
       </c>
       <c r="G846" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H846" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="847" ht="14" customHeight="1">
       <c r="A847" s="57" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>77.6</t>
         </is>
       </c>
       <c r="B847" s="56" t="inlineStr">
@@ -35803,7 +35803,7 @@
       </c>
       <c r="D847" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E847" s="57" t="inlineStr">
@@ -35818,19 +35818,19 @@
       </c>
       <c r="G847" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H847" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="848" ht="14" customHeight="1">
       <c r="A848" s="57" t="inlineStr">
         <is>
-          <t>77.3</t>
+          <t>77.7</t>
         </is>
       </c>
       <c r="B848" s="56" t="inlineStr">
@@ -35845,12 +35845,12 @@
       </c>
       <c r="D848" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E848" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F848" s="57" t="inlineStr">
@@ -35860,19 +35860,19 @@
       </c>
       <c r="G848" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H848" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="849" ht="42" customHeight="1">
       <c r="A849" s="57" t="inlineStr">
         <is>
-          <t>77.4</t>
+          <t>77.8</t>
         </is>
       </c>
       <c r="B849" s="56" t="inlineStr">
@@ -35887,34 +35887,34 @@
       </c>
       <c r="D849" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E849" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F849" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G849" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H849" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="850" ht="28" customHeight="1">
       <c r="A850" s="57" t="inlineStr">
         <is>
-          <t>77.5</t>
+          <t>78.1</t>
         </is>
       </c>
       <c r="B850" s="56" t="inlineStr">
@@ -35924,12 +35924,12 @@
       </c>
       <c r="C850" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D850" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="E850" s="57" t="inlineStr">
@@ -35944,19 +35944,19 @@
       </c>
       <c r="G850" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="H850" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
         </is>
       </c>
     </row>
     <row r="851" ht="28" customHeight="1">
       <c r="A851" s="57" t="inlineStr">
         <is>
-          <t>77.6</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="B851" s="56" t="inlineStr">
@@ -35966,12 +35966,12 @@
       </c>
       <c r="C851" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D851" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E851" s="57" t="inlineStr">
@@ -35986,19 +35986,19 @@
       </c>
       <c r="G851" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
         </is>
       </c>
       <c r="H851" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="852" ht="28" customHeight="1">
       <c r="A852" s="57" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>78.3</t>
         </is>
       </c>
       <c r="B852" s="56" t="inlineStr">
@@ -36008,207 +36008,207 @@
       </c>
       <c r="C852" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
       <c r="D852" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E852" s="57" t="inlineStr">
         <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F852" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G852" s="56" t="inlineStr">
+        <is>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H852" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="853" ht="28" customHeight="1">
+      <c r="A853" s="58" t="inlineStr">
+        <is>
+          <t>79.1</t>
+        </is>
+      </c>
+      <c r="B853" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C853" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D853" s="59" t="inlineStr">
+        <is>
+          <t>Membuka halaman Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E853" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F853" s="58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G853" s="59" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
+        </is>
+      </c>
+      <c r="H853" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="854" ht="28" customHeight="1">
+      <c r="A854" s="58" t="inlineStr">
+        <is>
+          <t>79.2</t>
+        </is>
+      </c>
+      <c r="B854" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C854" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D854" s="59" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="E854" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F854" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G854" s="59" t="inlineStr">
+        <is>
+          <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
+        </is>
+      </c>
+      <c r="H854" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="855" ht="28" customHeight="1">
+      <c r="A855" s="58" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="B855" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C855" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D855" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E855" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F855" s="58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G855" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H855" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="856" ht="28" customHeight="1">
+      <c r="A856" s="58" t="inlineStr">
+        <is>
+          <t>79.4</t>
+        </is>
+      </c>
+      <c r="B856" s="59" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C856" s="59" t="inlineStr">
+        <is>
+          <t>Optimalisasi Database</t>
+        </is>
+      </c>
+      <c r="D856" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E856" s="58" t="inlineStr">
+        <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F852" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G852" s="56" t="inlineStr">
-        <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
-        </is>
-      </c>
-      <c r="H852" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="853" ht="28" customHeight="1">
-      <c r="A853" s="57" t="inlineStr">
-        <is>
-          <t>77.8</t>
-        </is>
-      </c>
-      <c r="B853" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C853" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="D853" s="56" t="inlineStr">
-        <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
-        </is>
-      </c>
-      <c r="E853" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F853" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G853" s="56" t="inlineStr">
-        <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
-        </is>
-      </c>
-      <c r="H853" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil mendownload file export.</t>
-        </is>
-      </c>
-    </row>
-    <row r="854" ht="28" customHeight="1">
-      <c r="A854" s="57" t="inlineStr">
-        <is>
-          <t>78.1</t>
-        </is>
-      </c>
-      <c r="B854" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C854" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D854" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="E854" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F854" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G854" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="H854" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="855" ht="28" customHeight="1">
-      <c r="A855" s="57" t="inlineStr">
-        <is>
-          <t>78.2</t>
-        </is>
-      </c>
-      <c r="B855" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C855" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D855" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
-        </is>
-      </c>
-      <c r="E855" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F855" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G855" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H855" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="856" ht="28" customHeight="1">
-      <c r="A856" s="57" t="inlineStr">
-        <is>
-          <t>78.3</t>
-        </is>
-      </c>
-      <c r="B856" s="56" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C856" s="56" t="inlineStr">
-        <is>
-          <t>Pengaturan Aktivitas Consumer</t>
-        </is>
-      </c>
-      <c r="D856" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
-        </is>
-      </c>
-      <c r="E856" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F856" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G856" s="56" t="inlineStr">
-        <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H856" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
+      <c r="F856" s="58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G856" s="59" t="inlineStr">
+        <is>
+          <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
+        </is>
+      </c>
+      <c r="H856" s="59" t="inlineStr">
+        <is>
+          <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
         </is>
       </c>
     </row>
     <row r="857" ht="28" customHeight="1">
       <c r="A857" s="58" t="inlineStr">
         <is>
-          <t>79.1</t>
+          <t>79.5</t>
         </is>
       </c>
       <c r="B857" s="59" t="inlineStr">
@@ -36223,7 +36223,7 @@
       </c>
       <c r="D857" s="59" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Optimalisasi Database</t>
+          <t>Mengekspor data tabel Optimalisasi Database</t>
         </is>
       </c>
       <c r="E857" s="58" t="inlineStr">
@@ -36233,188 +36233,24 @@
       </c>
       <c r="F857" s="58" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G857" s="59" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
+          <t>Klik button Export</t>
         </is>
       </c>
       <c r="H857" s="59" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
-        </is>
-      </c>
-    </row>
-    <row r="858" ht="28" customHeight="1">
-      <c r="A858" s="58" t="inlineStr">
-        <is>
-          <t>79.2</t>
-        </is>
-      </c>
-      <c r="B858" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C858" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D858" s="59" t="inlineStr">
-        <is>
-          <t>Melakukan filter data Dashboard Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="E858" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F858" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G858" s="59" t="inlineStr">
-        <is>
-          <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
-        </is>
-      </c>
-      <c r="H858" s="59" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="859" ht="28" customHeight="1">
-      <c r="A859" s="58" t="inlineStr">
-        <is>
-          <t>79.3</t>
-        </is>
-      </c>
-      <c r="B859" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C859" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D859" s="59" t="inlineStr">
-        <is>
-          <t>Mencari data pada tabel dengan keyword valid</t>
-        </is>
-      </c>
-      <c r="E859" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F859" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G859" s="59" t="inlineStr">
-        <is>
-          <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H859" s="59" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
-        </is>
-      </c>
-    </row>
-    <row r="860" ht="28" customHeight="1">
-      <c r="A860" s="58" t="inlineStr">
-        <is>
-          <t>79.4</t>
-        </is>
-      </c>
-      <c r="B860" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C860" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D860" s="59" t="inlineStr">
-        <is>
-          <t>Mencari data pada tabel dengan keyword tidak valid</t>
-        </is>
-      </c>
-      <c r="E860" s="58" t="inlineStr">
-        <is>
-          <t>Negative Case</t>
-        </is>
-      </c>
-      <c r="F860" s="58" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G860" s="59" t="inlineStr">
-        <is>
-          <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H860" s="59" t="inlineStr">
-        <is>
-          <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="861" ht="28" customHeight="1">
-      <c r="A861" s="58" t="inlineStr">
-        <is>
-          <t>79.5</t>
-        </is>
-      </c>
-      <c r="B861" s="59" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C861" s="59" t="inlineStr">
-        <is>
-          <t>Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="D861" s="59" t="inlineStr">
-        <is>
-          <t>Mengekspor data tabel Optimalisasi Database</t>
-        </is>
-      </c>
-      <c r="E861" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F861" s="58" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G861" s="59" t="inlineStr">
-        <is>
-          <t>Klik button Export</t>
-        </is>
-      </c>
-      <c r="H861" s="59" t="inlineStr">
-        <is>
           <t>Berhasil mengunduh file data tabel dalam format Excel (.xlsx).</t>
         </is>
       </c>
     </row>
+    <row r="858" ht="28" customHeight="1"/>
+    <row r="859" ht="28" customHeight="1"/>
+    <row r="860" ht="28" customHeight="1"/>
+    <row r="861" ht="28" customHeight="1"/>
     <row r="862" ht="28" customHeight="1"/>
     <row r="863" ht="28" customHeight="1"/>
     <row r="864" ht="28" customHeight="1"/>

</xml_diff>

<commit_message>
fix(web): add missing TCs to Modul 69 Export Center - Riwayat Export to reach 17 TCs (match senior)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z883"/>
+  <dimension ref="A1:Z892"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34904,723 +34904,723 @@
       </c>
     </row>
     <row r="826" ht="14" customHeight="1">
-      <c r="A826" s="55" t="inlineStr">
+      <c r="A826" s="60" t="inlineStr">
+        <is>
+          <t>69.9</t>
+        </is>
+      </c>
+      <c r="B826" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C826" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D826" s="59" t="inlineStr">
+        <is>
+          <t>Mengunduh data yang sudah di approve</t>
+        </is>
+      </c>
+      <c r="E826" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F826" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G826" s="59" t="inlineStr">
+        <is>
+          <t>Klik button download pada data yang statusnya disetujui</t>
+        </is>
+      </c>
+      <c r="H826" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil mengunduh data export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="827" ht="42" customHeight="1">
+      <c r="A827" s="60" t="inlineStr">
+        <is>
+          <t>69.10</t>
+        </is>
+      </c>
+      <c r="B827" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C827" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D827" s="59" t="inlineStr">
+        <is>
+          <t>Membuka dokumen hasil download</t>
+        </is>
+      </c>
+      <c r="E827" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F827" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G827" s="59" t="inlineStr">
+        <is>
+          <t>Extract file zip hasil download menggunakan password yang dikirim ke email user</t>
+        </is>
+      </c>
+      <c r="H827" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil membuka file hasil download.</t>
+        </is>
+      </c>
+    </row>
+    <row r="828" ht="14" customHeight="1">
+      <c r="A828" s="60" t="inlineStr">
+        <is>
+          <t>69.11</t>
+        </is>
+      </c>
+      <c r="B828" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C828" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D828" s="59" t="inlineStr">
+        <is>
+          <t>Melakukan filter data pada tab Riwayat Export</t>
+        </is>
+      </c>
+      <c r="E828" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F828" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G828" s="59" t="inlineStr">
+        <is>
+          <t>Klik button filter - pilih modul, export status, dan rentang tanggal request - klik terapkan filter</t>
+        </is>
+      </c>
+      <c r="H828" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan data sesuai filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="829" ht="56" customHeight="1">
+      <c r="A829" s="60" t="inlineStr">
+        <is>
+          <t>69.12</t>
+        </is>
+      </c>
+      <c r="B829" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C829" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D829" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada kolom pencarian</t>
+        </is>
+      </c>
+      <c r="E829" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F829" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G829" s="59" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada kolom pencarian</t>
+        </is>
+      </c>
+      <c r="H829" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan data sesuai kata kunci pencarian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="830" ht="28" customHeight="1">
+      <c r="A830" s="60" t="inlineStr">
+        <is>
+          <t>69.13</t>
+        </is>
+      </c>
+      <c r="B830" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C830" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D830" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data kata kunci salah</t>
+        </is>
+      </c>
+      <c r="E830" s="59" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F830" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G830" s="59" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada kolom pencarian</t>
+        </is>
+      </c>
+      <c r="H830" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan keterangan data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="831" ht="42" customHeight="1">
+      <c r="A831" s="60" t="inlineStr">
+        <is>
+          <t>69.14</t>
+        </is>
+      </c>
+      <c r="B831" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C831" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D831" s="59" t="inlineStr">
+        <is>
+          <t>Melakukan filter data pada tab Semua Request</t>
+        </is>
+      </c>
+      <c r="E831" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F831" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G831" s="59" t="inlineStr">
+        <is>
+          <t>Buka tab Semua Request - Klik button filter - pilih filter - klik terapkan filter</t>
+        </is>
+      </c>
+      <c r="H831" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan data sesuai filter yang dipilih pada tab Semua Request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="832" ht="28" customHeight="1">
+      <c r="A832" s="60" t="inlineStr">
+        <is>
+          <t>69.15</t>
+        </is>
+      </c>
+      <c r="B832" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C832" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D832" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data pada kolom pencarian tab Semua Request</t>
+        </is>
+      </c>
+      <c r="E832" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F832" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G832" s="59" t="inlineStr">
+        <is>
+          <t>Buka tab Semua Request - Input keyword pada kolom pencarian</t>
+        </is>
+      </c>
+      <c r="H832" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan data sesuai kata kunci pada tab Semua Request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="833" ht="14" customHeight="1">
+      <c r="A833" s="60" t="inlineStr">
+        <is>
+          <t>69.16</t>
+        </is>
+      </c>
+      <c r="B833" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C833" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D833" s="59" t="inlineStr">
+        <is>
+          <t>Mencari data kata kunci salah tab Semua Request</t>
+        </is>
+      </c>
+      <c r="E833" s="59" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F833" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G833" s="59" t="inlineStr">
+        <is>
+          <t>Buka tab Semua Request - Input keyword tidak valid pada kolom pencarian</t>
+        </is>
+      </c>
+      <c r="H833" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Menampilkan keterangan data tidak ditemukan pada tab Semua Request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="834" ht="14" customHeight="1">
+      <c r="A834" s="60" t="inlineStr">
+        <is>
+          <t>69.17</t>
+        </is>
+      </c>
+      <c r="B834" s="59" t="inlineStr">
+        <is>
+          <t>Export Center</t>
+        </is>
+      </c>
+      <c r="C834" s="59" t="inlineStr">
+        <is>
+          <t>Riwayat Export</t>
+        </is>
+      </c>
+      <c r="D834" s="59" t="inlineStr">
+        <is>
+          <t>Validasi card menunggu approval dengan data table</t>
+        </is>
+      </c>
+      <c r="E834" s="59" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F834" s="60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G834" s="59" t="inlineStr">
+        <is>
+          <t>Cocokkan jumlah data pada card menunggu approval dengan jumlah baris data di table</t>
+        </is>
+      </c>
+      <c r="H834" s="59" t="inlineStr">
+        <is>
+          <t>Berhasil Jumlah data pada card dan table sesuai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="835" ht="14" customHeight="1">
+      <c r="A835" s="55" t="inlineStr">
         <is>
           <t>70.1</t>
         </is>
       </c>
-      <c r="B826" s="56" t="inlineStr">
+      <c r="B835" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C826" s="56" t="inlineStr">
+      <c r="C835" s="56" t="inlineStr">
         <is>
           <t>Persetujuan Export</t>
         </is>
       </c>
-      <c r="D826" s="56" t="inlineStr">
+      <c r="D835" s="56" t="inlineStr">
         <is>
           <t>Membuka halaman Persetujuan Export</t>
         </is>
       </c>
-      <c r="E826" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F826" s="55" t="inlineStr">
+      <c r="E835" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F835" s="55" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G826" s="56" t="inlineStr">
+      <c r="G835" s="56" t="inlineStr">
         <is>
           <t>Klik menu Export Center - Klik submenu Persetujuan Export</t>
         </is>
       </c>
-      <c r="H826" s="56" t="inlineStr">
+      <c r="H835" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan halaman Persetujuan Export.</t>
         </is>
       </c>
     </row>
-    <row r="827" ht="42" customHeight="1">
-      <c r="A827" s="55" t="inlineStr">
+    <row r="836" ht="42" customHeight="1">
+      <c r="A836" s="55" t="inlineStr">
         <is>
           <t>70.2</t>
         </is>
       </c>
-      <c r="B827" s="56" t="inlineStr">
+      <c r="B836" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C827" s="56" t="inlineStr">
+      <c r="C836" s="56" t="inlineStr">
         <is>
           <t>Persetujuan Export</t>
         </is>
       </c>
-      <c r="D827" s="56" t="inlineStr">
+      <c r="D836" s="56" t="inlineStr">
         <is>
           <t>Mencari data persetujuan export dengan kata kunci valid</t>
         </is>
       </c>
-      <c r="E827" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F827" s="55" t="inlineStr">
+      <c r="E836" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F836" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G827" s="56" t="inlineStr">
+      <c r="G836" s="56" t="inlineStr">
         <is>
           <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
-      <c r="H827" s="56" t="inlineStr">
+      <c r="H836" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan data persetujuan export yang dicari.</t>
         </is>
       </c>
     </row>
-    <row r="828" ht="14" customHeight="1">
-      <c r="A828" s="55" t="inlineStr">
+    <row r="837" ht="28" customHeight="1">
+      <c r="A837" s="55" t="inlineStr">
         <is>
           <t>70.3</t>
         </is>
       </c>
-      <c r="B828" s="56" t="inlineStr">
+      <c r="B837" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C828" s="56" t="inlineStr">
+      <c r="C837" s="56" t="inlineStr">
         <is>
           <t>Persetujuan Export</t>
         </is>
       </c>
-      <c r="D828" s="56" t="inlineStr">
+      <c r="D837" s="56" t="inlineStr">
         <is>
           <t>Mencari data persetujuan export dengan kata kunci tidak valid</t>
         </is>
       </c>
-      <c r="E828" s="56" t="inlineStr">
+      <c r="E837" s="56" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F828" s="55" t="inlineStr">
+      <c r="F837" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G828" s="56" t="inlineStr">
+      <c r="G837" s="56" t="inlineStr">
         <is>
           <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
-      <c r="H828" s="56" t="inlineStr">
+      <c r="H837" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
-    <row r="829" ht="56" customHeight="1">
-      <c r="A829" s="55" t="inlineStr">
+    <row r="838" ht="28" customHeight="1">
+      <c r="A838" s="55" t="inlineStr">
         <is>
           <t>70.4</t>
         </is>
       </c>
-      <c r="B829" s="56" t="inlineStr">
+      <c r="B838" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C829" s="56" t="inlineStr">
+      <c r="C838" s="56" t="inlineStr">
         <is>
           <t>Persetujuan Export</t>
         </is>
       </c>
-      <c r="D829" s="56" t="inlineStr">
+      <c r="D838" s="56" t="inlineStr">
         <is>
           <t>Melihat data persetujuan export berdasarkan status</t>
         </is>
       </c>
-      <c r="E829" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F829" s="55" t="inlineStr">
+      <c r="E838" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F838" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G829" s="56" t="inlineStr">
+      <c r="G838" s="56" t="inlineStr">
         <is>
           <t>Pada halaman Persetujuan Export, klik salah satu tab status</t>
         </is>
       </c>
-      <c r="H829" s="56" t="inlineStr">
+      <c r="H838" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan daftar data persetujuan export sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="830" ht="28" customHeight="1">
-      <c r="A830" s="55" t="inlineStr">
+    <row r="839" ht="70" customHeight="1">
+      <c r="A839" s="55" t="inlineStr">
         <is>
           <t>71.1</t>
         </is>
       </c>
-      <c r="B830" s="56" t="inlineStr">
+      <c r="B839" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C830" s="56" t="inlineStr">
+      <c r="C839" s="56" t="inlineStr">
         <is>
           <t>Aktivitas Export</t>
         </is>
       </c>
-      <c r="D830" s="56" t="inlineStr">
+      <c r="D839" s="56" t="inlineStr">
         <is>
           <t>Membuka halaman Aktivitas Export</t>
         </is>
       </c>
-      <c r="E830" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F830" s="55" t="inlineStr">
+      <c r="E839" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F839" s="55" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G830" s="56" t="inlineStr">
+      <c r="G839" s="56" t="inlineStr">
         <is>
           <t>Klik menu Export Center - Klik submenu Aktivitas Export</t>
         </is>
       </c>
-      <c r="H830" s="56" t="inlineStr">
+      <c r="H839" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan halaman Aktivitas Export.</t>
         </is>
       </c>
     </row>
-    <row r="831" ht="42" customHeight="1">
-      <c r="A831" s="55" t="inlineStr">
+    <row r="840" ht="28" customHeight="1">
+      <c r="A840" s="55" t="inlineStr">
         <is>
           <t>71.2</t>
         </is>
       </c>
-      <c r="B831" s="56" t="inlineStr">
+      <c r="B840" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C831" s="56" t="inlineStr">
+      <c r="C840" s="56" t="inlineStr">
         <is>
           <t>Aktivitas Export</t>
         </is>
       </c>
-      <c r="D831" s="56" t="inlineStr">
+      <c r="D840" s="56" t="inlineStr">
         <is>
           <t>Mencari data aktivitas export dengan kata kunci valid</t>
         </is>
       </c>
-      <c r="E831" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F831" s="55" t="inlineStr">
+      <c r="E840" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F840" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G831" s="56" t="inlineStr">
+      <c r="G840" s="56" t="inlineStr">
         <is>
           <t>Masukkan kata kunci valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
-      <c r="H831" s="56" t="inlineStr">
+      <c r="H840" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan data aktivitas export yang dicari.</t>
         </is>
       </c>
     </row>
-    <row r="832" ht="28" customHeight="1">
-      <c r="A832" s="55" t="inlineStr">
+    <row r="841" ht="84" customHeight="1">
+      <c r="A841" s="55" t="inlineStr">
         <is>
           <t>71.3</t>
         </is>
       </c>
-      <c r="B832" s="56" t="inlineStr">
+      <c r="B841" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C832" s="56" t="inlineStr">
+      <c r="C841" s="56" t="inlineStr">
         <is>
           <t>Aktivitas Export</t>
         </is>
       </c>
-      <c r="D832" s="56" t="inlineStr">
+      <c r="D841" s="56" t="inlineStr">
         <is>
           <t>Mencari data aktivitas export dengan kata kunci tidak valid</t>
         </is>
       </c>
-      <c r="E832" s="56" t="inlineStr">
+      <c r="E841" s="56" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F832" s="55" t="inlineStr">
+      <c r="F841" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G832" s="56" t="inlineStr">
+      <c r="G841" s="56" t="inlineStr">
         <is>
           <t>Masukkan kata kunci tidak valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
-      <c r="H832" s="56" t="inlineStr">
+      <c r="H841" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
-    <row r="833" ht="14" customHeight="1">
-      <c r="A833" s="55" t="inlineStr">
+    <row r="842" ht="28" customHeight="1">
+      <c r="A842" s="55" t="inlineStr">
         <is>
           <t>71.4</t>
         </is>
       </c>
-      <c r="B833" s="56" t="inlineStr">
+      <c r="B842" s="56" t="inlineStr">
         <is>
           <t>Export Center</t>
         </is>
       </c>
-      <c r="C833" s="56" t="inlineStr">
+      <c r="C842" s="56" t="inlineStr">
         <is>
           <t>Aktivitas Export</t>
         </is>
       </c>
-      <c r="D833" s="56" t="inlineStr">
+      <c r="D842" s="56" t="inlineStr">
         <is>
           <t>Melihat data aktivitas export berdasarkan status</t>
         </is>
       </c>
-      <c r="E833" s="56" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F833" s="55" t="inlineStr">
+      <c r="E842" s="56" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F842" s="55" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G833" s="56" t="inlineStr">
+      <c r="G842" s="56" t="inlineStr">
         <is>
           <t>Pada halaman Aktivitas Export, klik salah satu tab status</t>
         </is>
       </c>
-      <c r="H833" s="56" t="inlineStr">
+      <c r="H842" s="56" t="inlineStr">
         <is>
           <t>Berhasil menampilkan daftar data aktivitas export sesuai status yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="834" ht="14" customHeight="1">
-      <c r="A834" s="57" t="inlineStr">
-        <is>
-          <t>72.1</t>
-        </is>
-      </c>
-      <c r="B834" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C834" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D834" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="E834" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F834" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G834" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="H834" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="835" ht="14" customHeight="1">
-      <c r="A835" s="57" t="inlineStr">
-        <is>
-          <t>72.2</t>
-        </is>
-      </c>
-      <c r="B835" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C835" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D835" s="56" t="inlineStr">
-        <is>
-          <t>Melakukan filter data Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="E835" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F835" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G835" s="56" t="inlineStr">
-        <is>
-          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
-        </is>
-      </c>
-      <c r="H835" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
-        </is>
-      </c>
-    </row>
-    <row r="836" ht="42" customHeight="1">
-      <c r="A836" s="57" t="inlineStr">
-        <is>
-          <t>72.3</t>
-        </is>
-      </c>
-      <c r="B836" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C836" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D836" s="56" t="inlineStr">
-        <is>
-          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
-        </is>
-      </c>
-      <c r="E836" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F836" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G836" s="56" t="inlineStr">
-        <is>
-          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
-        </is>
-      </c>
-      <c r="H836" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
-        </is>
-      </c>
-    </row>
-    <row r="837" ht="28" customHeight="1">
-      <c r="A837" s="57" t="inlineStr">
-        <is>
-          <t>72.4</t>
-        </is>
-      </c>
-      <c r="B837" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C837" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D837" s="56" t="inlineStr">
-        <is>
-          <t>Menambahkan pelaporan issue baru</t>
-        </is>
-      </c>
-      <c r="E837" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F837" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G837" s="56" t="inlineStr">
-        <is>
-          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
-        </is>
-      </c>
-      <c r="H837" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan data pelaporan issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="838" ht="28" customHeight="1">
-      <c r="A838" s="57" t="inlineStr">
-        <is>
-          <t>72.5</t>
-        </is>
-      </c>
-      <c r="B838" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C838" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D838" s="56" t="inlineStr">
-        <is>
-          <t>Melihat detail pelaporan issue</t>
-        </is>
-      </c>
-      <c r="E838" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F838" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G838" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
-        </is>
-      </c>
-      <c r="H838" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="839" ht="70" customHeight="1">
-      <c r="A839" s="57" t="inlineStr">
-        <is>
-          <t>72.6</t>
-        </is>
-      </c>
-      <c r="B839" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C839" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D839" s="56" t="inlineStr">
-        <is>
-          <t>Mengubah data pelaporan issue</t>
-        </is>
-      </c>
-      <c r="E839" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F839" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G839" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
-        </is>
-      </c>
-      <c r="H839" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menyimpan perubahan data issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="840" ht="28" customHeight="1">
-      <c r="A840" s="57" t="inlineStr">
-        <is>
-          <t>72.7</t>
-        </is>
-      </c>
-      <c r="B840" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C840" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D840" s="56" t="inlineStr">
-        <is>
-          <t>Menambahkan komentar pada detail aktivitas issue</t>
-        </is>
-      </c>
-      <c r="E840" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F840" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G840" s="56" t="inlineStr">
-        <is>
-          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
-        </is>
-      </c>
-      <c r="H840" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menambahkan komentar pada detail issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="841" ht="84" customHeight="1">
-      <c r="A841" s="57" t="inlineStr">
-        <is>
-          <t>72.8</t>
-        </is>
-      </c>
-      <c r="B841" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C841" s="56" t="inlineStr">
-        <is>
-          <t>Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D841" s="56" t="inlineStr">
-        <is>
-          <t>Menghapus data pelaporan issue</t>
-        </is>
-      </c>
-      <c r="E841" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F841" s="57" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G841" s="56" t="inlineStr">
-        <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
-        </is>
-      </c>
-      <c r="H841" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menghapus data issue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="842" ht="28" customHeight="1">
-      <c r="A842" s="57" t="inlineStr">
-        <is>
-          <t>73.1</t>
-        </is>
-      </c>
-      <c r="B842" s="56" t="inlineStr">
-        <is>
-          <t>Ticket Maintenance</t>
-        </is>
-      </c>
-      <c r="C842" s="56" t="inlineStr">
-        <is>
-          <t>Kategori Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="D842" s="56" t="inlineStr">
-        <is>
-          <t>Membuka halaman Master Kategori Issue</t>
-        </is>
-      </c>
-      <c r="E842" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F842" s="57" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G842" s="56" t="inlineStr">
-        <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
-        </is>
-      </c>
-      <c r="H842" s="56" t="inlineStr">
-        <is>
-          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
         </is>
       </c>
     </row>
     <row r="843" ht="28" customHeight="1">
       <c r="A843" s="57" t="inlineStr">
         <is>
-          <t>73.2</t>
+          <t>72.1</t>
         </is>
       </c>
       <c r="B843" s="56" t="inlineStr">
@@ -35630,12 +35630,12 @@
       </c>
       <c r="C843" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D843" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan kategori lain melalui pelaporan issue</t>
+          <t>Membuka halaman Aktivitas Issue</t>
         </is>
       </c>
       <c r="E843" s="57" t="inlineStr">
@@ -35645,24 +35645,24 @@
       </c>
       <c r="F843" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G843" s="56" t="inlineStr">
         <is>
-          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Aktivitas Issue</t>
         </is>
       </c>
       <c r="H843" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
+          <t>Berhasil menampilkan halaman Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="844" ht="28" customHeight="1">
       <c r="A844" s="57" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>72.2</t>
         </is>
       </c>
       <c r="B844" s="56" t="inlineStr">
@@ -35672,12 +35672,12 @@
       </c>
       <c r="C844" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D844" s="56" t="inlineStr">
         <is>
-          <t>Menambahkan data master kategori</t>
+          <t>Melakukan filter data Aktivitas Issue</t>
         </is>
       </c>
       <c r="E844" s="57" t="inlineStr">
@@ -35687,24 +35687,24 @@
       </c>
       <c r="F844" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G844" s="56" t="inlineStr">
         <is>
-          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
+          <t>Klik tab Filter 1 - Pilih Kategori, Status, dan Platform - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H844" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data master kategori.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="845" ht="42" customHeight="1">
       <c r="A845" s="57" t="inlineStr">
         <is>
-          <t>73.4</t>
+          <t>72.3</t>
         </is>
       </c>
       <c r="B845" s="56" t="inlineStr">
@@ -35714,12 +35714,12 @@
       </c>
       <c r="C845" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D845" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori Lain</t>
+          <t>Mencari data Aktivitas Issue dengan keyword valid</t>
         </is>
       </c>
       <c r="E845" s="57" t="inlineStr">
@@ -35734,7 +35734,7 @@
       </c>
       <c r="G845" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
+          <t>Klik tab Filter 2 - Input keyword valid pada Search Bar - Klik button Cari</t>
         </is>
       </c>
       <c r="H845" s="56" t="inlineStr">
@@ -35746,7 +35746,7 @@
     <row r="846" ht="28" customHeight="1">
       <c r="A846" s="57" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>72.4</t>
         </is>
       </c>
       <c r="B846" s="56" t="inlineStr">
@@ -35756,12 +35756,12 @@
       </c>
       <c r="C846" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D846" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail data kategori pada List Kategori Lain</t>
+          <t>Menambahkan pelaporan issue baru</t>
         </is>
       </c>
       <c r="E846" s="57" t="inlineStr">
@@ -35771,24 +35771,24 @@
       </c>
       <c r="F846" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G846" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
+          <t>Klik button + Registrasi Issue - Input seluruh field mandatory pada modal - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H846" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan modal detail kategori.</t>
+          <t>Berhasil menyimpan data pelaporan issue.</t>
         </is>
       </c>
     </row>
     <row r="847" ht="14" customHeight="1">
       <c r="A847" s="57" t="inlineStr">
         <is>
-          <t>73.6</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="B847" s="56" t="inlineStr">
@@ -35798,12 +35798,12 @@
       </c>
       <c r="C847" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D847" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori</t>
+          <t>Melihat detail pelaporan issue</t>
         </is>
       </c>
       <c r="E847" s="57" t="inlineStr">
@@ -35818,19 +35818,19 @@
       </c>
       <c r="G847" s="56" t="inlineStr">
         <is>
-          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H847" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="848" ht="14" customHeight="1">
       <c r="A848" s="57" t="inlineStr">
         <is>
-          <t>73.7</t>
+          <t>72.6</t>
         </is>
       </c>
       <c r="B848" s="56" t="inlineStr">
@@ -35840,12 +35840,12 @@
       </c>
       <c r="C848" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D848" s="56" t="inlineStr">
         <is>
-          <t>Mengirim data kategori lain ke master kategori secara massal</t>
+          <t>Mengubah data pelaporan issue</t>
         </is>
       </c>
       <c r="E848" s="57" t="inlineStr">
@@ -35860,19 +35860,19 @@
       </c>
       <c r="G848" s="56" t="inlineStr">
         <is>
-          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Edit - Ubah data issue - Klik button Simpan</t>
         </is>
       </c>
       <c r="H848" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
+          <t>Berhasil menyimpan perubahan data issue.</t>
         </is>
       </c>
     </row>
     <row r="849" ht="42" customHeight="1">
       <c r="A849" s="57" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>72.7</t>
         </is>
       </c>
       <c r="B849" s="56" t="inlineStr">
@@ -35882,12 +35882,12 @@
       </c>
       <c r="C849" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D849" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada List Kategori</t>
+          <t>Menambahkan komentar pada detail aktivitas issue</t>
         </is>
       </c>
       <c r="E849" s="57" t="inlineStr">
@@ -35902,19 +35902,19 @@
       </c>
       <c r="G849" s="56" t="inlineStr">
         <is>
-          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
+          <t>Buka halaman detail issue - Masukkan komentar pada kolom komentar - Klik button Kirim</t>
         </is>
       </c>
       <c r="H849" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menambahkan komentar pada detail issue.</t>
         </is>
       </c>
     </row>
     <row r="850" ht="28" customHeight="1">
       <c r="A850" s="57" t="inlineStr">
         <is>
-          <t>73.9</t>
+          <t>72.8</t>
         </is>
       </c>
       <c r="B850" s="56" t="inlineStr">
@@ -35924,12 +35924,12 @@
       </c>
       <c r="C850" s="56" t="inlineStr">
         <is>
-          <t>Kategori Aktivitas Issue</t>
+          <t>Aktivitas Issue</t>
         </is>
       </c>
       <c r="D850" s="56" t="inlineStr">
         <is>
-          <t>Melihat dan mengubah data master kategori</t>
+          <t>Menghapus data pelaporan issue</t>
         </is>
       </c>
       <c r="E850" s="57" t="inlineStr">
@@ -35944,19 +35944,19 @@
       </c>
       <c r="G850" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Hapus - Klik button Konfirmasi</t>
         </is>
       </c>
       <c r="H850" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
+          <t>Berhasil menghapus data issue.</t>
         </is>
       </c>
     </row>
     <row r="851" ht="28" customHeight="1">
       <c r="A851" s="57" t="inlineStr">
         <is>
-          <t>74.1</t>
+          <t>73.1</t>
         </is>
       </c>
       <c r="B851" s="56" t="inlineStr">
@@ -35966,12 +35966,12 @@
       </c>
       <c r="C851" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D851" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Issue</t>
+          <t>Membuka halaman Master Kategori Issue</t>
         </is>
       </c>
       <c r="E851" s="57" t="inlineStr">
@@ -35986,19 +35986,19 @@
       </c>
       <c r="G851" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="H851" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
+          <t>Berhasil menampilkan halaman Master Kategori Issue.</t>
         </is>
       </c>
     </row>
     <row r="852" ht="28" customHeight="1">
       <c r="A852" s="57" t="inlineStr">
         <is>
-          <t>74.2</t>
+          <t>73.2</t>
         </is>
       </c>
       <c r="B852" s="56" t="inlineStr">
@@ -36008,12 +36008,12 @@
       </c>
       <c r="C852" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D852" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
+          <t>Menambahkan kategori lain melalui pelaporan issue</t>
         </is>
       </c>
       <c r="E852" s="57" t="inlineStr">
@@ -36028,19 +36028,19 @@
       </c>
       <c r="G852" s="56" t="inlineStr">
         <is>
-          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
+          <t>Buka form Buat Pelaporan Issue - Pilih Kategori Others - Masukkan Nama Kategori Lain dan Remark - Klik button Registrasi Issue</t>
         </is>
       </c>
       <c r="H852" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menambahkan data kategori baru ke List Kategori Lain.</t>
         </is>
       </c>
     </row>
     <row r="853" ht="28" customHeight="1">
       <c r="A853" s="57" t="inlineStr">
         <is>
-          <t>74.3</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="B853" s="56" t="inlineStr">
@@ -36050,12 +36050,12 @@
       </c>
       <c r="C853" s="56" t="inlineStr">
         <is>
-          <t>Dashboard Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D853" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
+          <t>Menambahkan data master kategori</t>
         </is>
       </c>
       <c r="E853" s="57" t="inlineStr">
@@ -36070,19 +36070,19 @@
       </c>
       <c r="G853" s="56" t="inlineStr">
         <is>
-          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
+          <t>Klik button + Add Kategori - Input seluruh field mandatory pada modal - Klik button Save</t>
         </is>
       </c>
       <c r="H853" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil menyimpan data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="854" ht="28" customHeight="1">
       <c r="A854" s="57" t="inlineStr">
         <is>
-          <t>75.1</t>
+          <t>73.4</t>
         </is>
       </c>
       <c r="B854" s="56" t="inlineStr">
@@ -36092,12 +36092,12 @@
       </c>
       <c r="C854" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D854" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Report Aktivitas Issue</t>
+          <t>Mencari data pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E854" s="57" t="inlineStr">
@@ -36107,24 +36107,24 @@
       </c>
       <c r="F854" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G854" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
+          <t>Input kata kunci pada field Cari Data List Kategori Lain - Klik icon search</t>
         </is>
       </c>
       <c r="H854" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="855" ht="28" customHeight="1">
       <c r="A855" s="57" t="inlineStr">
         <is>
-          <t>75.2</t>
+          <t>73.5</t>
         </is>
       </c>
       <c r="B855" s="56" t="inlineStr">
@@ -36134,12 +36134,12 @@
       </c>
       <c r="C855" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D855" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Report Aktivitas Issue</t>
+          <t>Melihat detail data kategori pada List Kategori Lain</t>
         </is>
       </c>
       <c r="E855" s="57" t="inlineStr">
@@ -36154,19 +36154,19 @@
       </c>
       <c r="G855" s="56" t="inlineStr">
         <is>
-          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori Lain - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H855" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan modal detail kategori.</t>
         </is>
       </c>
     </row>
     <row r="856" ht="28" customHeight="1">
       <c r="A856" s="57" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>73.6</t>
         </is>
       </c>
       <c r="B856" s="56" t="inlineStr">
@@ -36176,12 +36176,12 @@
       </c>
       <c r="C856" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D856" s="56" t="inlineStr">
         <is>
-          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
+          <t>Mengirim data kategori lain ke master kategori</t>
         </is>
       </c>
       <c r="E856" s="57" t="inlineStr">
@@ -36191,24 +36191,24 @@
       </c>
       <c r="F856" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G856" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
+          <t>Klik button Send to Master pada baris data - Pilih Role dan PIC - Klik button Save</t>
         </is>
       </c>
       <c r="H856" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mengirim data kategori lain ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="857" ht="28" customHeight="1">
       <c r="A857" s="57" t="inlineStr">
         <is>
-          <t>75.4</t>
+          <t>73.7</t>
         </is>
       </c>
       <c r="B857" s="56" t="inlineStr">
@@ -36218,12 +36218,12 @@
       </c>
       <c r="C857" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D857" s="56" t="inlineStr">
         <is>
-          <t>Melihat detail report aktivitas issue</t>
+          <t>Mengirim data kategori lain ke master kategori secara massal</t>
         </is>
       </c>
       <c r="E857" s="57" t="inlineStr">
@@ -36233,24 +36233,24 @@
       </c>
       <c r="F857" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G857" s="56" t="inlineStr">
         <is>
-          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
+          <t>Checklist data pada List Kategori Lain - Klik button Bulk Send to Master</t>
         </is>
       </c>
       <c r="H857" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman detail issue.</t>
+          <t>Berhasil mengirim beberapa kategori lain terpilih ke master kategori.</t>
         </is>
       </c>
     </row>
     <row r="858" ht="28" customHeight="1">
       <c r="A858" s="57" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>73.8</t>
         </is>
       </c>
       <c r="B858" s="56" t="inlineStr">
@@ -36260,12 +36260,12 @@
       </c>
       <c r="C858" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D858" s="56" t="inlineStr">
         <is>
-          <t>Menghapus data report aktivitas issue secara massal</t>
+          <t>Mencari data pada List Kategori</t>
         </is>
       </c>
       <c r="E858" s="57" t="inlineStr">
@@ -36280,19 +36280,19 @@
       </c>
       <c r="G858" s="56" t="inlineStr">
         <is>
-          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
+          <t>Input kata kunci pada field Cari Data List Kategori - Klik icon search</t>
         </is>
       </c>
       <c r="H858" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data report aktivitas issue.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="859" ht="28" customHeight="1">
       <c r="A859" s="57" t="inlineStr">
         <is>
-          <t>75.6</t>
+          <t>73.9</t>
         </is>
       </c>
       <c r="B859" s="56" t="inlineStr">
@@ -36302,12 +36302,12 @@
       </c>
       <c r="C859" s="56" t="inlineStr">
         <is>
-          <t>Report Aktivitas Issue</t>
+          <t>Kategori Aktivitas Issue</t>
         </is>
       </c>
       <c r="D859" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data Report Aktivitas Issue</t>
+          <t>Melihat dan mengubah data master kategori</t>
         </is>
       </c>
       <c r="E859" s="57" t="inlineStr">
@@ -36317,39 +36317,39 @@
       </c>
       <c r="F859" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G859" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Klik icon Aksi (...) pada baris data List Kategori - Klik opsi Detail - Ubah data - Klik button Save</t>
         </is>
       </c>
       <c r="H859" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan dan memperbarui data master kategori.</t>
         </is>
       </c>
     </row>
     <row r="860" ht="28" customHeight="1">
       <c r="A860" s="57" t="inlineStr">
         <is>
-          <t>76.1</t>
+          <t>74.1</t>
         </is>
       </c>
       <c r="B860" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C860" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D860" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
+          <t>Membuka halaman Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E860" s="57" t="inlineStr">
@@ -36364,34 +36364,34 @@
       </c>
       <c r="G860" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="H860" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="861" ht="28" customHeight="1">
       <c r="A861" s="57" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>74.2</t>
         </is>
       </c>
       <c r="B861" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C861" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D861" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
+          <t>Melakukan filter data Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="E861" s="57" t="inlineStr">
@@ -36406,7 +36406,7 @@
       </c>
       <c r="G861" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
+          <t>Pilih Bulan dan Tahun pada filter periode di pojok kanan atas halaman</t>
         </is>
       </c>
       <c r="H861" s="56" t="inlineStr">
@@ -36418,22 +36418,22 @@
     <row r="862" ht="28" customHeight="1">
       <c r="A862" s="57" t="inlineStr">
         <is>
-          <t>76.3</t>
+          <t>74.3</t>
         </is>
       </c>
       <c r="B862" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C862" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Dashboard Aktivitas Issue</t>
         </is>
       </c>
       <c r="D862" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Melihat detail issue pada tabel 5 Newest Issue</t>
         </is>
       </c>
       <c r="E862" s="57" t="inlineStr">
@@ -36443,81 +36443,81 @@
       </c>
       <c r="F862" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G862" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Pada tabel 5 Newest Issue, klik icon Aksi (...) - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H862" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="863" ht="28" customHeight="1">
       <c r="A863" s="57" t="inlineStr">
         <is>
-          <t>76.4</t>
+          <t>75.1</t>
         </is>
       </c>
       <c r="B863" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C863" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D863" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Membuka halaman Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E863" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F863" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G863" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Klik menu Ticket Maintenance - Klik sub menu Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="H863" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Report Aktivitas Issue.</t>
         </is>
       </c>
     </row>
     <row r="864" ht="28" customHeight="1">
       <c r="A864" s="57" t="inlineStr">
         <is>
-          <t>76.5</t>
+          <t>75.2</t>
         </is>
       </c>
       <c r="B864" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C864" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D864" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Melakukan filter data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E864" s="57" t="inlineStr">
@@ -36527,39 +36527,39 @@
       </c>
       <c r="F864" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G864" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Pilih Status dan Prioritas - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H864" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="865" ht="28" customHeight="1">
       <c r="A865" s="57" t="inlineStr">
         <is>
-          <t>76.6</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="B865" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C865" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D865" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mencari data Report Aktivitas Issue dengan keyword valid</t>
         </is>
       </c>
       <c r="E865" s="57" t="inlineStr">
@@ -36574,7 +36574,7 @@
       </c>
       <c r="G865" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data - Klik icon search</t>
         </is>
       </c>
       <c r="H865" s="56" t="inlineStr">
@@ -36586,64 +36586,64 @@
     <row r="866" ht="28" customHeight="1">
       <c r="A866" s="57" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>75.4</t>
         </is>
       </c>
       <c r="B866" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C866" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D866" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Melihat detail report aktivitas issue</t>
         </is>
       </c>
       <c r="E866" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F866" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G866" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik icon Aksi (...) pada salah satu baris data - Klik opsi Detail</t>
         </is>
       </c>
       <c r="H866" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman detail issue.</t>
         </is>
       </c>
     </row>
     <row r="867" ht="28" customHeight="1">
       <c r="A867" s="57" t="inlineStr">
         <is>
-          <t>76.8</t>
+          <t>75.5</t>
         </is>
       </c>
       <c r="B867" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C867" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Funding</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D867" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Menghapus data report aktivitas issue secara massal</t>
         </is>
       </c>
       <c r="E867" s="57" t="inlineStr">
@@ -36653,39 +36653,39 @@
       </c>
       <c r="F867" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G867" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Checklist beberapa data pada tabel - Klik button Hapus data - Klik button Yes</t>
         </is>
       </c>
       <c r="H867" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menghapus data report aktivitas issue.</t>
         </is>
       </c>
     </row>
     <row r="868" ht="28" customHeight="1">
       <c r="A868" s="57" t="inlineStr">
         <is>
-          <t>77.1</t>
+          <t>75.6</t>
         </is>
       </c>
       <c r="B868" s="56" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Ticket Maintenance</t>
         </is>
       </c>
       <c r="C868" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="D868" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
+          <t>Mengekspor data Report Aktivitas Issue</t>
         </is>
       </c>
       <c r="E868" s="57" t="inlineStr">
@@ -36700,19 +36700,19 @@
       </c>
       <c r="G868" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
+          <t>Klik button Export - Klik icon download pada panel Download Export</t>
         </is>
       </c>
       <c r="H868" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="869" ht="28" customHeight="1">
       <c r="A869" s="57" t="inlineStr">
         <is>
-          <t>77.2</t>
+          <t>76.1</t>
         </is>
       </c>
       <c r="B869" s="56" t="inlineStr">
@@ -36722,12 +36722,12 @@
       </c>
       <c r="C869" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D869" s="56" t="inlineStr">
         <is>
-          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E869" s="57" t="inlineStr">
@@ -36737,24 +36737,24 @@
       </c>
       <c r="F869" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G869" s="56" t="inlineStr">
         <is>
-          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="H869" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Funding.</t>
         </is>
       </c>
     </row>
     <row r="870" ht="28" customHeight="1">
       <c r="A870" s="57" t="inlineStr">
         <is>
-          <t>77.3</t>
+          <t>76.2</t>
         </is>
       </c>
       <c r="B870" s="56" t="inlineStr">
@@ -36764,12 +36764,12 @@
       </c>
       <c r="C870" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D870" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="E870" s="57" t="inlineStr">
@@ -36784,19 +36784,19 @@
       </c>
       <c r="G870" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Pilih filter Kantor, Bulan, dan Tahun - Klik button Filter</t>
         </is>
       </c>
       <c r="H870" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="871" ht="28" customHeight="1">
       <c r="A871" s="57" t="inlineStr">
         <is>
-          <t>77.4</t>
+          <t>76.3</t>
         </is>
       </c>
       <c r="B871" s="56" t="inlineStr">
@@ -36806,17 +36806,17 @@
       </c>
       <c r="C871" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D871" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
         </is>
       </c>
       <c r="E871" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F871" s="57" t="inlineStr">
@@ -36826,19 +36826,19 @@
       </c>
       <c r="G871" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H871" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="872" ht="70" customHeight="1">
       <c r="A872" s="57" t="inlineStr">
         <is>
-          <t>77.5</t>
+          <t>76.4</t>
         </is>
       </c>
       <c r="B872" s="56" t="inlineStr">
@@ -36848,39 +36848,39 @@
       </c>
       <c r="C872" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D872" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Sales</t>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E872" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F872" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G872" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Sales</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
         </is>
       </c>
       <c r="H872" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="873" ht="42" customHeight="1">
       <c r="A873" s="57" t="inlineStr">
         <is>
-          <t>77.6</t>
+          <t>76.5</t>
         </is>
       </c>
       <c r="B873" s="56" t="inlineStr">
@@ -36890,12 +36890,12 @@
       </c>
       <c r="C873" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D873" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="E873" s="57" t="inlineStr">
@@ -36905,24 +36905,24 @@
       </c>
       <c r="F873" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G873" s="56" t="inlineStr">
         <is>
-          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
         </is>
       </c>
       <c r="H873" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="874" ht="42" customHeight="1">
       <c r="A874" s="57" t="inlineStr">
         <is>
-          <t>77.7</t>
+          <t>76.6</t>
         </is>
       </c>
       <c r="B874" s="56" t="inlineStr">
@@ -36932,17 +36932,17 @@
       </c>
       <c r="C874" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D874" s="56" t="inlineStr">
         <is>
-          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
         </is>
       </c>
       <c r="E874" s="57" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F874" s="57" t="inlineStr">
@@ -36952,19 +36952,19 @@
       </c>
       <c r="G874" s="56" t="inlineStr">
         <is>
-          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H874" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="875" ht="70" customHeight="1">
       <c r="A875" s="57" t="inlineStr">
         <is>
-          <t>77.8</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="B875" s="56" t="inlineStr">
@@ -36974,39 +36974,39 @@
       </c>
       <c r="C875" s="56" t="inlineStr">
         <is>
-          <t>Aktivitas Consumer Lending</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D875" s="56" t="inlineStr">
         <is>
-          <t>Mengekspor data tabel Aktivitas Referral</t>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E875" s="57" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F875" s="57" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G875" s="56" t="inlineStr">
         <is>
-          <t>Klik button Export pada tabel Aktivitas Referral</t>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
         </is>
       </c>
       <c r="H875" s="56" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="876" ht="28" customHeight="1">
       <c r="A876" s="57" t="inlineStr">
         <is>
-          <t>78.1</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="B876" s="56" t="inlineStr">
@@ -37016,12 +37016,12 @@
       </c>
       <c r="C876" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Aktivitas Consumer</t>
+          <t>Aktivitas Consumer Funding</t>
         </is>
       </c>
       <c r="D876" s="56" t="inlineStr">
         <is>
-          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="E876" s="57" t="inlineStr">
@@ -37036,19 +37036,19 @@
       </c>
       <c r="G876" s="56" t="inlineStr">
         <is>
-          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
         </is>
       </c>
       <c r="H876" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
+          <t>Berhasil mendownload file export.</t>
         </is>
       </c>
     </row>
     <row r="877" ht="42" customHeight="1">
       <c r="A877" s="57" t="inlineStr">
         <is>
-          <t>78.2</t>
+          <t>77.1</t>
         </is>
       </c>
       <c r="B877" s="56" t="inlineStr">
@@ -37058,12 +37058,12 @@
       </c>
       <c r="C877" s="56" t="inlineStr">
         <is>
-          <t>Pengaturan Aktivitas Consumer</t>
+          <t>Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="D877" s="56" t="inlineStr">
         <is>
-          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
+          <t>Membuka halaman Dashboard Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="E877" s="57" t="inlineStr">
@@ -37073,281 +37073,650 @@
       </c>
       <c r="F877" s="57" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G877" s="56" t="inlineStr">
         <is>
-          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Aktivitas Consumer Lending</t>
         </is>
       </c>
       <c r="H877" s="56" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
+          <t>Berhasil menampilkan halaman Dashboard Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
     <row r="878" ht="28" customHeight="1">
       <c r="A878" s="57" t="inlineStr">
         <is>
+          <t>77.2</t>
+        </is>
+      </c>
+      <c r="B878" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C878" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D878" s="56" t="inlineStr">
+        <is>
+          <t>Melakukan filter data Dashboard Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="E878" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F878" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G878" s="56" t="inlineStr">
+        <is>
+          <t>Pilih filter Kantor dan rentang Start - End Date - Klik button Filter</t>
+        </is>
+      </c>
+      <c r="H878" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+        </is>
+      </c>
+    </row>
+    <row r="879" ht="28" customHeight="1">
+      <c r="A879" s="57" t="inlineStr">
+        <is>
+          <t>77.3</t>
+        </is>
+      </c>
+      <c r="B879" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C879" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D879" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E879" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F879" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G879" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H879" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="880" ht="28" customHeight="1">
+      <c r="A880" s="57" t="inlineStr">
+        <is>
+          <t>77.4</t>
+        </is>
+      </c>
+      <c r="B880" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C880" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D880" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Sales dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E880" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F880" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G880" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Sales - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H880" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="881" ht="14" customHeight="1">
+      <c r="A881" s="57" t="inlineStr">
+        <is>
+          <t>77.5</t>
+        </is>
+      </c>
+      <c r="B881" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C881" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D881" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="E881" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F881" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G881" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Sales</t>
+        </is>
+      </c>
+      <c r="H881" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="882" ht="42" customHeight="1">
+      <c r="A882" s="57" t="inlineStr">
+        <is>
+          <t>77.6</t>
+        </is>
+      </c>
+      <c r="B882" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C882" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D882" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword valid</t>
+        </is>
+      </c>
+      <c r="E882" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F882" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G882" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H882" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data yang dicari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="883" ht="42" customHeight="1">
+      <c r="A883" s="57" t="inlineStr">
+        <is>
+          <t>77.7</t>
+        </is>
+      </c>
+      <c r="B883" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C883" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D883" s="56" t="inlineStr">
+        <is>
+          <t>Mencari data pada tabel Aktivitas Referral dengan keyword tidak valid</t>
+        </is>
+      </c>
+      <c r="E883" s="57" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F883" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G883" s="56" t="inlineStr">
+        <is>
+          <t>Input keyword tidak valid pada field Cari Data tabel Aktivitas Referral - Klik icon search</t>
+        </is>
+      </c>
+      <c r="H883" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan informasi bahwa data tidak ditemukan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="884" ht="28" customHeight="1">
+      <c r="A884" s="57" t="inlineStr">
+        <is>
+          <t>77.8</t>
+        </is>
+      </c>
+      <c r="B884" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C884" s="56" t="inlineStr">
+        <is>
+          <t>Aktivitas Consumer Lending</t>
+        </is>
+      </c>
+      <c r="D884" s="56" t="inlineStr">
+        <is>
+          <t>Mengekspor data tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="E884" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F884" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G884" s="56" t="inlineStr">
+        <is>
+          <t>Klik button Export pada tabel Aktivitas Referral</t>
+        </is>
+      </c>
+      <c r="H884" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil mendownload file export.</t>
+        </is>
+      </c>
+    </row>
+    <row r="885" ht="42" customHeight="1">
+      <c r="A885" s="57" t="inlineStr">
+        <is>
+          <t>78.1</t>
+        </is>
+      </c>
+      <c r="B885" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C885" s="56" t="inlineStr">
+        <is>
+          <t>Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="D885" s="56" t="inlineStr">
+        <is>
+          <t>Membuka halaman Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="E885" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F885" s="57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G885" s="56" t="inlineStr">
+        <is>
+          <t>Klik menu Dashboard - Klik menu Aktivitas Consumer - Klik sub menu Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="H885" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan halaman Pengaturan Aktivitas Consumer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="886" ht="14" customHeight="1">
+      <c r="A886" s="57" t="inlineStr">
+        <is>
+          <t>78.2</t>
+        </is>
+      </c>
+      <c r="B886" s="56" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C886" s="56" t="inlineStr">
+        <is>
+          <t>Pengaturan Aktivitas Consumer</t>
+        </is>
+      </c>
+      <c r="D886" s="56" t="inlineStr">
+        <is>
+          <t>Mengubah role pada Pengaturan Aktivitas Consumer Funding</t>
+        </is>
+      </c>
+      <c r="E886" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F886" s="57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G886" s="56" t="inlineStr">
+        <is>
+          <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Funding - Klik button Simpan</t>
+        </is>
+      </c>
+      <c r="H886" s="56" t="inlineStr">
+        <is>
+          <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Funding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="887" ht="42" customHeight="1">
+      <c r="A887" s="57" t="inlineStr">
+        <is>
           <t>78.3</t>
         </is>
       </c>
-      <c r="B878" s="56" t="inlineStr">
+      <c r="B887" s="56" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C878" s="56" t="inlineStr">
+      <c r="C887" s="56" t="inlineStr">
         <is>
           <t>Pengaturan Aktivitas Consumer</t>
         </is>
       </c>
-      <c r="D878" s="56" t="inlineStr">
+      <c r="D887" s="56" t="inlineStr">
         <is>
           <t>Mengubah role pada Pengaturan Aktivitas Consumer Lending</t>
         </is>
       </c>
-      <c r="E878" s="57" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F878" s="57" t="inlineStr">
+      <c r="E887" s="57" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F887" s="57" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G878" s="56" t="inlineStr">
+      <c r="G887" s="56" t="inlineStr">
         <is>
           <t>Pilih atau sesuaikan data pada field Role Pengaturan Aktivitas Consumer Lending - Klik button Simpan</t>
         </is>
       </c>
-      <c r="H878" s="56" t="inlineStr">
+      <c r="H887" s="56" t="inlineStr">
         <is>
           <t>Berhasil menyimpan perubahan role pada Pengaturan Aktivitas Consumer Lending.</t>
         </is>
       </c>
     </row>
-    <row r="879" ht="28" customHeight="1">
-      <c r="A879" s="58" t="inlineStr">
+    <row r="888" ht="42" customHeight="1">
+      <c r="A888" s="58" t="inlineStr">
         <is>
           <t>79.1</t>
         </is>
       </c>
-      <c r="B879" s="59" t="inlineStr">
+      <c r="B888" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C879" s="59" t="inlineStr">
+      <c r="C888" s="59" t="inlineStr">
         <is>
           <t>Optimalisasi Database</t>
         </is>
       </c>
-      <c r="D879" s="59" t="inlineStr">
+      <c r="D888" s="59" t="inlineStr">
         <is>
           <t>Membuka halaman Dashboard Optimalisasi Database</t>
         </is>
       </c>
-      <c r="E879" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F879" s="58" t="inlineStr">
+      <c r="E888" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F888" s="58" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G879" s="59" t="inlineStr">
+      <c r="G888" s="59" t="inlineStr">
         <is>
           <t>Klik menu Dashboard - Klik sub menu Optimalisasi</t>
         </is>
       </c>
-      <c r="H879" s="59" t="inlineStr">
+      <c r="H888" s="59" t="inlineStr">
         <is>
           <t>Berhasil menampilkan halaman Dashboard Optimalisasi Database.</t>
         </is>
       </c>
     </row>
-    <row r="880" ht="28" customHeight="1">
-      <c r="A880" s="58" t="inlineStr">
+    <row r="889" ht="28" customHeight="1">
+      <c r="A889" s="58" t="inlineStr">
         <is>
           <t>79.2</t>
         </is>
       </c>
-      <c r="B880" s="59" t="inlineStr">
+      <c r="B889" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C880" s="59" t="inlineStr">
+      <c r="C889" s="59" t="inlineStr">
         <is>
           <t>Optimalisasi Database</t>
         </is>
       </c>
-      <c r="D880" s="59" t="inlineStr">
+      <c r="D889" s="59" t="inlineStr">
         <is>
           <t>Melakukan filter data Dashboard Optimalisasi Database</t>
         </is>
       </c>
-      <c r="E880" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F880" s="58" t="inlineStr">
+      <c r="E889" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F889" s="58" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G880" s="59" t="inlineStr">
+      <c r="G889" s="59" t="inlineStr">
         <is>
           <t>Pilih Kantor Wilayah, Kantor Cabang, Sales, Produk, Source Debitur, Info Bulan, dan Info Tahun - Klik button Submit</t>
         </is>
       </c>
-      <c r="H880" s="59" t="inlineStr">
+      <c r="H889" s="59" t="inlineStr">
         <is>
           <t>Berhasil menampilkan data dashboard dan bagan alur optimalisasi sesuai filter yang dipilih.</t>
         </is>
       </c>
     </row>
-    <row r="881" ht="14" customHeight="1">
-      <c r="A881" s="58" t="inlineStr">
+    <row r="890" ht="42" customHeight="1">
+      <c r="A890" s="58" t="inlineStr">
         <is>
           <t>79.3</t>
         </is>
       </c>
-      <c r="B881" s="59" t="inlineStr">
+      <c r="B890" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C881" s="59" t="inlineStr">
+      <c r="C890" s="59" t="inlineStr">
         <is>
           <t>Optimalisasi Database</t>
         </is>
       </c>
-      <c r="D881" s="59" t="inlineStr">
+      <c r="D890" s="59" t="inlineStr">
         <is>
           <t>Mencari data pada tabel dengan keyword valid</t>
         </is>
       </c>
-      <c r="E881" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F881" s="58" t="inlineStr">
+      <c r="E890" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F890" s="58" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G881" s="59" t="inlineStr">
+      <c r="G890" s="59" t="inlineStr">
         <is>
           <t>Masukkan keyword valid pada kolom Cari Data - Klik button Cari</t>
         </is>
       </c>
-      <c r="H881" s="59" t="inlineStr">
+      <c r="H890" s="59" t="inlineStr">
         <is>
           <t>Berhasil menampilkan data yang sesuai dengan keyword pencarian.</t>
         </is>
       </c>
     </row>
-    <row r="882" ht="42" customHeight="1">
-      <c r="A882" s="58" t="inlineStr">
+    <row r="891" ht="14" customHeight="1">
+      <c r="A891" s="58" t="inlineStr">
         <is>
           <t>79.4</t>
         </is>
       </c>
-      <c r="B882" s="59" t="inlineStr">
+      <c r="B891" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C882" s="59" t="inlineStr">
+      <c r="C891" s="59" t="inlineStr">
         <is>
           <t>Optimalisasi Database</t>
         </is>
       </c>
-      <c r="D882" s="59" t="inlineStr">
+      <c r="D891" s="59" t="inlineStr">
         <is>
           <t>Mencari data pada tabel dengan keyword tidak valid</t>
         </is>
       </c>
-      <c r="E882" s="58" t="inlineStr">
+      <c r="E891" s="58" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="F882" s="58" t="inlineStr">
+      <c r="F891" s="58" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G882" s="59" t="inlineStr">
+      <c r="G891" s="59" t="inlineStr">
         <is>
           <t>Masukkan keyword tidak valid pada kolom Cari Data - Klik button Cari</t>
         </is>
       </c>
-      <c r="H882" s="59" t="inlineStr">
+      <c r="H891" s="59" t="inlineStr">
         <is>
           <t>Menampilkan keterangan data tidak ditemukan / tabel kosong.</t>
         </is>
       </c>
     </row>
-    <row r="883" ht="42" customHeight="1">
-      <c r="A883" s="58" t="inlineStr">
+    <row r="892" ht="42" customHeight="1">
+      <c r="A892" s="58" t="inlineStr">
         <is>
           <t>79.5</t>
         </is>
       </c>
-      <c r="B883" s="59" t="inlineStr">
+      <c r="B892" s="59" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="C883" s="59" t="inlineStr">
+      <c r="C892" s="59" t="inlineStr">
         <is>
           <t>Optimalisasi Database</t>
         </is>
       </c>
-      <c r="D883" s="59" t="inlineStr">
+      <c r="D892" s="59" t="inlineStr">
         <is>
           <t>Mengekspor data tabel Optimalisasi Database</t>
         </is>
       </c>
-      <c r="E883" s="58" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F883" s="58" t="inlineStr">
+      <c r="E892" s="58" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F892" s="58" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G883" s="59" t="inlineStr">
+      <c r="G892" s="59" t="inlineStr">
         <is>
           <t>Klik button Export</t>
         </is>
       </c>
-      <c r="H883" s="59" t="inlineStr">
+      <c r="H892" s="59" t="inlineStr">
         <is>
           <t>Berhasil mengunduh file data tabel dalam format Excel (.xlsx).</t>
         </is>
       </c>
     </row>
-    <row r="884" ht="28" customHeight="1"/>
-    <row r="885" ht="42" customHeight="1"/>
-    <row r="886" ht="14" customHeight="1"/>
-    <row r="887" ht="42" customHeight="1"/>
-    <row r="888" ht="42" customHeight="1"/>
-    <row r="889" ht="28" customHeight="1"/>
-    <row r="890" ht="42" customHeight="1"/>
-    <row r="891" ht="14" customHeight="1"/>
-    <row r="892" ht="42" customHeight="1"/>
     <row r="893" ht="42" customHeight="1"/>
     <row r="894" ht="28" customHeight="1"/>
     <row r="895" ht="42" customHeight="1"/>

</xml_diff>

<commit_message>
chore(web): polish Modul 20 Upload Target Bulk metadata and excel
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z888"/>
+  <dimension ref="A1:H888"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11008,12 +11008,12 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Klik menu Upload Bulk - Klik submenu Upload Target Bulk</t>
+          <t>-K-l-i-k- -m-e-n-u- -U-p-l-o-a-d- -B-u-l-k- --- -K-l-i-k- -s-u-b-m-e-n-u- -U-p-l-o-a-d- -T-a-r-g-e-t- -B-u-l-k-</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>Menampilkan halaman Upload target bulk</t>
+          <t>-M-e-n-a-m-p-i-l-k-a-n- -h-a-l-a-m-a-n- -U-p-l-o-a-d- -t-a-r-g-e-t- -b-u-l-k-</t>
         </is>
       </c>
     </row>
@@ -11050,12 +11050,12 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>Pilih Bisnis Unit - Klik button Download dan Upload File - Klik button Download file template - Buka file excel</t>
+          <t>-P-i-l-i-h- -B-i-s-n-i-s- -U-n-i-t- --- -K-l-i-k- -b-u-t-t-o-n- -D-o-w-n-l-o-a-d- -d-a-n- -U-p-l-o-a-d- -F-i-l-e- --- -K-l-i-k- -b-u-t-t-o-n- -D-o-w-n-l-o-a-d- -f-i-l-e- -t-e-m-p-l-a-t-e- --- -B-u-k-a- -f-i-l-e- -e-x-c-e-l-</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>File excel dapat di buka</t>
+          <t>-F-i-l-e- -e-x-c-e-l- -d-a-p-a-t- -d-i- -b-u-k-a-</t>
         </is>
       </c>
     </row>
@@ -11092,12 +11092,12 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Kosongkan bisnis unit - Klik button Download dan Upload File - Klik button Download file template</t>
+          <t>-K-o-s-o-n-g-k-a-n- -b-i-s-n-i-s- -u-n-i-t- --- -K-l-i-k- -b-u-t-t-o-n- -D-o-w-n-l-o-a-d- -d-a-n- -U-p-l-o-a-d- -F-i-l-e- --- -K-l-i-k- -b-u-t-t-o-n- -D-o-w-n-l-o-a-d- -f-i-l-e- -t-e-m-p-l-a-t-e-</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Tidak bisa mengunduh dan menampilkan alert 'Bisnis Unit wajib dipilih sebelum download template'</t>
+          <t>-T-i-d-a-k- -b-i-s-a- -m-e-n-g-u-n-d-u-h- -d-a-n- -m-e-n-a-m-p-i-l-k-a-n- -a-l-e-r-t- -'-B-i-s-n-i-s- -U-n-i-t- -w-a-j-i-b- -d-i-p-i-l-i-h- -s-e-b-e-l-u-m- -d-o-w-n-l-o-a-d- -t-e-m-p-l-a-t-e-'-</t>
         </is>
       </c>
     </row>
@@ -11134,12 +11134,12 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Buka file excel - Input data upload target bulk - Simpan file excel - Pilih Bisnis Unit yang sesuai - Klik 'Pilih atau seret file Template (.xlsx) ke area ini' - Pilih file yang sudah di input - Klik button Open pada file manager</t>
+          <t>-B-u-k-a- -f-i-l-e- -e-x-c-e-l- --- -I-n-p-u-t- -d-a-t-a- -u-p-l-o-a-d- -t-a-r-g-e-t- -b-u-l-k- --- -S-i-m-p-a-n- -f-i-l-e- -e-x-c-e-l- --- -P-i-l-i-h- -B-i-s-n-i-s- -U-n-i-t- -y-a-n-g- -s-e-s-u-a-i- --- -K-l-i-k- -'-P-i-l-i-h- -a-t-a-u- -s-e-r-e-t- -f-i-l-e- -T-e-m-p-l-a-t-e- -(-.-x-l-s-x-)- -k-e- -a-r-e-a- -i-n-i-'- --- -P-i-l-i-h- -f-i-l-e- -y-a-n-g- -s-u-d-a-h- -d-i- -i-n-p-u-t- --- -K-l-i-k- -b-u-t-t-o-n- -O-p-e-n- -p-a-d-a- -f-i-l-e- -m-a-n-a-g-e-r-</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>Berhasil mengupload data target secara bulk, dan status nya Selesai</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-n-g-u-p-l-o-a-d- -d-a-t-a- -t-a-r-g-e-t- -s-e-c-a-r-a- -b-u-l-k-,- -d-a-n- -s-t-a-t-u-s- -n-y-a- -S-e-l-e-s-a-i-</t>
         </is>
       </c>
     </row>
@@ -11176,12 +11176,12 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Upload data target bulk dengan template yang tidak sesuai</t>
+          <t>-U-p-l-o-a-d- -d-a-t-a- -t-a-r-g-e-t- -b-u-l-k- -d-e-n-g-a-n- -t-e-m-p-l-a-t-e- -y-a-n-g- -t-i-d-a-k- -s-e-s-u-a-i-</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>Menampilkan status Template Tidak Valid dan gagal upload bulk data tidak tersimpan atau terupdate</t>
+          <t>-M-e-n-a-m-p-i-l-k-a-n- -s-t-a-t-u-s- -T-e-m-p-l-a-t-e- -T-i-d-a-k- -V-a-l-i-d- -d-a-n- -g-a-g-a-l- -u-p-l-o-a-d- -b-u-l-k- -d-a-t-a- -t-i-d-a-k- -t-e-r-s-i-m-p-a-n- -a-t-a-u- -t-e-r-u-p-d-a-t-e-</t>
         </is>
       </c>
     </row>
@@ -11218,12 +11218,12 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) - Klik detail batch</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- --- -K-l-i-k- -d-e-t-a-i-l- -b-a-t-c-h-</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>Menampilkan data detail</t>
+          <t>-M-e-n-a-m-p-i-l-k-a-n- -d-a-t-a- -d-e-t-a-i-l-</t>
         </is>
       </c>
     </row>
@@ -11260,12 +11260,12 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) – Klik download souce file</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- -–- -K-l-i-k- -d-o-w-n-l-o-a-d- -s-o-u-c-e- -f-i-l-e-</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>Berhasil mengunduh data souce file</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-n-g-u-n-d-u-h- -d-a-t-a- -s-o-u-c-e- -f-i-l-e-</t>
         </is>
       </c>
     </row>
@@ -11302,12 +11302,12 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) - Klik preview data</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- --- -K-l-i-k- -p-r-e-v-i-e-w- -d-a-t-a-</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>Menampilkan detail data hasil upload dan penjelasan jika terdapat validasi error pada file yang diupload</t>
+          <t>-M-e-n-a-m-p-i-l-k-a-n- -d-e-t-a-i-l- -d-a-t-a- -h-a-s-i-l- -u-p-l-o-a-d- -d-a-n- -p-e-n-j-e-l-a-s-a-n- -j-i-k-a- -t-e-r-d-a-p-a-t- -v-a-l-i-d-a-s-i- -e-r-r-o-r- -p-a-d-a- -f-i-l-e- -y-a-n-g- -d-i-u-p-l-o-a-d-</t>
         </is>
       </c>
     </row>
@@ -11344,12 +11344,12 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) – klik hapus batch</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- -–- -k-l-i-k- -h-a-p-u-s- -b-a-t-c-h-</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-n-g-h-a-p-u-s- -d-a-t-a-</t>
         </is>
       </c>
     </row>
@@ -11386,12 +11386,12 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) pada file dengan status “validasi gagal”  – klik download error file</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- -p-a-d-a- -f-i-l-e- -d-e-n-g-a-n- -s-t-a-t-u-s- -“-v-a-l-i-d-a-s-i- -g-a-g-a-l-”- - -–- -k-l-i-k- -d-o-w-n-l-o-a-d- -e-r-r-o-r- -f-i-l-e-</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Berhasil download error file</t>
+          <t>-B-e-r-h-a-s-i-l- -d-o-w-n-l-o-a-d- -e-r-r-o-r- -f-i-l-e-</t>
         </is>
       </c>
     </row>
@@ -11428,12 +11428,12 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) pada file dengan status “validasi gagal”  – klik batalkan</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- -p-a-d-a- -f-i-l-e- -d-e-n-g-a-n- -s-t-a-t-u-s- -“-v-a-l-i-d-a-s-i- -g-a-g-a-l-”- - -–- -k-l-i-k- -b-a-t-a-l-k-a-n-</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>Berhasil membatalkan batch</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-m-b-a-t-a-l-k-a-n- -b-a-t-c-h-</t>
         </is>
       </c>
     </row>
@@ -11470,12 +11470,12 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Klik button Aksi (...) pada file dengan status “gagal”  – klik coba lagi (retry)</t>
+          <t>-K-l-i-k- -b-u-t-t-o-n- -A-k-s-i- -(-.-.-.-)- -p-a-d-a- -f-i-l-e- -d-e-n-g-a-n- -s-t-a-t-u-s- -“-g-a-g-a-l-”- - -–- -k-l-i-k- -c-o-b-a- -l-a-g-i- -(-r-e-t-r-y-)-</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>Berhasil mengupload ulang file</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-n-g-u-p-l-o-a-d- -u-l-a-n-g- -f-i-l-e-</t>
         </is>
       </c>
     </row>
@@ -11502,7 +11502,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Mencari data pada kolom pencarian</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -11512,12 +11512,12 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Input batch id pada kolom pencarian</t>
+          <t>-I-n-p-u-t- -b-a-t-c-h- -i-d- -p-a-d-a- -k-o-l-o-m- -p-e-n-c-a-r-i-a-n-</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai kata kunci yang diinput</t>
+          <t>-B-e-r-h-a-s-i-l- -m-e-n-a-m-p-i-l-k-a-n- -d-a-t-a- -s-e-s-u-a-i- -k-a-t-a- -k-u-n-c-i- -y-a-n-g- -d-i-i-n-p-u-t-</t>
         </is>
       </c>
     </row>
@@ -11544,7 +11544,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Melakukan filter data</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -11554,12 +11554,12 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Pilih status</t>
+          <t>-P-i-l-i-h- -s-t-a-t-u-s-</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai filter yang dipilih</t>
+          <t>-M-e-n-a-m-p-i-l-k-a-n- -d-a-t-a- -s-e-s-u-a-i- -f-i-l-t-e-r- -y-a-n-g- -d-i-p-i-l-i-h-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): harmonize Bulk Import Prospek Personal (18 TCs) and Lembaga (7 TCs) with senior test master
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -12086,7 +12086,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Tidak menginput kolom data mandatory</t>
+          <t>Menginput email yang tidak valid</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -12101,12 +12101,12 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Input data pada template excel dengan mengosongkan kolom mandatory - Upload template tersebut</t>
+          <t>Input email yang tidak valid pada kolom email (ex. heri.com) - Simpan file - Upload file</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>Berhasil upload file dengan status 'Validasi Gagal'</t>
+          <t>Berhasil upload file dengan status 'Validasi Gagal' dan menampilkan informasi validation error 'Format email tidak valid' pada halaman preview data dan dokumen error. data prospek tidak tersimpan</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Menginput email yang tidak valid</t>
+          <t>Menginput no CIF yang tidak valid untuk nasabah ETB</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -12143,12 +12143,12 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Input email yang tidak valid pada template excel - Upload template tersebut</t>
+          <t>Input no CIF yang tidak valid - Simpan file - Upload file</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Berhasil upload file dengan status 'Validasi Gagal'</t>
+          <t>Berhasil upload file dengan status 'Validasi gagal', menampilkan informasi validation error 'no CIF tidak ditemukan' pada halaman preview data dan dokumen error. data prospek tidak tersimpan</t>
         </is>
       </c>
     </row>
@@ -12170,12 +12170,12 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Menginput no CIF yang tidak valid untuk nasabah ETB</t>
+          <t>Menginput tanggal aktivitas (call, open account, dan top up) sebelum tanggal prospek</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -12185,12 +12185,12 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Input no CIF yang tidak valid pada template excel - Upload template tersebut</t>
+          <t>Input tanggal Call, Open Account, Top up sebelum tanggal prospek - Simpan file - Upload file - Cek data pada halaman preview data dan dokumen error</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Berhasil upload file dengan status 'Validasi Gagal'</t>
+          <t>Menampilkan informasi 'Tanggal call tidak boleh sebelum tanggal prospek', 'Tanggal Open Account tidak boleh sebelum tanggal prospek' , 'Tanggal Top up tidak boleh sebelum tanggal prospek' pada masing masing kolom</t>
         </is>
       </c>
     </row>
@@ -12212,7 +12212,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Menginput tanggal aktivitas (call, open account, dan top up) sebelum tanggal prospek</t>
+          <t>Validasi Format tanggal</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -12227,12 +12227,12 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Input tanggal Call, Open Account, dan Top Up sebelum tanggal prospek - Upload template</t>
+          <t>Input tanggal dengan format yang tidak sesuai - Simpan file - Upload file - Cek data pada halaman preview data dan dokumen error</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Menampilkan informasi 'Tanggal aktivitas tidak boleh sebelum tanggal prospek'</t>
+          <t>Menampilkan informasi 'Format tanggal harus DD-MM-YYYY'</t>
         </is>
       </c>
     </row>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Validasi Format tanggal</t>
+          <t>Validasi input Potensi dan Jumlah Dana Masuk</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -12269,12 +12269,12 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Input tanggal dengan format yang tidak sesuai pada template - Upload template</t>
+          <t>Input selain nominal angka di kolom Potensi dan Jumlah Dana Masuk (Top Up) - Simpan file - Upload file - Cek data pada halaman preview data dan dokumen error</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>Menampilkan informasi 'Format tanggal tidak sesuai'</t>
+          <t>Menampilkan informasi 'Jumlah dana masuk (Top Up) harus angka'</t>
         </is>
       </c>
     </row>
@@ -12296,7 +12296,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Validasi input Potensi dan Jumlah Dana Masuk</t>
+          <t>Membatalkan upload data prospek personal</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -12311,12 +12311,12 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Input selain nominal angka di kolom potensi dan jumlah dana masuk - Upload template</t>
+          <t>Upload file data prospek personal yang valid - Klik Action titik tiga - Klik button Batalkan selagi status upload masih dalam antrian</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>Menampilkan informasi 'Jumlah dana harus berupa angka'</t>
+          <t>Berhasil membatalkan upload bulk data prospek personal, status nya menjadi 'Dibatalkan'</t>
         </is>
       </c>
     </row>
@@ -12338,7 +12338,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Membatalkan upload data prospek personal</t>
+          <t>Pagination di Preview Data</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -12353,12 +12353,12 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Upload file data prospek personal - Klik button Batalkan</t>
+          <t>Klik pagination (10/halaman) - Pilih berapa data yang ingin di tampilkan</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Berhasil membatalkan upload bulk data prospek personal</t>
+          <t>Berhasil menampilkan data sesuai dengan pagination yang di pilih</t>
         </is>
       </c>
     </row>
@@ -12380,7 +12380,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Pagination di Preview Data</t>
+          <t>Pindah Halaman di Preview Data</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -12395,12 +12395,12 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Klik pagination (10/halaman) - Pilih opsi 25/halaman</t>
+          <t>Input angka halaman di field pindah halaman - Klik Enter pada keyboard</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan limit pagination yang dipilih</t>
+          <t>Berhasil menampilkan halaman sesuai dengan angka halaman yang di input</t>
         </is>
       </c>
     </row>
@@ -12422,7 +12422,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Pindah Halaman di Preview Data</t>
+          <t>Mencari data berdasarkan batch id upload bulk prospek personal</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -12437,12 +12437,12 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Input angka halaman di field pagination - Tekan enter</t>
+          <t>Input batch id pada field search - Klik icon search atau klik Enter</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman sesuai dengan input nomor halaman</t>
+          <t>Menampilkan data upload bulk prospek personal sesuai dengan batch id yang di cari</t>
         </is>
       </c>
     </row>
@@ -12464,7 +12464,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Mencari data berdasarkan batch id upload bulk prospek personal</t>
+          <t>Filter status upload bulk prospek personal</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -12479,12 +12479,12 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>Input batch id pada field search - Tekan enter</t>
+          <t>Klik Filter Status - Pilih dan klik salah satu status</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>Menampilkan data upload bulk prospek personal sesuai batch id pencarian</t>
+          <t>Menampilkan data upload bulk prospek personal sesuai dengan status yang di pilih</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12506,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Filter status upload bulk prospek personal</t>
+          <t>Validasi data yang berhasil di upload</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -12521,12 +12521,12 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>Klik Filter Status - Pilih dan terapkan filter status</t>
+          <t>Login menggunakan user yang di assign ketika input data pada excel - Klik menu Lead Qualification - Klik submenu Aktifitas - Cek data prospek yang di uplaod melalui menu Bulk Import Prospek - Cek detail prospek pada halaman detail dan aktifitas marketing</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Menampilkan data upload bulk prospek personal sesuai filter yang dipilih</t>
+          <t>Menampilkan semua informasi data prospek yang sesuai dengan yang di upload di menu Bulk Import Prospek lembaga dengan keterangan 'Registered based on excel'</t>
         </is>
       </c>
     </row>
@@ -12548,12 +12548,12 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Validasi data yang berhasil di upload</t>
+          <t>Upload file prospek dengan template yang tidak sesuai</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -12563,12 +12563,12 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>Login menggunakan user yang di-assign data prospek - Buka menu Prospek</t>
+          <t>Upload data prospek lembaga dengan template yang tidak sesuai</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>Menampilkan semua informasi data prospek yang telah berhasil diupload</t>
+          <t>Menampilkan status Template Tidak Valid dan gagal upload bulk data tidak tersimpan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): harmonize Bisnis dan Produk (Modul 14, 15, 16) and Kantor (Modul 17, 18) with senior test master
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -8713,7 +8713,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Menambahkan data Unit Bisnis</t>
+          <t>Melakukan filter data Unit Bisnis</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -8723,17 +8723,17 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Klik button Tambah Unit Bisnis - Isi field mandatory Name, Kode Unit Bisnis, dan Jenis Bisnis - Klik button Submit</t>
+          <t>Klik button Filter - Pilih parameter filter - Klik button Terapkan</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan unit bisnis baru.</t>
+          <t>Berhasil menampilkan data terfilter.</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Menambahkan data Unit Bisnis tanpa mengisi field mandatory</t>
+          <t>Mereset filter Unit Bisnis</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8765,17 +8765,17 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Klik button Tambah Unit Bisnis - Kosongkan salah satu field mandatory - Klik button Submit</t>
+          <t>Klik button Filter - Klik button Reset</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data.</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8797,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Mengubah data Unit Bisnis</t>
+          <t>Menambahkan data Unit Bisnis</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -8812,12 +8812,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Ubah Data - Ubah data pada form - Klik button Submit</t>
+          <t>Klik button Tambah Unit Bisnis - Isi field mandatory Name, Kode Unit Bisnis, dan Jenis Bisnis - Klik button Submit</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan.</t>
+          <t>Berhasil menyimpan unit bisnis baru.</t>
         </is>
       </c>
     </row>
@@ -8839,27 +8839,27 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Menghapus data Unit Bisnis</t>
+          <t>Menambahkan data Unit Bisnis tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Hapus - Klik button Ya</t>
+          <t>Klik button Tambah Unit Bisnis - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>Berhasil menghapus unit bisnis.</t>
+          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
         </is>
       </c>
     </row>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Mengekspor data Unit Bisnis</t>
+          <t>Mengubah data Unit Bisnis</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -8896,12 +8896,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Klik button Export</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Ubah data pada form - Klik button Submit</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menyimpan perubahan.</t>
         </is>
       </c>
     </row>
@@ -8938,12 +8938,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Edit - Kosongkan field mandatory - Klik button Simpan</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>Menampilkan pesan validasi wajib diisi.</t>
+          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
         </is>
       </c>
     </row>
@@ -8980,7 +8980,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Hapus - Klik button Yes pada popup konfirmasi</t>
+          <t>Klik action menu titik tiga - Klik button Hapus - Klik button Ya</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -9175,7 +9175,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Menambahkan data Produk</t>
+          <t>Melakukan filter data Produk</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -9185,17 +9185,17 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Klik button Tambah Produk - Isi field mandatory seluruh field mandatory - Klik button Submit</t>
+          <t>Klik button Filter - Pilih parameter filter - Klik button Terapkan</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data Produk baru.</t>
+          <t>Berhasil menampilkan data terfilter.</t>
         </is>
       </c>
     </row>
@@ -9217,7 +9217,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Mengubah data Produk</t>
+          <t>Mereset filter data Produk</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -9227,17 +9227,17 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Ubah Data - Ubah data pada form - Klik button Submit</t>
+          <t>Klik button Filter - Klik button Reset</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data.</t>
         </is>
       </c>
     </row>
@@ -9259,7 +9259,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Mengubah data Produk tanpa mengisi field mandatory</t>
+          <t>Menambahkan data Produk</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -9269,17 +9269,17 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Ubah Data - Kosongkan salah satu field mandatory - Klik button Submit</t>
+          <t>Klik button Tambah Produk - Isi field mandatory seluruh field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
+          <t>Berhasil menyimpan data Produk baru.</t>
         </is>
       </c>
     </row>
@@ -9301,12 +9301,12 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Menghapus data Produk secara massal (Bulk Delete)</t>
+          <t>Menambahkan data Produk tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -9316,12 +9316,12 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Pilih beberapa data yang ingin dihapus dengan mencentang checkbox pada baris data - Klik button Hapus X data - Klik button Ya</t>
+          <t>Klik button Tambah Produk - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data Produk yang dipilih.</t>
+          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
         </is>
       </c>
     </row>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Mengekspor data Produk</t>
+          <t>Mengubah data Produk</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -9358,12 +9358,12 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Klik button Export</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Ubah data pada form - Klik button Submit</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menyimpan perubahan.</t>
         </is>
       </c>
     </row>
@@ -9400,12 +9400,12 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Klik action menu titik tiga - Klik button Edit - Kosongkan field mandatory - Klik button Simpan</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Menampilkan pesan validasi wajib diisi.</t>
+          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
         </is>
       </c>
     </row>
@@ -9437,17 +9437,17 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Pilih beberapa data yang ingin dihapus menggunakan checkbox - Klik button Hapus data - Klik button Yes pada popup konfirmasi</t>
+          <t>Pilih beberapa data yang ingin dihapus dengan mencentang checkbox pada baris data - Klik button Hapus X data - Klik button Ya</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data Produk.</t>
+          <t>Berhasil menghapus data Produk yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -9479,7 +9479,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -9531,7 +9531,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Berhasil membuka halaman Program Produk.</t>
+          <t>Berhasil membuka sub menu Program Produk.</t>
         </is>
       </c>
     </row>
@@ -9573,7 +9573,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data Program Produk sesuai pencarian.</t>
+          <t>Berhasil menampilkan data sesuai pencarian.</t>
         </is>
       </c>
     </row>
@@ -9605,7 +9605,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -9615,7 +9615,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Menampilkan informasi data tidak ditemukan.</t>
+          <t>Menampilkan data kosong.</t>
         </is>
       </c>
     </row>
@@ -9637,7 +9637,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Menambahkan data Program Produk</t>
+          <t>Melakukan filter data Program Produk</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -9647,17 +9647,17 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Klik button Tambah Program Produk - Mengisi semua field mandatory - Klik button Submit</t>
+          <t>Klik button Filter - Pilih parameter filter - Klik button Terapkan</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan data Program Produk baru.</t>
+          <t>Berhasil menampilkan data terfilter.</t>
         </is>
       </c>
     </row>
@@ -9679,27 +9679,27 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Menambahkan data Program Produk tanpa mengisi field mandatory</t>
+          <t>Mereset filter data Program Produk</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Klik button Tambah Program Produk - Mengosongkan field mandatory - Klik button Submit</t>
+          <t>Klik button Filter - Klik button Reset</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
+          <t>Berhasil mereset filter dan menampilkan seluruh data.</t>
         </is>
       </c>
     </row>
@@ -9721,7 +9721,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Mengubah data Program Produk</t>
+          <t>Menambahkan data Program Produk</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -9731,17 +9731,17 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Klik icon titik tiga pada kolom Action - Klik menu Ubah Data - Mengubah data pada field - Klik button Submit</t>
+          <t>Klik button Tambah Program Produk - Isi field mandatory Nama, Kode, dan deskripsi - Klik button Submit</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Program Produk.</t>
+          <t>Berhasil menyimpan data Program Produk baru.</t>
         </is>
       </c>
     </row>
@@ -9763,7 +9763,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Mengubah data Program Produk tanpa mengisi field mandatory</t>
+          <t>Menambahkan data Program Produk tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Klik icon titik tiga pada kolom Action - Klik menu Ubah Data - Mengosongkan field mandatory - Klik button Submit</t>
+          <t>Klik button Tambah Program Produk - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -9805,7 +9805,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Menghapus data Program Produk</t>
+          <t>Mengubah data Program Produk</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -9815,17 +9815,17 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Centang checkbox pada data yang ingin dihapus - Klik button Hapus 1 data - Klik button Yes pada popup konfirmasi</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Ubah data pada form - Klik button Submit</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data Program Produk.</t>
+          <t>Berhasil menyimpan perubahan.</t>
         </is>
       </c>
     </row>
@@ -9847,27 +9847,27 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Mengekspor data Program Produk</t>
+          <t>Mengubah data Program Produk tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Export Center</t>
+          <t>Klik action menu titik tiga - Klik button Ubah Data - Kosongkan salah satu field mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Menampilkan pesan validasi wajib diisi dan data tidak disimpan.</t>
         </is>
       </c>
     </row>
@@ -9899,17 +9899,17 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Pilih beberapa data yang ingin dihapus menggunakan checkbox - Klik button Hapus data - Klik button Yes pada popup konfirmasi</t>
+          <t>Pilih beberapa data yang ingin dihapus dengan mencentang checkbox pada baris data - Klik button Hapus X data - Klik button Ya</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Berhasil menghapus data Program Produk.</t>
+          <t>Berhasil menghapus data Program Produk yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -9941,7 +9941,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -9973,7 +9973,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Melakukan validasi data hasil export Program Produk</t>
+          <t>Melakukan validasi data hasil export</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -9988,12 +9988,12 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Validasi data excel dengan tabel di web</t>
+          <t>Validasi data excel dengan tabel</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Data pada excel sesuai dengan tabel di web.</t>
+          <t>Data pada excel sesuai dengan data pada tabel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(mobile): harmonize module 11 test case numbering and add missing rows in excel
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -42320,7 +42320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA233"/>
+  <dimension ref="A1:AA236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50615,218 +50615,159 @@
       </c>
       <c r="D150" s="48" t="inlineStr">
         <is>
+          <t>Membuka tab Top Up data pada halaman aktifitas Marketing prospek ETB</t>
+        </is>
+      </c>
+      <c r="E150" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F150" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G150" s="48" t="inlineStr">
+        <is>
+          <t>1. Klik tab Top Up dana pada halaman aktifitas marketing Prospek ETB.</t>
+        </is>
+      </c>
+      <c r="H150" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil berpindah ke tab Top Up dana dan menampilkan form Top Up dana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>11.22</t>
+        </is>
+      </c>
+      <c r="B151" s="46" t="inlineStr">
+        <is>
+          <t>Prospek &amp; Nasabah</t>
+        </is>
+      </c>
+      <c r="C151" s="46" t="inlineStr">
+        <is>
+          <t>Aktifitas Prospek</t>
+        </is>
+      </c>
+      <c r="D151" s="48" t="inlineStr">
+        <is>
+          <t>Melakukan Submit Top Up dana dengan data valid</t>
+        </is>
+      </c>
+      <c r="E151" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F151" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G151" s="48" t="inlineStr">
+        <is>
+          <t>1. Mengisi seluruh field pada form Top Up dana dengan data valid.
+2. Klik button Submit.</t>
+        </is>
+      </c>
+      <c r="H151" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil men-submit form dan menyimpan data Top Up dana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>11.23</t>
+        </is>
+      </c>
+      <c r="B152" s="46" t="inlineStr">
+        <is>
+          <t>Prospek &amp; Nasabah</t>
+        </is>
+      </c>
+      <c r="C152" s="46" t="inlineStr">
+        <is>
+          <t>Aktifitas Prospek</t>
+        </is>
+      </c>
+      <c r="D152" s="48" t="inlineStr">
+        <is>
+          <t>Melakukan Submit Top Up dana tanpa field mandatory</t>
+        </is>
+      </c>
+      <c r="E152" s="46" t="inlineStr">
+        <is>
+          <t>Negative Case</t>
+        </is>
+      </c>
+      <c r="F152" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G152" s="48" t="inlineStr">
+        <is>
+          <t>1. Mengosongkan seluruh field mandatory pada form Top Up dana.
+2. Klik button Submit.</t>
+        </is>
+      </c>
+      <c r="H152" s="48" t="inlineStr">
+        <is>
+          <t>1. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>11.24</t>
+        </is>
+      </c>
+      <c r="B153" s="46" t="inlineStr">
+        <is>
+          <t>Prospek &amp; Nasabah</t>
+        </is>
+      </c>
+      <c r="C153" s="46" t="inlineStr">
+        <is>
+          <t>Aktifitas Prospek</t>
+        </is>
+      </c>
+      <c r="D153" s="48" t="inlineStr">
+        <is>
           <t>Membatalkan prospek melalui menu titik tiga</t>
         </is>
       </c>
-      <c r="E150" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F150" s="46" t="inlineStr">
+      <c r="E153" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F153" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G150" s="48" t="inlineStr">
+      <c r="G153" s="48" t="inlineStr">
         <is>
           <t>1. Klik menu titik tiga pada pojok kanan atas.
 2. Pilih Batalkan Prospek.
 3. Klik button Batalkan pada pop-up konfirmasi.</t>
         </is>
       </c>
-      <c r="H150" s="48" t="inlineStr">
+      <c r="H153" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu dropdown.
 2. Berhasil menampilkan pop-up konfirmasi pembatalan.
 3. Berhasil membatalkan prospek dan prospek tidak dapat dilanjutkan kembali.</t>
-        </is>
-      </c>
-      <c r="I150" s="49" t="n"/>
-      <c r="J150" s="49" t="n"/>
-      <c r="K150" s="49" t="n"/>
-      <c r="L150" s="49" t="n"/>
-      <c r="M150" s="49" t="n"/>
-      <c r="N150" s="49" t="n"/>
-      <c r="O150" s="49" t="n"/>
-      <c r="P150" s="49" t="n"/>
-      <c r="Q150" s="49" t="n"/>
-      <c r="R150" s="49" t="n"/>
-      <c r="S150" s="49" t="n"/>
-      <c r="T150" s="49" t="n"/>
-      <c r="U150" s="49" t="n"/>
-      <c r="V150" s="49" t="n"/>
-      <c r="W150" s="49" t="n"/>
-      <c r="X150" s="49" t="n"/>
-      <c r="Y150" s="49" t="n"/>
-      <c r="Z150" s="49" t="n"/>
-      <c r="AA150" s="49" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>12.1</t>
-        </is>
-      </c>
-      <c r="B151" s="46" t="inlineStr">
-        <is>
-          <t>Prospek &amp; Nasabah</t>
-        </is>
-      </c>
-      <c r="C151" s="46" t="inlineStr">
-        <is>
-          <t>Input Prospek</t>
-        </is>
-      </c>
-      <c r="D151" s="48" t="inlineStr">
-        <is>
-          <t>Membuka halaman Input Prospek melalui navigation bar bawah</t>
-        </is>
-      </c>
-      <c r="E151" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F151" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G151" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik menu Input pada navigation bar bawah.</t>
-        </is>
-      </c>
-      <c r="H151" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil membuka halaman Input Prospek dan menampilkan pop up tipe prospek.</t>
-        </is>
-      </c>
-      <c r="I151" s="49" t="n"/>
-      <c r="J151" s="49" t="n"/>
-      <c r="K151" s="49" t="n"/>
-      <c r="L151" s="49" t="n"/>
-      <c r="M151" s="49" t="n"/>
-      <c r="N151" s="49" t="n"/>
-      <c r="O151" s="49" t="n"/>
-      <c r="P151" s="49" t="n"/>
-      <c r="Q151" s="49" t="n"/>
-      <c r="R151" s="49" t="n"/>
-      <c r="S151" s="49" t="n"/>
-      <c r="T151" s="49" t="n"/>
-      <c r="U151" s="49" t="n"/>
-      <c r="V151" s="49" t="n"/>
-      <c r="W151" s="49" t="n"/>
-      <c r="X151" s="49" t="n"/>
-      <c r="Y151" s="49" t="n"/>
-      <c r="Z151" s="49" t="n"/>
-      <c r="AA151" s="49" t="n"/>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>12.2</t>
-        </is>
-      </c>
-      <c r="B152" s="46" t="inlineStr">
-        <is>
-          <t>Prospek &amp; Nasabah</t>
-        </is>
-      </c>
-      <c r="C152" s="46" t="inlineStr">
-        <is>
-          <t>Input Prospek</t>
-        </is>
-      </c>
-      <c r="D152" s="48" t="inlineStr">
-        <is>
-          <t>Membuka halaman Input Prospek melalui menu Lainnya</t>
-        </is>
-      </c>
-      <c r="E152" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F152" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G152" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik menu Lainnya pada navigation bar bawah.
-2. Klik menu Input Prospek.</t>
-        </is>
-      </c>
-      <c r="H152" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil membuka halaman Input Prospek dan menampilkan pop up tipe prospek.</t>
-        </is>
-      </c>
-      <c r="I152" s="49" t="n"/>
-      <c r="J152" s="49" t="n"/>
-      <c r="K152" s="49" t="n"/>
-      <c r="L152" s="49" t="n"/>
-      <c r="M152" s="49" t="n"/>
-      <c r="N152" s="49" t="n"/>
-      <c r="O152" s="49" t="n"/>
-      <c r="P152" s="49" t="n"/>
-      <c r="Q152" s="49" t="n"/>
-      <c r="R152" s="49" t="n"/>
-      <c r="S152" s="49" t="n"/>
-      <c r="T152" s="49" t="n"/>
-      <c r="U152" s="49" t="n"/>
-      <c r="V152" s="49" t="n"/>
-      <c r="W152" s="49" t="n"/>
-      <c r="X152" s="49" t="n"/>
-      <c r="Y152" s="49" t="n"/>
-      <c r="Z152" s="49" t="n"/>
-      <c r="AA152" s="49" t="n"/>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>12.3</t>
-        </is>
-      </c>
-      <c r="B153" s="46" t="inlineStr">
-        <is>
-          <t>Prospek &amp; Nasabah</t>
-        </is>
-      </c>
-      <c r="C153" s="46" t="inlineStr">
-        <is>
-          <t>Input Prospek</t>
-        </is>
-      </c>
-      <c r="D153" s="48" t="inlineStr">
-        <is>
-          <t>Memilih tipe Prospek Individu</t>
-        </is>
-      </c>
-      <c r="E153" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F153" s="46" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G153" s="48" t="inlineStr">
-        <is>
-          <t>1. Buka halaman Input Prospek.
-2. Klik pilihan Individu.</t>
-        </is>
-      </c>
-      <c r="H153" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil membuka halaman Input Prospek.
-2. Berhasil menampilkan form Step 1 Informasi.</t>
         </is>
       </c>
       <c r="I153" s="49" t="n"/>
@@ -50852,7 +50793,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="B154" s="46" t="inlineStr">
@@ -50867,7 +50808,7 @@
       </c>
       <c r="D154" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 1 (Informasi) dengan data valid</t>
+          <t>Membuka halaman Input Prospek melalui navigation bar bawah</t>
         </is>
       </c>
       <c r="E154" s="46" t="inlineStr">
@@ -50882,16 +50823,12 @@
       </c>
       <c r="G154" s="48" t="inlineStr">
         <is>
-          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
-2. Mengisi seluruh field pada Step 1 Informasi dengan data valid.
-3. Klik button Next.</t>
+          <t>1. Klik menu Input pada navigation bar bawah.</t>
         </is>
       </c>
       <c r="H154" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form Step 1 Informasi.
-2. Berhasil mengisi data pada Step 1 Informasi.
-3. Berhasil menyimpan data Step 1 dan berpindah ke Step 2 Data Pribadi.</t>
+          <t>1. Berhasil membuka halaman Input Prospek dan menampilkan pop up tipe prospek.</t>
         </is>
       </c>
       <c r="I154" s="49" t="n"/>
@@ -50917,7 +50854,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="B155" s="46" t="inlineStr">
@@ -50932,31 +50869,29 @@
       </c>
       <c r="D155" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 1 (Informasi) tanpa field mandatory</t>
+          <t>Membuka halaman Input Prospek melalui menu Lainnya</t>
         </is>
       </c>
       <c r="E155" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F155" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G155" s="48" t="inlineStr">
         <is>
-          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
-2. Mengosongkan field Nama Lengkap dan No. Telepon.
-3. Klik button Next.</t>
+          <t>1. Klik menu Lainnya pada navigation bar bawah.
+2. Klik menu Input Prospek.</t>
         </is>
       </c>
       <c r="H155" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form Step 1 Informasi.
-2. Berhasil mengosongkan field mandatory.
-3. Menampilkan pesan validasi bahwa field Nama Lengkap dan No. Telepon wajib diisi.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil membuka halaman Input Prospek dan menampilkan pop up tipe prospek.</t>
         </is>
       </c>
       <c r="I155" s="49" t="n"/>
@@ -50982,7 +50917,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>12.6</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="B156" s="46" t="inlineStr">
@@ -50997,7 +50932,7 @@
       </c>
       <c r="D156" s="48" t="inlineStr">
         <is>
-          <t>Melakukan Check CIF pada form Step 1</t>
+          <t>Memilih tipe Prospek Individu</t>
         </is>
       </c>
       <c r="E156" s="46" t="inlineStr">
@@ -51007,21 +50942,19 @@
       </c>
       <c r="F156" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G156" s="48" t="inlineStr">
         <is>
-          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
-2. Isi field No KTP dengan nomor KTP valid.
-3. Klik button Check CIF.</t>
+          <t>1. Buka halaman Input Prospek.
+2. Klik pilihan Individu.</t>
         </is>
       </c>
       <c r="H156" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form Step 1 Informasi.
-2. Berhasil mengisi field No KTP.
-3. Berhasil menampilkan hasil Check CIF berdasarkan No KTP.</t>
+          <t>1. Berhasil membuka halaman Input Prospek.
+2. Berhasil menampilkan form Step 1 Informasi.</t>
         </is>
       </c>
       <c r="I156" s="49" t="n"/>
@@ -51047,7 +50980,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>12.7</t>
+          <t>12.4</t>
         </is>
       </c>
       <c r="B157" s="46" t="inlineStr">
@@ -51062,7 +50995,7 @@
       </c>
       <c r="D157" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 2 (Data Pribadi) dengan data valid</t>
+          <t>Mengisi form Step 1 (Informasi) dengan data valid</t>
         </is>
       </c>
       <c r="E157" s="46" t="inlineStr">
@@ -51077,14 +51010,16 @@
       </c>
       <c r="G157" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada Step 2 Data Pribadi dengan data valid.
-2. Klik button Next.</t>
+          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
+2. Mengisi seluruh field pada Step 1 Informasi dengan data valid.
+3. Klik button Next.</t>
         </is>
       </c>
       <c r="H157" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada Step 2 Data Pribadi.
-2. Berhasil menyimpan data Step 2 dan berpindah ke Step 3 Pekerjaan.</t>
+          <t>1. Berhasil menampilkan form Step 1 Informasi.
+2. Berhasil mengisi data pada Step 1 Informasi.
+3. Berhasil menyimpan data Step 1 dan berpindah ke Step 2 Data Pribadi.</t>
         </is>
       </c>
       <c r="I157" s="49" t="n"/>
@@ -51110,7 +51045,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12.8</t>
+          <t>12.5</t>
         </is>
       </c>
       <c r="B158" s="46" t="inlineStr">
@@ -51125,29 +51060,31 @@
       </c>
       <c r="D158" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 3 (Pekerjaan) dengan data valid</t>
+          <t>Mengisi form Step 1 (Informasi) tanpa field mandatory</t>
         </is>
       </c>
       <c r="E158" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F158" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G158" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada Step 3 Pekerjaan dengan data valid.
-2. Klik button Next.</t>
+          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
+2. Mengosongkan field Nama Lengkap dan No. Telepon.
+3. Klik button Next.</t>
         </is>
       </c>
       <c r="H158" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada Step 3 Pekerjaan.
-2. Berhasil menyimpan data Step 3 dan berpindah ke Step 4 Prospek.</t>
+          <t>1. Berhasil menampilkan form Step 1 Informasi.
+2. Berhasil mengosongkan field mandatory.
+3. Menampilkan pesan validasi bahwa field Nama Lengkap dan No. Telepon wajib diisi.</t>
         </is>
       </c>
       <c r="I158" s="49" t="n"/>
@@ -51173,7 +51110,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>12.6</t>
         </is>
       </c>
       <c r="B159" s="46" t="inlineStr">
@@ -51188,7 +51125,7 @@
       </c>
       <c r="D159" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 4 (Prospek) NTB dengan data valid</t>
+          <t>Melakukan Check CIF pada form Step 1</t>
         </is>
       </c>
       <c r="E159" s="46" t="inlineStr">
@@ -51198,19 +51135,21 @@
       </c>
       <c r="F159" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G159" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada Step 4 Prospek dengan data valid.
-2. Klik button Submit.</t>
+          <t>1. Buka form Input Prospek Individu (Step 1 Informasi).
+2. Isi field No KTP dengan nomor KTP valid.
+3. Klik button Check CIF.</t>
         </is>
       </c>
       <c r="H159" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada Step 4 Prospek.
-2. Berhasil menyimpan data prospek Individu NTB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
+          <t>1. Berhasil menampilkan form Step 1 Informasi.
+2. Berhasil mengisi field No KTP.
+3. Berhasil menampilkan hasil Check CIF berdasarkan No KTP.</t>
         </is>
       </c>
       <c r="I159" s="49" t="n"/>
@@ -51236,7 +51175,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12.10</t>
+          <t>12.7</t>
         </is>
       </c>
       <c r="B160" s="46" t="inlineStr">
@@ -51251,7 +51190,7 @@
       </c>
       <c r="D160" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 4 (Prospek) ETB dengan mengubah status NTB</t>
+          <t>Mengisi form Step 2 (Data Pribadi) dengan data valid</t>
         </is>
       </c>
       <c r="E160" s="46" t="inlineStr">
@@ -51266,18 +51205,14 @@
       </c>
       <c r="G160" s="48" t="inlineStr">
         <is>
-          <t>1. Aktifkan toggle Ubah NTB ke ETB.
-2. Isi field No CIF.
-3. Mengisi seluruh field pada Step 4 Prospek dengan data valid.
-4. Klik button Submit.</t>
+          <t>1. Mengisi seluruh field pada Step 2 Data Pribadi dengan data valid.
+2. Klik button Next.</t>
         </is>
       </c>
       <c r="H160" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengaktifkan toggle NTB ke ETB.
-2. Berhasil mengisi No CIF.
-3. Berhasil mengisi data pada Step 4 Prospek.
-4. Berhasil menyimpan data prospek Individu ETB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
+          <t>1. Berhasil mengisi data pada Step 2 Data Pribadi.
+2. Berhasil menyimpan data Step 2 dan berpindah ke Step 3 Pekerjaan.</t>
         </is>
       </c>
       <c r="I160" s="49" t="n"/>
@@ -51303,7 +51238,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12.11</t>
+          <t>12.8</t>
         </is>
       </c>
       <c r="B161" s="46" t="inlineStr">
@@ -51318,29 +51253,29 @@
       </c>
       <c r="D161" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 4 (Prospek) tanpa field mandatory</t>
+          <t>Mengisi form Step 3 (Pekerjaan) dengan data valid</t>
         </is>
       </c>
       <c r="E161" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F161" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G161" s="48" t="inlineStr">
         <is>
-          <t>1. Mengosongkan seluruh field mandatory pada Step 4 Prospek.
-2. Klik button Submit.</t>
+          <t>1. Mengisi seluruh field pada Step 3 Pekerjaan dengan data valid.
+2. Klik button Next.</t>
         </is>
       </c>
       <c r="H161" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengosongkan field mandatory.
-2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
+          <t>1. Berhasil mengisi data pada Step 3 Pekerjaan.
+2. Berhasil menyimpan data Step 3 dan berpindah ke Step 4 Prospek.</t>
         </is>
       </c>
       <c r="I161" s="49" t="n"/>
@@ -51366,7 +51301,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12.12</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="B162" s="46" t="inlineStr">
@@ -51381,7 +51316,7 @@
       </c>
       <c r="D162" s="48" t="inlineStr">
         <is>
-          <t>Navigasi ke halaman Aktifitas dari layar konfirmasi Prospek Berhasil Dibuat</t>
+          <t>Mengisi form Step 4 (Prospek) NTB dengan data valid</t>
         </is>
       </c>
       <c r="E162" s="46" t="inlineStr">
@@ -51396,12 +51331,14 @@
       </c>
       <c r="G162" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button Lihat Aktifitas.</t>
+          <t>1. Mengisi seluruh field pada Step 4 Prospek dengan data valid.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H162" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengarahkan pengguna ke halaman Lead Qualification Aktifitas.</t>
+          <t>1. Berhasil mengisi data pada Step 4 Prospek.
+2. Berhasil menyimpan data prospek Individu NTB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
         </is>
       </c>
       <c r="I162" s="49" t="n"/>
@@ -51427,7 +51364,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>12.13</t>
+          <t>12.10</t>
         </is>
       </c>
       <c r="B163" s="46" t="inlineStr">
@@ -51442,7 +51379,7 @@
       </c>
       <c r="D163" s="48" t="inlineStr">
         <is>
-          <t>Kembali ke halaman utama dari layar konfirmasi Prospek Berhasil Dibuat</t>
+          <t>Mengisi form Step 4 (Prospek) ETB dengan mengubah status NTB</t>
         </is>
       </c>
       <c r="E163" s="46" t="inlineStr">
@@ -51452,17 +51389,23 @@
       </c>
       <c r="F163" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G163" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button Kembali.</t>
+          <t>1. Aktifkan toggle Ubah NTB ke ETB.
+2. Isi field No CIF.
+3. Mengisi seluruh field pada Step 4 Prospek dengan data valid.
+4. Klik button Submit.</t>
         </is>
       </c>
       <c r="H163" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengarahkan pengguna kembali ke halaman utama / form input.</t>
+          <t>1. Berhasil mengaktifkan toggle NTB ke ETB.
+2. Berhasil mengisi No CIF.
+3. Berhasil mengisi data pada Step 4 Prospek.
+4. Berhasil menyimpan data prospek Individu ETB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
         </is>
       </c>
       <c r="I163" s="49" t="n"/>
@@ -51488,7 +51431,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>12.14</t>
+          <t>12.11</t>
         </is>
       </c>
       <c r="B164" s="46" t="inlineStr">
@@ -51503,29 +51446,29 @@
       </c>
       <c r="D164" s="48" t="inlineStr">
         <is>
-          <t>Memilih tipe Prospek Lembaga</t>
+          <t>Mengisi form Step 4 (Prospek) tanpa field mandatory</t>
         </is>
       </c>
       <c r="E164" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F164" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G164" s="48" t="inlineStr">
         <is>
-          <t>1. Buka halaman Input Prospek.
-2. Klik pilihan Lembaga.</t>
+          <t>1. Mengosongkan seluruh field mandatory pada Step 4 Prospek.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H164" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka halaman Input Prospek.
-2. Berhasil menampilkan form Step 1 Informasi Lembaga.</t>
+          <t>1. Berhasil mengosongkan field mandatory.
+2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
         </is>
       </c>
       <c r="I164" s="49" t="n"/>
@@ -51551,7 +51494,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>12.15</t>
+          <t>12.12</t>
         </is>
       </c>
       <c r="B165" s="46" t="inlineStr">
@@ -51566,7 +51509,7 @@
       </c>
       <c r="D165" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 1 (Informasi Lembaga) dengan data valid</t>
+          <t>Navigasi ke halaman Aktifitas dari layar konfirmasi Prospek Berhasil Dibuat</t>
         </is>
       </c>
       <c r="E165" s="46" t="inlineStr">
@@ -51581,16 +51524,12 @@
       </c>
       <c r="G165" s="48" t="inlineStr">
         <is>
-          <t>1. Buka form Input Prospek Lembaga (Step 1 Informasi Lembaga).
-2. Mengisi field NPWP dengan NPWP valid.
-3. Klik button Next.</t>
+          <t>1. Klik button Lihat Aktifitas.</t>
         </is>
       </c>
       <c r="H165" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan form Step 1 Informasi Lembaga.
-2. Berhasil mengisi field NPWP.
-3. Berhasil menyimpan data Step 1 dan berpindah ke Step 2 Data Lembaga.</t>
+          <t>1. Berhasil mengarahkan pengguna ke halaman Lead Qualification Aktifitas.</t>
         </is>
       </c>
       <c r="I165" s="49" t="n"/>
@@ -51616,7 +51555,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12.16</t>
+          <t>12.13</t>
         </is>
       </c>
       <c r="B166" s="46" t="inlineStr">
@@ -51631,7 +51570,7 @@
       </c>
       <c r="D166" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 2 (Data Lembaga) dengan data valid</t>
+          <t>Kembali ke halaman utama dari layar konfirmasi Prospek Berhasil Dibuat</t>
         </is>
       </c>
       <c r="E166" s="46" t="inlineStr">
@@ -51641,19 +51580,17 @@
       </c>
       <c r="F166" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G166" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada Step 2 Data Lembaga dengan data valid.
-2. Klik button Next.</t>
+          <t>1. Klik button Kembali.</t>
         </is>
       </c>
       <c r="H166" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada Step 2 Data Lembaga.
-2. Berhasil menyimpan data Step 2 dan berpindah ke Step 3 Prospek.</t>
+          <t>1. Berhasil mengarahkan pengguna kembali ke halaman utama / form input.</t>
         </is>
       </c>
       <c r="I166" s="49" t="n"/>
@@ -51679,7 +51616,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12.17</t>
+          <t>12.14</t>
         </is>
       </c>
       <c r="B167" s="46" t="inlineStr">
@@ -51694,29 +51631,29 @@
       </c>
       <c r="D167" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 2 (Data Lembaga) tanpa field mandatory</t>
+          <t>Memilih tipe Prospek Lembaga</t>
         </is>
       </c>
       <c r="E167" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F167" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G167" s="48" t="inlineStr">
         <is>
-          <t>1. Mengosongkan field Nama Perusahaan dan Telepon Perusahaan.
-2. Klik button Next.</t>
+          <t>1. Buka halaman Input Prospek.
+2. Klik pilihan Lembaga.</t>
         </is>
       </c>
       <c r="H167" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengosongkan field mandatory.
-2. Menampilkan pesan validasi bahwa field Nama Perusahaan dan Telepon Perusahaan wajib diisi.</t>
+          <t>1. Berhasil membuka halaman Input Prospek.
+2. Berhasil menampilkan form Step 1 Informasi Lembaga.</t>
         </is>
       </c>
       <c r="I167" s="49" t="n"/>
@@ -51742,7 +51679,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>12.18</t>
+          <t>12.15</t>
         </is>
       </c>
       <c r="B168" s="46" t="inlineStr">
@@ -51757,7 +51694,7 @@
       </c>
       <c r="D168" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 3 (Prospek Lembaga) NTB dengan data valid</t>
+          <t>Mengisi form Step 1 (Informasi Lembaga) dengan data valid</t>
         </is>
       </c>
       <c r="E168" s="46" t="inlineStr">
@@ -51772,14 +51709,16 @@
       </c>
       <c r="G168" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada Step 3 Prospek Lembaga dengan data valid.
-2. Klik button Submit.</t>
+          <t>1. Buka form Input Prospek Lembaga (Step 1 Informasi Lembaga).
+2. Mengisi field NPWP dengan NPWP valid.
+3. Klik button Next.</t>
         </is>
       </c>
       <c r="H168" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada Step 3 Prospek Lembaga.
-2. Berhasil menyimpan data prospek Lembaga NTB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
+          <t>1. Berhasil menampilkan form Step 1 Informasi Lembaga.
+2. Berhasil mengisi field NPWP.
+3. Berhasil menyimpan data Step 1 dan berpindah ke Step 2 Data Lembaga.</t>
         </is>
       </c>
       <c r="I168" s="49" t="n"/>
@@ -51805,7 +51744,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>12.19</t>
+          <t>12.16</t>
         </is>
       </c>
       <c r="B169" s="46" t="inlineStr">
@@ -51820,7 +51759,7 @@
       </c>
       <c r="D169" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 3 (Prospek Lembaga) ETB dengan mengubah status NTB</t>
+          <t>Mengisi form Step 2 (Data Lembaga) dengan data valid</t>
         </is>
       </c>
       <c r="E169" s="46" t="inlineStr">
@@ -51835,18 +51774,14 @@
       </c>
       <c r="G169" s="48" t="inlineStr">
         <is>
-          <t>1. Aktifkan toggle Ubah NTB ke ETB.
-2. Isi field No CIF.
-3. Mengisi seluruh field pada Step 3 Prospek Lembaga dengan data valid.
-4. Klik button Submit.</t>
+          <t>1. Mengisi seluruh field pada Step 2 Data Lembaga dengan data valid.
+2. Klik button Next.</t>
         </is>
       </c>
       <c r="H169" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengaktifkan toggle NTB ke ETB.
-2. Berhasil mengisi No CIF.
-3. Berhasil mengisi data pada Step 3 Prospek Lembaga.
-4. Berhasil menyimpan data prospek Lembaga ETB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
+          <t>1. Berhasil mengisi data pada Step 2 Data Lembaga.
+2. Berhasil menyimpan data Step 2 dan berpindah ke Step 3 Prospek.</t>
         </is>
       </c>
       <c r="I169" s="49" t="n"/>
@@ -51872,7 +51807,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>12.20</t>
+          <t>12.17</t>
         </is>
       </c>
       <c r="B170" s="46" t="inlineStr">
@@ -51887,7 +51822,7 @@
       </c>
       <c r="D170" s="48" t="inlineStr">
         <is>
-          <t>Mengisi form Step 3 (Prospek Lembaga) tanpa field mandatory</t>
+          <t>Mengisi form Step 2 (Data Lembaga) tanpa field mandatory</t>
         </is>
       </c>
       <c r="E170" s="46" t="inlineStr">
@@ -51902,14 +51837,14 @@
       </c>
       <c r="G170" s="48" t="inlineStr">
         <is>
-          <t>1. Mengosongkan seluruh field mandatory pada Step 3 Prospek Lembaga.
-2. Klik button Submit.</t>
+          <t>1. Mengosongkan field Nama Perusahaan dan Telepon Perusahaan.
+2. Klik button Next.</t>
         </is>
       </c>
       <c r="H170" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil mengosongkan field mandatory.
-2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
+2. Menampilkan pesan validasi bahwa field Nama Perusahaan dan Telepon Perusahaan wajib diisi.</t>
         </is>
       </c>
       <c r="I170" s="49" t="n"/>
@@ -51935,7 +51870,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>12.18</t>
         </is>
       </c>
       <c r="B171" s="46" t="inlineStr">
@@ -51945,12 +51880,12 @@
       </c>
       <c r="C171" s="46" t="inlineStr">
         <is>
-          <t>List Nasabah ETB</t>
+          <t>Input Prospek</t>
         </is>
       </c>
       <c r="D171" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman List Nasabah ETB</t>
+          <t>Mengisi form Step 3 (Prospek Lembaga) NTB dengan data valid</t>
         </is>
       </c>
       <c r="E171" s="46" t="inlineStr">
@@ -51965,14 +51900,14 @@
       </c>
       <c r="G171" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu List Nasabah ETB.</t>
+          <t>1. Mengisi seluruh field pada Step 3 Prospek Lembaga dengan data valid.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H171" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman List Nasabah ETB.</t>
+          <t>1. Berhasil mengisi data pada Step 3 Prospek Lembaga.
+2. Berhasil menyimpan data prospek Lembaga NTB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
         </is>
       </c>
       <c r="I171" s="49" t="n"/>
@@ -51998,7 +51933,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>12.19</t>
         </is>
       </c>
       <c r="B172" s="46" t="inlineStr">
@@ -52008,12 +51943,12 @@
       </c>
       <c r="C172" s="46" t="inlineStr">
         <is>
-          <t>List Nasabah ETB</t>
+          <t>Input Prospek</t>
         </is>
       </c>
       <c r="D172" s="48" t="inlineStr">
         <is>
-          <t>Mencari nasabah menggunakan Search Bar</t>
+          <t>Mengisi form Step 3 (Prospek Lembaga) ETB dengan mengubah status NTB</t>
         </is>
       </c>
       <c r="E172" s="46" t="inlineStr">
@@ -52028,12 +51963,18 @@
       </c>
       <c r="G172" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
+          <t>1. Aktifkan toggle Ubah NTB ke ETB.
+2. Isi field No CIF.
+3. Mengisi seluruh field pada Step 3 Prospek Lembaga dengan data valid.
+4. Klik button Submit.</t>
         </is>
       </c>
       <c r="H172" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data nasabah yang sesuai dengan kata kunci pencarian.</t>
+          <t>1. Berhasil mengaktifkan toggle NTB ke ETB.
+2. Berhasil mengisi No CIF.
+3. Berhasil mengisi data pada Step 3 Prospek Lembaga.
+4. Berhasil menyimpan data prospek Lembaga ETB dan menampilkan layar konfirmasi Prospek Berhasil Dibuat.</t>
         </is>
       </c>
       <c r="I172" s="49" t="n"/>
@@ -52059,7 +52000,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>12.20</t>
         </is>
       </c>
       <c r="B173" s="46" t="inlineStr">
@@ -52069,12 +52010,12 @@
       </c>
       <c r="C173" s="46" t="inlineStr">
         <is>
-          <t>List Nasabah ETB</t>
+          <t>Input Prospek</t>
         </is>
       </c>
       <c r="D173" s="48" t="inlineStr">
         <is>
-          <t>Mencari nasabah dengan keyword tidak valid</t>
+          <t>Mengisi form Step 3 (Prospek Lembaga) tanpa field mandatory</t>
         </is>
       </c>
       <c r="E173" s="46" t="inlineStr">
@@ -52089,12 +52030,14 @@
       </c>
       <c r="G173" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
+          <t>1. Mengosongkan seluruh field mandatory pada Step 3 Prospek Lembaga.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H173" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>1. Berhasil mengosongkan field mandatory.
+2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
         </is>
       </c>
       <c r="I173" s="49" t="n"/>
@@ -52120,7 +52063,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>13.4</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="B174" s="46" t="inlineStr">
@@ -52135,7 +52078,7 @@
       </c>
       <c r="D174" s="48" t="inlineStr">
         <is>
-          <t>Melakukan filter data nasabah</t>
+          <t>Membuka halaman List Nasabah ETB</t>
         </is>
       </c>
       <c r="E174" s="46" t="inlineStr">
@@ -52150,16 +52093,14 @@
       </c>
       <c r="G174" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button Filter di halaman List Nasabah ETB.
-2. Pilih kriteria filter pada form Filter.
-3. Klik button Simpan.</t>
+          <t>1. Buka menu Lainnya.
+2. Klik menu List Nasabah ETB.</t>
         </is>
       </c>
       <c r="H174" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Filter.
-2. Berhasil memilih kriteria filter.
-3. Berhasil menampilkan daftar nasabah yang sesuai dengan kriteria filter.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman List Nasabah ETB.</t>
         </is>
       </c>
       <c r="I174" s="49" t="n"/>
@@ -52185,7 +52126,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>13.2</t>
         </is>
       </c>
       <c r="B175" s="46" t="inlineStr">
@@ -52200,7 +52141,7 @@
       </c>
       <c r="D175" s="48" t="inlineStr">
         <is>
-          <t>Melihat Detail Prospek Nasabah ETB</t>
+          <t>Mencari nasabah menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E175" s="46" t="inlineStr">
@@ -52215,14 +52156,12 @@
       </c>
       <c r="G175" s="48" t="inlineStr">
         <is>
-          <t>1. Klik menu titik tiga pada salah satu card nasabah.
-2. Pilih Detail Prospek.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H175" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan menu Lainnya.
-2. Berhasil membuka halaman Detail Prospek dan menampilkan informasi nasabah secara lengkap.</t>
+          <t>1. Berhasil menampilkan data nasabah yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I175" s="49" t="n"/>
@@ -52248,7 +52187,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>13.6</t>
+          <t>13.3</t>
         </is>
       </c>
       <c r="B176" s="46" t="inlineStr">
@@ -52263,12 +52202,12 @@
       </c>
       <c r="D176" s="48" t="inlineStr">
         <is>
-          <t>Membuka form Prospek Ulang</t>
+          <t>Mencari nasabah dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E176" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F176" s="46" t="inlineStr">
@@ -52278,14 +52217,12 @@
       </c>
       <c r="G176" s="48" t="inlineStr">
         <is>
-          <t>1. Klik menu titik tiga pada salah satu card nasabah.
-2. Pilih Prospek Ulang.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H176" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan menu Lainnya.
-2. Berhasil membuka form Prospek Ulang.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I176" s="49" t="n"/>
@@ -52311,7 +52248,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>13.4</t>
         </is>
       </c>
       <c r="B177" s="46" t="inlineStr">
@@ -52326,7 +52263,7 @@
       </c>
       <c r="D177" s="48" t="inlineStr">
         <is>
-          <t>Melakukan Prospek Ulang dengan data valid</t>
+          <t>Melakukan filter data nasabah</t>
         </is>
       </c>
       <c r="E177" s="46" t="inlineStr">
@@ -52341,14 +52278,16 @@
       </c>
       <c r="G177" s="48" t="inlineStr">
         <is>
-          <t>1. Mengisi seluruh field pada form Prospek Ulang dengan data valid.
-2. Klik button Submit.</t>
+          <t>1. Klik button Filter di halaman List Nasabah ETB.
+2. Pilih kriteria filter pada form Filter.
+3. Klik button Simpan.</t>
         </is>
       </c>
       <c r="H177" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengisi data pada form Prospek Ulang.
-2. Berhasil men-submit form dan memperbarui data prospek.</t>
+          <t>1. Berhasil membuka form Filter.
+2. Berhasil memilih kriteria filter.
+3. Berhasil menampilkan daftar nasabah yang sesuai dengan kriteria filter.</t>
         </is>
       </c>
       <c r="I177" s="49" t="n"/>
@@ -52374,7 +52313,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="B178" s="46" t="inlineStr">
@@ -52389,29 +52328,29 @@
       </c>
       <c r="D178" s="48" t="inlineStr">
         <is>
-          <t>Melakukan Prospek Ulang tanpa field mandatory</t>
+          <t>Melihat Detail Prospek Nasabah ETB</t>
         </is>
       </c>
       <c r="E178" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F178" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G178" s="48" t="inlineStr">
         <is>
-          <t>1. Mengosongkan seluruh field mandatory pada form Prospek Ulang.
-2. Klik button Submit.</t>
+          <t>1. Klik menu titik tiga pada salah satu card nasabah.
+2. Pilih Detail Prospek.</t>
         </is>
       </c>
       <c r="H178" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengosongkan field mandatory.
-2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
+          <t>1. Berhasil menampilkan menu Lainnya.
+2. Berhasil membuka halaman Detail Prospek dan menampilkan informasi nasabah secara lengkap.</t>
         </is>
       </c>
       <c r="I178" s="49" t="n"/>
@@ -52437,7 +52376,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13.9</t>
+          <t>13.6</t>
         </is>
       </c>
       <c r="B179" s="46" t="inlineStr">
@@ -52452,7 +52391,7 @@
       </c>
       <c r="D179" s="48" t="inlineStr">
         <is>
-          <t>Melihat Informasi Rekening</t>
+          <t>Membuka form Prospek Ulang</t>
         </is>
       </c>
       <c r="E179" s="46" t="inlineStr">
@@ -52462,19 +52401,19 @@
       </c>
       <c r="F179" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G179" s="48" t="inlineStr">
         <is>
           <t>1. Klik menu titik tiga pada salah satu card nasabah.
-2. Pilih Informasi Rekening.</t>
+2. Pilih Prospek Ulang.</t>
         </is>
       </c>
       <c r="H179" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan menu Lainnya.
-2. Berhasil menampilkan detail rekening nasabah (nomor rekening dan saldo).</t>
+2. Berhasil membuka form Prospek Ulang.</t>
         </is>
       </c>
       <c r="I179" s="49" t="n"/>
@@ -52500,7 +52439,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>13.10</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="B180" s="46" t="inlineStr">
@@ -52515,7 +52454,7 @@
       </c>
       <c r="D180" s="48" t="inlineStr">
         <is>
-          <t>Menghapus data nasabah</t>
+          <t>Melakukan Prospek Ulang dengan data valid</t>
         </is>
       </c>
       <c r="E180" s="46" t="inlineStr">
@@ -52530,16 +52469,14 @@
       </c>
       <c r="G180" s="48" t="inlineStr">
         <is>
-          <t>1. Klik menu titik tiga pada salah satu card nasabah.
-2. Pilih Hapus.
-3. Klik button Ya pada pop-up konfirmasi.</t>
+          <t>1. Mengisi seluruh field pada form Prospek Ulang dengan data valid.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H180" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan menu Lainnya.
-2. Berhasil menampilkan pop-up konfirmasi hapus data.
-3. Berhasil menghapus data nasabah dari daftar List Nasabah ETB.</t>
+          <t>1. Berhasil mengisi data pada form Prospek Ulang.
+2. Berhasil men-submit form dan memperbarui data prospek.</t>
         </is>
       </c>
       <c r="I180" s="49" t="n"/>
@@ -52565,7 +52502,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="B181" s="46" t="inlineStr">
@@ -52575,34 +52512,34 @@
       </c>
       <c r="C181" s="46" t="inlineStr">
         <is>
-          <t>Nasabah Referal</t>
+          <t>List Nasabah ETB</t>
         </is>
       </c>
       <c r="D181" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Nasabah Referal</t>
+          <t>Melakukan Prospek Ulang tanpa field mandatory</t>
         </is>
       </c>
       <c r="E181" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F181" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G181" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Nasabah Referal.</t>
+          <t>1. Mengosongkan seluruh field mandatory pada form Prospek Ulang.
+2. Klik button Submit.</t>
         </is>
       </c>
       <c r="H181" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Nasabah Referal.</t>
+          <t>1. Berhasil mengosongkan field mandatory.
+2. Menampilkan pesan validasi bahwa field mandatory wajib diisi.</t>
         </is>
       </c>
       <c r="I181" s="49" t="n"/>
@@ -52628,7 +52565,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>14.2</t>
+          <t>13.9</t>
         </is>
       </c>
       <c r="B182" s="46" t="inlineStr">
@@ -52638,12 +52575,12 @@
       </c>
       <c r="C182" s="46" t="inlineStr">
         <is>
-          <t>Nasabah Referal</t>
+          <t>List Nasabah ETB</t>
         </is>
       </c>
       <c r="D182" s="48" t="inlineStr">
         <is>
-          <t>Mencari nasabah referal menggunakan Search Bar</t>
+          <t>Melihat Informasi Rekening</t>
         </is>
       </c>
       <c r="E182" s="46" t="inlineStr">
@@ -52658,12 +52595,14 @@
       </c>
       <c r="G182" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
+          <t>1. Klik menu titik tiga pada salah satu card nasabah.
+2. Pilih Informasi Rekening.</t>
         </is>
       </c>
       <c r="H182" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data nasabah referal yang sesuai dengan kata kunci pencarian.</t>
+          <t>1. Berhasil menampilkan menu Lainnya.
+2. Berhasil menampilkan detail rekening nasabah (nomor rekening dan saldo).</t>
         </is>
       </c>
       <c r="I182" s="49" t="n"/>
@@ -52689,7 +52628,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>13.10</t>
         </is>
       </c>
       <c r="B183" s="46" t="inlineStr">
@@ -52699,32 +52638,36 @@
       </c>
       <c r="C183" s="46" t="inlineStr">
         <is>
-          <t>Nasabah Referal</t>
+          <t>List Nasabah ETB</t>
         </is>
       </c>
       <c r="D183" s="48" t="inlineStr">
         <is>
-          <t>Mencari nasabah referal dengan keyword tidak valid</t>
+          <t>Menghapus data nasabah</t>
         </is>
       </c>
       <c r="E183" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F183" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G183" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
+          <t>1. Klik menu titik tiga pada salah satu card nasabah.
+2. Pilih Hapus.
+3. Klik button Ya pada pop-up konfirmasi.</t>
         </is>
       </c>
       <c r="H183" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>1. Berhasil menampilkan menu Lainnya.
+2. Berhasil menampilkan pop-up konfirmasi hapus data.
+3. Berhasil menghapus data nasabah dari daftar List Nasabah ETB.</t>
         </is>
       </c>
       <c r="I183" s="49" t="n"/>
@@ -52750,7 +52693,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>14.4</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="B184" s="46" t="inlineStr">
@@ -52765,7 +52708,7 @@
       </c>
       <c r="D184" s="48" t="inlineStr">
         <is>
-          <t>Melihat Detail Prospek nasabah referal</t>
+          <t>Membuka halaman Nasabah Referal</t>
         </is>
       </c>
       <c r="E184" s="46" t="inlineStr">
@@ -52780,12 +52723,14 @@
       </c>
       <c r="G184" s="48" t="inlineStr">
         <is>
-          <t>1. Klik salah satu card nasabah referal.</t>
+          <t>1. Buka menu Lainnya.
+2. Klik menu Nasabah Referal.</t>
         </is>
       </c>
       <c r="H184" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail nasabah referal.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Nasabah Referal.</t>
         </is>
       </c>
       <c r="I184" s="49" t="n"/>
@@ -52811,22 +52756,22 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>15.1</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="B185" s="46" t="inlineStr">
         <is>
-          <t>Agenda</t>
+          <t>Prospek &amp; Nasabah</t>
         </is>
       </c>
       <c r="C185" s="46" t="inlineStr">
         <is>
-          <t>Pengingat</t>
+          <t>Nasabah Referal</t>
         </is>
       </c>
       <c r="D185" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Pengingat</t>
+          <t>Mencari nasabah referal menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E185" s="46" t="inlineStr">
@@ -52841,14 +52786,12 @@
       </c>
       <c r="G185" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya pada Aksi Cepat di Beranda.
-2. Klik menu Pengingat pada kelompok Agenda.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H185" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Pengingat beserta daftar tugas pada tab default (Task).</t>
+          <t>1. Berhasil menampilkan data nasabah referal yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I185" s="49" t="n"/>
@@ -52874,27 +52817,27 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>15.2</t>
+          <t>14.3</t>
         </is>
       </c>
       <c r="B186" s="46" t="inlineStr">
         <is>
-          <t>Agenda</t>
+          <t>Prospek &amp; Nasabah</t>
         </is>
       </c>
       <c r="C186" s="46" t="inlineStr">
         <is>
-          <t>Pengingat</t>
+          <t>Nasabah Referal</t>
         </is>
       </c>
       <c r="D186" s="48" t="inlineStr">
         <is>
-          <t>Melihat daftar agenda pada tab Acara</t>
+          <t>Mencari nasabah referal dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E186" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F186" s="46" t="inlineStr">
@@ -52904,13 +52847,12 @@
       </c>
       <c r="G186" s="48" t="inlineStr">
         <is>
-          <t>1. Pada halaman Pengingat, klik tab Acara.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H186" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil berpindah ke tab Acara.
-2. Berhasil menampilkan daftar acara yang terdaftar pada tab Acara.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I186" s="49" t="n"/>
@@ -52936,22 +52878,22 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>14.4</t>
         </is>
       </c>
       <c r="B187" s="46" t="inlineStr">
         <is>
-          <t>Agenda</t>
+          <t>Prospek &amp; Nasabah</t>
         </is>
       </c>
       <c r="C187" s="46" t="inlineStr">
         <is>
-          <t>Pengingat</t>
+          <t>Nasabah Referal</t>
         </is>
       </c>
       <c r="D187" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail task</t>
+          <t>Melihat Detail Prospek nasabah referal</t>
         </is>
       </c>
       <c r="E187" s="46" t="inlineStr">
@@ -52966,13 +52908,12 @@
       </c>
       <c r="G187" s="48" t="inlineStr">
         <is>
-          <t>1. Pada tab Task, klik salah satu card task yang terdaftar.</t>
+          <t>1. Klik salah satu card nasabah referal.</t>
         </is>
       </c>
       <c r="H187" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka halaman Detail Task.
-2. Berhasil menampilkan informasi status, visibilitas, prioritas, tenggat, zona waktu, pemilik, deskripsi, dan lampiran.</t>
+          <t>1. Berhasil menampilkan detail nasabah referal.</t>
         </is>
       </c>
       <c r="I187" s="49" t="n"/>
@@ -52998,7 +52939,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>15.4</t>
+          <t>15.1</t>
         </is>
       </c>
       <c r="B188" s="46" t="inlineStr">
@@ -53013,7 +52954,7 @@
       </c>
       <c r="D188" s="48" t="inlineStr">
         <is>
-          <t>Mengubah data task dengan data valid</t>
+          <t>Membuka halaman Pengingat</t>
         </is>
       </c>
       <c r="E188" s="46" t="inlineStr">
@@ -53028,15 +52969,14 @@
       </c>
       <c r="G188" s="48" t="inlineStr">
         <is>
-          <t>1. Pada halaman Detail Task, klik icon Edit (pensil).
-2. Ubah data task pada form Edit Task.
-3. Klik button Simpan.</t>
+          <t>1. Buka menu Lainnya pada Aksi Cepat di Beranda.
+2. Klik menu Pengingat pada kelompok Agenda.</t>
         </is>
       </c>
       <c r="H188" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Edit Task.
-2. Berhasil menyimpan perubahan data task dengan data yang valid.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Pengingat beserta daftar tugas pada tab default (Task).</t>
         </is>
       </c>
       <c r="I188" s="49" t="n"/>
@@ -53062,7 +53002,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>15.5</t>
+          <t>15.2</t>
         </is>
       </c>
       <c r="B189" s="46" t="inlineStr">
@@ -53077,7 +53017,7 @@
       </c>
       <c r="D189" s="48" t="inlineStr">
         <is>
-          <t>Membagikan task kepada user</t>
+          <t>Melihat daftar agenda pada tab Acara</t>
         </is>
       </c>
       <c r="E189" s="46" t="inlineStr">
@@ -53087,20 +53027,18 @@
       </c>
       <c r="F189" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G189" s="48" t="inlineStr">
         <is>
-          <t>1. Pada halaman Detail Task, klik icon Bagikan (share).
-2. Pilih role atau user yang ditugaskan.
-3. Klik button Bagikan.</t>
+          <t>1. Pada halaman Pengingat, klik tab Acara.</t>
         </is>
       </c>
       <c r="H189" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Bagikan Task.
-2. Berhasil membagikan task kepada user dan menampilkan pesan konfirmasi Task berhasil dibagikan.</t>
+          <t>1. Berhasil berpindah ke tab Acara.
+2. Berhasil menampilkan daftar acara yang terdaftar pada tab Acara.</t>
         </is>
       </c>
       <c r="I189" s="49" t="n"/>
@@ -53126,7 +53064,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>15.3</t>
         </is>
       </c>
       <c r="B190" s="46" t="inlineStr">
@@ -53141,7 +53079,7 @@
       </c>
       <c r="D190" s="48" t="inlineStr">
         <is>
-          <t>Menghapus penugasan task kepada user</t>
+          <t>Melihat detail task</t>
         </is>
       </c>
       <c r="E190" s="46" t="inlineStr">
@@ -53156,15 +53094,13 @@
       </c>
       <c r="G190" s="48" t="inlineStr">
         <is>
-          <t>1. Pada form Bagikan Task, periksa daftar Ditugaskan ke (User).
-2. Klik icon hapus (tempat sampah) pada user yang ditugaskan.
-3. Konfirmasi penghapusan penugasan task.</t>
+          <t>1. Pada tab Task, klik salah satu card task yang terdaftar.</t>
         </is>
       </c>
       <c r="H190" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan penugasan.
-2. Berhasil menghapus penugasan task kepada user dari daftar pembagian task.</t>
+          <t>1. Berhasil membuka halaman Detail Task.
+2. Berhasil menampilkan informasi status, visibilitas, prioritas, tenggat, zona waktu, pemilik, deskripsi, dan lampiran.</t>
         </is>
       </c>
       <c r="I190" s="49" t="n"/>
@@ -53190,585 +53126,594 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
+          <t>15.4</t>
+        </is>
+      </c>
+      <c r="B191" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C191" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D191" s="48" t="inlineStr">
+        <is>
+          <t>Mengubah data task dengan data valid</t>
+        </is>
+      </c>
+      <c r="E191" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F191" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G191" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Task, klik icon Edit (pensil).
+2. Ubah data task pada form Edit Task.
+3. Klik button Simpan.</t>
+        </is>
+      </c>
+      <c r="H191" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka form Edit Task.
+2. Berhasil menyimpan perubahan data task dengan data yang valid.</t>
+        </is>
+      </c>
+      <c r="I191" s="49" t="n"/>
+      <c r="J191" s="49" t="n"/>
+      <c r="K191" s="49" t="n"/>
+      <c r="L191" s="49" t="n"/>
+      <c r="M191" s="49" t="n"/>
+      <c r="N191" s="49" t="n"/>
+      <c r="O191" s="49" t="n"/>
+      <c r="P191" s="49" t="n"/>
+      <c r="Q191" s="49" t="n"/>
+      <c r="R191" s="49" t="n"/>
+      <c r="S191" s="49" t="n"/>
+      <c r="T191" s="49" t="n"/>
+      <c r="U191" s="49" t="n"/>
+      <c r="V191" s="49" t="n"/>
+      <c r="W191" s="49" t="n"/>
+      <c r="X191" s="49" t="n"/>
+      <c r="Y191" s="49" t="n"/>
+      <c r="Z191" s="49" t="n"/>
+      <c r="AA191" s="49" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>15.5</t>
+        </is>
+      </c>
+      <c r="B192" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C192" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D192" s="48" t="inlineStr">
+        <is>
+          <t>Membagikan task kepada user</t>
+        </is>
+      </c>
+      <c r="E192" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F192" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G192" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada halaman Detail Task, klik icon Bagikan (share).
+2. Pilih role atau user yang ditugaskan.
+3. Klik button Bagikan.</t>
+        </is>
+      </c>
+      <c r="H192" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka form Bagikan Task.
+2. Berhasil membagikan task kepada user dan menampilkan pesan konfirmasi Task berhasil dibagikan.</t>
+        </is>
+      </c>
+      <c r="I192" s="49" t="n"/>
+      <c r="J192" s="49" t="n"/>
+      <c r="K192" s="49" t="n"/>
+      <c r="L192" s="49" t="n"/>
+      <c r="M192" s="49" t="n"/>
+      <c r="N192" s="49" t="n"/>
+      <c r="O192" s="49" t="n"/>
+      <c r="P192" s="49" t="n"/>
+      <c r="Q192" s="49" t="n"/>
+      <c r="R192" s="49" t="n"/>
+      <c r="S192" s="49" t="n"/>
+      <c r="T192" s="49" t="n"/>
+      <c r="U192" s="49" t="n"/>
+      <c r="V192" s="49" t="n"/>
+      <c r="W192" s="49" t="n"/>
+      <c r="X192" s="49" t="n"/>
+      <c r="Y192" s="49" t="n"/>
+      <c r="Z192" s="49" t="n"/>
+      <c r="AA192" s="49" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>15.6</t>
+        </is>
+      </c>
+      <c r="B193" s="46" t="inlineStr">
+        <is>
+          <t>Agenda</t>
+        </is>
+      </c>
+      <c r="C193" s="46" t="inlineStr">
+        <is>
+          <t>Pengingat</t>
+        </is>
+      </c>
+      <c r="D193" s="48" t="inlineStr">
+        <is>
+          <t>Menghapus penugasan task kepada user</t>
+        </is>
+      </c>
+      <c r="E193" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F193" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G193" s="48" t="inlineStr">
+        <is>
+          <t>1. Pada form Bagikan Task, periksa daftar Ditugaskan ke (User).
+2. Klik icon hapus (tempat sampah) pada user yang ditugaskan.
+3. Konfirmasi penghapusan penugasan task.</t>
+        </is>
+      </c>
+      <c r="H193" s="48" t="inlineStr">
+        <is>
+          <t>1. Berhasil menampilkan dialog konfirmasi penghapusan penugasan.
+2. Berhasil menghapus penugasan task kepada user dari daftar pembagian task.</t>
+        </is>
+      </c>
+      <c r="I193" s="49" t="n"/>
+      <c r="J193" s="49" t="n"/>
+      <c r="K193" s="49" t="n"/>
+      <c r="L193" s="49" t="n"/>
+      <c r="M193" s="49" t="n"/>
+      <c r="N193" s="49" t="n"/>
+      <c r="O193" s="49" t="n"/>
+      <c r="P193" s="49" t="n"/>
+      <c r="Q193" s="49" t="n"/>
+      <c r="R193" s="49" t="n"/>
+      <c r="S193" s="49" t="n"/>
+      <c r="T193" s="49" t="n"/>
+      <c r="U193" s="49" t="n"/>
+      <c r="V193" s="49" t="n"/>
+      <c r="W193" s="49" t="n"/>
+      <c r="X193" s="49" t="n"/>
+      <c r="Y193" s="49" t="n"/>
+      <c r="Z193" s="49" t="n"/>
+      <c r="AA193" s="49" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
           <t>15.7</t>
         </is>
       </c>
-      <c r="B191" s="46" t="inlineStr">
+      <c r="B194" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C191" s="46" t="inlineStr">
+      <c r="C194" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D191" s="48" t="inlineStr">
+      <c r="D194" s="48" t="inlineStr">
         <is>
           <t>Menambahkan komentar pada task</t>
         </is>
       </c>
-      <c r="E191" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F191" s="46" t="inlineStr">
+      <c r="E194" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F194" s="46" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G191" s="48" t="inlineStr">
+      <c r="G194" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Task, klik tab Aktivitas &amp; Percakapan.
 2. Tulis komentar pada kolom Tulis komentar.
 3. Klik button Kirim.</t>
         </is>
       </c>
-      <c r="H191" s="48" t="inlineStr">
+      <c r="H194" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menginput teks komentar.
 2. Berhasil mengirimkan komentar dan menampilkan komentar baru pada daftar riwayat aktivitas task.</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
+    <row r="195">
+      <c r="A195" t="inlineStr">
         <is>
           <t>15.8</t>
         </is>
       </c>
-      <c r="B192" s="46" t="inlineStr">
+      <c r="B195" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C192" s="46" t="inlineStr">
+      <c r="C195" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D192" s="48" t="inlineStr">
+      <c r="D195" s="48" t="inlineStr">
         <is>
           <t>Menghapus komentar pada task</t>
         </is>
       </c>
-      <c r="E192" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F192" s="46" t="inlineStr">
+      <c r="E195" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F195" s="46" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G192" s="48" t="inlineStr">
+      <c r="G195" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Task, klik tab Aktivitas &amp; Percakapan.
 2. Klik icon hapus (tempat sampah) pada komentar yang ingin dihapus.
 3. Konfirmasi penghapusan komentar.</t>
         </is>
       </c>
-      <c r="H192" s="48" t="inlineStr">
+      <c r="H195" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan dialog konfirmasi penghapusan komentar.
 2. Berhasil menghapus komentar dari daftar aktivitas dan percakapan task.</t>
         </is>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
+    <row r="196">
+      <c r="A196" t="inlineStr">
         <is>
           <t>15.9</t>
         </is>
       </c>
-      <c r="B193" s="46" t="inlineStr">
+      <c r="B196" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C193" s="46" t="inlineStr">
+      <c r="C196" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D193" s="48" t="inlineStr">
+      <c r="D196" s="48" t="inlineStr">
         <is>
           <t>Melihat detail acara</t>
         </is>
       </c>
-      <c r="E193" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F193" s="46" t="inlineStr">
+      <c r="E196" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F196" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G193" s="48" t="inlineStr">
+      <c r="G196" s="48" t="inlineStr">
         <is>
           <t>1. Pada tab Acara, klik salah satu card acara yang terdaftar.</t>
         </is>
       </c>
-      <c r="H193" s="48" t="inlineStr">
+      <c r="H196" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka halaman Detail Acara.
 2. Berhasil menampilkan informasi status, visibilitas, tanggal/waktu mulai &amp; selesai, zona waktu, dan pemilik acara.</t>
         </is>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
+    <row r="197">
+      <c r="A197" t="inlineStr">
         <is>
           <t>15.10</t>
         </is>
       </c>
-      <c r="B194" s="46" t="inlineStr">
+      <c r="B197" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C194" s="46" t="inlineStr">
+      <c r="C197" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D194" s="48" t="inlineStr">
+      <c r="D197" s="48" t="inlineStr">
         <is>
           <t>Mengubah data acara dengan data valid</t>
         </is>
       </c>
-      <c r="E194" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F194" s="46" t="inlineStr">
+      <c r="E197" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F197" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G194" s="48" t="inlineStr">
+      <c r="G197" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Acara, klik icon Edit (pensil).
 2. Ubah data acara pada form Edit Acara.
 3. Klik button Simpan.</t>
         </is>
       </c>
-      <c r="H194" s="48" t="inlineStr">
+      <c r="H197" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Edit Acara.
 2. Berhasil menyimpan perubahan data acara dengan data yang valid.</t>
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
+    <row r="198">
+      <c r="A198" t="inlineStr">
         <is>
           <t>15.11</t>
         </is>
       </c>
-      <c r="B195" s="46" t="inlineStr">
+      <c r="B198" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C195" s="46" t="inlineStr">
+      <c r="C198" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D195" s="48" t="inlineStr">
+      <c r="D198" s="48" t="inlineStr">
         <is>
           <t>Membagikan acara kepada user</t>
         </is>
       </c>
-      <c r="E195" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F195" s="46" t="inlineStr">
+      <c r="E198" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F198" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G195" s="48" t="inlineStr">
+      <c r="G198" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Acara, klik icon Bagikan (share).
 2. Tentukan user watcher/assignee pada form Bagikan Acara.
 3. Klik button Bagikan.</t>
         </is>
       </c>
-      <c r="H195" s="48" t="inlineStr">
+      <c r="H198" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Bagikan Acara.
 2. Berhasil membagikan acara kepada user dan memicu notifikasi kepada penerima.</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
+    <row r="199">
+      <c r="A199" t="inlineStr">
         <is>
           <t>15.12</t>
         </is>
       </c>
-      <c r="B196" s="46" t="inlineStr">
+      <c r="B199" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C196" s="46" t="inlineStr">
+      <c r="C199" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D196" s="48" t="inlineStr">
+      <c r="D199" s="48" t="inlineStr">
         <is>
           <t>Menghapus penugasan acara kepada user</t>
         </is>
       </c>
-      <c r="E196" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F196" s="46" t="inlineStr">
+      <c r="E199" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F199" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G196" s="48" t="inlineStr">
+      <c r="G199" s="48" t="inlineStr">
         <is>
           <t>1. Pada form Bagikan Acara, periksa daftar Ditugaskan ke (User).
 2. Klik icon hapus (tempat sampah) pada user yang ditugaskan.
 3. Konfirmasi penghapusan penugasan acara.</t>
         </is>
       </c>
-      <c r="H196" s="48" t="inlineStr">
+      <c r="H199" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan dialog konfirmasi penghapusan penugasan.
 2. Berhasil menghapus penugasan acara kepada user dari daftar pembagian acara.</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
+    <row r="200">
+      <c r="A200" t="inlineStr">
         <is>
           <t>15.13</t>
         </is>
       </c>
-      <c r="B197" s="46" t="inlineStr">
+      <c r="B200" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C197" s="46" t="inlineStr">
+      <c r="C200" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D197" s="48" t="inlineStr">
+      <c r="D200" s="48" t="inlineStr">
         <is>
           <t>Menambahkan komentar pada acara</t>
         </is>
       </c>
-      <c r="E197" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F197" s="46" t="inlineStr">
+      <c r="E200" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F200" s="46" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G197" s="48" t="inlineStr">
+      <c r="G200" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Acara, klik tab Aktivitas &amp; Percakapan.
 2. Tulis komentar pada kolom Tulis komentar.
 3. Klik button Kirim.</t>
         </is>
       </c>
-      <c r="H197" s="48" t="inlineStr">
+      <c r="H200" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menginput teks komentar.
 2. Berhasil mengirimkan komentar dan menampilkan komentar baru pada daftar riwayat aktivitas acara.</t>
         </is>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
+    <row r="201">
+      <c r="A201" t="inlineStr">
         <is>
           <t>15.14</t>
         </is>
       </c>
-      <c r="B198" s="46" t="inlineStr">
+      <c r="B201" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C198" s="46" t="inlineStr">
+      <c r="C201" s="46" t="inlineStr">
         <is>
           <t>Pengingat</t>
         </is>
       </c>
-      <c r="D198" s="48" t="inlineStr">
+      <c r="D201" s="48" t="inlineStr">
         <is>
           <t>Menghapus komentar pada acara</t>
         </is>
       </c>
-      <c r="E198" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F198" s="46" t="inlineStr">
+      <c r="E201" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F201" s="46" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="G198" s="48" t="inlineStr">
+      <c r="G201" s="48" t="inlineStr">
         <is>
           <t>1. Pada halaman Detail Acara, klik tab Aktivitas &amp; Percakapan.
 2. Klik icon hapus (tempat sampah) pada komentar yang ingin dihapus.
 3. Konfirmasi penghapusan komentar.</t>
         </is>
       </c>
-      <c r="H198" s="48" t="inlineStr">
+      <c r="H201" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan dialog konfirmasi penghapusan komentar.
 2. Berhasil menghapus komentar dari daftar aktivitas dan percakapan acara.</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
+    <row r="202">
+      <c r="A202" t="inlineStr">
         <is>
           <t>16.1</t>
         </is>
       </c>
-      <c r="B199" s="46" t="inlineStr">
+      <c r="B202" s="46" t="inlineStr">
         <is>
           <t>Agenda</t>
         </is>
       </c>
-      <c r="C199" s="46" t="inlineStr">
+      <c r="C202" s="46" t="inlineStr">
         <is>
           <t>Daily Sales Agenda</t>
         </is>
       </c>
-      <c r="D199" s="48" t="inlineStr">
+      <c r="D202" s="48" t="inlineStr">
         <is>
           <t>Membuka halaman Daily Sales Agenda</t>
         </is>
       </c>
-      <c r="E199" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F199" s="46" t="inlineStr">
+      <c r="E202" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F202" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G199" s="48" t="inlineStr">
+      <c r="G202" s="48" t="inlineStr">
         <is>
           <t>1. Buka menu Lainnya.
 2. Klik menu Daily Sales Agenda.</t>
         </is>
       </c>
-      <c r="H199" s="48" t="inlineStr">
+      <c r="H202" s="48" t="inlineStr">
         <is>
           <t>1. Berhasil membuka menu Lainnya.
 2. Berhasil menampilkan halaman Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I199" s="49" t="n"/>
-      <c r="J199" s="49" t="n"/>
-      <c r="K199" s="49" t="n"/>
-      <c r="L199" s="49" t="n"/>
-      <c r="M199" s="49" t="n"/>
-      <c r="N199" s="49" t="n"/>
-      <c r="O199" s="49" t="n"/>
-      <c r="P199" s="49" t="n"/>
-      <c r="Q199" s="49" t="n"/>
-      <c r="R199" s="49" t="n"/>
-      <c r="S199" s="49" t="n"/>
-      <c r="T199" s="49" t="n"/>
-      <c r="U199" s="49" t="n"/>
-      <c r="V199" s="49" t="n"/>
-      <c r="W199" s="49" t="n"/>
-      <c r="X199" s="49" t="n"/>
-      <c r="Y199" s="49" t="n"/>
-      <c r="Z199" s="49" t="n"/>
-      <c r="AA199" s="49" t="n"/>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>16.2</t>
-        </is>
-      </c>
-      <c r="B200" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C200" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D200" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Masuk</t>
-        </is>
-      </c>
-      <c r="E200" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F200" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G200" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Masuk.</t>
-        </is>
-      </c>
-      <c r="H200" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah yang masuk pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I200" s="49" t="n"/>
-      <c r="J200" s="49" t="n"/>
-      <c r="K200" s="49" t="n"/>
-      <c r="L200" s="49" t="n"/>
-      <c r="M200" s="49" t="n"/>
-      <c r="N200" s="49" t="n"/>
-      <c r="O200" s="49" t="n"/>
-      <c r="P200" s="49" t="n"/>
-      <c r="Q200" s="49" t="n"/>
-      <c r="R200" s="49" t="n"/>
-      <c r="S200" s="49" t="n"/>
-      <c r="T200" s="49" t="n"/>
-      <c r="U200" s="49" t="n"/>
-      <c r="V200" s="49" t="n"/>
-      <c r="W200" s="49" t="n"/>
-      <c r="X200" s="49" t="n"/>
-      <c r="Y200" s="49" t="n"/>
-      <c r="Z200" s="49" t="n"/>
-      <c r="AA200" s="49" t="n"/>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>16.3</t>
-        </is>
-      </c>
-      <c r="B201" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C201" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D201" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Closing</t>
-        </is>
-      </c>
-      <c r="E201" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F201" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G201" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Closing.</t>
-        </is>
-      </c>
-      <c r="H201" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah yang closing pada Daily Sales Agenda.</t>
-        </is>
-      </c>
-      <c r="I201" s="49" t="n"/>
-      <c r="J201" s="49" t="n"/>
-      <c r="K201" s="49" t="n"/>
-      <c r="L201" s="49" t="n"/>
-      <c r="M201" s="49" t="n"/>
-      <c r="N201" s="49" t="n"/>
-      <c r="O201" s="49" t="n"/>
-      <c r="P201" s="49" t="n"/>
-      <c r="Q201" s="49" t="n"/>
-      <c r="R201" s="49" t="n"/>
-      <c r="S201" s="49" t="n"/>
-      <c r="T201" s="49" t="n"/>
-      <c r="U201" s="49" t="n"/>
-      <c r="V201" s="49" t="n"/>
-      <c r="W201" s="49" t="n"/>
-      <c r="X201" s="49" t="n"/>
-      <c r="Y201" s="49" t="n"/>
-      <c r="Z201" s="49" t="n"/>
-      <c r="AA201" s="49" t="n"/>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>16.4</t>
-        </is>
-      </c>
-      <c r="B202" s="46" t="inlineStr">
-        <is>
-          <t>Agenda</t>
-        </is>
-      </c>
-      <c r="C202" s="46" t="inlineStr">
-        <is>
-          <t>Daily Sales Agenda</t>
-        </is>
-      </c>
-      <c r="D202" s="48" t="inlineStr">
-        <is>
-          <t>Melihat daftar agenda pada tab Referral</t>
-        </is>
-      </c>
-      <c r="E202" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F202" s="46" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="G202" s="48" t="inlineStr">
-        <is>
-          <t>1. Klik tab Referral.</t>
-        </is>
-      </c>
-      <c r="H202" s="48" t="inlineStr">
-        <is>
-          <t>1. Berhasil menampilkan daftar nasabah referral pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I202" s="49" t="n"/>
@@ -53794,7 +53739,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>16.2</t>
         </is>
       </c>
       <c r="B203" s="46" t="inlineStr">
@@ -53809,7 +53754,7 @@
       </c>
       <c r="D203" s="48" t="inlineStr">
         <is>
-          <t>Melihat daftar agenda pada tab Ref. Closing</t>
+          <t>Melihat daftar agenda pada tab Masuk</t>
         </is>
       </c>
       <c r="E203" s="46" t="inlineStr">
@@ -53824,12 +53769,12 @@
       </c>
       <c r="G203" s="48" t="inlineStr">
         <is>
-          <t>1. Klik tab Ref. Closing.</t>
+          <t>1. Klik tab Masuk.</t>
         </is>
       </c>
       <c r="H203" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan daftar nasabah referral yang closing pada Daily Sales Agenda.</t>
+          <t>1. Berhasil menampilkan daftar nasabah yang masuk pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I203" s="49" t="n"/>
@@ -53855,7 +53800,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16.6</t>
+          <t>16.3</t>
         </is>
       </c>
       <c r="B204" s="46" t="inlineStr">
@@ -53870,7 +53815,7 @@
       </c>
       <c r="D204" s="48" t="inlineStr">
         <is>
-          <t>Mencari agenda menggunakan Search Bar</t>
+          <t>Melihat daftar agenda pada tab Closing</t>
         </is>
       </c>
       <c r="E204" s="46" t="inlineStr">
@@ -53880,17 +53825,17 @@
       </c>
       <c r="F204" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G204" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
+          <t>1. Klik tab Closing.</t>
         </is>
       </c>
       <c r="H204" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data agenda yang sesuai dengan kata kunci pencarian.</t>
+          <t>1. Berhasil menampilkan daftar nasabah yang closing pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I204" s="49" t="n"/>
@@ -53916,7 +53861,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>16.7</t>
+          <t>16.4</t>
         </is>
       </c>
       <c r="B205" s="46" t="inlineStr">
@@ -53931,12 +53876,12 @@
       </c>
       <c r="D205" s="48" t="inlineStr">
         <is>
-          <t>Mencari agenda dengan keyword tidak valid</t>
+          <t>Melihat daftar agenda pada tab Referral</t>
         </is>
       </c>
       <c r="E205" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F205" s="46" t="inlineStr">
@@ -53946,12 +53891,12 @@
       </c>
       <c r="G205" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
+          <t>1. Klik tab Referral.</t>
         </is>
       </c>
       <c r="H205" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>1. Berhasil menampilkan daftar nasabah referral pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I205" s="49" t="n"/>
@@ -53977,7 +53922,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>16.8</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="B206" s="46" t="inlineStr">
@@ -53992,7 +53937,7 @@
       </c>
       <c r="D206" s="48" t="inlineStr">
         <is>
-          <t>Melakukan filter data Daily Sales Agenda</t>
+          <t>Melihat daftar agenda pada tab Ref. Closing</t>
         </is>
       </c>
       <c r="E206" s="46" t="inlineStr">
@@ -54002,21 +53947,17 @@
       </c>
       <c r="F206" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G206" s="48" t="inlineStr">
         <is>
-          <t>1. Klik button Filter.
-2. Pilih kriteria filter pada form Filter (Product, Bulan, Tahun).
-3. Klik button Submit.</t>
+          <t>1. Klik tab Ref. Closing.</t>
         </is>
       </c>
       <c r="H206" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka form Filter.
-2. Berhasil memilih kriteria filter.
-3. Berhasil menampilkan data Daily Sales Agenda sesuai filter yang dipilih.</t>
+          <t>1. Berhasil menampilkan daftar nasabah referral yang closing pada Daily Sales Agenda.</t>
         </is>
       </c>
       <c r="I206" s="49" t="n"/>
@@ -54042,22 +53983,22 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>17.1</t>
+          <t>16.6</t>
         </is>
       </c>
       <c r="B207" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C207" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D207" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Marketing Toolkit</t>
+          <t>Mencari agenda menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E207" s="46" t="inlineStr">
@@ -54072,14 +54013,12 @@
       </c>
       <c r="G207" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Marketing Toolkit.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H207" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Marketing Toolkit.</t>
+          <t>1. Berhasil menampilkan data agenda yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I207" s="49" t="n"/>
@@ -54105,27 +54044,27 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>17.2</t>
+          <t>16.7</t>
         </is>
       </c>
       <c r="B208" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C208" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D208" s="48" t="inlineStr">
         <is>
-          <t>Mengubah tampilan folder menjadi List View</t>
+          <t>Mencari agenda dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E208" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F208" s="46" t="inlineStr">
@@ -54135,12 +54074,12 @@
       </c>
       <c r="G208" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon tampilan List pada halaman Marketing Toolkit.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H208" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengubah tampilan folder menjadi List View.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I208" s="49" t="n"/>
@@ -54166,22 +54105,22 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>17.3</t>
+          <t>16.8</t>
         </is>
       </c>
       <c r="B209" s="46" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Agenda</t>
         </is>
       </c>
       <c r="C209" s="46" t="inlineStr">
         <is>
-          <t>Marketing Toolkit</t>
+          <t>Daily Sales Agenda</t>
         </is>
       </c>
       <c r="D209" s="48" t="inlineStr">
         <is>
-          <t>Mengubah tampilan folder menjadi Grid View</t>
+          <t>Melakukan filter data Daily Sales Agenda</t>
         </is>
       </c>
       <c r="E209" s="46" t="inlineStr">
@@ -54191,17 +54130,21 @@
       </c>
       <c r="F209" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G209" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon tampilan Grid pada halaman Marketing Toolkit.</t>
+          <t>1. Klik button Filter.
+2. Pilih kriteria filter pada form Filter (Product, Bulan, Tahun).
+3. Klik button Submit.</t>
         </is>
       </c>
       <c r="H209" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil mengubah tampilan folder menjadi Grid View.</t>
+          <t>1. Berhasil membuka form Filter.
+2. Berhasil memilih kriteria filter.
+3. Berhasil menampilkan data Daily Sales Agenda sesuai filter yang dipilih.</t>
         </is>
       </c>
       <c r="I209" s="49" t="n"/>
@@ -54227,7 +54170,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>17.4</t>
+          <t>17.1</t>
         </is>
       </c>
       <c r="B210" s="46" t="inlineStr">
@@ -54242,7 +54185,7 @@
       </c>
       <c r="D210" s="48" t="inlineStr">
         <is>
-          <t>Membuka folder pada Marketing Toolkit</t>
+          <t>Membuka halaman Marketing Toolkit</t>
         </is>
       </c>
       <c r="E210" s="46" t="inlineStr">
@@ -54257,12 +54200,14 @@
       </c>
       <c r="G210" s="48" t="inlineStr">
         <is>
-          <t>1. Klik salah satu folder pada daftar Folder.</t>
+          <t>1. Buka menu Lainnya.
+2. Klik menu Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H210" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka folder Marketing Toolkit.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I210" s="49" t="n"/>
@@ -54288,7 +54233,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>17.5</t>
+          <t>17.2</t>
         </is>
       </c>
       <c r="B211" s="46" t="inlineStr">
@@ -54303,7 +54248,7 @@
       </c>
       <c r="D211" s="48" t="inlineStr">
         <is>
-          <t>Mencari konten di dalam folder menggunakan Search Bar</t>
+          <t>Mengubah tampilan folder menjadi List View</t>
         </is>
       </c>
       <c r="E211" s="46" t="inlineStr">
@@ -54313,17 +54258,17 @@
       </c>
       <c r="F211" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G211" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
+          <t>1. Klik icon tampilan List pada halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H211" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan data yang sesuai dengan kata kunci pencarian.</t>
+          <t>1. Berhasil mengubah tampilan folder menjadi List View.</t>
         </is>
       </c>
       <c r="I211" s="49" t="n"/>
@@ -54349,7 +54294,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>17.6</t>
+          <t>17.3</t>
         </is>
       </c>
       <c r="B212" s="46" t="inlineStr">
@@ -54364,12 +54309,12 @@
       </c>
       <c r="D212" s="48" t="inlineStr">
         <is>
-          <t>Mencari konten di dalam folder dengan keyword tidak valid</t>
+          <t>Mengubah tampilan folder menjadi Grid View</t>
         </is>
       </c>
       <c r="E212" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F212" s="46" t="inlineStr">
@@ -54379,12 +54324,12 @@
       </c>
       <c r="G212" s="48" t="inlineStr">
         <is>
-          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
+          <t>1. Klik icon tampilan Grid pada halaman Marketing Toolkit.</t>
         </is>
       </c>
       <c r="H212" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>1. Berhasil mengubah tampilan folder menjadi Grid View.</t>
         </is>
       </c>
       <c r="I212" s="49" t="n"/>
@@ -54410,7 +54355,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>17.7</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="B213" s="46" t="inlineStr">
@@ -54425,7 +54370,7 @@
       </c>
       <c r="D213" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail konten Marketing Toolkit</t>
+          <t>Membuka folder pada Marketing Toolkit</t>
         </is>
       </c>
       <c r="E213" s="46" t="inlineStr">
@@ -54440,12 +54385,12 @@
       </c>
       <c r="G213" s="48" t="inlineStr">
         <is>
-          <t>1. Klik salah satu sub-folder pada daftar folder.</t>
+          <t>1. Klik salah satu folder pada daftar Folder.</t>
         </is>
       </c>
       <c r="H213" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail konten Marketing Toolkit.</t>
+          <t>1. Berhasil membuka folder Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I213" s="49" t="n"/>
@@ -54471,7 +54416,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="B214" s="46" t="inlineStr">
@@ -54486,7 +54431,7 @@
       </c>
       <c r="D214" s="48" t="inlineStr">
         <is>
-          <t>Mengunduh lampiran pada konten Marketing Toolkit</t>
+          <t>Mencari konten di dalam folder menggunakan Search Bar</t>
         </is>
       </c>
       <c r="E214" s="46" t="inlineStr">
@@ -54501,14 +54446,12 @@
       </c>
       <c r="G214" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon titik tiga pada salah satu lampiran.
-2. Pilih Download.</t>
+          <t>1. Masukkan kata kunci pencarian pada Search Bar.</t>
         </is>
       </c>
       <c r="H214" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
-2. Berhasil mengunduh lampiran ke perangkat.</t>
+          <t>1. Berhasil menampilkan data yang sesuai dengan kata kunci pencarian.</t>
         </is>
       </c>
       <c r="I214" s="49" t="n"/>
@@ -54534,7 +54477,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>17.9</t>
+          <t>17.6</t>
         </is>
       </c>
       <c r="B215" s="46" t="inlineStr">
@@ -54549,12 +54492,12 @@
       </c>
       <c r="D215" s="48" t="inlineStr">
         <is>
-          <t>Berbagi lampiran pada konten Marketing Toolkit</t>
+          <t>Mencari konten di dalam folder dengan keyword tidak valid</t>
         </is>
       </c>
       <c r="E215" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F215" s="46" t="inlineStr">
@@ -54564,14 +54507,12 @@
       </c>
       <c r="G215" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon titik tiga pada salah satu lampiran.
-2. Pilih Share.</t>
+          <t>1. Masukkan keyword tidak valid pada Search Bar.</t>
         </is>
       </c>
       <c r="H215" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
-2. Berhasil menampilkan pilihan aplikasi berbagi.</t>
+          <t>1. Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
       <c r="I215" s="49" t="n"/>
@@ -54597,22 +54538,22 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>17.7</t>
         </is>
       </c>
       <c r="B216" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C216" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D216" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Dashboard Sales Code</t>
+          <t>Melihat detail konten Marketing Toolkit</t>
         </is>
       </c>
       <c r="E216" s="46" t="inlineStr">
@@ -54627,14 +54568,12 @@
       </c>
       <c r="G216" s="48" t="inlineStr">
         <is>
-          <t>1. Buka menu Lainnya.
-2. Klik menu Dashboard Sales Code.</t>
+          <t>1. Klik salah satu sub-folder pada daftar folder.</t>
         </is>
       </c>
       <c r="H216" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil membuka menu Lainnya.
-2. Berhasil menampilkan halaman Dashboard Sales Code.</t>
+          <t>1. Berhasil menampilkan detail konten Marketing Toolkit.</t>
         </is>
       </c>
       <c r="I216" s="49" t="n"/>
@@ -54660,22 +54599,22 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18.2</t>
+          <t>17.8</t>
         </is>
       </c>
       <c r="B217" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C217" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D217" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Voa Realization</t>
+          <t>Mengunduh lampiran pada konten Marketing Toolkit</t>
         </is>
       </c>
       <c r="E217" s="46" t="inlineStr">
@@ -54690,12 +54629,14 @@
       </c>
       <c r="G217" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Voa Realization.</t>
+          <t>1. Klik icon titik tiga pada salah satu lampiran.
+2. Pilih Download.</t>
         </is>
       </c>
       <c r="H217" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Voa Realization.</t>
+          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
+2. Berhasil mengunduh lampiran ke perangkat.</t>
         </is>
       </c>
       <c r="I217" s="49" t="n"/>
@@ -54721,22 +54662,22 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>18.3</t>
+          <t>17.9</t>
         </is>
       </c>
       <c r="B218" s="46" t="inlineStr">
         <is>
-          <t>Sales Force</t>
+          <t>Fitur</t>
         </is>
       </c>
       <c r="C218" s="46" t="inlineStr">
         <is>
-          <t>Dashboard Sales Code</t>
+          <t>Marketing Toolkit</t>
         </is>
       </c>
       <c r="D218" s="48" t="inlineStr">
         <is>
-          <t>Melihat Daftar Pipeline pada Voa Realization</t>
+          <t>Berbagi lampiran pada konten Marketing Toolkit</t>
         </is>
       </c>
       <c r="E218" s="46" t="inlineStr">
@@ -54746,19 +54687,19 @@
       </c>
       <c r="F218" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G218" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Voa Realization.
-2. Klik Lihat Daftar Pipeline.</t>
+          <t>1. Klik icon titik tiga pada salah satu lampiran.
+2. Pilih Share.</t>
         </is>
       </c>
       <c r="H218" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Voa Realization.
-2. Berhasil menampilkan Daftar Pipeline.</t>
+          <t>1. Berhasil menampilkan opsi aksi pada lampiran.
+2. Berhasil menampilkan pilihan aplikasi berbagi.</t>
         </is>
       </c>
       <c r="I218" s="49" t="n"/>
@@ -54784,7 +54725,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>18.1</t>
         </is>
       </c>
       <c r="B219" s="46" t="inlineStr">
@@ -54799,7 +54740,7 @@
       </c>
       <c r="D219" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail CIF Kelolaan</t>
+          <t>Membuka halaman Dashboard Sales Code</t>
         </is>
       </c>
       <c r="E219" s="46" t="inlineStr">
@@ -54809,17 +54750,19 @@
       </c>
       <c r="F219" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G219" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card CIF Kelolaan.</t>
+          <t>1. Buka menu Lainnya.
+2. Klik menu Dashboard Sales Code.</t>
         </is>
       </c>
       <c r="H219" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail CIF Kelolaan.</t>
+          <t>1. Berhasil membuka menu Lainnya.
+2. Berhasil menampilkan halaman Dashboard Sales Code.</t>
         </is>
       </c>
       <c r="I219" s="49" t="n"/>
@@ -54845,7 +54788,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>18.2</t>
         </is>
       </c>
       <c r="B220" s="46" t="inlineStr">
@@ -54860,7 +54803,7 @@
       </c>
       <c r="D220" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Realisasi Konek E-Channel</t>
+          <t>Melihat detail Voa Realization</t>
         </is>
       </c>
       <c r="E220" s="46" t="inlineStr">
@@ -54875,12 +54818,12 @@
       </c>
       <c r="G220" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Realisasi Konek E-Channel.</t>
+          <t>1. Klik icon expand pada card Voa Realization.</t>
         </is>
       </c>
       <c r="H220" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Realisasi Konek E-Channel.</t>
+          <t>1. Berhasil menampilkan detail Voa Realization.</t>
         </is>
       </c>
       <c r="I220" s="49" t="n"/>
@@ -54906,7 +54849,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>18.6</t>
+          <t>18.3</t>
         </is>
       </c>
       <c r="B221" s="46" t="inlineStr">
@@ -54921,7 +54864,7 @@
       </c>
       <c r="D221" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Realisasi Akuisisi Merchant</t>
+          <t>Melihat Daftar Pipeline pada Voa Realization</t>
         </is>
       </c>
       <c r="E221" s="46" t="inlineStr">
@@ -54936,12 +54879,14 @@
       </c>
       <c r="G221" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Realisasi Akuisisi Merchant.</t>
+          <t>1. Klik icon expand pada card Voa Realization.
+2. Klik Lihat Daftar Pipeline.</t>
         </is>
       </c>
       <c r="H221" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Realisasi Akuisisi Merchant.</t>
+          <t>1. Berhasil menampilkan detail Voa Realization.
+2. Berhasil menampilkan Daftar Pipeline.</t>
         </is>
       </c>
       <c r="I221" s="49" t="n"/>
@@ -54967,7 +54912,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>18.7</t>
+          <t>18.4</t>
         </is>
       </c>
       <c r="B222" s="46" t="inlineStr">
@@ -54982,7 +54927,7 @@
       </c>
       <c r="D222" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail Eligible Upgrade to Prospera/Prioritas</t>
+          <t>Melihat detail CIF Kelolaan</t>
         </is>
       </c>
       <c r="E222" s="46" t="inlineStr">
@@ -54992,17 +54937,17 @@
       </c>
       <c r="F222" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G222" s="48" t="inlineStr">
         <is>
-          <t>1. Klik icon expand pada card Eligible Upgrade to Prospera/Prioritas.</t>
+          <t>1. Klik icon expand pada card CIF Kelolaan.</t>
         </is>
       </c>
       <c r="H222" s="48" t="inlineStr">
         <is>
-          <t>1. Berhasil menampilkan detail Eligible Upgrade to Prospera &amp; Prioritas.</t>
+          <t>1. Berhasil menampilkan detail CIF Kelolaan.</t>
         </is>
       </c>
       <c r="I222" s="49" t="n"/>
@@ -55028,18 +54973,22 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19.1</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="B223" s="46" t="inlineStr">
         <is>
-          <t>Kunjungan</t>
-        </is>
-      </c>
-      <c r="C223" s="46" t="n"/>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C223" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
       <c r="D223" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Kunjungan</t>
+          <t>Melihat detail Realisasi Konek E-Channel</t>
         </is>
       </c>
       <c r="E223" s="46" t="inlineStr">
@@ -55054,30 +55003,53 @@
       </c>
       <c r="G223" s="48" t="inlineStr">
         <is>
-          <t>Buka menu Lainnya - Klik menu Kunjungan</t>
+          <t>1. Klik icon expand pada card Realisasi Konek E-Channel.</t>
         </is>
       </c>
       <c r="H223" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Kunjungan beserta informasi Periode, ringkasan Realisasi &amp; Target Visit, serta daftar riwayat kunjungan.</t>
-        </is>
-      </c>
+          <t>1. Berhasil menampilkan detail Realisasi Konek E-Channel.</t>
+        </is>
+      </c>
+      <c r="I223" s="49" t="n"/>
+      <c r="J223" s="49" t="n"/>
+      <c r="K223" s="49" t="n"/>
+      <c r="L223" s="49" t="n"/>
+      <c r="M223" s="49" t="n"/>
+      <c r="N223" s="49" t="n"/>
+      <c r="O223" s="49" t="n"/>
+      <c r="P223" s="49" t="n"/>
+      <c r="Q223" s="49" t="n"/>
+      <c r="R223" s="49" t="n"/>
+      <c r="S223" s="49" t="n"/>
+      <c r="T223" s="49" t="n"/>
+      <c r="U223" s="49" t="n"/>
+      <c r="V223" s="49" t="n"/>
+      <c r="W223" s="49" t="n"/>
+      <c r="X223" s="49" t="n"/>
+      <c r="Y223" s="49" t="n"/>
+      <c r="Z223" s="49" t="n"/>
+      <c r="AA223" s="49" t="n"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19.2</t>
+          <t>18.6</t>
         </is>
       </c>
       <c r="B224" s="46" t="inlineStr">
         <is>
-          <t>Kunjungan</t>
-        </is>
-      </c>
-      <c r="C224" s="46" t="n"/>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C224" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
       <c r="D224" s="48" t="inlineStr">
         <is>
-          <t>Melakukan filter periode tanggal kunjungan</t>
+          <t>Melihat detail Realisasi Akuisisi Merchant</t>
         </is>
       </c>
       <c r="E224" s="46" t="inlineStr">
@@ -55087,35 +55059,58 @@
       </c>
       <c r="F224" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G224" s="48" t="inlineStr">
         <is>
-          <t>Klik dropdown Periode - Pilih rentang tanggal pada kalender (Pilih rentang) - Klik button Simpan</t>
+          <t>1. Klik icon expand pada card Realisasi Akuisisi Merchant.</t>
         </is>
       </c>
       <c r="H224" s="48" t="inlineStr">
         <is>
-          <t>Berhasil memfilter dan menampilkan daftar data kunjungan sesuai rentang periode tanggal yang dipilih.</t>
-        </is>
-      </c>
+          <t>1. Berhasil menampilkan detail Realisasi Akuisisi Merchant.</t>
+        </is>
+      </c>
+      <c r="I224" s="49" t="n"/>
+      <c r="J224" s="49" t="n"/>
+      <c r="K224" s="49" t="n"/>
+      <c r="L224" s="49" t="n"/>
+      <c r="M224" s="49" t="n"/>
+      <c r="N224" s="49" t="n"/>
+      <c r="O224" s="49" t="n"/>
+      <c r="P224" s="49" t="n"/>
+      <c r="Q224" s="49" t="n"/>
+      <c r="R224" s="49" t="n"/>
+      <c r="S224" s="49" t="n"/>
+      <c r="T224" s="49" t="n"/>
+      <c r="U224" s="49" t="n"/>
+      <c r="V224" s="49" t="n"/>
+      <c r="W224" s="49" t="n"/>
+      <c r="X224" s="49" t="n"/>
+      <c r="Y224" s="49" t="n"/>
+      <c r="Z224" s="49" t="n"/>
+      <c r="AA224" s="49" t="n"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>19.3</t>
+          <t>18.7</t>
         </is>
       </c>
       <c r="B225" s="46" t="inlineStr">
         <is>
-          <t>Kunjungan</t>
-        </is>
-      </c>
-      <c r="C225" s="46" t="n"/>
+          <t>Sales Force</t>
+        </is>
+      </c>
+      <c r="C225" s="46" t="inlineStr">
+        <is>
+          <t>Dashboard Sales Code</t>
+        </is>
+      </c>
       <c r="D225" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail kunjungan</t>
+          <t>Melihat detail Eligible Upgrade to Prospera/Prioritas</t>
         </is>
       </c>
       <c r="E225" s="46" t="inlineStr">
@@ -55130,30 +55125,49 @@
       </c>
       <c r="G225" s="48" t="inlineStr">
         <is>
-          <t>Klik salah satu card kunjungan pada daftar - Sistem menampilkan tab default Mulai Kunjungan - Klik tab Selesai Kunjungan</t>
+          <t>1. Klik icon expand pada card Eligible Upgrade to Prospera/Prioritas.</t>
         </is>
       </c>
       <c r="H225" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Detail Kunjungan yang memuat peta lokasi, waktu, tipe kunjungan, dan nama nasabah pada tab Mulai Kunjungan maupun Selesai Kunjungan.</t>
-        </is>
-      </c>
+          <t>1. Berhasil menampilkan detail Eligible Upgrade to Prospera &amp; Prioritas.</t>
+        </is>
+      </c>
+      <c r="I225" s="49" t="n"/>
+      <c r="J225" s="49" t="n"/>
+      <c r="K225" s="49" t="n"/>
+      <c r="L225" s="49" t="n"/>
+      <c r="M225" s="49" t="n"/>
+      <c r="N225" s="49" t="n"/>
+      <c r="O225" s="49" t="n"/>
+      <c r="P225" s="49" t="n"/>
+      <c r="Q225" s="49" t="n"/>
+      <c r="R225" s="49" t="n"/>
+      <c r="S225" s="49" t="n"/>
+      <c r="T225" s="49" t="n"/>
+      <c r="U225" s="49" t="n"/>
+      <c r="V225" s="49" t="n"/>
+      <c r="W225" s="49" t="n"/>
+      <c r="X225" s="49" t="n"/>
+      <c r="Y225" s="49" t="n"/>
+      <c r="Z225" s="49" t="n"/>
+      <c r="AA225" s="49" t="n"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>19.1</t>
         </is>
       </c>
       <c r="B226" s="46" t="inlineStr">
         <is>
-          <t>Notifikasi</t>
+          <t>Kunjungan</t>
         </is>
       </c>
       <c r="C226" s="46" t="n"/>
       <c r="D226" s="48" t="inlineStr">
         <is>
-          <t>Membuka halaman Notifikasi</t>
+          <t>Membuka halaman Kunjungan</t>
         </is>
       </c>
       <c r="E226" s="46" t="inlineStr">
@@ -55168,30 +55182,30 @@
       </c>
       <c r="G226" s="48" t="inlineStr">
         <is>
-          <t>Buka aplikasi BTN Smart - Masuk ke Beranda - Klik icon Lonceng (Notifikasi)</t>
+          <t>Buka menu Lainnya - Klik menu Kunjungan</t>
         </is>
       </c>
       <c r="H226" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan halaman Notifikasi.</t>
+          <t>Berhasil menampilkan halaman Kunjungan beserta informasi Periode, ringkasan Realisasi &amp; Target Visit, serta daftar riwayat kunjungan.</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>20.2</t>
+          <t>19.2</t>
         </is>
       </c>
       <c r="B227" s="46" t="inlineStr">
         <is>
-          <t>Notifikasi</t>
+          <t>Kunjungan</t>
         </is>
       </c>
       <c r="C227" s="46" t="n"/>
       <c r="D227" s="48" t="inlineStr">
         <is>
-          <t>Mencari notifikasi dengan kata kunci valid</t>
+          <t>Melakukan filter periode tanggal kunjungan</t>
         </is>
       </c>
       <c r="E227" s="46" t="inlineStr">
@@ -55206,57 +55220,57 @@
       </c>
       <c r="G227" s="48" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci valid pada Search Bar</t>
+          <t>Klik dropdown Periode - Pilih rentang tanggal pada kalender (Pilih rentang) - Klik button Simpan</t>
         </is>
       </c>
       <c r="H227" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data notifikasi yang dicari.</t>
+          <t>Berhasil memfilter dan menampilkan daftar data kunjungan sesuai rentang periode tanggal yang dipilih.</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>20.3</t>
+          <t>19.3</t>
         </is>
       </c>
       <c r="B228" s="46" t="inlineStr">
         <is>
-          <t>Notifikasi</t>
+          <t>Kunjungan</t>
         </is>
       </c>
       <c r="C228" s="46" t="n"/>
       <c r="D228" s="48" t="inlineStr">
         <is>
-          <t>Mencari notifikasi dengan kata kunci tidak valid</t>
+          <t>Melihat detail kunjungan</t>
         </is>
       </c>
       <c r="E228" s="46" t="inlineStr">
         <is>
-          <t>Negative Case</t>
+          <t>Positive Case</t>
         </is>
       </c>
       <c r="F228" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G228" s="48" t="inlineStr">
         <is>
-          <t>Masukkan kata kunci tidak valid pada Search Bar</t>
+          <t>Klik salah satu card kunjungan pada daftar - Sistem menampilkan tab default Mulai Kunjungan - Klik tab Selesai Kunjungan</t>
         </is>
       </c>
       <c r="H228" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
+          <t>Berhasil menampilkan halaman Detail Kunjungan yang memuat peta lokasi, waktu, tipe kunjungan, dan nama nasabah pada tab Mulai Kunjungan maupun Selesai Kunjungan.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>20.4</t>
+          <t>20.1</t>
         </is>
       </c>
       <c r="B229" s="46" t="inlineStr">
@@ -55267,7 +55281,7 @@
       <c r="C229" s="46" t="n"/>
       <c r="D229" s="48" t="inlineStr">
         <is>
-          <t>Melihat data notifikasi Belum Dibaca</t>
+          <t>Membuka halaman Notifikasi</t>
         </is>
       </c>
       <c r="E229" s="46" t="inlineStr">
@@ -55277,24 +55291,24 @@
       </c>
       <c r="F229" s="46" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G229" s="48" t="inlineStr">
         <is>
-          <t>Pada halaman Notifikasi, klik tab Belum Dibaca</t>
+          <t>Buka aplikasi BTN Smart - Masuk ke Beranda - Klik icon Lonceng (Notifikasi)</t>
         </is>
       </c>
       <c r="H229" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data notifikasi belum dibaca.</t>
+          <t>Berhasil menampilkan halaman Notifikasi.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>20.2</t>
         </is>
       </c>
       <c r="B230" s="46" t="inlineStr">
@@ -55305,7 +55319,7 @@
       <c r="C230" s="46" t="n"/>
       <c r="D230" s="48" t="inlineStr">
         <is>
-          <t>Melihat data notifikasi Diarsipkan</t>
+          <t>Mencari notifikasi dengan kata kunci valid</t>
         </is>
       </c>
       <c r="E230" s="46" t="inlineStr">
@@ -55320,19 +55334,19 @@
       </c>
       <c r="G230" s="48" t="inlineStr">
         <is>
-          <t>Pada halaman Notifikasi, klik tab Diarsipkan</t>
+          <t>Masukkan kata kunci valid pada Search Bar</t>
         </is>
       </c>
       <c r="H230" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data notifikasi diarsipkan.</t>
+          <t>Berhasil menampilkan data notifikasi yang dicari.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>20.6</t>
+          <t>20.3</t>
         </is>
       </c>
       <c r="B231" s="46" t="inlineStr">
@@ -55343,34 +55357,34 @@
       <c r="C231" s="46" t="n"/>
       <c r="D231" s="48" t="inlineStr">
         <is>
-          <t>Melihat detail notifikasi</t>
+          <t>Mencari notifikasi dengan kata kunci tidak valid</t>
         </is>
       </c>
       <c r="E231" s="46" t="inlineStr">
         <is>
-          <t>Positive Case</t>
+          <t>Negative Case</t>
         </is>
       </c>
       <c r="F231" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G231" s="48" t="inlineStr">
         <is>
-          <t>Pada halaman Notifikasi, klik salah satu notifikasi</t>
+          <t>Masukkan kata kunci tidak valid pada Search Bar</t>
         </is>
       </c>
       <c r="H231" s="48" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan detail notifikasi.</t>
+          <t>Berhasil menampilkan informasi data tidak ditemukan.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="B232" s="46" t="inlineStr">
@@ -55381,7 +55395,7 @@
       <c r="C232" s="46" t="n"/>
       <c r="D232" s="48" t="inlineStr">
         <is>
-          <t>Mengarsipkan notifikasi</t>
+          <t>Melihat data notifikasi Belum Dibaca</t>
         </is>
       </c>
       <c r="E232" s="46" t="inlineStr">
@@ -55391,24 +55405,24 @@
       </c>
       <c r="F232" s="46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="G232" s="48" t="inlineStr">
         <is>
-          <t>Pada halaman Detail Notifikasi, klik icon Arsipkan</t>
+          <t>Pada halaman Notifikasi, klik tab Belum Dibaca</t>
         </is>
       </c>
       <c r="H232" s="48" t="inlineStr">
         <is>
-          <t>Berhasil mengarsipkan notifikasi.</t>
+          <t>Berhasil menampilkan data notifikasi belum dibaca.</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>20.5</t>
         </is>
       </c>
       <c r="B233" s="46" t="inlineStr">
@@ -55419,25 +55433,139 @@
       <c r="C233" s="46" t="n"/>
       <c r="D233" s="48" t="inlineStr">
         <is>
+          <t>Melihat data notifikasi Diarsipkan</t>
+        </is>
+      </c>
+      <c r="E233" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F233" s="46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G233" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Notifikasi, klik tab Diarsipkan</t>
+        </is>
+      </c>
+      <c r="H233" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan data notifikasi diarsipkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20.6</t>
+        </is>
+      </c>
+      <c r="B234" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C234" s="46" t="n"/>
+      <c r="D234" s="48" t="inlineStr">
+        <is>
+          <t>Melihat detail notifikasi</t>
+        </is>
+      </c>
+      <c r="E234" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F234" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G234" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Notifikasi, klik salah satu notifikasi</t>
+        </is>
+      </c>
+      <c r="H234" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil menampilkan detail notifikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>20.7</t>
+        </is>
+      </c>
+      <c r="B235" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C235" s="46" t="n"/>
+      <c r="D235" s="48" t="inlineStr">
+        <is>
+          <t>Mengarsipkan notifikasi</t>
+        </is>
+      </c>
+      <c r="E235" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F235" s="46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G235" s="48" t="inlineStr">
+        <is>
+          <t>Pada halaman Detail Notifikasi, klik icon Arsipkan</t>
+        </is>
+      </c>
+      <c r="H235" s="48" t="inlineStr">
+        <is>
+          <t>Berhasil mengarsipkan notifikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="B236" s="46" t="inlineStr">
+        <is>
+          <t>Notifikasi</t>
+        </is>
+      </c>
+      <c r="C236" s="46" t="n"/>
+      <c r="D236" s="48" t="inlineStr">
+        <is>
           <t>Membatalkan arsip notifikasi</t>
         </is>
       </c>
-      <c r="E233" s="46" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="F233" s="46" t="inlineStr">
+      <c r="E236" s="46" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="F236" s="46" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G233" s="48" t="inlineStr">
+      <c r="G236" s="48" t="inlineStr">
         <is>
           <t>Pada detail notifikasi di tab Diarsipkan, klik icon Buka Arsip</t>
         </is>
       </c>
-      <c r="H233" s="48" t="inlineStr">
+      <c r="H236" s="48" t="inlineStr">
         <is>
           <t>Berhasil membatalkan arsip notifikasi.</t>
         </is>

</xml_diff>

<commit_message>
feat(sit): fix formatting, move heading 79, center TC numbers, and sync Excel numbering
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -23574,7 +23574,7 @@
     <row r="555" ht="28" customHeight="1">
       <c r="A555" t="inlineStr">
         <is>
-          <t>50.10</t>
+          <t>50.1</t>
         </is>
       </c>
       <c r="B555" t="inlineStr">
@@ -23616,7 +23616,7 @@
     <row r="556" ht="28" customHeight="1">
       <c r="A556" t="inlineStr">
         <is>
-          <t>50.1</t>
+          <t>50.2</t>
         </is>
       </c>
       <c r="B556" t="inlineStr">
@@ -23658,7 +23658,7 @@
     <row r="557" ht="28" customHeight="1">
       <c r="A557" t="inlineStr">
         <is>
-          <t>50.2</t>
+          <t>50.3</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
@@ -23700,7 +23700,7 @@
     <row r="558" ht="28" customHeight="1">
       <c r="A558" t="inlineStr">
         <is>
-          <t>50.3</t>
+          <t>50.4</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
@@ -23742,7 +23742,7 @@
     <row r="559" ht="28" customHeight="1">
       <c r="A559" t="inlineStr">
         <is>
-          <t>50.4</t>
+          <t>50.5</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
@@ -23784,7 +23784,7 @@
     <row r="560" ht="28" customHeight="1">
       <c r="A560" t="inlineStr">
         <is>
-          <t>50.5</t>
+          <t>50.6</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
@@ -23826,7 +23826,7 @@
     <row r="561" ht="14" customHeight="1">
       <c r="A561" t="inlineStr">
         <is>
-          <t>50.6</t>
+          <t>50.7</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
@@ -23868,7 +23868,7 @@
     <row r="562" ht="14" customHeight="1">
       <c r="A562" t="inlineStr">
         <is>
-          <t>50.7</t>
+          <t>50.8</t>
         </is>
       </c>
       <c r="B562" t="inlineStr">
@@ -23910,7 +23910,7 @@
     <row r="563" ht="14" customHeight="1">
       <c r="A563" t="inlineStr">
         <is>
-          <t>50.8</t>
+          <t>50.9</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
@@ -23952,7 +23952,7 @@
     <row r="564" ht="14" customHeight="1">
       <c r="A564" t="inlineStr">
         <is>
-          <t>50.9</t>
+          <t>50.10</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
@@ -23994,7 +23994,7 @@
     <row r="565" ht="42" customHeight="1">
       <c r="A565" t="inlineStr">
         <is>
-          <t>50.10</t>
+          <t>50.11</t>
         </is>
       </c>
       <c r="B565" t="inlineStr">
@@ -24036,7 +24036,7 @@
     <row r="566" ht="42" customHeight="1">
       <c r="A566" t="inlineStr">
         <is>
-          <t>50.11</t>
+          <t>50.12</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
@@ -24078,7 +24078,7 @@
     <row r="567" ht="42" customHeight="1">
       <c r="A567" t="inlineStr">
         <is>
-          <t>50.12</t>
+          <t>50.13</t>
         </is>
       </c>
       <c r="B567" t="inlineStr">
@@ -24120,7 +24120,7 @@
     <row r="568" ht="42" customHeight="1">
       <c r="A568" t="inlineStr">
         <is>
-          <t>50.13</t>
+          <t>50.14</t>
         </is>
       </c>
       <c r="B568" t="inlineStr">
@@ -24162,7 +24162,7 @@
     <row r="569" ht="28" customHeight="1">
       <c r="A569" t="inlineStr">
         <is>
-          <t>50.14</t>
+          <t>50.15</t>
         </is>
       </c>
       <c r="B569" t="inlineStr">
@@ -24204,7 +24204,7 @@
     <row r="570" ht="28" customHeight="1">
       <c r="A570" t="inlineStr">
         <is>
-          <t>50.15</t>
+          <t>50.16</t>
         </is>
       </c>
       <c r="B570" t="inlineStr">
@@ -24246,7 +24246,7 @@
     <row r="571" ht="28" customHeight="1">
       <c r="A571" t="inlineStr">
         <is>
-          <t>50.16</t>
+          <t>50.17</t>
         </is>
       </c>
       <c r="B571" t="inlineStr">
@@ -24288,7 +24288,7 @@
     <row r="572" ht="28" customHeight="1">
       <c r="A572" t="inlineStr">
         <is>
-          <t>50.17</t>
+          <t>50.18</t>
         </is>
       </c>
       <c r="B572" t="inlineStr">
@@ -24330,7 +24330,7 @@
     <row r="573" ht="28" customHeight="1">
       <c r="A573" t="inlineStr">
         <is>
-          <t>50.18</t>
+          <t>50.19</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
@@ -24372,7 +24372,7 @@
     <row r="574" ht="42" customHeight="1">
       <c r="A574" t="inlineStr">
         <is>
-          <t>50.19</t>
+          <t>50.20</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
@@ -24414,7 +24414,7 @@
     <row r="575" ht="42" customHeight="1">
       <c r="A575" t="inlineStr">
         <is>
-          <t>50.20</t>
+          <t>50.21</t>
         </is>
       </c>
       <c r="B575" t="inlineStr">
@@ -24456,7 +24456,7 @@
     <row r="576" ht="28" customHeight="1">
       <c r="A576" t="inlineStr">
         <is>
-          <t>50.21</t>
+          <t>50.22</t>
         </is>
       </c>
       <c r="B576" t="inlineStr">
@@ -24498,7 +24498,7 @@
     <row r="577" ht="14" customHeight="1">
       <c r="A577" t="inlineStr">
         <is>
-          <t>50.22</t>
+          <t>50.23</t>
         </is>
       </c>
       <c r="B577" t="inlineStr">
@@ -24540,7 +24540,7 @@
     <row r="578" ht="42" customHeight="1">
       <c r="A578" t="inlineStr">
         <is>
-          <t>50.23</t>
+          <t>50.24</t>
         </is>
       </c>
       <c r="B578" t="inlineStr">
@@ -24582,7 +24582,7 @@
     <row r="579" ht="42" customHeight="1">
       <c r="A579" t="inlineStr">
         <is>
-          <t>50.24</t>
+          <t>50.25</t>
         </is>
       </c>
       <c r="B579" t="inlineStr">
@@ -24624,7 +24624,7 @@
     <row r="580" ht="28" customHeight="1">
       <c r="A580" t="inlineStr">
         <is>
-          <t>50.25</t>
+          <t>50.26</t>
         </is>
       </c>
       <c r="B580" t="inlineStr">
@@ -24666,7 +24666,7 @@
     <row r="581" ht="28" customHeight="1">
       <c r="A581" t="inlineStr">
         <is>
-          <t>50.26</t>
+          <t>50.27</t>
         </is>
       </c>
       <c r="B581" t="inlineStr">
@@ -24708,7 +24708,7 @@
     <row r="582" ht="28" customHeight="1">
       <c r="A582" t="inlineStr">
         <is>
-          <t>50.27</t>
+          <t>50.28</t>
         </is>
       </c>
       <c r="B582" t="inlineStr">
@@ -24750,7 +24750,7 @@
     <row r="583" ht="70" customHeight="1">
       <c r="A583" t="inlineStr">
         <is>
-          <t>50.28</t>
+          <t>50.29</t>
         </is>
       </c>
       <c r="B583" t="inlineStr">
@@ -24792,7 +24792,7 @@
     <row r="584" ht="28" customHeight="1">
       <c r="A584" t="inlineStr">
         <is>
-          <t>50.29</t>
+          <t>50.30</t>
         </is>
       </c>
       <c r="B584" t="inlineStr">
@@ -24834,7 +24834,7 @@
     <row r="585" ht="28" customHeight="1">
       <c r="A585" t="inlineStr">
         <is>
-          <t>50.30</t>
+          <t>50.31</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
@@ -24876,7 +24876,7 @@
     <row r="586" ht="70" customHeight="1">
       <c r="A586" t="inlineStr">
         <is>
-          <t>50.31</t>
+          <t>50.32</t>
         </is>
       </c>
       <c r="B586" t="inlineStr">
@@ -24918,7 +24918,7 @@
     <row r="587" ht="28" customHeight="1">
       <c r="A587" t="inlineStr">
         <is>
-          <t>50.32</t>
+          <t>50.33</t>
         </is>
       </c>
       <c r="B587" t="inlineStr">
@@ -27018,7 +27018,7 @@
     <row r="637" ht="28" customHeight="1">
       <c r="A637" t="inlineStr">
         <is>
-          <t>55.3</t>
+          <t>55.4</t>
         </is>
       </c>
       <c r="B637" t="inlineStr">
@@ -27060,7 +27060,7 @@
     <row r="638" ht="14" customHeight="1">
       <c r="A638" t="inlineStr">
         <is>
-          <t>55.4</t>
+          <t>55.5</t>
         </is>
       </c>
       <c r="B638" t="inlineStr">
@@ -27102,7 +27102,7 @@
     <row r="639" ht="28" customHeight="1">
       <c r="A639" t="inlineStr">
         <is>
-          <t>55.5</t>
+          <t>55.6</t>
         </is>
       </c>
       <c r="B639" t="inlineStr">
@@ -27144,7 +27144,7 @@
     <row r="640" ht="28" customHeight="1">
       <c r="A640" t="inlineStr">
         <is>
-          <t>55.6</t>
+          <t>55.7</t>
         </is>
       </c>
       <c r="B640" t="inlineStr">
@@ -27186,7 +27186,7 @@
     <row r="641" ht="28" customHeight="1">
       <c r="A641" t="inlineStr">
         <is>
-          <t>55.7</t>
+          <t>55.8</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
@@ -27228,7 +27228,7 @@
     <row r="642" ht="28" customHeight="1">
       <c r="A642" t="inlineStr">
         <is>
-          <t>55.8</t>
+          <t>55.9</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
@@ -27270,7 +27270,7 @@
     <row r="643" ht="42" customHeight="1">
       <c r="A643" t="inlineStr">
         <is>
-          <t>55.9</t>
+          <t>55.10</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
@@ -27312,7 +27312,7 @@
     <row r="644" ht="28" customHeight="1">
       <c r="A644" t="inlineStr">
         <is>
-          <t>55.10</t>
+          <t>55.11</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">

</xml_diff>

<commit_message>
fix(web): Part 2 - harmonisasi 16 pasang TC Funnel, Referal, dan Approval Target Growth (73/79 modul 100% match)
</commit_message>
<xml_diff>
--- a/SIT/Test Case.xlsx
+++ b/SIT/Test Case.xlsx
@@ -13596,7 +13596,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Melihat data tab Prospek yang direferalkan ke saya</t>
+          <t>Melihat detail tab Prospek yang saya referalkan</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -13611,12 +13611,12 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>Klik tab Prospek yang direferalkan ke saya</t>
+          <t>Klik icon aksi detail pada salah satu baris tab Prospek yang saya referalkan</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pada tab Prospek yang direferalkan ke saya.</t>
+          <t>Berhasil menampilkan detail prospek.</t>
         </is>
       </c>
     </row>
@@ -13638,7 +13638,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Mencari data tab Prospek yang direferalkan ke saya dengan keyword valid</t>
+          <t>Melihat data tab Prospek yang direferalkan ke saya</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -13653,12 +13653,12 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>Mengisi field Search dengan keyword valid - Klik button Search</t>
+          <t>Klik tab Prospek yang direferalkan ke saya</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data yang dicari.</t>
+          <t>Berhasil menampilkan data pada tab Prospek yang direferalkan ke saya.</t>
         </is>
       </c>
     </row>
@@ -13680,7 +13680,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Mencari data tab Prospek yang direferalkan ke saya dengan keyword tidak valid</t>
+          <t>Mencari data tab Prospek yang direferalkan ke saya dengan keyword valid</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -13695,12 +13695,12 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>Mengisi field Search dengan keyword tidak valid - Klik button Search</t>
+          <t>Mengisi field Search dengan keyword valid - Klik button Search</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Menampilkan pesan data tidak ditemukan.</t>
+          <t>Berhasil menampilkan data yang dicari.</t>
         </is>
       </c>
     </row>
@@ -21321,7 +21321,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Membuka menu approval cif kelolaan</t>
+          <t>Melihat detail</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
@@ -21336,12 +21336,12 @@
       </c>
       <c r="G501" t="inlineStr">
         <is>
-          <t>Klik menu sales force - klik menu approval - Klik submenu Appoval cif kelolaan</t>
+          <t>Klik icon mata pada salah satu data Target Growth</t>
         </is>
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>Menampilkan halaman approval cif kelolaan</t>
+          <t>Menampilkan detail data Approval Target Growth.</t>
         </is>
       </c>
     </row>
@@ -21363,14 +21363,14 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
+          <t>Melakukan approval data</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
           <t>Melakukan filter data</t>
         </is>
       </c>
-      <c r="E502" t="inlineStr">
-        <is>
-          <t>Melakukan filter data</t>
-        </is>
-      </c>
       <c r="F502" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21378,12 +21378,12 @@
       </c>
       <c r="G502" t="inlineStr">
         <is>
-          <t>Pilih bulan tahun dan tipe – kemudia klik button filter</t>
+          <t>Klik icon ceklis pada table dengan status data pending request - input remark - klik button submit</t>
         </is>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai dengan filter yang dipilih</t>
+          <t>Berhasil melakukan approval data Target Growth.</t>
         </is>
       </c>
     </row>
@@ -21405,14 +21405,14 @@
       </c>
       <c r="D503" t="inlineStr">
         <is>
+          <t>Melakukan reject data</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
           <t>Melakukan approval data</t>
         </is>
       </c>
-      <c r="E503" t="inlineStr">
-        <is>
-          <t>Melakukan approval data</t>
-        </is>
-      </c>
       <c r="F503" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21420,12 +21420,12 @@
       </c>
       <c r="G503" t="inlineStr">
         <is>
-          <t>Klik icon ceklis pada table dengan status data pending request - input remark - klik button submit</t>
+          <t>Klik icon silang pada table dengan status data pending request - input remark - Klik button submit</t>
         </is>
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>Berhasil melakukan approval data CIF Kelolaan</t>
+          <t>Berhasil melakukan reject data Target Growth.</t>
         </is>
       </c>
     </row>
@@ -21447,14 +21447,14 @@
       </c>
       <c r="D504" t="inlineStr">
         <is>
+          <t>Membuka tab status ( pending request/approved/Rejected/expired)</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
           <t>Melakukan reject data</t>
         </is>
       </c>
-      <c r="E504" t="inlineStr">
-        <is>
-          <t>Melakukan reject data</t>
-        </is>
-      </c>
       <c r="F504" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21462,12 +21462,12 @@
       </c>
       <c r="G504" t="inlineStr">
         <is>
-          <t>Klik icon silang pada table dengan status data pending request - input remark - KLik button submit</t>
+          <t>Klik tab status ( pending request/approved/Rejected/ expired)</t>
         </is>
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>Berhasil melakukan reject data CIF Kelolaan</t>
+          <t>Menampilkan list data sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -21489,14 +21489,14 @@
       </c>
       <c r="D505" t="inlineStr">
         <is>
+          <t>Melihat detail data</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
           <t>Membuka tab status ( pending request/approved/Rejected/expired)</t>
         </is>
       </c>
-      <c r="E505" t="inlineStr">
-        <is>
-          <t>Membuka tab status ( pending request/approved/Rejected/expired)</t>
-        </is>
-      </c>
       <c r="F505" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21504,12 +21504,12 @@
       </c>
       <c r="G505" t="inlineStr">
         <is>
-          <t>Klik tab status ( pending request/approved/Rejected/ expired)</t>
+          <t>Klik icon mata pada salah satu data Target Growth</t>
         </is>
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>Menampilkan list data sesuai status yang dipilih</t>
+          <t>Menampilkan detail data.</t>
         </is>
       </c>
     </row>
@@ -21531,14 +21531,14 @@
       </c>
       <c r="D506" t="inlineStr">
         <is>
+          <t>Melakukan approval data</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
           <t>Melihat detail data</t>
         </is>
       </c>
-      <c r="E506" t="inlineStr">
-        <is>
-          <t>Melihat detail data</t>
-        </is>
-      </c>
       <c r="F506" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21546,12 +21546,12 @@
       </c>
       <c r="G506" t="inlineStr">
         <is>
-          <t>Klik icon mata</t>
+          <t>Klik icon ceklis pada table dengan status data pending request - input remark - klik button submit</t>
         </is>
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>Menampilkan detail data</t>
+          <t>Berhasil melakukan approval data Target Growth.</t>
         </is>
       </c>
     </row>
@@ -21573,14 +21573,14 @@
       </c>
       <c r="D507" t="inlineStr">
         <is>
+          <t>Melakukan reject data</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
           <t>Mencari data pada kolom pencarian</t>
         </is>
       </c>
-      <c r="E507" t="inlineStr">
-        <is>
-          <t>Mencari data pada kolom pencarian</t>
-        </is>
-      </c>
       <c r="F507" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -21588,12 +21588,12 @@
       </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>Input data pada kolom pencarian</t>
+          <t>Klik icon silang pada table dengan status data pending request - input remark - Klik button submit</t>
         </is>
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>Menampilkan data sesuai kata kunci yang diinput</t>
+          <t>Berhasil melakukan reject data Target Growth.</t>
         </is>
       </c>
     </row>
@@ -21615,7 +21615,7 @@
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>Mencari data kata kunci yang tidak sesuai</t>
+          <t>Membuka tab status ( pending request/approved/Rejected/expired)</t>
         </is>
       </c>
       <c r="E508" t="inlineStr">
@@ -21630,12 +21630,12 @@
       </c>
       <c r="G508" t="inlineStr">
         <is>
-          <t>Input data yang belun terdaftar</t>
+          <t>Klik tab status ( pending request/approved/Rejected/ expired)</t>
         </is>
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>Data tidak ditemukan</t>
+          <t>Menampilkan list data sesuai status yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -29369,7 +29369,7 @@
       </c>
       <c r="D695" t="inlineStr">
         <is>
-          <t>Menampilkan data Rekap Funnel</t>
+          <t>Melakukan filter data Rekap Funnel</t>
         </is>
       </c>
       <c r="E695" t="inlineStr">
@@ -29384,12 +29384,12 @@
       </c>
       <c r="G695" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory (Kantor Wilayah, Unit Bisnis, Produk, Info Bulan, Info Tahun) - Klik button Filter Data</t>
+          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H695" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan daftar data Rekap Funnel di dalam tabel.</t>
+          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -29411,7 +29411,7 @@
       </c>
       <c r="D696" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel</t>
+          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E696" t="inlineStr">
@@ -29426,12 +29426,12 @@
       </c>
       <c r="G696" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
+          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H696" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
@@ -29453,7 +29453,7 @@
       </c>
       <c r="D697" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
+          <t>Mereset filter data Rekap Funnel</t>
         </is>
       </c>
       <c r="E697" t="inlineStr">
@@ -29468,12 +29468,12 @@
       </c>
       <c r="G697" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
+          <t>Klik button Reset Filter</t>
         </is>
       </c>
       <c r="H697" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil mengosongkan kriteria filter dan mengembalikan kondisi filter ke default.</t>
         </is>
       </c>
     </row>
@@ -29495,7 +29495,7 @@
       </c>
       <c r="D698" t="inlineStr">
         <is>
-          <t>Mengunduh data Rekap Funnel</t>
+          <t>Mengekspor data Rekap Funnel</t>
         </is>
       </c>
       <c r="E698" t="inlineStr">
@@ -29579,7 +29579,7 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>Menampilkan data Pengaturan Funnel Funding berdasarkan section</t>
+          <t>Mengubah data Pengaturan Funnel Funding</t>
         </is>
       </c>
       <c r="E700" t="inlineStr">
@@ -29594,12 +29594,12 @@
       </c>
       <c r="G700" t="inlineStr">
         <is>
-          <t>Klik salah satu daftar section pada tabel</t>
+          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
         </is>
       </c>
       <c r="H700" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pengaturan funnel Funding.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -29621,7 +29621,7 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Funding</t>
+          <t>Mengubah data Pengaturan Funnel Funding tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E701" t="inlineStr">
@@ -29636,12 +29636,12 @@
       </c>
       <c r="G701" t="inlineStr">
         <is>
-          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
+          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
         </is>
       </c>
       <c r="H701" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
@@ -29663,7 +29663,7 @@
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Funding tanpa mengisi field mandatory</t>
+          <t>Menambahkan Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E702" t="inlineStr">
@@ -29678,12 +29678,12 @@
       </c>
       <c r="G702" t="inlineStr">
         <is>
-          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
         </is>
       </c>
     </row>
@@ -29705,7 +29705,7 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Menghapus Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E703" t="inlineStr">
@@ -29720,12 +29720,12 @@
       </c>
       <c r="G703" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
         </is>
       </c>
       <c r="H703" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -29747,7 +29747,7 @@
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
+          <t>Menambahkan Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E704" t="inlineStr">
@@ -29762,12 +29762,12 @@
       </c>
       <c r="G704" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik button Add Operator pada condition yang dipilih - Memilih operator - Klik button Submit</t>
         </is>
       </c>
       <c r="H704" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Funding.</t>
         </is>
       </c>
     </row>
@@ -29789,7 +29789,7 @@
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Menghapus Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E705" t="inlineStr">
@@ -29804,7 +29804,7 @@
       </c>
       <c r="G705" t="inlineStr">
         <is>
-          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
+          <t>Klik button Remove pada salah satu operator di condition - Klik button Submit</t>
         </is>
       </c>
       <c r="H705" t="inlineStr">
@@ -30839,7 +30839,7 @@
       </c>
       <c r="D730" t="inlineStr">
         <is>
-          <t>Melakukan filter data Personal Funnel</t>
+          <t>Menampilkan data Personal Funnel berdasarkan tab</t>
         </is>
       </c>
       <c r="E730" t="inlineStr">
@@ -30854,12 +30854,12 @@
       </c>
       <c r="G730" t="inlineStr">
         <is>
-          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
+          <t>Klik salah satu daftar tab (Semua, Non PKS, PKS) pada halaman Personal Funnel</t>
         </is>
       </c>
       <c r="H730" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
+          <t>Berhasil menampilkan data Personal Funnel pada tab Semua, Non PKS, dan PKS.</t>
         </is>
       </c>
     </row>
@@ -30881,7 +30881,7 @@
       </c>
       <c r="D731" t="inlineStr">
         <is>
-          <t>Melakukan filter data Personal Funnel tanpa mengisi field mandatory</t>
+          <t>Melakukan filter data Personal Funnel</t>
         </is>
       </c>
       <c r="E731" t="inlineStr">
@@ -30896,12 +30896,12 @@
       </c>
       <c r="G731" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
+          <t>Mengisi semua field filter mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H731" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil menampilkan data sesuai dengan filter yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -30923,7 +30923,7 @@
       </c>
       <c r="D732" t="inlineStr">
         <is>
-          <t>Mengekspor data Personal Funnel</t>
+          <t>Melakukan filter data Personal Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E732" t="inlineStr">
@@ -30938,12 +30938,12 @@
       </c>
       <c r="G732" t="inlineStr">
         <is>
-          <t>Klik button Export - Klik icon download pada panel Download Export</t>
+          <t>Mengosongkan field filter mandatory - Klik button Submit</t>
         </is>
       </c>
       <c r="H732" t="inlineStr">
         <is>
-          <t>Berhasil mendownload file export.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
@@ -31007,7 +31007,7 @@
       </c>
       <c r="D734" t="inlineStr">
         <is>
-          <t>Menampilkan data Rekap Funnel</t>
+          <t>Melakukan filter data Rekap Funnel</t>
         </is>
       </c>
       <c r="E734" t="inlineStr">
@@ -31022,12 +31022,12 @@
       </c>
       <c r="G734" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory (Kantor Wilayah, Unit Bisnis, Produk, Info Bulan, Info Tahun) - Klik button Filter Data</t>
+          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H734" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan daftar data Rekap Funnel di dalam tabel.</t>
+          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
         </is>
       </c>
     </row>
@@ -31049,7 +31049,7 @@
       </c>
       <c r="D735" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel</t>
+          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E735" t="inlineStr">
@@ -31064,12 +31064,12 @@
       </c>
       <c r="G735" t="inlineStr">
         <is>
-          <t>Mengisi field filter mandatory beserta kriteria filter spesifik (seperti Kantor Cabang/Role) - Klik button Filter Data</t>
+          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
         </is>
       </c>
       <c r="H735" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data Rekap Funnel yang sesuai dengan kriteria filter yang dipilih.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
         </is>
       </c>
     </row>
@@ -31091,7 +31091,7 @@
       </c>
       <c r="D736" t="inlineStr">
         <is>
-          <t>Melakukan filter data Rekap Funnel tanpa mengisi field mandatory</t>
+          <t>Mereset filter data Rekap Funnel</t>
         </is>
       </c>
       <c r="E736" t="inlineStr">
@@ -31106,12 +31106,12 @@
       </c>
       <c r="G736" t="inlineStr">
         <is>
-          <t>Mengosongkan field filter mandatory - Klik button Filter Data</t>
+          <t>Klik button Reset Filter</t>
         </is>
       </c>
       <c r="H736" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field filter mandatory wajib diisi.</t>
+          <t>Berhasil mengosongkan kriteria filter dan mengembalikan kondisi filter ke default.</t>
         </is>
       </c>
     </row>
@@ -31133,7 +31133,7 @@
       </c>
       <c r="D737" t="inlineStr">
         <is>
-          <t>Mengunduh data Rekap Funnel</t>
+          <t>Mengekspor data Rekap Funnel</t>
         </is>
       </c>
       <c r="E737" t="inlineStr">
@@ -31217,7 +31217,7 @@
       </c>
       <c r="D739" t="inlineStr">
         <is>
-          <t>Menampilkan data Pengaturan Funnel Lending berdasarkan section</t>
+          <t>Mengubah data Pengaturan Funnel Lending</t>
         </is>
       </c>
       <c r="E739" t="inlineStr">
@@ -31232,12 +31232,12 @@
       </c>
       <c r="G739" t="inlineStr">
         <is>
-          <t>Klik salah satu daftar section pada tabel</t>
+          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
         </is>
       </c>
       <c r="H739" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan data pengaturan funnel Lending.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -31259,7 +31259,7 @@
       </c>
       <c r="D740" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending</t>
+          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
         </is>
       </c>
       <c r="E740" t="inlineStr">
@@ -31274,12 +31274,12 @@
       </c>
       <c r="G740" t="inlineStr">
         <is>
-          <t>Mengisi semua field mandatory Performance Percentage pada setiap tahapan funnel - Klik button Submit</t>
+          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
         </is>
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
+          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
         </is>
       </c>
     </row>
@@ -31301,7 +31301,7 @@
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>Mengubah data Pengaturan Funnel Lending tanpa mengisi field mandatory</t>
+          <t>Menambahkan Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
@@ -31316,12 +31316,12 @@
       </c>
       <c r="G741" t="inlineStr">
         <is>
-          <t>Mengosongkan field mandatory Performance Percentage - Klik button Submit</t>
+          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
         </is>
       </c>
       <c r="H741" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
         </is>
       </c>
     </row>
@@ -31343,7 +31343,7 @@
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator</t>
+          <t>Menghapus Kondisi pada Indikator Performa</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
@@ -31358,12 +31358,12 @@
       </c>
       <c r="G742" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengisi semua field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
         </is>
       </c>
       <c r="H742" t="inlineStr">
         <is>
-          <t>Berhasil menyimpan condition baru pada Performance Indicator.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -31385,7 +31385,7 @@
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>Menambahkan Condition pada Performance Indicator tanpa mengisi field mandatory</t>
+          <t>Menambahkan Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E743" t="inlineStr">
@@ -31400,12 +31400,12 @@
       </c>
       <c r="G743" t="inlineStr">
         <is>
-          <t>Klik button Add Condition pada bagian Performance Indicator - Mengosongkan field mandatory pada condition baru - Klik button Submit</t>
+          <t>Klik button Add Operator pada condition yang dipilih - Memilih operator - Klik button Submit</t>
         </is>
       </c>
       <c r="H743" t="inlineStr">
         <is>
-          <t>Berhasil menampilkan pesan validasi bahwa field mandatory harus diisi.</t>
+          <t>Berhasil menyimpan perubahan data Pengaturan Funnel Lending.</t>
         </is>
       </c>
     </row>
@@ -31427,7 +31427,7 @@
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>Menghapus Condition pada Performance Indicator</t>
+          <t>Menghapus Operator pada Kondisi</t>
         </is>
       </c>
       <c r="E744" t="inlineStr">
@@ -31442,7 +31442,7 @@
       </c>
       <c r="G744" t="inlineStr">
         <is>
-          <t>Klik button Remove pada salah satu condition di Performance Indicator - Klik button Submit</t>
+          <t>Klik button Remove pada salah satu operator di condition - Klik button Submit</t>
         </is>
       </c>
       <c r="H744" t="inlineStr">

</xml_diff>